<commit_message>
article fix + qa fix + storyboard
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1552" uniqueCount="894">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1552" uniqueCount="891">
   <si>
     <t>LEGEND</t>
   </si>
@@ -2635,24 +2635,18 @@
     <t>Title, excerpt, canonical managed image URL and Article HTML persist once; admin list requests medium and the admin viewer body requests large</t>
   </si>
   <si>
-    <t>IN PROGRESS</t>
-  </si>
-  <si>
-    <t>Backend admin idea/content HTTP coverage plus frontend Article list/viewer and managed-HTML variant unit coverage</t>
-  </si>
-  <si>
-    <t>Finish the open draft, save once, reopen and compare the persisted DTO plus Network URLs</t>
-  </si>
-  <si>
-    <t>Started from a new English Article editor after MEDIA-IMG-001 closure. Do not classify upload as a separate producer; the Article Save owns title, excerpt, HTML and image persistence.</t>
+    <t>Backend admin idea/content HTTP coverage plus frontend Article list/viewer, managed-HTML variant, paste and focused Article service coverage</t>
+  </si>
+  <si>
+    <t>Proceed to LANDING-ARTICLE-001 with the retained draft; keep publication outside this checkpoint</t>
+  </si>
+  <si>
+    <t>ARTICLE-SRC-002 saved and reopened with title, excerpt, body and one canonical large.webp URL in Mongo imageUrl/imageUrls plus HTML. The list requested medium.webp; the viewer requested large.webp 200 and rendered without a broken link. Source 1229x706; variants 128x74, 640x368 and 1229x706, all HTTP 200. Delete-without-replacement removed the HTML reference and all four stored objects while preserving the body. Raw-HTML and URL copy-paste regressions were fixed and focused frontend 5/5 plus IdeaPostsService tests passed.</t>
   </si>
   <si>
     <t>LANDING-ARTICLE-001</t>
   </si>
   <si>
-    <t>Queued checkpoint</t>
-  </si>
-  <si>
     <t>Public landing / Articles</t>
   </si>
   <si>
@@ -2662,16 +2656,13 @@
     <t>A fresh landing load shows the published Article exactly once with the expected count, medium card image and large body image; refresh/live-update behavior is recorded explicitly</t>
   </si>
   <si>
-    <t>QUEUED</t>
-  </si>
-  <si>
     <t>Backend ContentMedia HTTP E2E proves published inclusion and deleted exclusion; frontend landing specs cover featured/regular lists and large body-image rendering</t>
   </si>
   <si>
-    <t>After ARTICLE-EDITOR-001, capture pre-publish landing state, publish once, then compare already-open and fresh landing views</t>
-  </si>
-  <si>
-    <t>No existing browser test proves the complete Admin publish to rendered landing transition; do not assume an already-open landing updates live.</t>
+    <t>Proceed to CHAT-AUTH-001; no Article republish or landing retest is required</t>
+  </si>
+  <si>
+    <t>Pre-publish landing content and full list both reported 5 and excluded ARTICLE-SRC-002. One publish kept All 7 and Featured 4 stable while Published changed 5-&gt;6 and Drafts 2-&gt;1. Fresh APIs reported total 6 and exactly one QA article. The already-open list stayed at 5 without live update; hard refresh showed 6 and the QA card once. Card medium.webp and detail large.webp both returned 200; landing detail rendered title, body and image without a broken link.</t>
   </si>
   <si>
     <t>QA-RESET-001</t>
@@ -7656,150 +7647,150 @@
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="13" t="s">
+      <c r="A95" s="12" t="s">
         <v>867</v>
       </c>
-      <c r="B95" s="13" t="s">
+      <c r="B95" s="12" t="s">
         <v>445</v>
       </c>
-      <c r="C95" s="13" t="s">
+      <c r="C95" s="12" t="s">
         <v>868</v>
       </c>
-      <c r="D95" s="13" t="s">
+      <c r="D95" s="12" t="s">
         <v>869</v>
       </c>
-      <c r="E95" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="F95" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="G95" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="H95" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="I95" s="13" t="s">
+      <c r="E95" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="F95" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="G95" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H95" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="I95" s="12" t="s">
         <v>870</v>
       </c>
-      <c r="J95" s="13" t="s">
+      <c r="J95" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="K95" s="12" t="s">
+        <v>863</v>
+      </c>
+      <c r="L95" s="12" t="s">
         <v>871</v>
       </c>
-      <c r="K95" s="13" t="s">
+      <c r="M95" s="12" t="s">
+        <v>872</v>
+      </c>
+      <c r="N95" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="O95" s="12" t="s">
+        <v>873</v>
+      </c>
+      <c r="P95" s="12" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="12" t="s">
+        <v>874</v>
+      </c>
+      <c r="B96" s="12" t="s">
+        <v>445</v>
+      </c>
+      <c r="C96" s="12" t="s">
+        <v>875</v>
+      </c>
+      <c r="D96" s="12" t="s">
+        <v>876</v>
+      </c>
+      <c r="E96" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="F96" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="G96" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H96" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="I96" s="12" t="s">
+        <v>877</v>
+      </c>
+      <c r="J96" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="K96" s="12" t="s">
         <v>863</v>
       </c>
-      <c r="L95" s="13" t="s">
-        <v>872</v>
-      </c>
-      <c r="M95" s="13" t="s">
-        <v>873</v>
-      </c>
-      <c r="N95" s="13" t="s">
-        <v>429</v>
-      </c>
-      <c r="O95" s="13" t="s">
-        <v>874</v>
-      </c>
-      <c r="P95" s="13" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="0" t="s">
-        <v>875</v>
-      </c>
-      <c r="B96" s="0" t="s">
-        <v>876</v>
-      </c>
-      <c r="C96" s="0" t="s">
-        <v>877</v>
-      </c>
-      <c r="D96" s="0" t="s">
+      <c r="L96" s="12" t="s">
         <v>878</v>
       </c>
-      <c r="E96" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="F96" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="G96" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="H96" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="I96" s="0" t="s">
+      <c r="M96" s="12" t="s">
         <v>879</v>
       </c>
-      <c r="J96" s="0" t="s">
+      <c r="N96" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="O96" s="12" t="s">
         <v>880</v>
       </c>
-      <c r="K96" s="0" t="s">
-        <v>1</v>
-      </c>
-      <c r="L96" s="0" t="s">
-        <v>881</v>
-      </c>
-      <c r="M96" s="0" t="s">
-        <v>882</v>
-      </c>
-      <c r="N96" s="0" t="s">
-        <v>1</v>
-      </c>
-      <c r="O96" s="0" t="s">
-        <v>883</v>
-      </c>
-      <c r="P96" s="0" t="s">
+      <c r="P96" s="12" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="13" t="s">
+        <v>881</v>
+      </c>
+      <c r="B97" s="13" t="s">
+        <v>882</v>
+      </c>
+      <c r="C97" s="13" t="s">
+        <v>883</v>
+      </c>
+      <c r="D97" s="13" t="s">
         <v>884</v>
       </c>
-      <c r="B97" s="13" t="s">
+      <c r="E97" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="F97" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="G97" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="H97" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="I97" s="13" t="s">
         <v>885</v>
       </c>
-      <c r="C97" s="13" t="s">
+      <c r="J97" s="13" t="s">
         <v>886</v>
-      </c>
-      <c r="D97" s="13" t="s">
-        <v>887</v>
-      </c>
-      <c r="E97" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="F97" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="G97" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="H97" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="I97" s="13" t="s">
-        <v>888</v>
-      </c>
-      <c r="J97" s="13" t="s">
-        <v>889</v>
       </c>
       <c r="K97" s="13" t="s">
         <v>47</v>
       </c>
       <c r="L97" s="13" t="s">
+        <v>887</v>
+      </c>
+      <c r="M97" s="13" t="s">
+        <v>888</v>
+      </c>
+      <c r="N97" s="13" t="s">
+        <v>889</v>
+      </c>
+      <c r="O97" s="13" t="s">
         <v>890</v>
-      </c>
-      <c r="M97" s="13" t="s">
-        <v>891</v>
-      </c>
-      <c r="N97" s="13" t="s">
-        <v>892</v>
-      </c>
-      <c r="O97" s="13" t="s">
-        <v>893</v>
       </c>
       <c r="P97" s="13" t="s">
         <v>241</v>

</xml_diff>

<commit_message>
qa + storyboard fix
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1552" uniqueCount="891">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1552" uniqueCount="890">
   <si>
     <t>LEGEND</t>
   </si>
@@ -277,13 +277,13 @@
     <t>STAT-011</t>
   </si>
   <si>
-    <t>Send one ordinary chat message</t>
-  </si>
-  <si>
-    <t>Messages timeline +1; Communication +1</t>
-  </si>
-  <si>
-    <t>Chat flow +1; outbox conditional</t>
+    <t>Send controlled ordinary chat messages</t>
+  </si>
+  <si>
+    <t>Messages timeline +1 per message; Communication +1 per message</t>
+  </si>
+  <si>
+    <t>Chat flow +1 per message; outbox conditional</t>
   </si>
   <si>
     <t>Notification outbox conditional</t>
@@ -295,13 +295,16 @@
     <t>MANUAL UI + FUNCTIONAL PASS</t>
   </si>
   <si>
-    <t>Chat/realtime E2E support</t>
-  </si>
-  <si>
-    <t>Continue with STAT-012; retain this unique-message oracle</t>
-  </si>
-  <si>
-    <t>Farkas Anna sent one unique ordinary message in Host Circle Ops. UI showed one bubble; API showed chat total 41-&gt;42 and exactly one matching non-system message. The real Statistics worker changed today's Messages 0-&gt;1, Communication/Messages 417-&gt;418 and Communication total 426-&gt;427. Browser screenshots at 06:53 confirmed Messages 1 and Messages 418; Ratings, Moderation and the pre-message Events value stayed stable.</t>
+    <t>2026-08-05</t>
+  </si>
+  <si>
+    <t>Chat/realtime E2E support; focused WebSocket handshake regression PASS</t>
+  </si>
+  <si>
+    <t>Closed; retain both historical one-message and current two-message causal samples, and repeat only after chat/statistics changes</t>
+  </si>
+  <si>
+    <t>Historical 2026-08-04 sample: one Farkas Anna message changed chat 41-&gt;42, today's Messages 0-&gt;1, Communication/Messages 417-&gt;418 and Communication 426-&gt;427. Current 2026-08-05 replay reused the two deliberate Riley messages from CHAT-AUTH-001 without another write: the real worker snapshot at 08:42 reported daily Messages 2, chat.message.sent 419 and Communication 428 (Messages 419 + Warnings 9). Admin Statistics screenshots from snapshot 08:43 independently showed Daily usage Message 2 and Segments Communication 428 / Messages 419 / Warnings 9. Other visible daily metrics were Activity 18, New 0, Ratings 0, Event/assets 1306 and Moderation 0; no unrelated delta was attributed to the chat operation.</t>
   </si>
   <si>
     <t>P1 66</t>
@@ -2005,31 +2008,28 @@
     <t>Compare Admin, accepted, pending and left membership against the same event chat</t>
   </si>
   <si>
-    <t>INDIRECT only for the one proof message</t>
-  </si>
-  <si>
-    <t>DELTA chat write only after accepted state</t>
-  </si>
-  <si>
-    <t>X unless the message creates documented delivery work</t>
+    <t>INDIRECT only for the controlled proof messages; causal Statistics replay is STAT-011</t>
+  </si>
+  <si>
+    <t>DELTA chat writes only after accepted state</t>
+  </si>
+  <si>
+    <t>X unless a message creates documented delivery work</t>
   </si>
   <si>
     <t>Admin and accepted member share history; pending/left users have no channel and are server-denied</t>
   </si>
   <si>
-    <t>MANUAL POSITIVE AUTHORIZATION FAIL; NEGATIVE CONTROL PASS</t>
-  </si>
-  <si>
-    <t>Chat/access-control coverage partial; regression required for event-chat materialization on terminal acceptance</t>
-  </si>
-  <si>
-    <t>After the backend fix, keep Casey Admin, Riley accepted and Nova pending isolated sessions open; prove Casey/Riley channel visibility, send one unique Riley message to Casey, and retain Nova absence plus direct denial</t>
-  </si>
-  <si>
-    <t>FAIL / PARTIAL PASS</t>
-  </si>
-  <si>
-    <t>After Riley reached terminal accepted membership, all three open Chats lists were empty. Nova pending correctly had no channel, but Riley accepted and Casey Admin also lacked the event channel, so the positive materialization/authorization branch failed before a proof message could be sent. This is a backend projection defect, not a UI fallback opportunity.</t>
+    <t>MANUAL UI + FUNCTIONAL PASS; WEBSOCKET DEFECT FIXED</t>
+  </si>
+  <si>
+    <t>Chat/access-control coverage plus focused ChatHandshakeInterceptorTest PASS</t>
+  </si>
+  <si>
+    <t>Proceed to retained-message Statistics checkpoint STAT-011; repeat authorization only after chat-id, membership or access-policy changes</t>
+  </si>
+  <si>
+    <t>Casey Admin and Riley accepted shared one mainEvent chat with only their two avatars; Nova stayed pending with an empty Chats UI and no chat-message notification. The first send exposed encoded %3A being used as the WebSocket database key; it persisted nothing. Query-param decoding was fixed, its focused test passed and hot deploy loaded. Riley then sent two deliberate messages: the second separately proved the Event bucket after the first was read. Each message persisted once and created one Casey-only notification/outbox row. Casey UI proved Chats/All/Event unread cycles 0-&gt;1-&gt;0, both messages in shared history and Notification Center 5-&gt;6; final unread was 0. Nova received neither message, retained no chat owner copy, and direct history access returned 404 Chat not found.</t>
   </si>
   <si>
     <t>EVENT-FEEDBACK-001</t>
@@ -2609,9 +2609,6 @@
   </si>
   <si>
     <t>MANUAL UI + ORACLE PASS; FIX VERIFIED</t>
-  </si>
-  <si>
-    <t>2026-08-05</t>
   </si>
   <si>
     <t>Backend response/strict distinct-rendition HTTP E2E plus frontend URL/carousel coverage; focused editor-slot regression 1 file 3/3</t>
@@ -3528,27 +3525,27 @@
         <v>90</v>
       </c>
       <c r="K12" s="12" t="s">
-        <v>47</v>
+        <v>91</v>
       </c>
       <c r="L12" s="12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="M12" s="12" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="N12" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O12" s="12" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="P12" s="12" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B13" s="12" t="s">
         <v>71</v>
@@ -3557,22 +3554,22 @@
         <v>30</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G13" s="12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H13" s="12" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I13" s="12" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="J13" s="12" t="s">
         <v>90</v>
@@ -3581,24 +3578,24 @@
         <v>47</v>
       </c>
       <c r="L13" s="12" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="M13" s="12" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="N13" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O13" s="12" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="P13" s="12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B14" s="15" t="s">
         <v>71</v>
@@ -3607,13 +3604,13 @@
         <v>30</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F14" s="15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G14" s="15" t="s">
         <v>6</v>
@@ -3622,7 +3619,7 @@
         <v>76</v>
       </c>
       <c r="I14" s="15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J14" s="15" t="s">
         <v>57</v>
@@ -3631,10 +3628,10 @@
         <v>1</v>
       </c>
       <c r="L14" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="M14" s="15" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="N14" s="15" t="s">
         <v>1</v>
@@ -3643,12 +3640,12 @@
         <v>1</v>
       </c>
       <c r="P14" s="15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B15" s="13" t="s">
         <v>71</v>
@@ -3657,13 +3654,13 @@
         <v>30</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G15" s="13" t="s">
         <v>6</v>
@@ -3672,83 +3669,83 @@
         <v>6</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J15" s="13" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K15" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L15" s="13" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="M15" s="13" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N15" s="13" t="s">
         <v>1</v>
       </c>
       <c r="O15" s="13" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="P15" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B16" s="13" t="s">
         <v>71</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H16" s="13" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I16" s="13" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J16" s="13" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="K16" s="13" t="s">
         <v>47</v>
       </c>
       <c r="L16" s="13" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="M16" s="13" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="N16" s="13" t="s">
         <v>81</v>
       </c>
       <c r="O16" s="13" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="P16" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="15" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B17" s="15" t="s">
         <v>71</v>
@@ -3757,22 +3754,22 @@
         <v>54</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G17" s="15" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H17" s="15" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I17" s="15" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="J17" s="15" t="s">
         <v>57</v>
@@ -3781,10 +3778,10 @@
         <v>1</v>
       </c>
       <c r="L17" s="15" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="M17" s="15" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="N17" s="15" t="s">
         <v>1</v>
@@ -3793,12 +3790,12 @@
         <v>1</v>
       </c>
       <c r="P17" s="15" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B18" s="13" t="s">
         <v>71</v>
@@ -3807,122 +3804,122 @@
         <v>54</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E18" s="13" t="s">
         <v>6</v>
       </c>
       <c r="F18" s="13" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G18" s="13" t="s">
         <v>6</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I18" s="13" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J18" s="13" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K18" s="13" t="s">
         <v>47</v>
       </c>
       <c r="L18" s="13" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="M18" s="13" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="N18" s="13" t="s">
         <v>81</v>
       </c>
       <c r="O18" s="13" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="P18" s="13" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E19" s="15" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F19" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="G19" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="G19" s="15" t="s">
-        <v>160</v>
-      </c>
       <c r="H19" s="15" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I19" s="15" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J19" s="15" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="K19" s="15" t="s">
         <v>1</v>
       </c>
       <c r="L19" s="15" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="M19" s="15" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="N19" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O19" s="15" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="P19" s="15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E20" s="15" t="s">
         <v>6</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G20" s="15" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H20" s="15" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I20" s="15" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="J20" s="15" t="s">
         <v>57</v>
@@ -3931,33 +3928,33 @@
         <v>1</v>
       </c>
       <c r="L20" s="15" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="M20" s="15" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="N20" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O20" s="15" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="P20" s="15" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C21" s="15" t="s">
         <v>32</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E21" s="15" t="s">
         <v>6</v>
@@ -3966,7 +3963,7 @@
         <v>6</v>
       </c>
       <c r="G21" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H21" s="15" t="s">
         <v>6</v>
@@ -3981,10 +3978,10 @@
         <v>1</v>
       </c>
       <c r="L21" s="15" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="M21" s="15" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="N21" s="15" t="s">
         <v>1</v>
@@ -3998,16 +3995,16 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C22" s="15" t="s">
         <v>32</v>
       </c>
       <c r="D22" s="15" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E22" s="15" t="s">
         <v>6</v>
@@ -4016,13 +4013,13 @@
         <v>6</v>
       </c>
       <c r="G22" s="15" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H22" s="15" t="s">
         <v>6</v>
       </c>
       <c r="I22" s="15" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="J22" s="15" t="s">
         <v>57</v>
@@ -4031,10 +4028,10 @@
         <v>1</v>
       </c>
       <c r="L22" s="15" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="M22" s="15" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="N22" s="15" t="s">
         <v>1</v>
@@ -4043,30 +4040,30 @@
         <v>1</v>
       </c>
       <c r="P22" s="15" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C23" s="15" t="s">
         <v>32</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F23" s="15" t="s">
         <v>6</v>
       </c>
       <c r="G23" s="15" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H23" s="15" t="s">
         <v>6</v>
@@ -4081,10 +4078,10 @@
         <v>1</v>
       </c>
       <c r="L23" s="15" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="M23" s="15" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="N23" s="15" t="s">
         <v>1</v>
@@ -4093,21 +4090,21 @@
         <v>1</v>
       </c>
       <c r="P23" s="15" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C24" s="15" t="s">
         <v>32</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E24" s="15" t="s">
         <v>6</v>
@@ -4116,13 +4113,13 @@
         <v>6</v>
       </c>
       <c r="G24" s="15" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H24" s="15" t="s">
         <v>6</v>
       </c>
       <c r="I24" s="15" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="J24" s="15" t="s">
         <v>57</v>
@@ -4131,10 +4128,10 @@
         <v>1</v>
       </c>
       <c r="L24" s="15" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="M24" s="15" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="N24" s="15" t="s">
         <v>1</v>
@@ -4143,12 +4140,12 @@
         <v>1</v>
       </c>
       <c r="P24" s="15" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B25" s="15" t="s">
         <v>71</v>
@@ -4157,22 +4154,22 @@
         <v>32</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G25" s="15" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="H25" s="15" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I25" s="15" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J25" s="15" t="s">
         <v>57</v>
@@ -4181,10 +4178,10 @@
         <v>1</v>
       </c>
       <c r="L25" s="15" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="M25" s="15" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="N25" s="15" t="s">
         <v>1</v>
@@ -4193,36 +4190,36 @@
         <v>1</v>
       </c>
       <c r="P25" s="15" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E26" s="15" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F26" s="15" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="G26" s="15" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H26" s="15" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I26" s="15" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="J26" s="15" t="s">
         <v>57</v>
@@ -4231,33 +4228,33 @@
         <v>1</v>
       </c>
       <c r="L26" s="15" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="M26" s="15" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="N26" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O26" s="15" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="P26" s="15" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C27" s="15" t="s">
         <v>32</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E27" s="15" t="s">
         <v>6</v>
@@ -4266,13 +4263,13 @@
         <v>6</v>
       </c>
       <c r="G27" s="15" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H27" s="15" t="s">
         <v>6</v>
       </c>
       <c r="I27" s="15" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J27" s="15" t="s">
         <v>57</v>
@@ -4281,10 +4278,10 @@
         <v>1</v>
       </c>
       <c r="L27" s="15" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="M27" s="15" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="N27" s="15" t="s">
         <v>1</v>
@@ -4298,31 +4295,31 @@
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="15" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E28" s="15" t="s">
         <v>6</v>
       </c>
       <c r="F28" s="15" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G28" s="15" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H28" s="15" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I28" s="15" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="J28" s="15" t="s">
         <v>57</v>
@@ -4331,10 +4328,10 @@
         <v>1</v>
       </c>
       <c r="L28" s="15" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="M28" s="15" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="N28" s="15" t="s">
         <v>1</v>
@@ -4343,36 +4340,36 @@
         <v>1</v>
       </c>
       <c r="P28" s="15" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="15" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E29" s="15" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F29" s="15" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="G29" s="15" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="H29" s="15" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I29" s="15" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="J29" s="15" t="s">
         <v>57</v>
@@ -4381,10 +4378,10 @@
         <v>1</v>
       </c>
       <c r="L29" s="15" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="M29" s="15" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="N29" s="15" t="s">
         <v>1</v>
@@ -4393,36 +4390,36 @@
         <v>1</v>
       </c>
       <c r="P29" s="15" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="15" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E30" s="15" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F30" s="15" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="G30" s="15" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="H30" s="15" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I30" s="15" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="J30" s="15" t="s">
         <v>57</v>
@@ -4431,10 +4428,10 @@
         <v>1</v>
       </c>
       <c r="L30" s="15" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="M30" s="15" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="N30" s="15" t="s">
         <v>1</v>
@@ -4443,36 +4440,36 @@
         <v>1</v>
       </c>
       <c r="P30" s="15" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="15" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E31" s="15" t="s">
         <v>6</v>
       </c>
       <c r="F31" s="15" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G31" s="15" t="s">
         <v>6</v>
       </c>
       <c r="H31" s="15" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="I31" s="15" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="J31" s="15" t="s">
         <v>57</v>
@@ -4481,16 +4478,16 @@
         <v>1</v>
       </c>
       <c r="L31" s="15" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="M31" s="15" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="N31" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O31" s="15" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="P31" s="15" t="s">
         <v>83</v>
@@ -4498,31 +4495,31 @@
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="15" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E32" s="15" t="s">
         <v>6</v>
       </c>
       <c r="F32" s="15" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G32" s="15" t="s">
         <v>6</v>
       </c>
       <c r="H32" s="15" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="I32" s="15" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J32" s="15" t="s">
         <v>57</v>
@@ -4531,48 +4528,48 @@
         <v>1</v>
       </c>
       <c r="L32" s="15" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="M32" s="15" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="N32" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O32" s="15" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="P32" s="15" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="15" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E33" s="15" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F33" s="15" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="G33" s="15" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="H33" s="15" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I33" s="15" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="J33" s="15" t="s">
         <v>57</v>
@@ -4581,10 +4578,10 @@
         <v>1</v>
       </c>
       <c r="L33" s="15" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="M33" s="15" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="N33" s="15" t="s">
         <v>1</v>
@@ -4593,86 +4590,86 @@
         <v>1</v>
       </c>
       <c r="P33" s="15" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="15" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E34" s="15" t="s">
         <v>6</v>
       </c>
       <c r="F34" s="15" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G34" s="15" t="s">
         <v>6</v>
       </c>
       <c r="H34" s="15" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="I34" s="15" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="J34" s="15" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="K34" s="15" t="s">
         <v>1</v>
       </c>
       <c r="L34" s="15" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="M34" s="15" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="N34" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O34" s="15" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="P34" s="15" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="15" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E35" s="15" t="s">
         <v>6</v>
       </c>
       <c r="F35" s="15" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G35" s="15" t="s">
         <v>6</v>
       </c>
       <c r="H35" s="15" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="I35" s="15" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="J35" s="15" t="s">
         <v>57</v>
@@ -4681,10 +4678,10 @@
         <v>1</v>
       </c>
       <c r="L35" s="15" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="M35" s="15" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="N35" s="15" t="s">
         <v>1</v>
@@ -4693,21 +4690,21 @@
         <v>1</v>
       </c>
       <c r="P35" s="15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="15" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E36" s="15" t="s">
         <v>6</v>
@@ -4719,10 +4716,10 @@
         <v>6</v>
       </c>
       <c r="H36" s="15" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="I36" s="15" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="J36" s="15" t="s">
         <v>57</v>
@@ -4731,10 +4728,10 @@
         <v>1</v>
       </c>
       <c r="L36" s="15" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="M36" s="15" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="N36" s="15" t="s">
         <v>1</v>
@@ -4743,86 +4740,86 @@
         <v>1</v>
       </c>
       <c r="P36" s="15" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B37" s="13" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E37" s="13" t="s">
         <v>6</v>
       </c>
       <c r="F37" s="13" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="G37" s="13" t="s">
         <v>6</v>
       </c>
       <c r="H37" s="13" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="I37" s="13" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="J37" s="13" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="K37" s="13" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="L37" s="13" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="M37" s="13" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="N37" s="13" t="s">
         <v>81</v>
       </c>
       <c r="O37" s="13" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="P37" s="13" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F38" s="12" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="G38" s="12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H38" s="12" t="s">
         <v>12</v>
       </c>
       <c r="I38" s="12" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="J38" s="12" t="s">
         <v>90</v>
@@ -4831,39 +4828,39 @@
         <v>47</v>
       </c>
       <c r="L38" s="12" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="M38" s="12" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="N38" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O38" s="12" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="P38" s="12" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="13" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B39" s="13" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E39" s="13" t="s">
         <v>6</v>
       </c>
       <c r="F39" s="13" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G39" s="13" t="s">
         <v>6</v>
@@ -4872,48 +4869,48 @@
         <v>12</v>
       </c>
       <c r="I39" s="13" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="J39" s="13" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K39" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L39" s="13" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="M39" s="13" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="N39" s="13" t="s">
         <v>81</v>
       </c>
       <c r="O39" s="13" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="P39" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="13" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B40" s="13" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D40" s="13" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="E40" s="13" t="s">
         <v>6</v>
       </c>
       <c r="F40" s="13" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G40" s="13" t="s">
         <v>6</v>
@@ -4922,25 +4919,25 @@
         <v>12</v>
       </c>
       <c r="I40" s="13" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="J40" s="13" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K40" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L40" s="13" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="M40" s="13" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="N40" s="13" t="s">
         <v>81</v>
       </c>
       <c r="O40" s="13" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="P40" s="13" t="s">
         <v>61</v>
@@ -4948,22 +4945,22 @@
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="13" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E41" s="13" t="s">
         <v>6</v>
       </c>
       <c r="F41" s="13" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G41" s="13" t="s">
         <v>6</v>
@@ -4972,48 +4969,48 @@
         <v>12</v>
       </c>
       <c r="I41" s="13" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="J41" s="13" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K41" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L41" s="13" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="M41" s="13" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="N41" s="13" t="s">
         <v>81</v>
       </c>
       <c r="O41" s="13" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="P41" s="13" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="13" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E42" s="13" t="s">
         <v>6</v>
       </c>
       <c r="F42" s="13" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G42" s="13" t="s">
         <v>6</v>
@@ -5022,101 +5019,101 @@
         <v>12</v>
       </c>
       <c r="I42" s="13" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="J42" s="13" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K42" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L42" s="13" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="M42" s="13" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="N42" s="13" t="s">
         <v>81</v>
       </c>
       <c r="O42" s="13" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="P42" s="13" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="13" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B43" s="13" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D43" s="13" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F43" s="13" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G43" s="13" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="H43" s="13" t="s">
         <v>12</v>
       </c>
       <c r="I43" s="13" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="J43" s="13" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K43" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L43" s="13" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="M43" s="13" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="N43" s="13" t="s">
         <v>81</v>
       </c>
       <c r="O43" s="13" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="P43" s="13" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="15" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B44" s="15" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C44" s="15" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D44" s="15" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E44" s="15" t="s">
         <v>6</v>
       </c>
       <c r="F44" s="15" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G44" s="15" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="H44" s="15" t="s">
         <v>12</v>
@@ -5131,39 +5128,39 @@
         <v>1</v>
       </c>
       <c r="L44" s="15" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="M44" s="15" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="N44" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O44" s="15" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="P44" s="15" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="13" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B45" s="13" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D45" s="13" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E45" s="13" t="s">
         <v>6</v>
       </c>
       <c r="F45" s="13" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="G45" s="13" t="s">
         <v>6</v>
@@ -5172,242 +5169,242 @@
         <v>12</v>
       </c>
       <c r="I45" s="13" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="J45" s="13" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K45" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L45" s="13" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="M45" s="13" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="N45" s="13" t="s">
         <v>81</v>
       </c>
       <c r="O45" s="13" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="P45" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="13" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B46" s="13" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F46" s="13" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G46" s="13" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="H46" s="13" t="s">
         <v>12</v>
       </c>
       <c r="I46" s="13" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="J46" s="13" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K46" s="13" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L46" s="13" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="M46" s="13" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="N46" s="13" t="s">
         <v>81</v>
       </c>
       <c r="O46" s="13" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="P46" s="13" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="13" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B47" s="13" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D47" s="13" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="F47" s="13" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="G47" s="13" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="H47" s="13" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="I47" s="13" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="J47" s="13" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="K47" s="13" t="s">
         <v>47</v>
       </c>
       <c r="L47" s="13" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="M47" s="13" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="N47" s="13" t="s">
         <v>81</v>
       </c>
       <c r="O47" s="13" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="P47" s="13" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="15" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B48" s="15" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C48" s="15" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="D48" s="15" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="E48" s="15" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="F48" s="15" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="G48" s="15" t="s">
         <v>6</v>
       </c>
       <c r="H48" s="15" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="I48" s="15" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="J48" s="15" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="K48" s="15" t="s">
         <v>1</v>
       </c>
       <c r="L48" s="15" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="M48" s="15" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="N48" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O48" s="15" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="P48" s="15" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="13" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B49" s="13" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D49" s="13" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="E49" s="13" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="F49" s="13" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="G49" s="13" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="H49" s="13" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="I49" s="13" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="J49" s="13" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="K49" s="13" t="s">
         <v>47</v>
       </c>
       <c r="L49" s="13" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="M49" s="13" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="N49" s="13" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="O49" s="13" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="P49" s="13" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="13" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="E50" s="13" t="s">
         <v>6</v>
@@ -5419,60 +5416,60 @@
         <v>6</v>
       </c>
       <c r="H50" s="13" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="I50" s="13" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="J50" s="13" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="K50" s="13" t="s">
         <v>47</v>
       </c>
       <c r="L50" s="13" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="M50" s="13" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="N50" s="13" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="O50" s="13" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="P50" s="13" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="12" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B51" s="12" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D51" s="12" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E51" s="12" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="F51" s="12" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="G51" s="12" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="H51" s="12" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="I51" s="12" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="J51" s="12" t="s">
         <v>90</v>
@@ -5481,48 +5478,48 @@
         <v>47</v>
       </c>
       <c r="L51" s="12" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="M51" s="12" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="N51" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O51" s="12" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="P51" s="12" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="12" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B52" s="12" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="D52" s="12" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="E52" s="12" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="F52" s="12" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="G52" s="12" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="H52" s="12" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="I52" s="12" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="J52" s="12" t="s">
         <v>90</v>
@@ -5531,48 +5528,48 @@
         <v>47</v>
       </c>
       <c r="L52" s="12" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="M52" s="12" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="N52" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O52" s="12" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="P52" s="12" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="12" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B53" s="12" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D53" s="12" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E53" s="12" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="F53" s="12" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="G53" s="12" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="H53" s="12" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="I53" s="12" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="J53" s="12" t="s">
         <v>90</v>
@@ -5581,98 +5578,98 @@
         <v>47</v>
       </c>
       <c r="L53" s="12" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="M53" s="12" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="N53" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O53" s="12" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="P53" s="12" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="14" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B54" s="14" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="D54" s="14" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="E54" s="14" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="F54" s="14" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="G54" s="14" t="s">
         <v>6</v>
       </c>
       <c r="H54" s="14" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="I54" s="14" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J54" s="14" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="K54" s="14" t="s">
         <v>47</v>
       </c>
       <c r="L54" s="14" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="M54" s="14" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="N54" s="14" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="O54" s="14" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="P54" s="14" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="12" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="B55" s="12" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C55" s="12" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="D55" s="12" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="E55" s="12" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="F55" s="12" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G55" s="12" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="H55" s="12" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="I55" s="12" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="J55" s="12" t="s">
         <v>90</v>
@@ -5681,66 +5678,66 @@
         <v>47</v>
       </c>
       <c r="L55" s="12" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="M55" s="12" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="N55" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O55" s="12" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="P55" s="12" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="12" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="B56" s="12" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="C56" s="12" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="D56" s="12" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="E56" s="12" t="s">
         <v>6</v>
       </c>
       <c r="F56" s="12" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="G56" s="12" t="s">
         <v>6</v>
       </c>
       <c r="H56" s="12" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="I56" s="12" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="J56" s="12" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="K56" s="12" t="s">
         <v>47</v>
       </c>
       <c r="L56" s="12" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="M56" s="12" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="N56" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O56" s="12" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="P56" s="12" t="s">
         <v>83</v>
@@ -5748,72 +5745,72 @@
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="12" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B57" s="12" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="C57" s="12" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D57" s="12" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E57" s="12" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="F57" s="12" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="G57" s="12" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="H57" s="12" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="I57" s="12" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="J57" s="12" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="K57" s="12" t="s">
         <v>47</v>
       </c>
       <c r="L57" s="12" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="M57" s="12" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="N57" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O57" s="12" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="P57" s="12" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="12" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B58" s="12" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="C58" s="12" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="D58" s="12" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="E58" s="12" t="s">
         <v>6</v>
       </c>
       <c r="F58" s="12" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="G58" s="12" t="s">
         <v>6</v>
@@ -5822,57 +5819,57 @@
         <v>6</v>
       </c>
       <c r="I58" s="12" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="J58" s="12" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="K58" s="12" t="s">
         <v>47</v>
       </c>
       <c r="L58" s="12" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="M58" s="12" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="N58" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O58" s="12" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="P58" s="12" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="15" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B59" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C59" s="15" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="D59" s="15" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="E59" s="15" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="F59" s="15" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="G59" s="15" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="H59" s="15" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="I59" s="15" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="J59" s="15" t="s">
         <v>57</v>
@@ -5881,48 +5878,48 @@
         <v>1</v>
       </c>
       <c r="L59" s="15" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="M59" s="15" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="N59" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O59" s="15" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="P59" s="15" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="15" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B60" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C60" s="15" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D60" s="15" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="E60" s="15" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="F60" s="15" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="G60" s="15" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="H60" s="15" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="I60" s="15" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="J60" s="15" t="s">
         <v>57</v>
@@ -5931,48 +5928,48 @@
         <v>1</v>
       </c>
       <c r="L60" s="15" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="M60" s="15" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="N60" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O60" s="15" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="P60" s="15" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="12" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="B61" s="12" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C61" s="12" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="D61" s="12" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="E61" s="12" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="F61" s="12" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="G61" s="12" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="H61" s="12" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="I61" s="12" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="J61" s="12" t="s">
         <v>90</v>
@@ -5981,48 +5978,48 @@
         <v>47</v>
       </c>
       <c r="L61" s="12" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="M61" s="12" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="N61" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O61" s="12" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="P61" s="12" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="15" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="B62" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C62" s="15" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="D62" s="15" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="E62" s="15" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="F62" s="15" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="G62" s="15" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="H62" s="15" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="I62" s="15" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="J62" s="15" t="s">
         <v>57</v>
@@ -6031,48 +6028,48 @@
         <v>1</v>
       </c>
       <c r="L62" s="15" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="M62" s="15" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="N62" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O62" s="15" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="P62" s="15" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="15" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="B63" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C63" s="15" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="D63" s="15" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="E63" s="15" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="F63" s="15" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="G63" s="15" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="H63" s="15" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="I63" s="15" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="J63" s="15" t="s">
         <v>57</v>
@@ -6081,48 +6078,48 @@
         <v>1</v>
       </c>
       <c r="L63" s="15" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="M63" s="15" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="N63" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O63" s="15" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="P63" s="15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="15" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="B64" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C64" s="15" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="D64" s="15" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E64" s="15" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="F64" s="15" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="G64" s="15" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="H64" s="15" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="I64" s="15" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="J64" s="15" t="s">
         <v>57</v>
@@ -6131,33 +6128,33 @@
         <v>1</v>
       </c>
       <c r="L64" s="15" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="M64" s="15" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="N64" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O64" s="15" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="P64" s="15" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="15" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="B65" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C65" s="15" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="D65" s="15" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="E65" s="15" t="s">
         <v>6</v>
@@ -6172,7 +6169,7 @@
         <v>6</v>
       </c>
       <c r="I65" s="15" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="J65" s="15" t="s">
         <v>57</v>
@@ -6181,48 +6178,48 @@
         <v>1</v>
       </c>
       <c r="L65" s="15" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="M65" s="15" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="N65" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O65" s="15" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="P65" s="15" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="15" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B66" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C66" s="15" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="D66" s="15" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="E66" s="15" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="F66" s="15" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="G66" s="15" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="H66" s="15" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="I66" s="15" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="J66" s="15" t="s">
         <v>57</v>
@@ -6231,33 +6228,33 @@
         <v>1</v>
       </c>
       <c r="L66" s="15" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="M66" s="15" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="N66" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O66" s="15" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="P66" s="15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="13" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="B67" s="13" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C67" s="13" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="D67" s="13" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E67" s="13" t="s">
         <v>6</v>
@@ -6272,107 +6269,107 @@
         <v>6</v>
       </c>
       <c r="I67" s="13" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="J67" s="13" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="K67" s="13" t="s">
         <v>47</v>
       </c>
       <c r="L67" s="13" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="M67" s="13" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="N67" s="13" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="O67" s="13" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="P67" s="13" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="12" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="B68" s="12" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C68" s="12" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="D68" s="12" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="E68" s="12" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="F68" s="12" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="G68" s="12" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="H68" s="12" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="I68" s="12" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="J68" s="12" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="K68" s="12" t="s">
         <v>47</v>
       </c>
       <c r="L68" s="12" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="M68" s="12" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="N68" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O68" s="12" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="P68" s="12" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="15" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="B69" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C69" s="15" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="D69" s="15" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="E69" s="15" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="F69" s="15" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="G69" s="15" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="H69" s="15" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="I69" s="15" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="J69" s="15" t="s">
         <v>57</v>
@@ -6381,48 +6378,48 @@
         <v>1</v>
       </c>
       <c r="L69" s="15" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="M69" s="15" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="N69" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O69" s="15" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="P69" s="15" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="15" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="B70" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C70" s="15" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D70" s="15" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E70" s="15" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="F70" s="15" t="s">
+        <v>644</v>
+      </c>
+      <c r="G70" s="15" t="s">
         <v>643</v>
       </c>
-      <c r="G70" s="15" t="s">
-        <v>642</v>
-      </c>
       <c r="H70" s="15" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="I70" s="15" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="J70" s="15" t="s">
         <v>57</v>
@@ -6431,48 +6428,48 @@
         <v>1</v>
       </c>
       <c r="L70" s="15" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="M70" s="15" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="N70" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O70" s="15" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="P70" s="15" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="15" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B71" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C71" s="15" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="D71" s="15" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="E71" s="15" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="F71" s="15" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="G71" s="15" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="H71" s="15" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="I71" s="15" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="J71" s="15" t="s">
         <v>57</v>
@@ -6481,69 +6478,69 @@
         <v>1</v>
       </c>
       <c r="L71" s="15" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="M71" s="15" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="N71" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O71" s="15" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="P71" s="15" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="14" t="s">
-        <v>658</v>
-      </c>
-      <c r="B72" s="14" t="s">
-        <v>445</v>
-      </c>
-      <c r="C72" s="14" t="s">
+      <c r="A72" s="12" t="s">
         <v>659</v>
       </c>
-      <c r="D72" s="14" t="s">
+      <c r="B72" s="12" t="s">
+        <v>446</v>
+      </c>
+      <c r="C72" s="12" t="s">
         <v>660</v>
       </c>
-      <c r="E72" s="14" t="s">
+      <c r="D72" s="12" t="s">
         <v>661</v>
       </c>
-      <c r="F72" s="14" t="s">
+      <c r="E72" s="12" t="s">
         <v>662</v>
       </c>
-      <c r="G72" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="H72" s="14" t="s">
+      <c r="F72" s="12" t="s">
         <v>663</v>
       </c>
-      <c r="I72" s="14" t="s">
+      <c r="G72" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H72" s="12" t="s">
         <v>664</v>
       </c>
-      <c r="J72" s="14" t="s">
+      <c r="I72" s="12" t="s">
         <v>665</v>
       </c>
-      <c r="K72" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="L72" s="14" t="s">
+      <c r="J72" s="12" t="s">
         <v>666</v>
       </c>
-      <c r="M72" s="14" t="s">
+      <c r="K72" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="L72" s="12" t="s">
         <v>667</v>
       </c>
-      <c r="N72" s="14" t="s">
+      <c r="M72" s="12" t="s">
         <v>668</v>
       </c>
-      <c r="O72" s="14" t="s">
+      <c r="N72" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="O72" s="12" t="s">
         <v>669</v>
       </c>
-      <c r="P72" s="14" t="s">
-        <v>431</v>
+      <c r="P72" s="12" t="s">
+        <v>432</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6551,7 +6548,7 @@
         <v>670</v>
       </c>
       <c r="B73" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C73" s="15" t="s">
         <v>671</v>
@@ -6593,7 +6590,7 @@
         <v>676</v>
       </c>
       <c r="P73" s="15" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6601,7 +6598,7 @@
         <v>677</v>
       </c>
       <c r="B74" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C74" s="15" t="s">
         <v>671</v>
@@ -6643,7 +6640,7 @@
         <v>686</v>
       </c>
       <c r="P74" s="15" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6651,7 +6648,7 @@
         <v>687</v>
       </c>
       <c r="B75" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C75" s="15" t="s">
         <v>671</v>
@@ -6693,7 +6690,7 @@
         <v>696</v>
       </c>
       <c r="P75" s="15" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6701,7 +6698,7 @@
         <v>697</v>
       </c>
       <c r="B76" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C76" s="15" t="s">
         <v>698</v>
@@ -6743,7 +6740,7 @@
         <v>705</v>
       </c>
       <c r="P76" s="15" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6751,7 +6748,7 @@
         <v>706</v>
       </c>
       <c r="B77" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C77" s="15" t="s">
         <v>707</v>
@@ -6793,7 +6790,7 @@
         <v>713</v>
       </c>
       <c r="P77" s="15" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6801,7 +6798,7 @@
         <v>714</v>
       </c>
       <c r="B78" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C78" s="15" t="s">
         <v>715</v>
@@ -6843,7 +6840,7 @@
         <v>722</v>
       </c>
       <c r="P78" s="15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6851,7 +6848,7 @@
         <v>723</v>
       </c>
       <c r="B79" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C79" s="15" t="s">
         <v>724</v>
@@ -6866,7 +6863,7 @@
         <v>727</v>
       </c>
       <c r="G79" s="15" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="H79" s="15" t="s">
         <v>728</v>
@@ -6893,7 +6890,7 @@
         <v>732</v>
       </c>
       <c r="P79" s="15" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6901,7 +6898,7 @@
         <v>733</v>
       </c>
       <c r="B80" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C80" s="15" t="s">
         <v>724</v>
@@ -6943,7 +6940,7 @@
         <v>738</v>
       </c>
       <c r="P80" s="15" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6951,7 +6948,7 @@
         <v>739</v>
       </c>
       <c r="B81" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C81" s="15" t="s">
         <v>724</v>
@@ -6993,7 +6990,7 @@
         <v>745</v>
       </c>
       <c r="P81" s="15" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7001,7 +6998,7 @@
         <v>746</v>
       </c>
       <c r="B82" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C82" s="15" t="s">
         <v>747</v>
@@ -7043,7 +7040,7 @@
         <v>756</v>
       </c>
       <c r="P82" s="15" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7051,7 +7048,7 @@
         <v>757</v>
       </c>
       <c r="B83" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C83" s="15" t="s">
         <v>758</v>
@@ -7081,7 +7078,7 @@
         <v>1</v>
       </c>
       <c r="L83" s="15" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="M83" s="15" t="s">
         <v>764</v>
@@ -7093,7 +7090,7 @@
         <v>765</v>
       </c>
       <c r="P83" s="15" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7101,7 +7098,7 @@
         <v>766</v>
       </c>
       <c r="B84" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C84" s="15" t="s">
         <v>758</v>
@@ -7110,7 +7107,7 @@
         <v>767</v>
       </c>
       <c r="E84" s="15" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="F84" s="15" t="s">
         <v>768</v>
@@ -7143,7 +7140,7 @@
         <v>774</v>
       </c>
       <c r="P84" s="15" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7151,7 +7148,7 @@
         <v>775</v>
       </c>
       <c r="B85" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C85" s="15" t="s">
         <v>758</v>
@@ -7193,7 +7190,7 @@
         <v>784</v>
       </c>
       <c r="P85" s="15" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7201,7 +7198,7 @@
         <v>785</v>
       </c>
       <c r="B86" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C86" s="15" t="s">
         <v>786</v>
@@ -7219,7 +7216,7 @@
         <v>6</v>
       </c>
       <c r="H86" s="15" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="I86" s="15" t="s">
         <v>790</v>
@@ -7243,7 +7240,7 @@
         <v>793</v>
       </c>
       <c r="P86" s="15" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7251,7 +7248,7 @@
         <v>794</v>
       </c>
       <c r="B87" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C87" s="15" t="s">
         <v>786</v>
@@ -7293,7 +7290,7 @@
         <v>801</v>
       </c>
       <c r="P87" s="15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7301,7 +7298,7 @@
         <v>802</v>
       </c>
       <c r="B88" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C88" s="15" t="s">
         <v>803</v>
@@ -7343,7 +7340,7 @@
         <v>811</v>
       </c>
       <c r="P88" s="15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7351,7 +7348,7 @@
         <v>812</v>
       </c>
       <c r="B89" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C89" s="15" t="s">
         <v>813</v>
@@ -7393,7 +7390,7 @@
         <v>820</v>
       </c>
       <c r="P89" s="15" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7401,7 +7398,7 @@
         <v>821</v>
       </c>
       <c r="B90" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C90" s="15" t="s">
         <v>822</v>
@@ -7443,7 +7440,7 @@
         <v>830</v>
       </c>
       <c r="P90" s="15" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7451,7 +7448,7 @@
         <v>831</v>
       </c>
       <c r="B91" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C91" s="15" t="s">
         <v>832</v>
@@ -7493,7 +7490,7 @@
         <v>837</v>
       </c>
       <c r="P91" s="15" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7501,7 +7498,7 @@
         <v>838</v>
       </c>
       <c r="B92" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C92" s="15" t="s">
         <v>839</v>
@@ -7516,7 +7513,7 @@
         <v>842</v>
       </c>
       <c r="G92" s="15" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="H92" s="15" t="s">
         <v>843</v>
@@ -7543,7 +7540,7 @@
         <v>847</v>
       </c>
       <c r="P92" s="15" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7551,7 +7548,7 @@
         <v>848</v>
       </c>
       <c r="B93" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="C93" s="15" t="s">
         <v>849</v>
@@ -7566,7 +7563,7 @@
         <v>852</v>
       </c>
       <c r="G93" s="15" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="H93" s="15" t="s">
         <v>853</v>
@@ -7593,7 +7590,7 @@
         <v>857</v>
       </c>
       <c r="P93" s="15" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7604,7 +7601,7 @@
         <v>859</v>
       </c>
       <c r="C94" s="12" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D94" s="12" t="s">
         <v>860</v>
@@ -7628,172 +7625,172 @@
         <v>862</v>
       </c>
       <c r="K94" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="L94" s="12" t="s">
         <v>863</v>
       </c>
-      <c r="L94" s="12" t="s">
+      <c r="M94" s="12" t="s">
         <v>864</v>
-      </c>
-      <c r="M94" s="12" t="s">
-        <v>865</v>
       </c>
       <c r="N94" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O94" s="12" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="P94" s="12" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="12" t="s">
+        <v>866</v>
+      </c>
+      <c r="B95" s="12" t="s">
+        <v>446</v>
+      </c>
+      <c r="C95" s="12" t="s">
         <v>867</v>
       </c>
-      <c r="B95" s="12" t="s">
-        <v>445</v>
-      </c>
-      <c r="C95" s="12" t="s">
+      <c r="D95" s="12" t="s">
         <v>868</v>
       </c>
-      <c r="D95" s="12" t="s">
+      <c r="E95" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="F95" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="G95" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H95" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="I95" s="12" t="s">
         <v>869</v>
-      </c>
-      <c r="E95" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="F95" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="G95" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="H95" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="I95" s="12" t="s">
-        <v>870</v>
       </c>
       <c r="J95" s="12" t="s">
         <v>46</v>
       </c>
       <c r="K95" s="12" t="s">
-        <v>863</v>
+        <v>91</v>
       </c>
       <c r="L95" s="12" t="s">
+        <v>870</v>
+      </c>
+      <c r="M95" s="12" t="s">
         <v>871</v>
-      </c>
-      <c r="M95" s="12" t="s">
-        <v>872</v>
       </c>
       <c r="N95" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O95" s="12" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="P95" s="12" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="12" t="s">
+        <v>873</v>
+      </c>
+      <c r="B96" s="12" t="s">
+        <v>446</v>
+      </c>
+      <c r="C96" s="12" t="s">
         <v>874</v>
       </c>
-      <c r="B96" s="12" t="s">
-        <v>445</v>
-      </c>
-      <c r="C96" s="12" t="s">
+      <c r="D96" s="12" t="s">
         <v>875</v>
       </c>
-      <c r="D96" s="12" t="s">
+      <c r="E96" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="F96" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="G96" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H96" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="I96" s="12" t="s">
         <v>876</v>
-      </c>
-      <c r="E96" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="F96" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="G96" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="H96" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="I96" s="12" t="s">
-        <v>877</v>
       </c>
       <c r="J96" s="12" t="s">
         <v>46</v>
       </c>
       <c r="K96" s="12" t="s">
-        <v>863</v>
+        <v>91</v>
       </c>
       <c r="L96" s="12" t="s">
+        <v>877</v>
+      </c>
+      <c r="M96" s="12" t="s">
         <v>878</v>
-      </c>
-      <c r="M96" s="12" t="s">
-        <v>879</v>
       </c>
       <c r="N96" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O96" s="12" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="P96" s="12" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="13" t="s">
+        <v>880</v>
+      </c>
+      <c r="B97" s="13" t="s">
         <v>881</v>
       </c>
-      <c r="B97" s="13" t="s">
+      <c r="C97" s="13" t="s">
         <v>882</v>
       </c>
-      <c r="C97" s="13" t="s">
+      <c r="D97" s="13" t="s">
         <v>883</v>
       </c>
-      <c r="D97" s="13" t="s">
+      <c r="E97" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="F97" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="G97" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="H97" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="I97" s="13" t="s">
         <v>884</v>
       </c>
-      <c r="E97" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="F97" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="G97" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="H97" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="I97" s="13" t="s">
+      <c r="J97" s="13" t="s">
         <v>885</v>
-      </c>
-      <c r="J97" s="13" t="s">
-        <v>886</v>
       </c>
       <c r="K97" s="13" t="s">
         <v>47</v>
       </c>
       <c r="L97" s="13" t="s">
+        <v>886</v>
+      </c>
+      <c r="M97" s="13" t="s">
         <v>887</v>
       </c>
-      <c r="M97" s="13" t="s">
+      <c r="N97" s="13" t="s">
         <v>888</v>
       </c>
-      <c r="N97" s="13" t="s">
+      <c r="O97" s="13" t="s">
         <v>889</v>
       </c>
-      <c r="O97" s="13" t="s">
-        <v>890</v>
-      </c>
       <c r="P97" s="13" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
qa - storyboard backup
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1552" uniqueCount="890">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1552" uniqueCount="893">
   <si>
     <t>LEGEND</t>
   </si>
@@ -2041,16 +2041,25 @@
     <t>Cross the feedback eligibility boundary</t>
   </si>
   <si>
-    <t>Accepted non-admin participant sees one item only after start plus two hours</t>
-  </si>
-  <si>
-    <t>Feedback eligibility service coverage partial</t>
-  </si>
-  <si>
-    <t>Compare before/after boundary, trashed, admin and pending controls</t>
-  </si>
-  <si>
-    <t>Current code uses start plus two hours, not event end or closed status</t>
+    <t>DELTA exact persisted users.activities.feedback and eventFeedback.pending at the eligibility write; popup/menu reads X</t>
+  </si>
+  <si>
+    <t>CONDITIONAL bounded due-event worker materializes the eligibility transition once; repeated pass X</t>
+  </si>
+  <si>
+    <t>Accepted non-admin participant sees one pending item only after start plus two hours; the independently reloaded profile menu shows the same actionable count</t>
+  </si>
+  <si>
+    <t>MANUAL UI + FUNCTIONAL PASS; MENU BADGE DEFECT FIXED</t>
+  </si>
+  <si>
+    <t>Focused UserActivityCountersService and EventCounterExpiryService eligibility/idempotence tests PASS; status oracle prints the exact main counter, four buckets and tracking markers</t>
+  </si>
+  <si>
+    <t>On any eligibility-policy change compare accepted participant against locked, trashed, admin and pending controls; require feedback=1 with ownEvents/pending/feedbacked/removed=0/1/0/0 before opening the popup</t>
+  </si>
+  <si>
+    <t>The popup showed exactly one eligible event and excluded the start+2h locked, trashed, admin and pending-member controls. The initial reload exposed a missing profile-menu badge because eligibility was computed only by the read projection. The fix materializes the transition through the existing bounded worker and owner service, with no frontend delta and no menu/popup recomputation. After hot deploy, reload independently showed red badge 1. Read-only Mongo proof: users.activities.feedback=1, eventFeedback ownEvents=0 pending=1 feedbacked=0 removed=0, exactly one eligible/counterTracked state, and the due source marked projected. The reusable checkpoint oracle now prints these exact values.</t>
   </si>
   <si>
     <t>EVENT-FEEDBACK-002</t>
@@ -6544,58 +6553,58 @@
       </c>
     </row>
     <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="15" t="s">
+      <c r="A73" s="12" t="s">
         <v>670</v>
       </c>
-      <c r="B73" s="15" t="s">
+      <c r="B73" s="12" t="s">
         <v>446</v>
       </c>
-      <c r="C73" s="15" t="s">
+      <c r="C73" s="12" t="s">
         <v>671</v>
       </c>
-      <c r="D73" s="15" t="s">
+      <c r="D73" s="12" t="s">
         <v>672</v>
       </c>
-      <c r="E73" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="F73" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="G73" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="H73" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="I73" s="15" t="s">
+      <c r="E73" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="F73" s="12" t="s">
         <v>673</v>
       </c>
-      <c r="J73" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="K73" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="L73" s="15" t="s">
+      <c r="G73" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="H73" s="12" t="s">
         <v>674</v>
       </c>
-      <c r="M73" s="15" t="s">
+      <c r="I73" s="12" t="s">
         <v>675</v>
       </c>
-      <c r="N73" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="O73" s="15" t="s">
+      <c r="J73" s="12" t="s">
         <v>676</v>
       </c>
-      <c r="P73" s="15" t="s">
+      <c r="K73" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="L73" s="12" t="s">
+        <v>677</v>
+      </c>
+      <c r="M73" s="12" t="s">
+        <v>678</v>
+      </c>
+      <c r="N73" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="O73" s="12" t="s">
+        <v>679</v>
+      </c>
+      <c r="P73" s="12" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="15" t="s">
-        <v>677</v>
+        <v>680</v>
       </c>
       <c r="B74" s="15" t="s">
         <v>446</v>
@@ -6604,22 +6613,22 @@
         <v>671</v>
       </c>
       <c r="D74" s="15" t="s">
-        <v>678</v>
+        <v>681</v>
       </c>
       <c r="E74" s="15" t="s">
-        <v>679</v>
+        <v>682</v>
       </c>
       <c r="F74" s="15" t="s">
-        <v>680</v>
+        <v>683</v>
       </c>
       <c r="G74" s="15" t="s">
-        <v>681</v>
+        <v>684</v>
       </c>
       <c r="H74" s="15" t="s">
-        <v>682</v>
+        <v>685</v>
       </c>
       <c r="I74" s="15" t="s">
-        <v>683</v>
+        <v>686</v>
       </c>
       <c r="J74" s="15" t="s">
         <v>57</v>
@@ -6628,16 +6637,16 @@
         <v>1</v>
       </c>
       <c r="L74" s="15" t="s">
-        <v>684</v>
+        <v>687</v>
       </c>
       <c r="M74" s="15" t="s">
-        <v>685</v>
+        <v>688</v>
       </c>
       <c r="N74" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O74" s="15" t="s">
-        <v>686</v>
+        <v>689</v>
       </c>
       <c r="P74" s="15" t="s">
         <v>226</v>
@@ -6645,7 +6654,7 @@
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="15" t="s">
-        <v>687</v>
+        <v>690</v>
       </c>
       <c r="B75" s="15" t="s">
         <v>446</v>
@@ -6654,22 +6663,22 @@
         <v>671</v>
       </c>
       <c r="D75" s="15" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="E75" s="15" t="s">
-        <v>689</v>
+        <v>692</v>
       </c>
       <c r="F75" s="15" t="s">
-        <v>690</v>
+        <v>693</v>
       </c>
       <c r="G75" s="15" t="s">
-        <v>691</v>
+        <v>694</v>
       </c>
       <c r="H75" s="15" t="s">
-        <v>692</v>
+        <v>695</v>
       </c>
       <c r="I75" s="15" t="s">
-        <v>693</v>
+        <v>696</v>
       </c>
       <c r="J75" s="15" t="s">
         <v>57</v>
@@ -6678,16 +6687,16 @@
         <v>1</v>
       </c>
       <c r="L75" s="15" t="s">
-        <v>694</v>
+        <v>697</v>
       </c>
       <c r="M75" s="15" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="N75" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O75" s="15" t="s">
-        <v>696</v>
+        <v>699</v>
       </c>
       <c r="P75" s="15" t="s">
         <v>146</v>
@@ -6695,22 +6704,22 @@
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="15" t="s">
-        <v>697</v>
+        <v>700</v>
       </c>
       <c r="B76" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C76" s="15" t="s">
-        <v>698</v>
+        <v>701</v>
       </c>
       <c r="D76" s="15" t="s">
-        <v>699</v>
+        <v>702</v>
       </c>
       <c r="E76" s="15" t="s">
-        <v>700</v>
+        <v>703</v>
       </c>
       <c r="F76" s="15" t="s">
-        <v>701</v>
+        <v>704</v>
       </c>
       <c r="G76" s="15" t="s">
         <v>6</v>
@@ -6719,7 +6728,7 @@
         <v>6</v>
       </c>
       <c r="I76" s="15" t="s">
-        <v>702</v>
+        <v>705</v>
       </c>
       <c r="J76" s="15" t="s">
         <v>57</v>
@@ -6728,16 +6737,16 @@
         <v>1</v>
       </c>
       <c r="L76" s="15" t="s">
-        <v>703</v>
+        <v>706</v>
       </c>
       <c r="M76" s="15" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
       <c r="N76" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O76" s="15" t="s">
-        <v>705</v>
+        <v>708</v>
       </c>
       <c r="P76" s="15" t="s">
         <v>156</v>
@@ -6745,22 +6754,22 @@
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="15" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="B77" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C77" s="15" t="s">
-        <v>707</v>
+        <v>710</v>
       </c>
       <c r="D77" s="15" t="s">
-        <v>708</v>
+        <v>711</v>
       </c>
       <c r="E77" s="15" t="s">
         <v>6</v>
       </c>
       <c r="F77" s="15" t="s">
-        <v>709</v>
+        <v>712</v>
       </c>
       <c r="G77" s="15" t="s">
         <v>6</v>
@@ -6769,7 +6778,7 @@
         <v>6</v>
       </c>
       <c r="I77" s="15" t="s">
-        <v>710</v>
+        <v>713</v>
       </c>
       <c r="J77" s="15" t="s">
         <v>57</v>
@@ -6778,16 +6787,16 @@
         <v>1</v>
       </c>
       <c r="L77" s="15" t="s">
-        <v>711</v>
+        <v>714</v>
       </c>
       <c r="M77" s="15" t="s">
-        <v>712</v>
+        <v>715</v>
       </c>
       <c r="N77" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O77" s="15" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="P77" s="15" t="s">
         <v>191</v>
@@ -6795,31 +6804,31 @@
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="15" t="s">
-        <v>714</v>
+        <v>717</v>
       </c>
       <c r="B78" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C78" s="15" t="s">
-        <v>715</v>
+        <v>718</v>
       </c>
       <c r="D78" s="15" t="s">
-        <v>716</v>
+        <v>719</v>
       </c>
       <c r="E78" s="15" t="s">
         <v>6</v>
       </c>
       <c r="F78" s="15" t="s">
-        <v>717</v>
+        <v>720</v>
       </c>
       <c r="G78" s="15" t="s">
-        <v>718</v>
+        <v>721</v>
       </c>
       <c r="H78" s="15" t="s">
         <v>6</v>
       </c>
       <c r="I78" s="15" t="s">
-        <v>719</v>
+        <v>722</v>
       </c>
       <c r="J78" s="15" t="s">
         <v>57</v>
@@ -6828,16 +6837,16 @@
         <v>1</v>
       </c>
       <c r="L78" s="15" t="s">
-        <v>720</v>
+        <v>723</v>
       </c>
       <c r="M78" s="15" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
       <c r="N78" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O78" s="15" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="P78" s="15" t="s">
         <v>169</v>
@@ -6845,31 +6854,31 @@
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="15" t="s">
-        <v>723</v>
+        <v>726</v>
       </c>
       <c r="B79" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C79" s="15" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
       <c r="D79" s="15" t="s">
-        <v>725</v>
+        <v>728</v>
       </c>
       <c r="E79" s="15" t="s">
-        <v>726</v>
+        <v>729</v>
       </c>
       <c r="F79" s="15" t="s">
-        <v>727</v>
+        <v>730</v>
       </c>
       <c r="G79" s="15" t="s">
         <v>451</v>
       </c>
       <c r="H79" s="15" t="s">
-        <v>728</v>
+        <v>731</v>
       </c>
       <c r="I79" s="15" t="s">
-        <v>729</v>
+        <v>732</v>
       </c>
       <c r="J79" s="15" t="s">
         <v>57</v>
@@ -6878,16 +6887,16 @@
         <v>1</v>
       </c>
       <c r="L79" s="15" t="s">
-        <v>730</v>
+        <v>733</v>
       </c>
       <c r="M79" s="15" t="s">
-        <v>731</v>
+        <v>734</v>
       </c>
       <c r="N79" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O79" s="15" t="s">
-        <v>732</v>
+        <v>735</v>
       </c>
       <c r="P79" s="15" t="s">
         <v>156</v>
@@ -6895,16 +6904,16 @@
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="15" t="s">
-        <v>733</v>
+        <v>736</v>
       </c>
       <c r="B80" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C80" s="15" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
       <c r="D80" s="15" t="s">
-        <v>734</v>
+        <v>737</v>
       </c>
       <c r="E80" s="15" t="s">
         <v>6</v>
@@ -6919,7 +6928,7 @@
         <v>6</v>
       </c>
       <c r="I80" s="15" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="J80" s="15" t="s">
         <v>57</v>
@@ -6928,16 +6937,16 @@
         <v>1</v>
       </c>
       <c r="L80" s="15" t="s">
-        <v>736</v>
+        <v>739</v>
       </c>
       <c r="M80" s="15" t="s">
-        <v>737</v>
+        <v>740</v>
       </c>
       <c r="N80" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O80" s="15" t="s">
-        <v>738</v>
+        <v>741</v>
       </c>
       <c r="P80" s="15" t="s">
         <v>226</v>
@@ -6945,19 +6954,19 @@
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="15" t="s">
-        <v>739</v>
+        <v>742</v>
       </c>
       <c r="B81" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C81" s="15" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
       <c r="D81" s="15" t="s">
-        <v>740</v>
+        <v>743</v>
       </c>
       <c r="E81" s="15" t="s">
-        <v>741</v>
+        <v>744</v>
       </c>
       <c r="F81" s="15" t="s">
         <v>6</v>
@@ -6969,7 +6978,7 @@
         <v>6</v>
       </c>
       <c r="I81" s="15" t="s">
-        <v>742</v>
+        <v>745</v>
       </c>
       <c r="J81" s="15" t="s">
         <v>57</v>
@@ -6978,16 +6987,16 @@
         <v>1</v>
       </c>
       <c r="L81" s="15" t="s">
-        <v>743</v>
+        <v>746</v>
       </c>
       <c r="M81" s="15" t="s">
-        <v>744</v>
+        <v>747</v>
       </c>
       <c r="N81" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O81" s="15" t="s">
-        <v>745</v>
+        <v>748</v>
       </c>
       <c r="P81" s="15" t="s">
         <v>391</v>
@@ -6995,31 +7004,31 @@
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="15" t="s">
-        <v>746</v>
+        <v>749</v>
       </c>
       <c r="B82" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C82" s="15" t="s">
-        <v>747</v>
+        <v>750</v>
       </c>
       <c r="D82" s="15" t="s">
-        <v>748</v>
+        <v>751</v>
       </c>
       <c r="E82" s="15" t="s">
-        <v>749</v>
+        <v>752</v>
       </c>
       <c r="F82" s="15" t="s">
-        <v>750</v>
+        <v>753</v>
       </c>
       <c r="G82" s="15" t="s">
-        <v>751</v>
+        <v>754</v>
       </c>
       <c r="H82" s="15" t="s">
-        <v>752</v>
+        <v>755</v>
       </c>
       <c r="I82" s="15" t="s">
-        <v>753</v>
+        <v>756</v>
       </c>
       <c r="J82" s="15" t="s">
         <v>57</v>
@@ -7028,16 +7037,16 @@
         <v>1</v>
       </c>
       <c r="L82" s="15" t="s">
-        <v>754</v>
+        <v>757</v>
       </c>
       <c r="M82" s="15" t="s">
-        <v>755</v>
+        <v>758</v>
       </c>
       <c r="N82" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O82" s="15" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="P82" s="15" t="s">
         <v>391</v>
@@ -7045,31 +7054,31 @@
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="15" t="s">
-        <v>757</v>
+        <v>760</v>
       </c>
       <c r="B83" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C83" s="15" t="s">
-        <v>758</v>
+        <v>761</v>
       </c>
       <c r="D83" s="15" t="s">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="E83" s="15" t="s">
-        <v>760</v>
+        <v>763</v>
       </c>
       <c r="F83" s="15" t="s">
-        <v>761</v>
+        <v>764</v>
       </c>
       <c r="G83" s="15" t="s">
-        <v>751</v>
+        <v>754</v>
       </c>
       <c r="H83" s="15" t="s">
-        <v>762</v>
+        <v>765</v>
       </c>
       <c r="I83" s="15" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
       <c r="J83" s="15" t="s">
         <v>57</v>
@@ -7081,13 +7090,13 @@
         <v>541</v>
       </c>
       <c r="M83" s="15" t="s">
-        <v>764</v>
+        <v>767</v>
       </c>
       <c r="N83" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O83" s="15" t="s">
-        <v>765</v>
+        <v>768</v>
       </c>
       <c r="P83" s="15" t="s">
         <v>146</v>
@@ -7095,31 +7104,31 @@
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="15" t="s">
-        <v>766</v>
+        <v>769</v>
       </c>
       <c r="B84" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C84" s="15" t="s">
-        <v>758</v>
+        <v>761</v>
       </c>
       <c r="D84" s="15" t="s">
-        <v>767</v>
+        <v>770</v>
       </c>
       <c r="E84" s="15" t="s">
         <v>493</v>
       </c>
       <c r="F84" s="15" t="s">
-        <v>768</v>
+        <v>771</v>
       </c>
       <c r="G84" s="15" t="s">
-        <v>769</v>
+        <v>772</v>
       </c>
       <c r="H84" s="15" t="s">
-        <v>770</v>
+        <v>773</v>
       </c>
       <c r="I84" s="15" t="s">
-        <v>771</v>
+        <v>774</v>
       </c>
       <c r="J84" s="15" t="s">
         <v>57</v>
@@ -7128,16 +7137,16 @@
         <v>1</v>
       </c>
       <c r="L84" s="15" t="s">
-        <v>772</v>
+        <v>775</v>
       </c>
       <c r="M84" s="15" t="s">
-        <v>773</v>
+        <v>776</v>
       </c>
       <c r="N84" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O84" s="15" t="s">
-        <v>774</v>
+        <v>777</v>
       </c>
       <c r="P84" s="15" t="s">
         <v>226</v>
@@ -7145,31 +7154,31 @@
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="15" t="s">
-        <v>775</v>
+        <v>778</v>
       </c>
       <c r="B85" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C85" s="15" t="s">
-        <v>758</v>
+        <v>761</v>
       </c>
       <c r="D85" s="15" t="s">
-        <v>776</v>
+        <v>779</v>
       </c>
       <c r="E85" s="15" t="s">
-        <v>777</v>
+        <v>780</v>
       </c>
       <c r="F85" s="15" t="s">
-        <v>778</v>
+        <v>781</v>
       </c>
       <c r="G85" s="15" t="s">
-        <v>779</v>
+        <v>782</v>
       </c>
       <c r="H85" s="15" t="s">
-        <v>780</v>
+        <v>783</v>
       </c>
       <c r="I85" s="15" t="s">
-        <v>781</v>
+        <v>784</v>
       </c>
       <c r="J85" s="15" t="s">
         <v>57</v>
@@ -7178,16 +7187,16 @@
         <v>1</v>
       </c>
       <c r="L85" s="15" t="s">
-        <v>782</v>
+        <v>785</v>
       </c>
       <c r="M85" s="15" t="s">
-        <v>783</v>
+        <v>786</v>
       </c>
       <c r="N85" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O85" s="15" t="s">
-        <v>784</v>
+        <v>787</v>
       </c>
       <c r="P85" s="15" t="s">
         <v>391</v>
@@ -7195,22 +7204,22 @@
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="15" t="s">
-        <v>785</v>
+        <v>788</v>
       </c>
       <c r="B86" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C86" s="15" t="s">
-        <v>786</v>
+        <v>789</v>
       </c>
       <c r="D86" s="15" t="s">
-        <v>787</v>
+        <v>790</v>
       </c>
       <c r="E86" s="15" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="F86" s="15" t="s">
-        <v>789</v>
+        <v>792</v>
       </c>
       <c r="G86" s="15" t="s">
         <v>6</v>
@@ -7219,7 +7228,7 @@
         <v>605</v>
       </c>
       <c r="I86" s="15" t="s">
-        <v>790</v>
+        <v>793</v>
       </c>
       <c r="J86" s="15" t="s">
         <v>57</v>
@@ -7228,16 +7237,16 @@
         <v>1</v>
       </c>
       <c r="L86" s="15" t="s">
-        <v>791</v>
+        <v>794</v>
       </c>
       <c r="M86" s="15" t="s">
-        <v>792</v>
+        <v>795</v>
       </c>
       <c r="N86" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O86" s="15" t="s">
-        <v>793</v>
+        <v>796</v>
       </c>
       <c r="P86" s="15" t="s">
         <v>146</v>
@@ -7245,31 +7254,31 @@
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="15" t="s">
-        <v>794</v>
+        <v>797</v>
       </c>
       <c r="B87" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C87" s="15" t="s">
-        <v>786</v>
+        <v>789</v>
       </c>
       <c r="D87" s="15" t="s">
-        <v>795</v>
+        <v>798</v>
       </c>
       <c r="E87" s="15" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="F87" s="15" t="s">
-        <v>796</v>
+        <v>799</v>
       </c>
       <c r="G87" s="15" t="s">
         <v>6</v>
       </c>
       <c r="H87" s="15" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="I87" s="15" t="s">
-        <v>798</v>
+        <v>801</v>
       </c>
       <c r="J87" s="15" t="s">
         <v>57</v>
@@ -7278,16 +7287,16 @@
         <v>1</v>
       </c>
       <c r="L87" s="15" t="s">
-        <v>799</v>
+        <v>802</v>
       </c>
       <c r="M87" s="15" t="s">
-        <v>800</v>
+        <v>803</v>
       </c>
       <c r="N87" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O87" s="15" t="s">
-        <v>801</v>
+        <v>804</v>
       </c>
       <c r="P87" s="15" t="s">
         <v>169</v>
@@ -7295,31 +7304,31 @@
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="15" t="s">
-        <v>802</v>
+        <v>805</v>
       </c>
       <c r="B88" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C88" s="15" t="s">
-        <v>803</v>
+        <v>806</v>
       </c>
       <c r="D88" s="15" t="s">
-        <v>804</v>
+        <v>807</v>
       </c>
       <c r="E88" s="15" t="s">
-        <v>805</v>
+        <v>808</v>
       </c>
       <c r="F88" s="15" t="s">
-        <v>806</v>
+        <v>809</v>
       </c>
       <c r="G88" s="15" t="s">
         <v>6</v>
       </c>
       <c r="H88" s="15" t="s">
-        <v>807</v>
+        <v>810</v>
       </c>
       <c r="I88" s="15" t="s">
-        <v>808</v>
+        <v>811</v>
       </c>
       <c r="J88" s="15" t="s">
         <v>57</v>
@@ -7328,16 +7337,16 @@
         <v>1</v>
       </c>
       <c r="L88" s="15" t="s">
-        <v>809</v>
+        <v>812</v>
       </c>
       <c r="M88" s="15" t="s">
-        <v>810</v>
+        <v>813</v>
       </c>
       <c r="N88" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O88" s="15" t="s">
-        <v>811</v>
+        <v>814</v>
       </c>
       <c r="P88" s="15" t="s">
         <v>169</v>
@@ -7345,31 +7354,31 @@
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="15" t="s">
-        <v>812</v>
+        <v>815</v>
       </c>
       <c r="B89" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C89" s="15" t="s">
-        <v>813</v>
+        <v>816</v>
       </c>
       <c r="D89" s="15" t="s">
-        <v>814</v>
+        <v>817</v>
       </c>
       <c r="E89" s="15" t="s">
         <v>6</v>
       </c>
       <c r="F89" s="15" t="s">
-        <v>815</v>
+        <v>818</v>
       </c>
       <c r="G89" s="15" t="s">
         <v>6</v>
       </c>
       <c r="H89" s="15" t="s">
-        <v>816</v>
+        <v>819</v>
       </c>
       <c r="I89" s="15" t="s">
-        <v>817</v>
+        <v>820</v>
       </c>
       <c r="J89" s="15" t="s">
         <v>57</v>
@@ -7378,16 +7387,16 @@
         <v>1</v>
       </c>
       <c r="L89" s="15" t="s">
-        <v>818</v>
+        <v>821</v>
       </c>
       <c r="M89" s="15" t="s">
-        <v>819</v>
+        <v>822</v>
       </c>
       <c r="N89" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O89" s="15" t="s">
-        <v>820</v>
+        <v>823</v>
       </c>
       <c r="P89" s="15" t="s">
         <v>432</v>
@@ -7395,31 +7404,31 @@
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="15" t="s">
-        <v>821</v>
+        <v>824</v>
       </c>
       <c r="B90" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C90" s="15" t="s">
-        <v>822</v>
+        <v>825</v>
       </c>
       <c r="D90" s="15" t="s">
-        <v>823</v>
+        <v>826</v>
       </c>
       <c r="E90" s="15" t="s">
-        <v>824</v>
+        <v>827</v>
       </c>
       <c r="F90" s="15" t="s">
-        <v>825</v>
+        <v>828</v>
       </c>
       <c r="G90" s="15" t="s">
-        <v>751</v>
+        <v>754</v>
       </c>
       <c r="H90" s="15" t="s">
-        <v>826</v>
+        <v>829</v>
       </c>
       <c r="I90" s="15" t="s">
-        <v>827</v>
+        <v>830</v>
       </c>
       <c r="J90" s="15" t="s">
         <v>57</v>
@@ -7428,16 +7437,16 @@
         <v>1</v>
       </c>
       <c r="L90" s="15" t="s">
-        <v>828</v>
+        <v>831</v>
       </c>
       <c r="M90" s="15" t="s">
-        <v>829</v>
+        <v>832</v>
       </c>
       <c r="N90" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O90" s="15" t="s">
-        <v>830</v>
+        <v>833</v>
       </c>
       <c r="P90" s="15" t="s">
         <v>169</v>
@@ -7445,16 +7454,16 @@
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="15" t="s">
-        <v>831</v>
+        <v>834</v>
       </c>
       <c r="B91" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C91" s="15" t="s">
-        <v>832</v>
+        <v>835</v>
       </c>
       <c r="D91" s="15" t="s">
-        <v>833</v>
+        <v>836</v>
       </c>
       <c r="E91" s="15" t="s">
         <v>6</v>
@@ -7469,7 +7478,7 @@
         <v>6</v>
       </c>
       <c r="I91" s="15" t="s">
-        <v>834</v>
+        <v>837</v>
       </c>
       <c r="J91" s="15" t="s">
         <v>57</v>
@@ -7478,16 +7487,16 @@
         <v>1</v>
       </c>
       <c r="L91" s="15" t="s">
-        <v>835</v>
+        <v>838</v>
       </c>
       <c r="M91" s="15" t="s">
-        <v>836</v>
+        <v>839</v>
       </c>
       <c r="N91" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O91" s="15" t="s">
-        <v>837</v>
+        <v>840</v>
       </c>
       <c r="P91" s="15" t="s">
         <v>226</v>
@@ -7495,31 +7504,31 @@
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="15" t="s">
-        <v>838</v>
+        <v>841</v>
       </c>
       <c r="B92" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C92" s="15" t="s">
-        <v>839</v>
+        <v>842</v>
       </c>
       <c r="D92" s="15" t="s">
-        <v>840</v>
+        <v>843</v>
       </c>
       <c r="E92" s="15" t="s">
-        <v>841</v>
+        <v>844</v>
       </c>
       <c r="F92" s="15" t="s">
-        <v>842</v>
+        <v>845</v>
       </c>
       <c r="G92" s="15" t="s">
         <v>451</v>
       </c>
       <c r="H92" s="15" t="s">
-        <v>843</v>
+        <v>846</v>
       </c>
       <c r="I92" s="15" t="s">
-        <v>844</v>
+        <v>847</v>
       </c>
       <c r="J92" s="15" t="s">
         <v>57</v>
@@ -7528,16 +7537,16 @@
         <v>1</v>
       </c>
       <c r="L92" s="15" t="s">
-        <v>845</v>
+        <v>848</v>
       </c>
       <c r="M92" s="15" t="s">
-        <v>846</v>
+        <v>849</v>
       </c>
       <c r="N92" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O92" s="15" t="s">
-        <v>847</v>
+        <v>850</v>
       </c>
       <c r="P92" s="15" t="s">
         <v>391</v>
@@ -7545,31 +7554,31 @@
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="15" t="s">
-        <v>848</v>
+        <v>851</v>
       </c>
       <c r="B93" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C93" s="15" t="s">
-        <v>849</v>
+        <v>852</v>
       </c>
       <c r="D93" s="15" t="s">
-        <v>850</v>
+        <v>853</v>
       </c>
       <c r="E93" s="15" t="s">
-        <v>851</v>
+        <v>854</v>
       </c>
       <c r="F93" s="15" t="s">
-        <v>852</v>
+        <v>855</v>
       </c>
       <c r="G93" s="15" t="s">
         <v>451</v>
       </c>
       <c r="H93" s="15" t="s">
-        <v>853</v>
+        <v>856</v>
       </c>
       <c r="I93" s="15" t="s">
-        <v>854</v>
+        <v>857</v>
       </c>
       <c r="J93" s="15" t="s">
         <v>57</v>
@@ -7578,16 +7587,16 @@
         <v>1</v>
       </c>
       <c r="L93" s="15" t="s">
-        <v>855</v>
+        <v>858</v>
       </c>
       <c r="M93" s="15" t="s">
-        <v>856</v>
+        <v>859</v>
       </c>
       <c r="N93" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O93" s="15" t="s">
-        <v>857</v>
+        <v>860</v>
       </c>
       <c r="P93" s="15" t="s">
         <v>391</v>
@@ -7595,16 +7604,16 @@
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="12" t="s">
-        <v>858</v>
+        <v>861</v>
       </c>
       <c r="B94" s="12" t="s">
-        <v>859</v>
+        <v>862</v>
       </c>
       <c r="C94" s="12" t="s">
         <v>447</v>
       </c>
       <c r="D94" s="12" t="s">
-        <v>860</v>
+        <v>863</v>
       </c>
       <c r="E94" s="12" t="s">
         <v>6</v>
@@ -7619,25 +7628,25 @@
         <v>6</v>
       </c>
       <c r="I94" s="12" t="s">
-        <v>861</v>
+        <v>864</v>
       </c>
       <c r="J94" s="12" t="s">
-        <v>862</v>
+        <v>865</v>
       </c>
       <c r="K94" s="12" t="s">
         <v>91</v>
       </c>
       <c r="L94" s="12" t="s">
-        <v>863</v>
+        <v>866</v>
       </c>
       <c r="M94" s="12" t="s">
-        <v>864</v>
+        <v>867</v>
       </c>
       <c r="N94" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O94" s="12" t="s">
-        <v>865</v>
+        <v>868</v>
       </c>
       <c r="P94" s="12" t="s">
         <v>226</v>
@@ -7645,16 +7654,16 @@
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="12" t="s">
-        <v>866</v>
+        <v>869</v>
       </c>
       <c r="B95" s="12" t="s">
         <v>446</v>
       </c>
       <c r="C95" s="12" t="s">
-        <v>867</v>
+        <v>870</v>
       </c>
       <c r="D95" s="12" t="s">
-        <v>868</v>
+        <v>871</v>
       </c>
       <c r="E95" s="12" t="s">
         <v>6</v>
@@ -7669,7 +7678,7 @@
         <v>6</v>
       </c>
       <c r="I95" s="12" t="s">
-        <v>869</v>
+        <v>872</v>
       </c>
       <c r="J95" s="12" t="s">
         <v>46</v>
@@ -7678,16 +7687,16 @@
         <v>91</v>
       </c>
       <c r="L95" s="12" t="s">
-        <v>870</v>
+        <v>873</v>
       </c>
       <c r="M95" s="12" t="s">
-        <v>871</v>
+        <v>874</v>
       </c>
       <c r="N95" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O95" s="12" t="s">
-        <v>872</v>
+        <v>875</v>
       </c>
       <c r="P95" s="12" t="s">
         <v>169</v>
@@ -7695,16 +7704,16 @@
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="12" t="s">
-        <v>873</v>
+        <v>876</v>
       </c>
       <c r="B96" s="12" t="s">
         <v>446</v>
       </c>
       <c r="C96" s="12" t="s">
-        <v>874</v>
+        <v>877</v>
       </c>
       <c r="D96" s="12" t="s">
-        <v>875</v>
+        <v>878</v>
       </c>
       <c r="E96" s="12" t="s">
         <v>6</v>
@@ -7719,7 +7728,7 @@
         <v>6</v>
       </c>
       <c r="I96" s="12" t="s">
-        <v>876</v>
+        <v>879</v>
       </c>
       <c r="J96" s="12" t="s">
         <v>46</v>
@@ -7728,16 +7737,16 @@
         <v>91</v>
       </c>
       <c r="L96" s="12" t="s">
-        <v>877</v>
+        <v>880</v>
       </c>
       <c r="M96" s="12" t="s">
-        <v>878</v>
+        <v>881</v>
       </c>
       <c r="N96" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O96" s="12" t="s">
-        <v>879</v>
+        <v>882</v>
       </c>
       <c r="P96" s="12" t="s">
         <v>156</v>
@@ -7745,16 +7754,16 @@
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="13" t="s">
-        <v>880</v>
+        <v>883</v>
       </c>
       <c r="B97" s="13" t="s">
-        <v>881</v>
+        <v>884</v>
       </c>
       <c r="C97" s="13" t="s">
-        <v>882</v>
+        <v>885</v>
       </c>
       <c r="D97" s="13" t="s">
-        <v>883</v>
+        <v>886</v>
       </c>
       <c r="E97" s="13" t="s">
         <v>6</v>
@@ -7769,25 +7778,25 @@
         <v>6</v>
       </c>
       <c r="I97" s="13" t="s">
-        <v>884</v>
+        <v>887</v>
       </c>
       <c r="J97" s="13" t="s">
-        <v>885</v>
+        <v>888</v>
       </c>
       <c r="K97" s="13" t="s">
         <v>47</v>
       </c>
       <c r="L97" s="13" t="s">
-        <v>886</v>
+        <v>889</v>
       </c>
       <c r="M97" s="13" t="s">
-        <v>887</v>
+        <v>890</v>
       </c>
       <c r="N97" s="13" t="s">
-        <v>888</v>
+        <v>891</v>
       </c>
       <c r="O97" s="13" t="s">
-        <v>889</v>
+        <v>892</v>
       </c>
       <c r="P97" s="13" t="s">
         <v>242</v>

</xml_diff>

<commit_message>
qa backup - event feedback
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1552" uniqueCount="893">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1552" uniqueCount="894">
   <si>
     <t>LEGEND</t>
   </si>
@@ -2065,7 +2065,7 @@
     <t>EVENT-FEEDBACK-002</t>
   </si>
   <si>
-    <t>Submit one controlled event feedback response</t>
+    <t>Submit one controlled event feedback response with an optional event opinion</t>
   </si>
   <si>
     <t>DELTA event feedback activity after snapshot</t>
@@ -2080,16 +2080,19 @@
     <t>DELTA affinity recompute; first-submit outbox</t>
   </si>
   <si>
-    <t>Submitted item, organizer received view and recipient notification agree</t>
-  </si>
-  <si>
-    <t>Feedback submit service tests</t>
-  </si>
-  <si>
-    <t>Match persisted answers, state, target IDs and first-submit notification</t>
-  </si>
-  <si>
-    <t>Continue to EVENT-IMPRESSION-001 for profile propagation</t>
+    <t>Before submit, Activities Event card, feedback-list card and feedback form use the same persisted image on both backend HTTP and frontend local/demo paths; when image is empty all three use neutral placeholders with no runtime stock photo. The first event page accepts an optional event opinion up to 160 characters. View my feedback and the organizer received view show that opinion separately from any note to organizer; submitted item and recipient notification agree</t>
+  </si>
+  <si>
+    <t>IN PROGRESS</t>
+  </si>
+  <si>
+    <t>Feedback submit service coverage; empty-image list/detail regressions added; event-opinion persistence/limit/view regressions authored but not separately run</t>
+  </si>
+  <si>
+    <t>Upload the generated event-feedback-002-cover.png fixture through the normal HTTP media endpoint, stage its returned canonical URL on the dedicated past event with the accepted participant, and do not repeat Event Editor. Compare the Activities Event source card against feedback list/form image semantics, then match persisted answers including eventComment, state, exact main/four-bucket counters, target IDs and first-submit notification</t>
+  </si>
+  <si>
+    <t>The original structured submission and post-submit oracle passed. The new event-opinion acceptance step still requires a fresh UI submission; feedback mapping must never manufacture an image or merge eventComment with organizerNote. Continue to EVENT-IMPRESSION-001 only after this visible proof.</t>
   </si>
   <si>
     <t>EVENT-FEEDBACK-003</t>
@@ -2155,19 +2158,19 @@
     <t>Event feedback metadata</t>
   </si>
   <si>
-    <t>Save and reopen one organizer note</t>
+    <t>Save and reopen one participant note to the organizer</t>
   </si>
   <si>
     <t>INDIRECT received-feedback counter refresh only</t>
   </si>
   <si>
-    <t>Exact note persists; participant answers and profile traits remain unchanged</t>
-  </si>
-  <si>
-    <t>Feedback note access tests partial</t>
-  </si>
-  <si>
-    <t>Use one unique note and unchanged answer/task controls</t>
+    <t>Add/Edit note remains available after feedback submission. The exact note persists in feedback state; View my feedback and the organizer received view show it separately from the event opinion; participant answers and profile traits remain unchanged</t>
+  </si>
+  <si>
+    <t>Feedback note access tests partial; submitted-card note action and separate viewer fields added</t>
+  </si>
+  <si>
+    <t>Use one unique note and unchanged answer/task controls; compare participant and organizer viewer text exactly</t>
   </si>
   <si>
     <t>No scheduler is part of this checkpoint</t>
@@ -6603,58 +6606,58 @@
       </c>
     </row>
     <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="15" t="s">
+      <c r="A74" s="0" t="s">
         <v>680</v>
       </c>
-      <c r="B74" s="15" t="s">
+      <c r="B74" s="0" t="s">
         <v>446</v>
       </c>
-      <c r="C74" s="15" t="s">
+      <c r="C74" s="0" t="s">
         <v>671</v>
       </c>
-      <c r="D74" s="15" t="s">
+      <c r="D74" s="0" t="s">
         <v>681</v>
       </c>
-      <c r="E74" s="15" t="s">
+      <c r="E74" s="0" t="s">
         <v>682</v>
       </c>
-      <c r="F74" s="15" t="s">
+      <c r="F74" s="0" t="s">
         <v>683</v>
       </c>
-      <c r="G74" s="15" t="s">
+      <c r="G74" s="0" t="s">
         <v>684</v>
       </c>
-      <c r="H74" s="15" t="s">
+      <c r="H74" s="0" t="s">
         <v>685</v>
       </c>
-      <c r="I74" s="15" t="s">
+      <c r="I74" s="0" t="s">
         <v>686</v>
       </c>
-      <c r="J74" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="K74" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="L74" s="15" t="s">
+      <c r="J74" s="0" t="s">
         <v>687</v>
       </c>
-      <c r="M74" s="15" t="s">
+      <c r="K74" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="L74" s="0" t="s">
         <v>688</v>
       </c>
-      <c r="N74" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="O74" s="15" t="s">
+      <c r="M74" s="0" t="s">
         <v>689</v>
       </c>
-      <c r="P74" s="15" t="s">
+      <c r="N74" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="O74" s="0" t="s">
+        <v>690</v>
+      </c>
+      <c r="P74" s="0" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="15" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="B75" s="15" t="s">
         <v>446</v>
@@ -6663,22 +6666,22 @@
         <v>671</v>
       </c>
       <c r="D75" s="15" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="E75" s="15" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="F75" s="15" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="G75" s="15" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="H75" s="15" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="I75" s="15" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="J75" s="15" t="s">
         <v>57</v>
@@ -6687,16 +6690,16 @@
         <v>1</v>
       </c>
       <c r="L75" s="15" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="M75" s="15" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="N75" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O75" s="15" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="P75" s="15" t="s">
         <v>146</v>
@@ -6704,22 +6707,22 @@
     </row>
     <row r="76" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="15" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B76" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C76" s="15" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="D76" s="15" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="E76" s="15" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="F76" s="15" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="G76" s="15" t="s">
         <v>6</v>
@@ -6728,7 +6731,7 @@
         <v>6</v>
       </c>
       <c r="I76" s="15" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="J76" s="15" t="s">
         <v>57</v>
@@ -6737,16 +6740,16 @@
         <v>1</v>
       </c>
       <c r="L76" s="15" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="M76" s="15" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="N76" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O76" s="15" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="P76" s="15" t="s">
         <v>156</v>
@@ -6754,22 +6757,22 @@
     </row>
     <row r="77" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="15" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B77" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C77" s="15" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="D77" s="15" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="E77" s="15" t="s">
         <v>6</v>
       </c>
       <c r="F77" s="15" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="G77" s="15" t="s">
         <v>6</v>
@@ -6778,7 +6781,7 @@
         <v>6</v>
       </c>
       <c r="I77" s="15" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="J77" s="15" t="s">
         <v>57</v>
@@ -6787,16 +6790,16 @@
         <v>1</v>
       </c>
       <c r="L77" s="15" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="M77" s="15" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="N77" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O77" s="15" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="P77" s="15" t="s">
         <v>191</v>
@@ -6804,31 +6807,31 @@
     </row>
     <row r="78" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="15" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="B78" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C78" s="15" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="D78" s="15" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="E78" s="15" t="s">
         <v>6</v>
       </c>
       <c r="F78" s="15" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="G78" s="15" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="H78" s="15" t="s">
         <v>6</v>
       </c>
       <c r="I78" s="15" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="J78" s="15" t="s">
         <v>57</v>
@@ -6837,16 +6840,16 @@
         <v>1</v>
       </c>
       <c r="L78" s="15" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="M78" s="15" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="N78" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O78" s="15" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="P78" s="15" t="s">
         <v>169</v>
@@ -6854,31 +6857,31 @@
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="15" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B79" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C79" s="15" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="D79" s="15" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="E79" s="15" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="F79" s="15" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="G79" s="15" t="s">
         <v>451</v>
       </c>
       <c r="H79" s="15" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="I79" s="15" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="J79" s="15" t="s">
         <v>57</v>
@@ -6887,16 +6890,16 @@
         <v>1</v>
       </c>
       <c r="L79" s="15" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="M79" s="15" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="N79" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O79" s="15" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="P79" s="15" t="s">
         <v>156</v>
@@ -6904,16 +6907,16 @@
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="15" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="B80" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C80" s="15" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="D80" s="15" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="E80" s="15" t="s">
         <v>6</v>
@@ -6928,7 +6931,7 @@
         <v>6</v>
       </c>
       <c r="I80" s="15" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="J80" s="15" t="s">
         <v>57</v>
@@ -6937,16 +6940,16 @@
         <v>1</v>
       </c>
       <c r="L80" s="15" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="M80" s="15" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="N80" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O80" s="15" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="P80" s="15" t="s">
         <v>226</v>
@@ -6954,19 +6957,19 @@
     </row>
     <row r="81" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="15" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="B81" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C81" s="15" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="D81" s="15" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="E81" s="15" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="F81" s="15" t="s">
         <v>6</v>
@@ -6978,7 +6981,7 @@
         <v>6</v>
       </c>
       <c r="I81" s="15" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="J81" s="15" t="s">
         <v>57</v>
@@ -6987,16 +6990,16 @@
         <v>1</v>
       </c>
       <c r="L81" s="15" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="M81" s="15" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="N81" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O81" s="15" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="P81" s="15" t="s">
         <v>391</v>
@@ -7004,31 +7007,31 @@
     </row>
     <row r="82" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="15" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B82" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C82" s="15" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="D82" s="15" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="E82" s="15" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="F82" s="15" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="G82" s="15" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="H82" s="15" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="I82" s="15" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="J82" s="15" t="s">
         <v>57</v>
@@ -7037,16 +7040,16 @@
         <v>1</v>
       </c>
       <c r="L82" s="15" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="M82" s="15" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="N82" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O82" s="15" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="P82" s="15" t="s">
         <v>391</v>
@@ -7054,31 +7057,31 @@
     </row>
     <row r="83" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="15" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="B83" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C83" s="15" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="D83" s="15" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
       <c r="E83" s="15" t="s">
-        <v>763</v>
+        <v>764</v>
       </c>
       <c r="F83" s="15" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="G83" s="15" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="H83" s="15" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="I83" s="15" t="s">
-        <v>766</v>
+        <v>767</v>
       </c>
       <c r="J83" s="15" t="s">
         <v>57</v>
@@ -7090,13 +7093,13 @@
         <v>541</v>
       </c>
       <c r="M83" s="15" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="N83" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O83" s="15" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="P83" s="15" t="s">
         <v>146</v>
@@ -7104,31 +7107,31 @@
     </row>
     <row r="84" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="15" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="B84" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C84" s="15" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="D84" s="15" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="E84" s="15" t="s">
         <v>493</v>
       </c>
       <c r="F84" s="15" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="G84" s="15" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="H84" s="15" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="I84" s="15" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="J84" s="15" t="s">
         <v>57</v>
@@ -7137,16 +7140,16 @@
         <v>1</v>
       </c>
       <c r="L84" s="15" t="s">
-        <v>775</v>
+        <v>776</v>
       </c>
       <c r="M84" s="15" t="s">
-        <v>776</v>
+        <v>777</v>
       </c>
       <c r="N84" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O84" s="15" t="s">
-        <v>777</v>
+        <v>778</v>
       </c>
       <c r="P84" s="15" t="s">
         <v>226</v>
@@ -7154,31 +7157,31 @@
     </row>
     <row r="85" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="15" t="s">
-        <v>778</v>
+        <v>779</v>
       </c>
       <c r="B85" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C85" s="15" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="D85" s="15" t="s">
-        <v>779</v>
+        <v>780</v>
       </c>
       <c r="E85" s="15" t="s">
-        <v>780</v>
+        <v>781</v>
       </c>
       <c r="F85" s="15" t="s">
-        <v>781</v>
+        <v>782</v>
       </c>
       <c r="G85" s="15" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
       <c r="H85" s="15" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="I85" s="15" t="s">
-        <v>784</v>
+        <v>785</v>
       </c>
       <c r="J85" s="15" t="s">
         <v>57</v>
@@ -7187,16 +7190,16 @@
         <v>1</v>
       </c>
       <c r="L85" s="15" t="s">
-        <v>785</v>
+        <v>786</v>
       </c>
       <c r="M85" s="15" t="s">
-        <v>786</v>
+        <v>787</v>
       </c>
       <c r="N85" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O85" s="15" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="P85" s="15" t="s">
         <v>391</v>
@@ -7204,22 +7207,22 @@
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="15" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="B86" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C86" s="15" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="D86" s="15" t="s">
-        <v>790</v>
+        <v>791</v>
       </c>
       <c r="E86" s="15" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="F86" s="15" t="s">
-        <v>792</v>
+        <v>793</v>
       </c>
       <c r="G86" s="15" t="s">
         <v>6</v>
@@ -7228,7 +7231,7 @@
         <v>605</v>
       </c>
       <c r="I86" s="15" t="s">
-        <v>793</v>
+        <v>794</v>
       </c>
       <c r="J86" s="15" t="s">
         <v>57</v>
@@ -7237,16 +7240,16 @@
         <v>1</v>
       </c>
       <c r="L86" s="15" t="s">
-        <v>794</v>
+        <v>795</v>
       </c>
       <c r="M86" s="15" t="s">
-        <v>795</v>
+        <v>796</v>
       </c>
       <c r="N86" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O86" s="15" t="s">
-        <v>796</v>
+        <v>797</v>
       </c>
       <c r="P86" s="15" t="s">
         <v>146</v>
@@ -7254,31 +7257,31 @@
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="15" t="s">
-        <v>797</v>
+        <v>798</v>
       </c>
       <c r="B87" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C87" s="15" t="s">
-        <v>789</v>
+        <v>790</v>
       </c>
       <c r="D87" s="15" t="s">
-        <v>798</v>
+        <v>799</v>
       </c>
       <c r="E87" s="15" t="s">
-        <v>791</v>
+        <v>792</v>
       </c>
       <c r="F87" s="15" t="s">
-        <v>799</v>
+        <v>800</v>
       </c>
       <c r="G87" s="15" t="s">
         <v>6</v>
       </c>
       <c r="H87" s="15" t="s">
-        <v>800</v>
+        <v>801</v>
       </c>
       <c r="I87" s="15" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="J87" s="15" t="s">
         <v>57</v>
@@ -7287,16 +7290,16 @@
         <v>1</v>
       </c>
       <c r="L87" s="15" t="s">
-        <v>802</v>
+        <v>803</v>
       </c>
       <c r="M87" s="15" t="s">
-        <v>803</v>
+        <v>804</v>
       </c>
       <c r="N87" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O87" s="15" t="s">
-        <v>804</v>
+        <v>805</v>
       </c>
       <c r="P87" s="15" t="s">
         <v>169</v>
@@ -7304,31 +7307,31 @@
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="15" t="s">
-        <v>805</v>
+        <v>806</v>
       </c>
       <c r="B88" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C88" s="15" t="s">
-        <v>806</v>
+        <v>807</v>
       </c>
       <c r="D88" s="15" t="s">
-        <v>807</v>
+        <v>808</v>
       </c>
       <c r="E88" s="15" t="s">
-        <v>808</v>
+        <v>809</v>
       </c>
       <c r="F88" s="15" t="s">
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="G88" s="15" t="s">
         <v>6</v>
       </c>
       <c r="H88" s="15" t="s">
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="I88" s="15" t="s">
-        <v>811</v>
+        <v>812</v>
       </c>
       <c r="J88" s="15" t="s">
         <v>57</v>
@@ -7337,16 +7340,16 @@
         <v>1</v>
       </c>
       <c r="L88" s="15" t="s">
-        <v>812</v>
+        <v>813</v>
       </c>
       <c r="M88" s="15" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="N88" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O88" s="15" t="s">
-        <v>814</v>
+        <v>815</v>
       </c>
       <c r="P88" s="15" t="s">
         <v>169</v>
@@ -7354,31 +7357,31 @@
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="15" t="s">
-        <v>815</v>
+        <v>816</v>
       </c>
       <c r="B89" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C89" s="15" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
       <c r="D89" s="15" t="s">
-        <v>817</v>
+        <v>818</v>
       </c>
       <c r="E89" s="15" t="s">
         <v>6</v>
       </c>
       <c r="F89" s="15" t="s">
-        <v>818</v>
+        <v>819</v>
       </c>
       <c r="G89" s="15" t="s">
         <v>6</v>
       </c>
       <c r="H89" s="15" t="s">
-        <v>819</v>
+        <v>820</v>
       </c>
       <c r="I89" s="15" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="J89" s="15" t="s">
         <v>57</v>
@@ -7387,16 +7390,16 @@
         <v>1</v>
       </c>
       <c r="L89" s="15" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
       <c r="M89" s="15" t="s">
-        <v>822</v>
+        <v>823</v>
       </c>
       <c r="N89" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O89" s="15" t="s">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="P89" s="15" t="s">
         <v>432</v>
@@ -7404,31 +7407,31 @@
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="15" t="s">
-        <v>824</v>
+        <v>825</v>
       </c>
       <c r="B90" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C90" s="15" t="s">
-        <v>825</v>
+        <v>826</v>
       </c>
       <c r="D90" s="15" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="E90" s="15" t="s">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="F90" s="15" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="G90" s="15" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="H90" s="15" t="s">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="I90" s="15" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="J90" s="15" t="s">
         <v>57</v>
@@ -7437,16 +7440,16 @@
         <v>1</v>
       </c>
       <c r="L90" s="15" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
       <c r="M90" s="15" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="N90" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O90" s="15" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="P90" s="15" t="s">
         <v>169</v>
@@ -7454,16 +7457,16 @@
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="15" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="B91" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C91" s="15" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="D91" s="15" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="E91" s="15" t="s">
         <v>6</v>
@@ -7478,7 +7481,7 @@
         <v>6</v>
       </c>
       <c r="I91" s="15" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="J91" s="15" t="s">
         <v>57</v>
@@ -7487,16 +7490,16 @@
         <v>1</v>
       </c>
       <c r="L91" s="15" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="M91" s="15" t="s">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="N91" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O91" s="15" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="P91" s="15" t="s">
         <v>226</v>
@@ -7504,31 +7507,31 @@
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="15" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="B92" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C92" s="15" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="D92" s="15" t="s">
-        <v>843</v>
+        <v>844</v>
       </c>
       <c r="E92" s="15" t="s">
-        <v>844</v>
+        <v>845</v>
       </c>
       <c r="F92" s="15" t="s">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="G92" s="15" t="s">
         <v>451</v>
       </c>
       <c r="H92" s="15" t="s">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="I92" s="15" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="J92" s="15" t="s">
         <v>57</v>
@@ -7537,16 +7540,16 @@
         <v>1</v>
       </c>
       <c r="L92" s="15" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="M92" s="15" t="s">
-        <v>849</v>
+        <v>850</v>
       </c>
       <c r="N92" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O92" s="15" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="P92" s="15" t="s">
         <v>391</v>
@@ -7554,31 +7557,31 @@
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="15" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="B93" s="15" t="s">
         <v>446</v>
       </c>
       <c r="C93" s="15" t="s">
-        <v>852</v>
+        <v>853</v>
       </c>
       <c r="D93" s="15" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="E93" s="15" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="F93" s="15" t="s">
-        <v>855</v>
+        <v>856</v>
       </c>
       <c r="G93" s="15" t="s">
         <v>451</v>
       </c>
       <c r="H93" s="15" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="I93" s="15" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="J93" s="15" t="s">
         <v>57</v>
@@ -7587,16 +7590,16 @@
         <v>1</v>
       </c>
       <c r="L93" s="15" t="s">
-        <v>858</v>
+        <v>859</v>
       </c>
       <c r="M93" s="15" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="N93" s="15" t="s">
         <v>1</v>
       </c>
       <c r="O93" s="15" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="P93" s="15" t="s">
         <v>391</v>
@@ -7604,16 +7607,16 @@
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="12" t="s">
-        <v>861</v>
+        <v>862</v>
       </c>
       <c r="B94" s="12" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="C94" s="12" t="s">
         <v>447</v>
       </c>
       <c r="D94" s="12" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="E94" s="12" t="s">
         <v>6</v>
@@ -7628,25 +7631,25 @@
         <v>6</v>
       </c>
       <c r="I94" s="12" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="J94" s="12" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="K94" s="12" t="s">
         <v>91</v>
       </c>
       <c r="L94" s="12" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="M94" s="12" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="N94" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O94" s="12" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="P94" s="12" t="s">
         <v>226</v>
@@ -7654,16 +7657,16 @@
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="12" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="B95" s="12" t="s">
         <v>446</v>
       </c>
       <c r="C95" s="12" t="s">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="D95" s="12" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="E95" s="12" t="s">
         <v>6</v>
@@ -7678,7 +7681,7 @@
         <v>6</v>
       </c>
       <c r="I95" s="12" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="J95" s="12" t="s">
         <v>46</v>
@@ -7687,16 +7690,16 @@
         <v>91</v>
       </c>
       <c r="L95" s="12" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="M95" s="12" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="N95" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O95" s="12" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="P95" s="12" t="s">
         <v>169</v>
@@ -7704,16 +7707,16 @@
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="12" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="B96" s="12" t="s">
         <v>446</v>
       </c>
       <c r="C96" s="12" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="D96" s="12" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="E96" s="12" t="s">
         <v>6</v>
@@ -7728,7 +7731,7 @@
         <v>6</v>
       </c>
       <c r="I96" s="12" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="J96" s="12" t="s">
         <v>46</v>
@@ -7737,16 +7740,16 @@
         <v>91</v>
       </c>
       <c r="L96" s="12" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="M96" s="12" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="N96" s="12" t="s">
         <v>50</v>
       </c>
       <c r="O96" s="12" t="s">
-        <v>882</v>
+        <v>883</v>
       </c>
       <c r="P96" s="12" t="s">
         <v>156</v>
@@ -7754,16 +7757,16 @@
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="13" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="B97" s="13" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="C97" s="13" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="D97" s="13" t="s">
-        <v>886</v>
+        <v>887</v>
       </c>
       <c r="E97" s="13" t="s">
         <v>6</v>
@@ -7778,25 +7781,25 @@
         <v>6</v>
       </c>
       <c r="I97" s="13" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="J97" s="13" t="s">
-        <v>888</v>
+        <v>889</v>
       </c>
       <c r="K97" s="13" t="s">
         <v>47</v>
       </c>
       <c r="L97" s="13" t="s">
-        <v>889</v>
+        <v>890</v>
       </c>
       <c r="M97" s="13" t="s">
-        <v>890</v>
+        <v>891</v>
       </c>
       <c r="N97" s="13" t="s">
-        <v>891</v>
+        <v>892</v>
       </c>
       <c r="O97" s="13" t="s">
-        <v>892</v>
+        <v>893</v>
       </c>
       <c r="P97" s="13" t="s">
         <v>242</v>

</xml_diff>

<commit_message>
qa fix - impression
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -2209,16 +2209,19 @@
     <t>INDIRECT because feedback submit queued target recompute</t>
   </si>
   <si>
-    <t>Correct Host or Attendee trait evidence changes; unrelated section X</t>
+    <t>Correct Host or Attendee trait evidence changes; unrelated user and section remain unchanged</t>
+  </si>
+  <si>
+    <t>FAIL</t>
   </si>
   <si>
     <t>Impressions merge code; frontend realtime support partial</t>
   </si>
   <si>
-    <t>Capture before popup, feedback oracle, recompute terminal and after popup</t>
-  </si>
-  <si>
-    <t>Popup open is read-only; stale data after the realtime window is a propagation defect</t>
+    <t>Capture target and second-user controls before submit; retain feedback oracle, recompute terminal and both after views</t>
+  </si>
+  <si>
+    <t>Casey Host correctly gained Creative Soul 18% after completed recompute and Attendee stayed unchanged, but Nova's prior participant presentation became no-data and remained absent through a poll and close/reopen</t>
   </si>
   <si>
     <t>EVENT-IMPRESSION-002</t>
@@ -2228,9 +2231,6 @@
   </si>
   <si>
     <t>Feedback badge remains unchanged immediately after open and after poll</t>
-  </si>
-  <si>
-    <t>FAIL</t>
   </si>
   <si>
     <t>Manual regression captured</t>
@@ -6898,58 +6898,58 @@
       </c>
     </row>
     <row r="79" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="15" t="s">
+      <c r="A79" s="14" t="s">
         <v>724</v>
       </c>
-      <c r="B79" s="15" t="s">
+      <c r="B79" s="14" t="s">
         <v>446</v>
       </c>
-      <c r="C79" s="15" t="s">
+      <c r="C79" s="14" t="s">
         <v>725</v>
       </c>
-      <c r="D79" s="15" t="s">
+      <c r="D79" s="14" t="s">
         <v>726</v>
       </c>
-      <c r="E79" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="F79" s="15" t="s">
+      <c r="E79" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="F79" s="14" t="s">
         <v>727</v>
       </c>
-      <c r="G79" s="15" t="s">
+      <c r="G79" s="14" t="s">
         <v>728</v>
       </c>
-      <c r="H79" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="I79" s="15" t="s">
+      <c r="H79" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="I79" s="14" t="s">
         <v>729</v>
       </c>
-      <c r="J79" s="15" t="s">
-        <v>57</v>
-      </c>
-      <c r="K79" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="L79" s="15" t="s">
+      <c r="J79" s="14" t="s">
         <v>730</v>
       </c>
-      <c r="M79" s="15" t="s">
+      <c r="K79" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="L79" s="14" t="s">
         <v>731</v>
       </c>
-      <c r="N79" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="O79" s="15" t="s">
+      <c r="M79" s="14" t="s">
         <v>732</v>
       </c>
-      <c r="P79" s="15" t="s">
+      <c r="N79" s="14" t="s">
+        <v>730</v>
+      </c>
+      <c r="O79" s="14" t="s">
+        <v>733</v>
+      </c>
+      <c r="P79" s="14" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="14" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="B80" s="14" t="s">
         <v>446</v>
@@ -6958,7 +6958,7 @@
         <v>725</v>
       </c>
       <c r="D80" s="14" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="E80" s="14" t="s">
         <v>6</v>
@@ -6973,10 +6973,10 @@
         <v>6</v>
       </c>
       <c r="I80" s="14" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="J80" s="14" t="s">
-        <v>736</v>
+        <v>730</v>
       </c>
       <c r="K80" s="14" t="s">
         <v>91</v>
@@ -6988,7 +6988,7 @@
         <v>738</v>
       </c>
       <c r="N80" s="14" t="s">
-        <v>736</v>
+        <v>730</v>
       </c>
       <c r="O80" s="14" t="s">
         <v>739</v>

</xml_diff>

<commit_message>
qa - ticketing fix
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -2275,16 +2275,16 @@
     <t>FAIL / RETEST REQUIRED</t>
   </si>
   <si>
-    <t>EventTicketServiceTest + EventParticipationTicketServiceTest PASS</t>
-  </si>
-  <si>
-    <t>Restage with Casey+Nova accepted and Riley pending, require 2 / 8, repeat Casey Unpublish -&gt; On -&gt; Publish, then prove one Nova A ticket and zero Casey/Riley tickets and users-table counters before opening Nova Ticket twice</t>
+    <t>EventTicketServiceTest + EventParticipationTicketServiceTest PASS; lifecycle publish regression added; hot-deploy BUILD SUCCESSFUL</t>
+  </si>
+  <si>
+    <t>Repeat Casey Unpublish -&gt; On -&gt; Publish on the clean 2026-08-06T05:01:50.062Z restage, then prove one Nova A ticket and zero Casey/Riley tickets and users-table counters before opening Nova Ticket twice</t>
   </si>
   <si>
     <t>FAIL</t>
   </si>
   <si>
-    <t>The first real publish correctly produced Nova's ticket and poll-driven badge, but the subsequent Casey read also manufactured an Admin credential. Creation has been moved to publish/terminal-acceptance write-side, read-side issuance removed, active-only uniqueness added, and focused tests pass. A later fixture defect stored acceptedMembers=1 despite two accepted membership documents; staging now keeps Casey+Nova accepted and Riley pending so the clean retest must show 2 / 8 with Riley ticketless.</t>
+    <t>The earlier read-side defect that manufactured an Admin credential was removed. The corrected 2 / 8 plus Riley-pending retest then exposed a separate backend defect before any Ticket read: the event was published Ticketing On, but tickets stayed empty and Nova counters stayed 0 / 0. The lifecycle publish() path omitted the ticket sync present in canonical save/sync. Publish now performs physical accepted-participant synchronization before users-table counter refresh; the same hot-deploy compiled and restarted successfully. Clean baseline restaged for retest.</t>
   </si>
   <si>
     <t>EVENT-TICKET-003</t>

</xml_diff>

<commit_message>
qa fix - event backup
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -2620,22 +2620,22 @@
     <t>DELTA event-definition scheduled task only for each lifecycle mutation; poll X</t>
   </si>
   <si>
-    <t>With Nova Ticket open, Casey Unpublish yields one under-review notification count/attention within one interval; Casey Republish yields one event-modified available-again row the same way; Casey receives neither; stable rows are preserved; closing Ticket resumes deferred ordinary side-menu reconciliation</t>
+    <t>With Nova chat open, Casey Unpublish yields one short bundle-resolved under-review notification within one interval; Casey Republish yields one green available-again row the same way; both titles are only the compact event name with no Manual/changed; Casey receives neither; stable rows are preserved; closing chat resumes deferred ordinary side-menu reconciliation</t>
   </si>
   <si>
     <t>FIX HOT-DEPLOYED; MANUAL RETEST PENDING</t>
   </si>
   <si>
-    <t>Backend publish/chat-creation regression plus ScheduledMessageTask message mapping; shared UiPollCoordinator independent notification-lane regressions; existing backend/frontend hot-deploy green</t>
-  </si>
-  <si>
-    <t>Keep Nova Ticket open; Casey Unpublish then Publish; capture notification count/attention and available-again row without reload, then close Ticket and prove normal side-menu poll resumes</t>
+    <t>Backend lifecycle scheduling plus Mongo/frontend en+hu i18n key mapping; shared UiPollCoordinator independent notification-lane regressions; existing backend/frontend hot-deploy green</t>
+  </si>
+  <si>
+    <t>Restage/reload, keep Nova chat open; Casey Unpublish then Publish; capture notification count/attention and concise rows without reload, then close chat and prove normal side-menu poll resumes</t>
   </si>
   <si>
     <t>OPEN / FIX READY</t>
   </si>
   <si>
-    <t>Observed Republish produced the replacement ticket but no event-modified task/row because actor-chat creation skipped lifecycle scheduling. Backend now schedules accepted non-actor participants in that branch. Frontend notification realtime now runs in its own coordinator lane during any popup and does not advance ordinary side-menu state until popup close.</t>
+    <t>Lifecycle messages are semantic bundle keys, not hard-coded UI strings. Notification template title is exactly @event_title; the event-domain QA fixture uses the compact QA prefix. All three Mongo i18n JSON seeds are generator-synchronized and audited; notification polling stays in its independent lane.</t>
   </si>
   <si>
     <t>EVENT-CHAT-LIFECYCLE-001</t>
@@ -2647,25 +2647,25 @@
     <t>Keep every physical event-bound chat and its history usable across Unpublish and Republish</t>
   </si>
   <si>
-    <t>DELTA one eventId-indexed physical-chat status batch per lifecycle mutation; chat reads X</t>
+    <t>DELTA one eventId-indexed physical-chat ownerStatus+revision batch per lifecycle mutation; indexed owner-copy header poll X</t>
   </si>
   <si>
     <t>X; direct event lifecycle write path</t>
   </si>
   <si>
-    <t>Capture main/optional/group/service chat owner-copy IDs and message IDs; Unpublish sets only ownerStatus=DR and shows compact inline/popup Under review while accepted users can still read/send; Republish sets the same documents A and removes the badge; no chat/message recreation, unread inflation, unauthorized pending access or cross-event change</t>
+    <t>Capture main/optional/group/service chat owner-copy IDs and message IDs; leave Nova chat open; Unpublish advances revision and the foreground 30-second header delta shows compact Under review without reload; Republish advances the same documents to A and removes the badge; no chat/message recreation, unread inflation, unauthorized pending access or cross-event change</t>
   </si>
   <si>
     <t>IMPLEMENTATION UPDATED; MANUAL RETEST PENDING</t>
   </si>
   <si>
-    <t>Backend physical Chat ownerStatus plus indexed Mongo updateMulti and mapper coverage; frontend HTTP/local physical-record mapping, lifecycle repository and SeedBuilder parity; row/popup badge regressions</t>
-  </si>
-  <si>
-    <t>Share the active notification checkpoint mutations: capture physical chat/history before Unpublish, exercise main plus a sub-event/service chat while DR, then compare exact IDs/history and badge removal after Publish</t>
-  </si>
-  <si>
-    <t>Read-side Event projection is forbidden. The denormalized owner status lives on each physical chats document and is changed only by the event lifecycle write path.</t>
+    <t>Backend physical Chat ownerStatus+revision and ownerUserId/chatId delta endpoint; frontend HTTP/local parity and shared foreground UiPollCoordinator scheduler; hot-deploy green</t>
+  </si>
+  <si>
+    <t>Restage/reload, open Nova chat, Casey Unpublish then Publish; verify both live badge transitions, independent notification polling and side-menu resume after chat close</t>
+  </si>
+  <si>
+    <t>Read-side Event projection is forbidden. The poll reads only the indexed physical chat owner copy and returns revision/changed/ownerStatus; it cannot reload the Event, chat list or history.</t>
   </si>
   <si>
     <t>AUTH-SESSION-001</t>

</xml_diff>

<commit_message>
qa fix - chat
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -55,7 +55,7 @@
     <t>Pending</t>
   </si>
   <si>
-    <t>20</t>
+    <t>19</t>
   </si>
   <si>
     <t>INDIRECT</t>
@@ -79,7 +79,7 @@
     <t>Failed</t>
   </si>
   <si>
-    <t>1</t>
+    <t>2</t>
   </si>
   <si>
     <t>Complete</t>
@@ -2653,19 +2653,19 @@
     <t>X; direct event lifecycle write path</t>
   </si>
   <si>
-    <t>Capture main/optional/group/service chat owner-copy IDs and message IDs; leave Nova chat open; Unpublish advances revision and the foreground 30-second header delta shows compact Under review without reload; Republish advances the same documents to A and removes the badge; no chat/message recreation, unread inflation, unauthorized pending access or cross-event change</t>
-  </si>
-  <si>
-    <t>IMPLEMENTATION UPDATED; MANUAL RETEST PENDING</t>
-  </si>
-  <si>
-    <t>Backend physical Chat ownerStatus+revision and ownerUserId/chatId delta endpoint; frontend HTTP/local parity and shared foreground UiPollCoordinator scheduler; hot-deploy green</t>
-  </si>
-  <si>
-    <t>Restage/reload, open Nova chat, Casey Unpublish then Publish; verify both live badge transitions, independent notification polling and side-menu resume after chat close</t>
-  </si>
-  <si>
-    <t>Read-side Event projection is forbidden. The poll reads only the indexed physical chat owner copy and returns revision/changed/ownerStatus; it cannot reload the Event, chat list or history.</t>
+    <t>Capture main/optional/group/service chat owner-copy IDs and message IDs; leave Nova Activities Chats list open; Unpublish advances revision and the foreground 30-second row delta shows compact Under review without reload; Republish advances the same documents to A and removes the badge; no chat/message recreation, unread inflation, unauthorized pending access or cross-event change</t>
+  </si>
+  <si>
+    <t>FIRST LIST RETEST FAILED; FIX HOT-DEPLOYED; RETEST PENDING</t>
+  </si>
+  <si>
+    <t>Persisted first-failure oracle proved both physical copies DR with matching advanced revision; backend ownerUserId/chatId delta endpoint; frontend HTTP/local parity and shared foreground UiPollCoordinator list scheduler; hot-deploy green</t>
+  </si>
+  <si>
+    <t>Restage/reload, leave Nova Activities Chats list open without entering the inner chat; Casey Unpublish then Publish; verify both live row-badge transitions, independent notification polling and side-menu resume after list close</t>
+  </si>
+  <si>
+    <t>Read-side Event projection is forbidden. The first concise notification poll passed. The fixed list poll sends known row revisions, patches only changed rows and cannot reload the Event, chat list or history.</t>
   </si>
   <si>
     <t>AUTH-SESSION-001</t>
@@ -8426,52 +8426,52 @@
       </c>
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="29" t="s">
+      <c r="A95" s="30" t="s">
         <v>872</v>
       </c>
-      <c r="B95" s="29" t="s">
+      <c r="B95" s="30" t="s">
         <v>861</v>
       </c>
-      <c r="C95" s="29" t="s">
+      <c r="C95" s="30" t="s">
         <v>873</v>
       </c>
-      <c r="D95" s="29" t="s">
+      <c r="D95" s="30" t="s">
         <v>874</v>
       </c>
-      <c r="E95" s="29" t="s">
-        <v>4</v>
-      </c>
-      <c r="F95" s="29" t="s">
+      <c r="E95" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="F95" s="30" t="s">
         <v>875</v>
       </c>
-      <c r="G95" s="29" t="s">
-        <v>4</v>
-      </c>
-      <c r="H95" s="29" t="s">
+      <c r="G95" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="H95" s="30" t="s">
         <v>876</v>
       </c>
-      <c r="I95" s="29" t="s">
+      <c r="I95" s="30" t="s">
         <v>877</v>
       </c>
-      <c r="J95" s="29" t="s">
+      <c r="J95" s="30" t="s">
         <v>878</v>
       </c>
-      <c r="K95" s="29" t="s">
+      <c r="K95" s="30" t="s">
         <v>737</v>
       </c>
-      <c r="L95" s="29" t="s">
+      <c r="L95" s="30" t="s">
         <v>879</v>
       </c>
-      <c r="M95" s="29" t="s">
+      <c r="M95" s="30" t="s">
         <v>880</v>
       </c>
-      <c r="N95" s="29" t="s">
+      <c r="N95" s="30" t="s">
         <v>870</v>
       </c>
-      <c r="O95" s="29" t="s">
+      <c r="O95" s="30" t="s">
         <v>881</v>
       </c>
-      <c r="P95" s="29" t="s">
+      <c r="P95" s="30" t="s">
         <v>429</v>
       </c>
     </row>

</xml_diff>

<commit_message>
qa fix - notification
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1824" uniqueCount="1051">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1824" uniqueCount="1053">
   <si>
     <t>EFFECT MARKERS</t>
   </si>
@@ -55,7 +55,7 @@
     <t>Pending</t>
   </si>
   <si>
-    <t>19</t>
+    <t>20</t>
   </si>
   <si>
     <t>INDIRECT</t>
@@ -67,7 +67,7 @@
     <t>Not started</t>
   </si>
   <si>
-    <t>55</t>
+    <t>54</t>
   </si>
   <si>
     <t>GAP</t>
@@ -2359,31 +2359,37 @@
     <t>Event ticket join approval</t>
   </si>
   <si>
-    <t>Discover a Public event in Explore, Join, then create the physical ticket when admin approval directly accepts the member-origin request</t>
-  </si>
-  <si>
-    <t>INDIRECT Join/approval counter deltas</t>
-  </si>
-  <si>
-    <t>DELTA pending Join membership, then approval-owned physical ticket and users-table counter creation</t>
-  </si>
-  <si>
-    <t>INDIRECT after Join/approval recompute</t>
-  </si>
-  <si>
-    <t>DELTA only for the owning Join and approval writes; Explore/Ticket reads X</t>
-  </si>
-  <si>
-    <t>Baseline has Casey accepted Admin only and Nova outside membership with no ticket/counter; Nova finds the event in Explore and Join creates requestKind=join pendingSource=member with no ticket/counter; Casey approval directly makes Nova accepted and creates one Nova A ticket; Casey gets none; two reads reuse it</t>
-  </si>
-  <si>
-    <t>EventParticipationTicketService pending/accepted focused tests PASS; local target-only join regression PASS</t>
-  </si>
-  <si>
-    <t>Stage a Public approval-required Ticketing On event with Casey only; as Nova find it in Explore and Join, prove pending plus zero ticket and both users counters, approve once as Casey, then observe Nova poll and open Ticket twice</t>
-  </si>
-  <si>
-    <t>Join is a pending non-producer; terminal admin approval is the ticket producer; Explore and Ticket reads are non-producers</t>
+    <t>Discover a Public event in Explore; prove Join, Cancel request, re-Join and terminal admin-approval ticket ownership</t>
+  </si>
+  <si>
+    <t>INDIRECT Join/cancel/approval counter deltas</t>
+  </si>
+  <si>
+    <t>DELTA pending Join membership; Cancel suppresses the pending audit record; re-Join reopens only that pending request; approval owns physical ticket and users-table counter creation</t>
+  </si>
+  <si>
+    <t>INDIRECT after Join/cancel/approval recompute</t>
+  </si>
+  <si>
+    <t>DELTA only for owning Join, cancel and approval writes; separate Pending/Cancelled admin notification intents; Explore/Ticket reads X</t>
+  </si>
+  <si>
+    <t>Baseline Casey-only; Nova Join creates one pending member-origin approval request, zero tickets and one Casey Pending notification; Cancel removes the visible pending activity, retains only suppressed membership plus T overlay audit, leaves tickets zero and adds a separate Casey Cancelled row; re-Join creates fresh pending plus a new Pending row, never accepted/ticketed; Casey approval directly accepts Nova and creates one A ticket; Casey gets none; reads reuse it</t>
+  </si>
+  <si>
+    <t>IN PROGRESS</t>
+  </si>
+  <si>
+    <t>Clean Join retest PASS with one Pending row and zero tickets. Clean Cancel retest PASS with a separate Cancelled row, suppressed-pending membership audit, T overlay, pending 0, trash 1 and all ticket objects/counters zero. Re-Join gate fix is hot-deployed</t>
+  </si>
+  <si>
+    <t>Nova joins again; prove one fresh pending/new Pending row/zero tickets; Casey approves once; prove one accepted Nova and one physical A ticket</t>
+  </si>
+  <si>
+    <t>JOIN + CANCEL PASS / RE-JOIN NEXT</t>
+  </si>
+  <si>
+    <t>Join and Cancel remain ticket non-producers. Notification rows are write-owned action occurrences, not read projections. Cancelled membership remains physical suppressed audit; only terminal admin approval creates the ticket</t>
   </si>
   <si>
     <t>EVENT-TICKET-006</t>
@@ -7973,67 +7979,67 @@
       </c>
     </row>
     <row r="86" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="31" t="s">
+      <c r="A86" s="0" t="s">
         <v>777</v>
       </c>
-      <c r="B86" s="31" t="s">
+      <c r="B86" s="0" t="s">
         <v>443</v>
       </c>
-      <c r="C86" s="31" t="s">
+      <c r="C86" s="0" t="s">
         <v>778</v>
       </c>
-      <c r="D86" s="31" t="s">
+      <c r="D86" s="0" t="s">
         <v>779</v>
       </c>
-      <c r="E86" s="31" t="s">
+      <c r="E86" s="0" t="s">
         <v>780</v>
       </c>
-      <c r="F86" s="31" t="s">
+      <c r="F86" s="0" t="s">
         <v>781</v>
       </c>
-      <c r="G86" s="31" t="s">
+      <c r="G86" s="0" t="s">
         <v>782</v>
       </c>
-      <c r="H86" s="31" t="s">
+      <c r="H86" s="0" t="s">
         <v>783</v>
       </c>
-      <c r="I86" s="31" t="s">
+      <c r="I86" s="0" t="s">
         <v>784</v>
       </c>
-      <c r="J86" s="31" t="s">
-        <v>54</v>
-      </c>
-      <c r="K86" s="31" t="s">
-        <v>1</v>
-      </c>
-      <c r="L86" s="31" t="s">
+      <c r="J86" s="0" t="s">
         <v>785</v>
       </c>
-      <c r="M86" s="31" t="s">
+      <c r="K86" s="0" t="s">
+        <v>737</v>
+      </c>
+      <c r="L86" s="0" t="s">
         <v>786</v>
       </c>
-      <c r="N86" s="31" t="s">
-        <v>1</v>
-      </c>
-      <c r="O86" s="31" t="s">
+      <c r="M86" s="0" t="s">
         <v>787</v>
       </c>
-      <c r="P86" s="31" t="s">
+      <c r="N86" s="0" t="s">
+        <v>788</v>
+      </c>
+      <c r="O86" s="0" t="s">
+        <v>789</v>
+      </c>
+      <c r="P86" s="0" t="s">
         <v>429</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="31" t="s">
-        <v>788</v>
+        <v>790</v>
       </c>
       <c r="B87" s="31" t="s">
         <v>443</v>
       </c>
       <c r="C87" s="31" t="s">
-        <v>789</v>
+        <v>791</v>
       </c>
       <c r="D87" s="31" t="s">
-        <v>790</v>
+        <v>792</v>
       </c>
       <c r="E87" s="31" t="s">
         <v>4</v>
@@ -8042,13 +8048,13 @@
         <v>4</v>
       </c>
       <c r="G87" s="31" t="s">
-        <v>791</v>
+        <v>793</v>
       </c>
       <c r="H87" s="31" t="s">
-        <v>792</v>
+        <v>794</v>
       </c>
       <c r="I87" s="31" t="s">
-        <v>793</v>
+        <v>795</v>
       </c>
       <c r="J87" s="31" t="s">
         <v>54</v>
@@ -8057,16 +8063,16 @@
         <v>1</v>
       </c>
       <c r="L87" s="31" t="s">
-        <v>794</v>
+        <v>796</v>
       </c>
       <c r="M87" s="31" t="s">
-        <v>795</v>
+        <v>797</v>
       </c>
       <c r="N87" s="31" t="s">
         <v>1</v>
       </c>
       <c r="O87" s="31" t="s">
-        <v>796</v>
+        <v>798</v>
       </c>
       <c r="P87" s="31" t="s">
         <v>223</v>
@@ -8074,31 +8080,31 @@
     </row>
     <row r="88" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="31" t="s">
-        <v>797</v>
+        <v>799</v>
       </c>
       <c r="B88" s="31" t="s">
         <v>443</v>
       </c>
       <c r="C88" s="31" t="s">
-        <v>798</v>
+        <v>800</v>
       </c>
       <c r="D88" s="31" t="s">
-        <v>799</v>
+        <v>801</v>
       </c>
       <c r="E88" s="31" t="s">
-        <v>800</v>
+        <v>802</v>
       </c>
       <c r="F88" s="31" t="s">
-        <v>801</v>
+        <v>803</v>
       </c>
       <c r="G88" s="31" t="s">
-        <v>802</v>
+        <v>804</v>
       </c>
       <c r="H88" s="31" t="s">
-        <v>803</v>
+        <v>805</v>
       </c>
       <c r="I88" s="31" t="s">
-        <v>804</v>
+        <v>806</v>
       </c>
       <c r="J88" s="31" t="s">
         <v>54</v>
@@ -8107,16 +8113,16 @@
         <v>1</v>
       </c>
       <c r="L88" s="31" t="s">
-        <v>805</v>
+        <v>807</v>
       </c>
       <c r="M88" s="31" t="s">
-        <v>806</v>
+        <v>808</v>
       </c>
       <c r="N88" s="31" t="s">
         <v>1</v>
       </c>
       <c r="O88" s="31" t="s">
-        <v>807</v>
+        <v>809</v>
       </c>
       <c r="P88" s="31" t="s">
         <v>429</v>
@@ -8124,31 +8130,31 @@
     </row>
     <row r="89" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="31" t="s">
-        <v>808</v>
+        <v>810</v>
       </c>
       <c r="B89" s="31" t="s">
         <v>443</v>
       </c>
       <c r="C89" s="31" t="s">
-        <v>809</v>
+        <v>811</v>
       </c>
       <c r="D89" s="31" t="s">
-        <v>810</v>
+        <v>812</v>
       </c>
       <c r="E89" s="31" t="s">
-        <v>811</v>
+        <v>813</v>
       </c>
       <c r="F89" s="31" t="s">
-        <v>812</v>
+        <v>814</v>
       </c>
       <c r="G89" s="31" t="s">
-        <v>813</v>
+        <v>815</v>
       </c>
       <c r="H89" s="31" t="s">
-        <v>814</v>
+        <v>816</v>
       </c>
       <c r="I89" s="31" t="s">
-        <v>815</v>
+        <v>817</v>
       </c>
       <c r="J89" s="31" t="s">
         <v>54</v>
@@ -8157,16 +8163,16 @@
         <v>1</v>
       </c>
       <c r="L89" s="31" t="s">
-        <v>816</v>
+        <v>818</v>
       </c>
       <c r="M89" s="31" t="s">
-        <v>817</v>
+        <v>819</v>
       </c>
       <c r="N89" s="31" t="s">
         <v>1</v>
       </c>
       <c r="O89" s="31" t="s">
-        <v>818</v>
+        <v>820</v>
       </c>
       <c r="P89" s="31" t="s">
         <v>429</v>
@@ -8174,49 +8180,49 @@
     </row>
     <row r="90" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="0" t="s">
-        <v>819</v>
+        <v>821</v>
       </c>
       <c r="B90" s="0" t="s">
         <v>443</v>
       </c>
       <c r="C90" s="0" t="s">
-        <v>820</v>
+        <v>822</v>
       </c>
       <c r="D90" s="0" t="s">
-        <v>821</v>
+        <v>823</v>
       </c>
       <c r="E90" s="0" t="s">
         <v>4</v>
       </c>
       <c r="F90" s="0" t="s">
-        <v>822</v>
+        <v>824</v>
       </c>
       <c r="G90" s="0" t="s">
         <v>4</v>
       </c>
       <c r="H90" s="0" t="s">
-        <v>823</v>
+        <v>825</v>
       </c>
       <c r="I90" s="0" t="s">
-        <v>824</v>
+        <v>826</v>
       </c>
       <c r="J90" s="0" t="s">
-        <v>825</v>
+        <v>827</v>
       </c>
       <c r="K90" s="0" t="s">
         <v>737</v>
       </c>
       <c r="L90" s="0" t="s">
-        <v>826</v>
+        <v>828</v>
       </c>
       <c r="M90" s="0" t="s">
-        <v>827</v>
+        <v>829</v>
       </c>
       <c r="N90" s="0" t="s">
         <v>1</v>
       </c>
       <c r="O90" s="0" t="s">
-        <v>828</v>
+        <v>830</v>
       </c>
       <c r="P90" s="0" t="s">
         <v>429</v>
@@ -8224,31 +8230,31 @@
     </row>
     <row r="91" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="28" t="s">
-        <v>829</v>
+        <v>831</v>
       </c>
       <c r="B91" s="28" t="s">
         <v>443</v>
       </c>
       <c r="C91" s="28" t="s">
-        <v>830</v>
+        <v>832</v>
       </c>
       <c r="D91" s="28" t="s">
-        <v>831</v>
+        <v>833</v>
       </c>
       <c r="E91" s="28" t="s">
         <v>4</v>
       </c>
       <c r="F91" s="28" t="s">
-        <v>832</v>
+        <v>834</v>
       </c>
       <c r="G91" s="28" t="s">
         <v>4</v>
       </c>
       <c r="H91" s="28" t="s">
-        <v>833</v>
+        <v>835</v>
       </c>
       <c r="I91" s="28" t="s">
-        <v>834</v>
+        <v>836</v>
       </c>
       <c r="J91" s="28" t="s">
         <v>633</v>
@@ -8257,16 +8263,16 @@
         <v>737</v>
       </c>
       <c r="L91" s="28" t="s">
-        <v>835</v>
+        <v>837</v>
       </c>
       <c r="M91" s="28" t="s">
-        <v>836</v>
+        <v>838</v>
       </c>
       <c r="N91" s="28" t="s">
         <v>47</v>
       </c>
       <c r="O91" s="28" t="s">
-        <v>837</v>
+        <v>839</v>
       </c>
       <c r="P91" s="28" t="s">
         <v>429</v>
@@ -8274,49 +8280,49 @@
     </row>
     <row r="92" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="0" t="s">
-        <v>838</v>
+        <v>840</v>
       </c>
       <c r="B92" s="0" t="s">
-        <v>839</v>
+        <v>841</v>
       </c>
       <c r="C92" s="0" t="s">
-        <v>840</v>
+        <v>842</v>
       </c>
       <c r="D92" s="0" t="s">
-        <v>841</v>
+        <v>843</v>
       </c>
       <c r="E92" s="0" t="s">
-        <v>842</v>
+        <v>844</v>
       </c>
       <c r="F92" s="0" t="s">
-        <v>843</v>
+        <v>845</v>
       </c>
       <c r="G92" s="0" t="s">
-        <v>844</v>
+        <v>846</v>
       </c>
       <c r="H92" s="0" t="s">
-        <v>845</v>
+        <v>847</v>
       </c>
       <c r="I92" s="0" t="s">
-        <v>846</v>
+        <v>848</v>
       </c>
       <c r="J92" s="0" t="s">
-        <v>847</v>
+        <v>849</v>
       </c>
       <c r="K92" s="0" t="s">
         <v>737</v>
       </c>
       <c r="L92" s="0" t="s">
-        <v>848</v>
+        <v>850</v>
       </c>
       <c r="M92" s="0" t="s">
-        <v>849</v>
+        <v>851</v>
       </c>
       <c r="N92" s="0" t="s">
         <v>16</v>
       </c>
       <c r="O92" s="0" t="s">
-        <v>850</v>
+        <v>852</v>
       </c>
       <c r="P92" s="0" t="s">
         <v>429</v>
@@ -8324,31 +8330,31 @@
     </row>
     <row r="93" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="28" t="s">
-        <v>851</v>
+        <v>853</v>
       </c>
       <c r="B93" s="28" t="s">
         <v>443</v>
       </c>
       <c r="C93" s="28" t="s">
-        <v>852</v>
+        <v>854</v>
       </c>
       <c r="D93" s="28" t="s">
-        <v>853</v>
+        <v>855</v>
       </c>
       <c r="E93" s="28" t="s">
         <v>4</v>
       </c>
       <c r="F93" s="28" t="s">
-        <v>854</v>
+        <v>856</v>
       </c>
       <c r="G93" s="28" t="s">
         <v>4</v>
       </c>
       <c r="H93" s="28" t="s">
-        <v>855</v>
+        <v>857</v>
       </c>
       <c r="I93" s="28" t="s">
-        <v>856</v>
+        <v>858</v>
       </c>
       <c r="J93" s="28" t="s">
         <v>633</v>
@@ -8357,16 +8363,16 @@
         <v>737</v>
       </c>
       <c r="L93" s="28" t="s">
-        <v>857</v>
+        <v>859</v>
       </c>
       <c r="M93" s="28" t="s">
-        <v>858</v>
+        <v>860</v>
       </c>
       <c r="N93" s="28" t="s">
         <v>47</v>
       </c>
       <c r="O93" s="28" t="s">
-        <v>859</v>
+        <v>861</v>
       </c>
       <c r="P93" s="28" t="s">
         <v>429</v>
@@ -8374,49 +8380,49 @@
     </row>
     <row r="94" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="29" t="s">
-        <v>860</v>
+        <v>862</v>
       </c>
       <c r="B94" s="29" t="s">
-        <v>861</v>
+        <v>863</v>
       </c>
       <c r="C94" s="29" t="s">
-        <v>862</v>
+        <v>864</v>
       </c>
       <c r="D94" s="29" t="s">
-        <v>863</v>
+        <v>865</v>
       </c>
       <c r="E94" s="29" t="s">
         <v>4</v>
       </c>
       <c r="F94" s="29" t="s">
-        <v>864</v>
+        <v>866</v>
       </c>
       <c r="G94" s="29" t="s">
         <v>4</v>
       </c>
       <c r="H94" s="29" t="s">
-        <v>865</v>
+        <v>867</v>
       </c>
       <c r="I94" s="29" t="s">
-        <v>866</v>
+        <v>868</v>
       </c>
       <c r="J94" s="29" t="s">
-        <v>867</v>
+        <v>869</v>
       </c>
       <c r="K94" s="29" t="s">
         <v>737</v>
       </c>
       <c r="L94" s="29" t="s">
-        <v>868</v>
+        <v>870</v>
       </c>
       <c r="M94" s="29" t="s">
-        <v>869</v>
+        <v>871</v>
       </c>
       <c r="N94" s="29" t="s">
-        <v>870</v>
+        <v>872</v>
       </c>
       <c r="O94" s="29" t="s">
-        <v>871</v>
+        <v>873</v>
       </c>
       <c r="P94" s="29" t="s">
         <v>429</v>
@@ -8424,31 +8430,31 @@
     </row>
     <row r="95" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="0" t="s">
-        <v>872</v>
+        <v>874</v>
       </c>
       <c r="B95" s="0" t="s">
-        <v>861</v>
+        <v>863</v>
       </c>
       <c r="C95" s="0" t="s">
-        <v>873</v>
+        <v>875</v>
       </c>
       <c r="D95" s="0" t="s">
-        <v>874</v>
+        <v>876</v>
       </c>
       <c r="E95" s="0" t="s">
         <v>4</v>
       </c>
       <c r="F95" s="0" t="s">
-        <v>875</v>
+        <v>877</v>
       </c>
       <c r="G95" s="0" t="s">
         <v>4</v>
       </c>
       <c r="H95" s="0" t="s">
-        <v>876</v>
+        <v>878</v>
       </c>
       <c r="I95" s="0" t="s">
-        <v>877</v>
+        <v>879</v>
       </c>
       <c r="J95" s="0" t="s">
         <v>47</v>
@@ -8457,16 +8463,16 @@
         <v>737</v>
       </c>
       <c r="L95" s="0" t="s">
-        <v>878</v>
+        <v>880</v>
       </c>
       <c r="M95" s="0" t="s">
-        <v>879</v>
+        <v>881</v>
       </c>
       <c r="N95" s="0" t="s">
         <v>633</v>
       </c>
       <c r="O95" s="0" t="s">
-        <v>880</v>
+        <v>882</v>
       </c>
       <c r="P95" s="0" t="s">
         <v>429</v>
@@ -8474,22 +8480,22 @@
     </row>
     <row r="96" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="31" t="s">
-        <v>881</v>
+        <v>883</v>
       </c>
       <c r="B96" s="31" t="s">
-        <v>882</v>
+        <v>884</v>
       </c>
       <c r="C96" s="31" t="s">
-        <v>883</v>
+        <v>885</v>
       </c>
       <c r="D96" s="31" t="s">
-        <v>884</v>
+        <v>886</v>
       </c>
       <c r="E96" s="31" t="s">
-        <v>885</v>
+        <v>887</v>
       </c>
       <c r="F96" s="31" t="s">
-        <v>886</v>
+        <v>888</v>
       </c>
       <c r="G96" s="31" t="s">
         <v>4</v>
@@ -8498,25 +8504,25 @@
         <v>4</v>
       </c>
       <c r="I96" s="31" t="s">
-        <v>887</v>
+        <v>889</v>
       </c>
       <c r="J96" s="31" t="s">
-        <v>888</v>
+        <v>890</v>
       </c>
       <c r="K96" s="31" t="s">
         <v>1</v>
       </c>
       <c r="L96" s="31" t="s">
-        <v>889</v>
+        <v>891</v>
       </c>
       <c r="M96" s="31" t="s">
-        <v>890</v>
+        <v>892</v>
       </c>
       <c r="N96" s="31" t="s">
         <v>1</v>
       </c>
       <c r="O96" s="31" t="s">
-        <v>891</v>
+        <v>893</v>
       </c>
       <c r="P96" s="31" t="s">
         <v>429</v>
@@ -8524,22 +8530,22 @@
     </row>
     <row r="97" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="31" t="s">
-        <v>892</v>
+        <v>894</v>
       </c>
       <c r="B97" s="31" t="s">
-        <v>882</v>
+        <v>884</v>
       </c>
       <c r="C97" s="31" t="s">
-        <v>893</v>
+        <v>895</v>
       </c>
       <c r="D97" s="31" t="s">
-        <v>894</v>
+        <v>896</v>
       </c>
       <c r="E97" s="31" t="s">
         <v>4</v>
       </c>
       <c r="F97" s="31" t="s">
-        <v>895</v>
+        <v>897</v>
       </c>
       <c r="G97" s="31" t="s">
         <v>4</v>
@@ -8548,25 +8554,25 @@
         <v>4</v>
       </c>
       <c r="I97" s="31" t="s">
-        <v>896</v>
+        <v>898</v>
       </c>
       <c r="J97" s="31" t="s">
-        <v>888</v>
+        <v>890</v>
       </c>
       <c r="K97" s="31" t="s">
         <v>1</v>
       </c>
       <c r="L97" s="31" t="s">
-        <v>897</v>
+        <v>899</v>
       </c>
       <c r="M97" s="31" t="s">
-        <v>898</v>
+        <v>900</v>
       </c>
       <c r="N97" s="31" t="s">
         <v>1</v>
       </c>
       <c r="O97" s="31" t="s">
-        <v>899</v>
+        <v>901</v>
       </c>
       <c r="P97" s="31" t="s">
         <v>429</v>
@@ -8574,31 +8580,31 @@
     </row>
     <row r="98" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="31" t="s">
-        <v>900</v>
+        <v>902</v>
       </c>
       <c r="B98" s="31" t="s">
         <v>443</v>
       </c>
       <c r="C98" s="31" t="s">
-        <v>901</v>
+        <v>903</v>
       </c>
       <c r="D98" s="31" t="s">
-        <v>902</v>
+        <v>904</v>
       </c>
       <c r="E98" s="31" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="F98" s="31" t="s">
-        <v>904</v>
+        <v>906</v>
       </c>
       <c r="G98" s="31" t="s">
         <v>771</v>
       </c>
       <c r="H98" s="31" t="s">
-        <v>905</v>
+        <v>907</v>
       </c>
       <c r="I98" s="31" t="s">
-        <v>906</v>
+        <v>908</v>
       </c>
       <c r="J98" s="31" t="s">
         <v>54</v>
@@ -8610,13 +8616,13 @@
         <v>549</v>
       </c>
       <c r="M98" s="31" t="s">
-        <v>907</v>
+        <v>909</v>
       </c>
       <c r="N98" s="31" t="s">
         <v>1</v>
       </c>
       <c r="O98" s="31" t="s">
-        <v>908</v>
+        <v>910</v>
       </c>
       <c r="P98" s="31" t="s">
         <v>143</v>
@@ -8624,31 +8630,31 @@
     </row>
     <row r="99" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="31" t="s">
-        <v>909</v>
+        <v>911</v>
       </c>
       <c r="B99" s="31" t="s">
         <v>443</v>
       </c>
       <c r="C99" s="31" t="s">
-        <v>901</v>
+        <v>903</v>
       </c>
       <c r="D99" s="31" t="s">
-        <v>910</v>
+        <v>912</v>
       </c>
       <c r="E99" s="31" t="s">
         <v>501</v>
       </c>
       <c r="F99" s="31" t="s">
-        <v>911</v>
+        <v>913</v>
       </c>
       <c r="G99" s="31" t="s">
-        <v>912</v>
+        <v>914</v>
       </c>
       <c r="H99" s="31" t="s">
-        <v>913</v>
+        <v>915</v>
       </c>
       <c r="I99" s="31" t="s">
-        <v>914</v>
+        <v>916</v>
       </c>
       <c r="J99" s="31" t="s">
         <v>54</v>
@@ -8657,16 +8663,16 @@
         <v>1</v>
       </c>
       <c r="L99" s="31" t="s">
-        <v>915</v>
+        <v>917</v>
       </c>
       <c r="M99" s="31" t="s">
-        <v>916</v>
+        <v>918</v>
       </c>
       <c r="N99" s="31" t="s">
         <v>1</v>
       </c>
       <c r="O99" s="31" t="s">
-        <v>917</v>
+        <v>919</v>
       </c>
       <c r="P99" s="31" t="s">
         <v>223</v>
@@ -8674,31 +8680,31 @@
     </row>
     <row r="100" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="31" t="s">
-        <v>918</v>
+        <v>920</v>
       </c>
       <c r="B100" s="31" t="s">
         <v>443</v>
       </c>
       <c r="C100" s="31" t="s">
-        <v>901</v>
+        <v>903</v>
       </c>
       <c r="D100" s="31" t="s">
-        <v>919</v>
+        <v>921</v>
       </c>
       <c r="E100" s="31" t="s">
-        <v>920</v>
+        <v>922</v>
       </c>
       <c r="F100" s="31" t="s">
-        <v>921</v>
+        <v>923</v>
       </c>
       <c r="G100" s="31" t="s">
-        <v>922</v>
+        <v>924</v>
       </c>
       <c r="H100" s="31" t="s">
-        <v>923</v>
+        <v>925</v>
       </c>
       <c r="I100" s="31" t="s">
-        <v>924</v>
+        <v>926</v>
       </c>
       <c r="J100" s="31" t="s">
         <v>54</v>
@@ -8707,16 +8713,16 @@
         <v>1</v>
       </c>
       <c r="L100" s="31" t="s">
-        <v>925</v>
+        <v>927</v>
       </c>
       <c r="M100" s="31" t="s">
-        <v>926</v>
+        <v>928</v>
       </c>
       <c r="N100" s="31" t="s">
         <v>1</v>
       </c>
       <c r="O100" s="31" t="s">
-        <v>927</v>
+        <v>929</v>
       </c>
       <c r="P100" s="31" t="s">
         <v>388</v>
@@ -8724,22 +8730,22 @@
     </row>
     <row r="101" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="31" t="s">
-        <v>928</v>
+        <v>930</v>
       </c>
       <c r="B101" s="31" t="s">
         <v>443</v>
       </c>
       <c r="C101" s="31" t="s">
-        <v>929</v>
+        <v>931</v>
       </c>
       <c r="D101" s="31" t="s">
-        <v>930</v>
+        <v>932</v>
       </c>
       <c r="E101" s="31" t="s">
-        <v>931</v>
+        <v>933</v>
       </c>
       <c r="F101" s="31" t="s">
-        <v>932</v>
+        <v>934</v>
       </c>
       <c r="G101" s="31" t="s">
         <v>4</v>
@@ -8748,7 +8754,7 @@
         <v>613</v>
       </c>
       <c r="I101" s="31" t="s">
-        <v>933</v>
+        <v>935</v>
       </c>
       <c r="J101" s="31" t="s">
         <v>54</v>
@@ -8757,16 +8763,16 @@
         <v>1</v>
       </c>
       <c r="L101" s="31" t="s">
-        <v>934</v>
+        <v>936</v>
       </c>
       <c r="M101" s="31" t="s">
-        <v>935</v>
+        <v>937</v>
       </c>
       <c r="N101" s="31" t="s">
         <v>1</v>
       </c>
       <c r="O101" s="31" t="s">
-        <v>936</v>
+        <v>938</v>
       </c>
       <c r="P101" s="31" t="s">
         <v>143</v>
@@ -8774,31 +8780,31 @@
     </row>
     <row r="102" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="31" t="s">
-        <v>937</v>
+        <v>939</v>
       </c>
       <c r="B102" s="31" t="s">
         <v>443</v>
       </c>
       <c r="C102" s="31" t="s">
-        <v>929</v>
+        <v>931</v>
       </c>
       <c r="D102" s="31" t="s">
-        <v>938</v>
+        <v>940</v>
       </c>
       <c r="E102" s="31" t="s">
-        <v>931</v>
+        <v>933</v>
       </c>
       <c r="F102" s="31" t="s">
-        <v>939</v>
+        <v>941</v>
       </c>
       <c r="G102" s="31" t="s">
         <v>4</v>
       </c>
       <c r="H102" s="31" t="s">
-        <v>940</v>
+        <v>942</v>
       </c>
       <c r="I102" s="31" t="s">
-        <v>941</v>
+        <v>943</v>
       </c>
       <c r="J102" s="31" t="s">
         <v>54</v>
@@ -8807,16 +8813,16 @@
         <v>1</v>
       </c>
       <c r="L102" s="31" t="s">
-        <v>942</v>
+        <v>944</v>
       </c>
       <c r="M102" s="31" t="s">
-        <v>943</v>
+        <v>945</v>
       </c>
       <c r="N102" s="31" t="s">
         <v>1</v>
       </c>
       <c r="O102" s="31" t="s">
-        <v>944</v>
+        <v>946</v>
       </c>
       <c r="P102" s="31" t="s">
         <v>166</v>
@@ -8824,31 +8830,31 @@
     </row>
     <row r="103" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="31" t="s">
-        <v>945</v>
+        <v>947</v>
       </c>
       <c r="B103" s="31" t="s">
         <v>443</v>
       </c>
       <c r="C103" s="31" t="s">
-        <v>946</v>
+        <v>948</v>
       </c>
       <c r="D103" s="31" t="s">
-        <v>947</v>
+        <v>949</v>
       </c>
       <c r="E103" s="31" t="s">
-        <v>948</v>
+        <v>950</v>
       </c>
       <c r="F103" s="31" t="s">
-        <v>949</v>
+        <v>951</v>
       </c>
       <c r="G103" s="31" t="s">
         <v>4</v>
       </c>
       <c r="H103" s="31" t="s">
-        <v>950</v>
+        <v>952</v>
       </c>
       <c r="I103" s="31" t="s">
-        <v>951</v>
+        <v>953</v>
       </c>
       <c r="J103" s="31" t="s">
         <v>54</v>
@@ -8857,16 +8863,16 @@
         <v>1</v>
       </c>
       <c r="L103" s="31" t="s">
-        <v>952</v>
+        <v>954</v>
       </c>
       <c r="M103" s="31" t="s">
-        <v>953</v>
+        <v>955</v>
       </c>
       <c r="N103" s="31" t="s">
         <v>1</v>
       </c>
       <c r="O103" s="31" t="s">
-        <v>954</v>
+        <v>956</v>
       </c>
       <c r="P103" s="31" t="s">
         <v>166</v>
@@ -8874,31 +8880,31 @@
     </row>
     <row r="104" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="31" t="s">
-        <v>955</v>
+        <v>957</v>
       </c>
       <c r="B104" s="31" t="s">
         <v>443</v>
       </c>
       <c r="C104" s="31" t="s">
-        <v>956</v>
+        <v>958</v>
       </c>
       <c r="D104" s="31" t="s">
-        <v>957</v>
+        <v>959</v>
       </c>
       <c r="E104" s="31" t="s">
         <v>4</v>
       </c>
       <c r="F104" s="31" t="s">
-        <v>958</v>
+        <v>960</v>
       </c>
       <c r="G104" s="31" t="s">
         <v>4</v>
       </c>
       <c r="H104" s="31" t="s">
-        <v>959</v>
+        <v>961</v>
       </c>
       <c r="I104" s="31" t="s">
-        <v>960</v>
+        <v>962</v>
       </c>
       <c r="J104" s="31" t="s">
         <v>54</v>
@@ -8907,16 +8913,16 @@
         <v>1</v>
       </c>
       <c r="L104" s="31" t="s">
-        <v>961</v>
+        <v>963</v>
       </c>
       <c r="M104" s="31" t="s">
-        <v>962</v>
+        <v>964</v>
       </c>
       <c r="N104" s="31" t="s">
         <v>1</v>
       </c>
       <c r="O104" s="31" t="s">
-        <v>963</v>
+        <v>965</v>
       </c>
       <c r="P104" s="31" t="s">
         <v>429</v>
@@ -8924,49 +8930,49 @@
     </row>
     <row r="105" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="0" t="s">
-        <v>964</v>
+        <v>966</v>
       </c>
       <c r="B105" s="0" t="s">
-        <v>882</v>
+        <v>884</v>
       </c>
       <c r="C105" s="0" t="s">
-        <v>965</v>
+        <v>967</v>
       </c>
       <c r="D105" s="0" t="s">
-        <v>966</v>
+        <v>968</v>
       </c>
       <c r="E105" s="0" t="s">
         <v>4</v>
       </c>
       <c r="F105" s="0" t="s">
-        <v>967</v>
+        <v>969</v>
       </c>
       <c r="G105" s="0" t="s">
         <v>4</v>
       </c>
       <c r="H105" s="0" t="s">
-        <v>968</v>
+        <v>970</v>
       </c>
       <c r="I105" s="0" t="s">
-        <v>969</v>
+        <v>971</v>
       </c>
       <c r="J105" s="0" t="s">
-        <v>970</v>
+        <v>972</v>
       </c>
       <c r="K105" s="0" t="s">
         <v>1</v>
       </c>
       <c r="L105" s="0" t="s">
-        <v>971</v>
+        <v>973</v>
       </c>
       <c r="M105" s="0" t="s">
-        <v>972</v>
+        <v>974</v>
       </c>
       <c r="N105" s="0" t="s">
         <v>1</v>
       </c>
       <c r="O105" s="0" t="s">
-        <v>973</v>
+        <v>975</v>
       </c>
       <c r="P105" s="0" t="s">
         <v>429</v>
@@ -8974,22 +8980,22 @@
     </row>
     <row r="106" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="0" t="s">
-        <v>974</v>
+        <v>976</v>
       </c>
       <c r="B106" s="0" t="s">
-        <v>882</v>
+        <v>884</v>
       </c>
       <c r="C106" s="0" t="s">
-        <v>975</v>
+        <v>977</v>
       </c>
       <c r="D106" s="0" t="s">
-        <v>976</v>
+        <v>978</v>
       </c>
       <c r="E106" s="0" t="s">
         <v>4</v>
       </c>
       <c r="F106" s="0" t="s">
-        <v>977</v>
+        <v>979</v>
       </c>
       <c r="G106" s="0" t="s">
         <v>4</v>
@@ -8998,25 +9004,25 @@
         <v>4</v>
       </c>
       <c r="I106" s="0" t="s">
-        <v>978</v>
+        <v>980</v>
       </c>
       <c r="J106" s="0" t="s">
-        <v>970</v>
+        <v>972</v>
       </c>
       <c r="K106" s="0" t="s">
         <v>1</v>
       </c>
       <c r="L106" s="0" t="s">
-        <v>979</v>
+        <v>981</v>
       </c>
       <c r="M106" s="0" t="s">
-        <v>980</v>
+        <v>982</v>
       </c>
       <c r="N106" s="0" t="s">
         <v>1</v>
       </c>
       <c r="O106" s="0" t="s">
-        <v>981</v>
+        <v>983</v>
       </c>
       <c r="P106" s="0" t="s">
         <v>429</v>
@@ -9024,31 +9030,31 @@
     </row>
     <row r="107" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="31" t="s">
-        <v>982</v>
+        <v>984</v>
       </c>
       <c r="B107" s="31" t="s">
         <v>443</v>
       </c>
       <c r="C107" s="31" t="s">
-        <v>983</v>
+        <v>985</v>
       </c>
       <c r="D107" s="31" t="s">
-        <v>984</v>
+        <v>986</v>
       </c>
       <c r="E107" s="31" t="s">
-        <v>985</v>
+        <v>987</v>
       </c>
       <c r="F107" s="31" t="s">
-        <v>986</v>
+        <v>988</v>
       </c>
       <c r="G107" s="31" t="s">
         <v>771</v>
       </c>
       <c r="H107" s="31" t="s">
-        <v>987</v>
+        <v>989</v>
       </c>
       <c r="I107" s="31" t="s">
-        <v>988</v>
+        <v>990</v>
       </c>
       <c r="J107" s="31" t="s">
         <v>54</v>
@@ -9057,16 +9063,16 @@
         <v>1</v>
       </c>
       <c r="L107" s="31" t="s">
-        <v>989</v>
+        <v>991</v>
       </c>
       <c r="M107" s="31" t="s">
-        <v>990</v>
+        <v>992</v>
       </c>
       <c r="N107" s="31" t="s">
         <v>1</v>
       </c>
       <c r="O107" s="31" t="s">
-        <v>991</v>
+        <v>993</v>
       </c>
       <c r="P107" s="31" t="s">
         <v>166</v>
@@ -9074,16 +9080,16 @@
     </row>
     <row r="108" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="31" t="s">
-        <v>992</v>
+        <v>994</v>
       </c>
       <c r="B108" s="31" t="s">
         <v>443</v>
       </c>
       <c r="C108" s="31" t="s">
-        <v>993</v>
+        <v>995</v>
       </c>
       <c r="D108" s="31" t="s">
-        <v>994</v>
+        <v>996</v>
       </c>
       <c r="E108" s="31" t="s">
         <v>4</v>
@@ -9098,7 +9104,7 @@
         <v>4</v>
       </c>
       <c r="I108" s="31" t="s">
-        <v>995</v>
+        <v>997</v>
       </c>
       <c r="J108" s="31" t="s">
         <v>54</v>
@@ -9107,16 +9113,16 @@
         <v>1</v>
       </c>
       <c r="L108" s="31" t="s">
-        <v>996</v>
+        <v>998</v>
       </c>
       <c r="M108" s="31" t="s">
-        <v>997</v>
+        <v>999</v>
       </c>
       <c r="N108" s="31" t="s">
         <v>1</v>
       </c>
       <c r="O108" s="31" t="s">
-        <v>998</v>
+        <v>1000</v>
       </c>
       <c r="P108" s="31" t="s">
         <v>223</v>
@@ -9124,31 +9130,31 @@
     </row>
     <row r="109" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="31" t="s">
-        <v>999</v>
+        <v>1001</v>
       </c>
       <c r="B109" s="31" t="s">
         <v>443</v>
       </c>
       <c r="C109" s="31" t="s">
-        <v>1000</v>
+        <v>1002</v>
       </c>
       <c r="D109" s="31" t="s">
-        <v>1001</v>
+        <v>1003</v>
       </c>
       <c r="E109" s="31" t="s">
-        <v>1002</v>
+        <v>1004</v>
       </c>
       <c r="F109" s="31" t="s">
-        <v>1003</v>
+        <v>1005</v>
       </c>
       <c r="G109" s="31" t="s">
         <v>448</v>
       </c>
       <c r="H109" s="31" t="s">
-        <v>1004</v>
+        <v>1006</v>
       </c>
       <c r="I109" s="31" t="s">
-        <v>1005</v>
+        <v>1007</v>
       </c>
       <c r="J109" s="31" t="s">
         <v>54</v>
@@ -9157,16 +9163,16 @@
         <v>1</v>
       </c>
       <c r="L109" s="31" t="s">
-        <v>1006</v>
+        <v>1008</v>
       </c>
       <c r="M109" s="31" t="s">
-        <v>1007</v>
+        <v>1009</v>
       </c>
       <c r="N109" s="31" t="s">
         <v>1</v>
       </c>
       <c r="O109" s="31" t="s">
-        <v>1008</v>
+        <v>1010</v>
       </c>
       <c r="P109" s="31" t="s">
         <v>388</v>
@@ -9174,31 +9180,31 @@
     </row>
     <row r="110" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="31" t="s">
-        <v>1009</v>
+        <v>1011</v>
       </c>
       <c r="B110" s="31" t="s">
         <v>443</v>
       </c>
       <c r="C110" s="31" t="s">
-        <v>1010</v>
+        <v>1012</v>
       </c>
       <c r="D110" s="31" t="s">
-        <v>1011</v>
+        <v>1013</v>
       </c>
       <c r="E110" s="31" t="s">
-        <v>1012</v>
+        <v>1014</v>
       </c>
       <c r="F110" s="31" t="s">
-        <v>1013</v>
+        <v>1015</v>
       </c>
       <c r="G110" s="31" t="s">
         <v>448</v>
       </c>
       <c r="H110" s="31" t="s">
-        <v>1014</v>
+        <v>1016</v>
       </c>
       <c r="I110" s="31" t="s">
-        <v>1015</v>
+        <v>1017</v>
       </c>
       <c r="J110" s="31" t="s">
         <v>54</v>
@@ -9207,16 +9213,16 @@
         <v>1</v>
       </c>
       <c r="L110" s="31" t="s">
-        <v>1016</v>
+        <v>1018</v>
       </c>
       <c r="M110" s="31" t="s">
-        <v>1017</v>
+        <v>1019</v>
       </c>
       <c r="N110" s="31" t="s">
         <v>1</v>
       </c>
       <c r="O110" s="31" t="s">
-        <v>1018</v>
+        <v>1020</v>
       </c>
       <c r="P110" s="31" t="s">
         <v>388</v>
@@ -9224,16 +9230,16 @@
     </row>
     <row r="111" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="28" t="s">
-        <v>1019</v>
+        <v>1021</v>
       </c>
       <c r="B111" s="28" t="s">
-        <v>1020</v>
+        <v>1022</v>
       </c>
       <c r="C111" s="28" t="s">
         <v>444</v>
       </c>
       <c r="D111" s="28" t="s">
-        <v>1021</v>
+        <v>1023</v>
       </c>
       <c r="E111" s="28" t="s">
         <v>4</v>
@@ -9248,25 +9254,25 @@
         <v>4</v>
       </c>
       <c r="I111" s="28" t="s">
-        <v>1022</v>
+        <v>1024</v>
       </c>
       <c r="J111" s="28" t="s">
-        <v>1023</v>
+        <v>1025</v>
       </c>
       <c r="K111" s="28" t="s">
         <v>88</v>
       </c>
       <c r="L111" s="28" t="s">
-        <v>1024</v>
+        <v>1026</v>
       </c>
       <c r="M111" s="28" t="s">
-        <v>1025</v>
+        <v>1027</v>
       </c>
       <c r="N111" s="28" t="s">
         <v>47</v>
       </c>
       <c r="O111" s="28" t="s">
-        <v>1026</v>
+        <v>1028</v>
       </c>
       <c r="P111" s="28" t="s">
         <v>223</v>
@@ -9274,16 +9280,16 @@
     </row>
     <row r="112" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="28" t="s">
-        <v>1027</v>
+        <v>1029</v>
       </c>
       <c r="B112" s="28" t="s">
         <v>443</v>
       </c>
       <c r="C112" s="28" t="s">
-        <v>1028</v>
+        <v>1030</v>
       </c>
       <c r="D112" s="28" t="s">
-        <v>1029</v>
+        <v>1031</v>
       </c>
       <c r="E112" s="28" t="s">
         <v>4</v>
@@ -9298,7 +9304,7 @@
         <v>4</v>
       </c>
       <c r="I112" s="28" t="s">
-        <v>1030</v>
+        <v>1032</v>
       </c>
       <c r="J112" s="28" t="s">
         <v>43</v>
@@ -9307,16 +9313,16 @@
         <v>88</v>
       </c>
       <c r="L112" s="28" t="s">
-        <v>1031</v>
+        <v>1033</v>
       </c>
       <c r="M112" s="28" t="s">
-        <v>1032</v>
+        <v>1034</v>
       </c>
       <c r="N112" s="28" t="s">
         <v>47</v>
       </c>
       <c r="O112" s="28" t="s">
-        <v>1033</v>
+        <v>1035</v>
       </c>
       <c r="P112" s="28" t="s">
         <v>166</v>
@@ -9324,16 +9330,16 @@
     </row>
     <row r="113" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="28" t="s">
-        <v>1034</v>
+        <v>1036</v>
       </c>
       <c r="B113" s="28" t="s">
         <v>443</v>
       </c>
       <c r="C113" s="28" t="s">
-        <v>1035</v>
+        <v>1037</v>
       </c>
       <c r="D113" s="28" t="s">
-        <v>1036</v>
+        <v>1038</v>
       </c>
       <c r="E113" s="28" t="s">
         <v>4</v>
@@ -9348,7 +9354,7 @@
         <v>4</v>
       </c>
       <c r="I113" s="28" t="s">
-        <v>1037</v>
+        <v>1039</v>
       </c>
       <c r="J113" s="28" t="s">
         <v>43</v>
@@ -9357,16 +9363,16 @@
         <v>88</v>
       </c>
       <c r="L113" s="28" t="s">
-        <v>1038</v>
+        <v>1040</v>
       </c>
       <c r="M113" s="28" t="s">
-        <v>1039</v>
+        <v>1041</v>
       </c>
       <c r="N113" s="28" t="s">
         <v>47</v>
       </c>
       <c r="O113" s="28" t="s">
-        <v>1040</v>
+        <v>1042</v>
       </c>
       <c r="P113" s="28" t="s">
         <v>153</v>
@@ -9374,16 +9380,16 @@
     </row>
     <row r="114" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="29" t="s">
-        <v>1041</v>
+        <v>1043</v>
       </c>
       <c r="B114" s="29" t="s">
-        <v>1042</v>
+        <v>1044</v>
       </c>
       <c r="C114" s="29" t="s">
-        <v>1043</v>
+        <v>1045</v>
       </c>
       <c r="D114" s="29" t="s">
-        <v>1044</v>
+        <v>1046</v>
       </c>
       <c r="E114" s="29" t="s">
         <v>4</v>
@@ -9398,25 +9404,25 @@
         <v>4</v>
       </c>
       <c r="I114" s="29" t="s">
-        <v>1045</v>
+        <v>1047</v>
       </c>
       <c r="J114" s="29" t="s">
-        <v>1046</v>
+        <v>1048</v>
       </c>
       <c r="K114" s="29" t="s">
         <v>44</v>
       </c>
       <c r="L114" s="29" t="s">
-        <v>1047</v>
+        <v>1049</v>
       </c>
       <c r="M114" s="29" t="s">
-        <v>1048</v>
+        <v>1050</v>
       </c>
       <c r="N114" s="29" t="s">
-        <v>1049</v>
+        <v>1051</v>
       </c>
       <c r="O114" s="29" t="s">
-        <v>1050</v>
+        <v>1052</v>
       </c>
       <c r="P114" s="29" t="s">
         <v>239</v>

</xml_diff>

<commit_message>
qa backup - 005
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -2359,13 +2359,13 @@
     <t>Event ticket join approval</t>
   </si>
   <si>
-    <t>Discover a Public event in Explore; prove Join, Cancel request, re-Join and terminal admin-approval ticket ownership</t>
+    <t>Discover a Public event in Explore; prove repeated Join/Cancel signal removal, visible-basket reload retention and terminal admin-approval ticket ownership</t>
   </si>
   <si>
     <t>INDIRECT Join/cancel/approval counter deltas</t>
   </si>
   <si>
-    <t>DELTA pending Join membership; Cancel suppresses the pending audit record; re-Join reopens only that pending request; approval owns physical ticket and users-table counter creation</t>
+    <t>DELTA pending Join membership; every Cancel emits one ID-scoped activity removal; re-Join reopens only that pending request; approval owns physical ticket and users-table counter creation</t>
   </si>
   <si>
     <t>INDIRECT after Join/cancel/approval recompute</t>
@@ -2374,22 +2374,22 @@
     <t>DELTA only for owning Join, cancel and approval writes; separate Pending/Cancelled admin notification intents; Explore/Ticket reads X</t>
   </si>
   <si>
-    <t>Baseline Casey-only; Nova Join creates one pending member-origin approval request, zero tickets and one Casey Pending notification; Cancel removes the visible pending activity, retains only suppressed membership plus T overlay audit, leaves tickets zero and adds a separate Casey Cancelled row; re-Join creates fresh pending plus a new Pending row, never accepted/ticketed; Casey approval directly accepts Nova and creates one A ticket; Casey gets none; reads reuse it</t>
+    <t>Baseline Casey-only; Nova Join creates one pending member-origin approval request, one physical approval-pending basket, zero tickets and one Casey Pending notification; prove the server basket exists before reload; while that basket is visible an Explore reload retains the Public event card, orange Continue booking and its other contextual actions independent of member pending status; run at least two Cancel/Join cycles and require every Cancel to remove only the matching pending Activity row while adjacent cards remain unchanged; Cancel returns currentUserMembershipStatus none with no basket/session and tickets zero; terminal Casey approval directly accepts Nova and creates one A ticket; Casey gets none; reads reuse it</t>
   </si>
   <si>
     <t>IN PROGRESS</t>
   </si>
   <si>
-    <t>Clean Join retest PASS with one Pending row and zero tickets. Clean Cancel retest PASS with a separate Cancelled row, suppressed-pending membership audit, T overlay, pending 0, trash 1 and all ticket objects/counters zero. Re-Join gate fix is hot-deployed</t>
-  </si>
-  <si>
-    <t>Nova joins again; prove one fresh pending/new Pending row/zero tickets; Casey approves once; prove one accepted Nova and one physical A ticket</t>
-  </si>
-  <si>
-    <t>JOIN + CANCEL PASS / RE-JOIN NEXT</t>
-  </si>
-  <si>
-    <t>Join and Cancel remain ticket non-producers. Notification rows are write-owned action occurrences, not read projections. Cancelled membership remains physical suppressed audit; only terminal admin approval creates the ticket</t>
+    <t>Physical basket omission fixed in authoritative Join payload. Repeated Cancel/Join then exposed stale Activity row retention because Cancel cleared the event-sync signal instead of emitting remove(eventId); both Cancel paths now emit the ID-scoped removal and frontend hot-deploy is green. Live state is already accepted/succeeded, so clean restage is required</t>
+  </si>
+  <si>
+    <t>Restage EVENT-TICKET-005; repeat Join -&gt; Cancel -&gt; Join -&gt; Cancel -&gt; Join; prove each Cancel removes only its event row and every Join remains pending with a physical basket and zero ticket; reload the last pending state, then approve once</t>
+  </si>
+  <si>
+    <t>PHYSICAL-BASKET + REMOVAL-SIGNAL RETEST</t>
+  </si>
+  <si>
+    <t>Visible physical basket owns pending-card retention; explicit eventId removal owns Cancel UI cleanup. Join and Cancel are ticket non-producers; only terminal admin approval creates the ticket</t>
   </si>
   <si>
     <t>EVENT-TICKET-006</t>

</xml_diff>

<commit_message>
[MSC-51, MSC-55, MSC-56, MSC-60] Publish the story editions and production planning packages
Consolidate the story manuscripts, books, scripts, prompt/storyboard
coverage and publication outputs. Preserve the event/image fixture updates
recorded alongside this work.

Original-snapshot: 6cd9f6b246e8bdd7e94061ef2ec7312b3e6edaaa

Tasks: fssrepository/myscoutee-roadmap#51, fssrepository/myscoutee-roadmap#55, fssrepository/myscoutee-roadmap#56, fssrepository/myscoutee-roadmap#60
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -2359,13 +2359,13 @@
     <t>Event ticket join approval</t>
   </si>
   <si>
-    <t>Discover a Public event in Explore; prove Join, Cancel request, re-Join and terminal admin-approval ticket ownership</t>
+    <t>Discover a Public event in Explore; prove repeated Join/Cancel signal removal, visible-basket reload retention and terminal admin-approval ticket ownership</t>
   </si>
   <si>
     <t>INDIRECT Join/cancel/approval counter deltas</t>
   </si>
   <si>
-    <t>DELTA pending Join membership; Cancel suppresses the pending audit record; re-Join reopens only that pending request; approval owns physical ticket and users-table counter creation</t>
+    <t>DELTA pending Join membership; every Cancel emits one ID-scoped activity removal; re-Join reopens only that pending request; approval owns physical ticket and users-table counter creation</t>
   </si>
   <si>
     <t>INDIRECT after Join/cancel/approval recompute</t>
@@ -2374,22 +2374,22 @@
     <t>DELTA only for owning Join, cancel and approval writes; separate Pending/Cancelled admin notification intents; Explore/Ticket reads X</t>
   </si>
   <si>
-    <t>Baseline Casey-only; Nova Join creates one pending member-origin approval request, zero tickets and one Casey Pending notification; Cancel removes the visible pending activity, retains only suppressed membership plus T overlay audit, leaves tickets zero and adds a separate Casey Cancelled row; re-Join creates fresh pending plus a new Pending row, never accepted/ticketed; Casey approval directly accepts Nova and creates one A ticket; Casey gets none; reads reuse it</t>
+    <t>Baseline Casey-only; Nova Join creates one pending member-origin approval request, one physical approval-pending basket, zero tickets and one Casey Pending notification; prove the server basket exists before reload; while that basket is visible an Explore reload retains the Public event card, orange Continue booking and its other contextual actions independent of member pending status; run at least two Cancel/Join cycles and require every Cancel to remove only the matching pending Activity row while adjacent cards remain unchanged; Cancel returns currentUserMembershipStatus none with no basket/session and tickets zero; terminal Casey approval directly accepts Nova and creates one A ticket; Casey gets none; reads reuse it</t>
   </si>
   <si>
     <t>IN PROGRESS</t>
   </si>
   <si>
-    <t>Clean Join retest PASS with one Pending row and zero tickets. Clean Cancel retest PASS with a separate Cancelled row, suppressed-pending membership audit, T overlay, pending 0, trash 1 and all ticket objects/counters zero. Re-Join gate fix is hot-deployed</t>
-  </si>
-  <si>
-    <t>Nova joins again; prove one fresh pending/new Pending row/zero tickets; Casey approves once; prove one accepted Nova and one physical A ticket</t>
-  </si>
-  <si>
-    <t>JOIN + CANCEL PASS / RE-JOIN NEXT</t>
-  </si>
-  <si>
-    <t>Join and Cancel remain ticket non-producers. Notification rows are write-owned action occurrences, not read projections. Cancelled membership remains physical suppressed audit; only terminal admin approval creates the ticket</t>
+    <t>Physical basket omission fixed in authoritative Join payload. Repeated Cancel/Join then exposed stale Activity row retention because Cancel cleared the event-sync signal instead of emitting remove(eventId); both Cancel paths now emit the ID-scoped removal and frontend hot-deploy is green. Live state is already accepted/succeeded, so clean restage is required</t>
+  </si>
+  <si>
+    <t>Restage EVENT-TICKET-005; repeat Join -&gt; Cancel -&gt; Join -&gt; Cancel -&gt; Join; prove each Cancel removes only its event row and every Join remains pending with a physical basket and zero ticket; reload the last pending state, then approve once</t>
+  </si>
+  <si>
+    <t>PHYSICAL-BASKET + REMOVAL-SIGNAL RETEST</t>
+  </si>
+  <si>
+    <t>Visible physical basket owns pending-card retention; explicit eventId removal owns Cancel UI cleanup. Join and Cancel are ticket non-producers; only terminal admin approval creates the ticket</t>
   </si>
   <si>
     <t>EVENT-TICKET-006</t>

</xml_diff>

<commit_message>
activity event - pending fix
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -2493,16 +2493,16 @@
     <t>Baseline Casey accepted Admin and Nova accepted Member with one stable Nova A ticket/counters 1, while Riley is outside membership with zero ticket/counters; Nova invite creates one pending invitation; Riley acceptance converts it to a pending Admin-approval request and remains ticketless; Casey approval creates one Riley A ticket and both Riley counters 1 without changing Nova's ticket; poll exposes Riley badge 1 and repeated reads reuse it</t>
   </si>
   <si>
-    <t>IN PROGRESS / NOVA INVITE PASS / RILEY RESPONSE PENDING</t>
-  </si>
-  <si>
-    <t>Backend accepted-eligibility ticket tests PASS; existing admin-before-invitee denial and ordinary-inviter approval-order regressions present; local invitation-boundary regression PASS; write-side terminal payment-finalization ordering/idempotence regressions added; invite-candidate fixture ownership and authenticated actor/owner preflight added; existing continuous compiler BUILD SUCCESSFUL and Spring hot restart PASS; separate Gradle test process intentionally not started</t>
-  </si>
-  <si>
-    <t>Riley opens Invitations -&gt; QA EVENT-TICKET-007 overflow -&gt; Accept -&gt; confirm Accept once; then prove the same row is pending requestKind approval and Riley ticket/counters remain 0 before touching Casey</t>
-  </si>
-  <si>
-    <t>NOVA INVITE PASS / QA SEQUENCE CORRECTED</t>
+    <t>IN PROGRESS / NOVA INVITE PASS / RILEY RESPONSE REPAIRED PASS</t>
+  </si>
+  <si>
+    <t>Backend accepted-eligibility ticket tests PASS; existing admin-before-invitee denial and ordinary-inviter approval-order regressions present; local invitation-boundary regression PASS; write-side terminal payment-finalization ordering/idempotence regressions added; invite-candidate fixture ownership and authenticated actor/owner preflight added; Java mutationApplied response and shared counter-revision regressions added; existing backend/frontend hot-deploy builds and Spring restart PASS; manual HTTP replay PASS in-place and after fresh document read; separate Gradle/npm test processes intentionally not started</t>
+  </si>
+  <si>
+    <t>Casey opens My Events -&gt; QA EVENT-TICKET-007 -&gt; 2 / 8 members -&gt; Riley Outside menu -&gt; Approve -&gt; confirm Approve once; then prove terminal accepted membership, exactly one Riley A ticket/counters 1/1 and unchanged Nova ticket</t>
+  </si>
+  <si>
+    <t>NOVA INVITE PASS / RILEY RESPONSE REPAIRED PASS</t>
   </si>
   <si>
     <t>• Baseline PASS: Casey accepted Admin/ticket 0; Nova accepted Member with sole A ticket manual-qa-checkpoint:v1:event-domain:ticket / TKT-d6bd7582-1849-46bb-ba09-24dd7fb92b44 and counters 1/1; Riley outside membership/counters 0/0.
@@ -2515,7 +2515,11 @@
 • Guarded candidate preparation at 18:54:03.858Z created one reset-owned Nova-Riley rate. Independent status retained membership/ticket/counter/payment/outbox/task baselines, and Nova-authenticated candidate API returned only Riley with total 1.
 • The already-open empty popup retained its prior response, so the replay resumed only at Invite popup close/reopen.
 • Nova invite PASS at 20:57:41+02:00: exactly one members/invite POST returned 200. Oracle shows Riley pending invite from Nova, no Riley ticket/counters, unchanged Nova ticket/counters and empty payments. In-place UI shows Nova 2 members + 1 pending, Casey 2/8 + pending 1, and untouched Riley Invitations 1 with no Ticket badge.
-• QA sequence corrected without resetting the live boundary: backend authorization and existing tests deliberately forbid Admin acceptance before the invitee responds. Riley must accept first and remain pending requestKind approval/ticketless; Casey's later approval is terminal and owns ticket creation.</t>
+• QA sequence corrected without resetting the live boundary: backend authorization and existing tests deliberately forbid Admin acceptance before the invitee responds. Riley must accept first and remain pending requestKind approval/ticketless; Casey's later approval is terminal and owns ticket creation.
+• Initial Riley response in-place FAIL: Invitations emptied, but Pending did not become 1. Persisted oracle/read PASS: pending requestKind approval/pendingSource member, stored Pending 1/Invitations 0, ticket counters 0/0, no Riley ticket, one Casey join-request; reload reconstructed the row.
+• Owning repair: Java requestJoin now reports its saved mutation so the response emits Invitations -1 and Pending +1; the shared frontend delta path advances the counter revision so older realtime state cannot overwrite it. Existing hot-deploy owners compiled/restarted successfully; no parallel build/test process ran.
+• Guarded focused replay PASS at 21:40:46+02:00: HTTP 200 returned changed=true plus Invitations -1 / event Pending +1 / event Invitations -1. Riley observed Pending 1 without reload; DOM showed Waiting for approval; oracle retained ticketless Riley and the exact Nova ticket. A later full document/fresh-filter read showed the same state.
+• Frontend-local runtime NOT EXECUTED: the active deterministic fixture uses HTTP; local adapter contract was inspected and the shared regression covers the affected store, but no local runtime PASS is claimed.</t>
   </si>
   <si>
     <t>EVENT-TICKET-008</t>
@@ -8468,7 +8472,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="165" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="146" t="s">
         <v>799</v>
       </c>

</xml_diff>

<commit_message>
ticket poll fix - offline mode
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1824" uniqueCount="1056">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1824" uniqueCount="1054">
   <si>
     <t>EFFECT MARKERS</t>
   </si>
@@ -43,7 +43,7 @@
     <t>Done</t>
   </si>
   <si>
-    <t>35</t>
+    <t>36</t>
   </si>
   <si>
     <t>DELTA</t>
@@ -79,13 +79,13 @@
     <t>Failed</t>
   </si>
   <si>
-    <t>2</t>
+    <t>1</t>
   </si>
   <si>
     <t>Complete</t>
   </si>
   <si>
-    <t>33%</t>
+    <t>34%</t>
   </si>
   <si>
     <t>QA TEST CASES</t>
@@ -2574,16 +2574,10 @@
     <t>Nova starts with two distinct A tickets bound to two event IDs. Unpublishing event A changes only A ticket A -&gt; D and total counters 2 -&gt; 1; event B ticket keeps the same id/code/A status and remains visible. Republishing A creates a new A id/code and counters return 1 -&gt; 2 without duplicating or reassigning B</t>
   </si>
   <si>
-    <t>UNPUBLISH SERVER PASS; OPEN TICKET POLL FAIL; SHARED CORE REVERTED; TICKET HTTP+LOCAL DELTA REPAIR BUILT; CLEAN BASELINE READY / REPLAY PENDING</t>
-  </si>
-  <si>
-    <t>A-only persisted isolation/fresh read and notification branches remain PASS; post-restart Unpublish reproduced split Ticket badge/list state; shared SmartList change is fully reverted; Ticket-specific Notification-style delta contract built in Java HTTP and local adapters with foreground ownership; clean reset/stage is independently verified</t>
-  </si>
-  <si>
-    <t>Replay A Unpublish -&gt; immediate Casey Publish + Nova B-only/header1/red1 via POST ticket sync, then A Republish -&gt; immediate Casey Unpublish + Nova A+B/header2/red2; compare exact A/B identities and republish oracle</t>
-  </si>
-  <si>
-    <t>IN PROGRESS</t>
+    <t>Removal and insertion replay passed through Java POST ticket sync plus exact persisted isolation; shared SmartList stays reverted; Ticket-specific Java HTTP and frontend-local delta adapters retain foreground ownership; independent Nova/Riley notification lane remained live</t>
+  </si>
+  <si>
+    <t>Closed; retain as regression checkpoint for Ticket delta removal/insertion, immediate publication menu sync and adjacent ticket identity isolation</t>
   </si>
   <si>
     <t>• Fresh stage owns event A manual-qa-checkpoint:v1:event-domain:event and event B manual-qa-checkpoint:v1:event-domain:ticket-isolation-control; both are A/Public/Ticketing On with Casey+Nova accepted, Riley pending and occupancy 2/8 (1).
@@ -2603,7 +2597,9 @@
 • Post-restart Unpublish server PASS / open Ticket UI FAIL: one A Unpublish at 11:43:46; oracle proved A DR + exact A ticket D, B exact ticket stable A and Nova 1/1. Ticket GET at 11:44:14 returned B-only/total1 and red Ticket badge became1, but screenshot retained popup header2 plus A+B. Later convergence does not erase this boundary.
 • Corrected diagnosis: no race was proven. The foreground Ticket list lacked the established delta reconciliation contract, while the notification-priority realtime path also applied non-notification domain counters under an open popup.
 • Scoped repair built: the prior SmartList core page-size edit and its core tests are exactly reverted. Ticket uses stable identity/revision + Notification-style pollDelta on authenticated Java POST /assets/tickets/sync and the equivalent frontend-local repository; open popups defer side-menu domain snapshots while notifications remain independent. Existing backend compile/restart and frontend build/sync passed; authenticated Java preflight returned removed A, B upsert, total1.
-• Clean delta replay READY: the first reset revealed that scheduledMessageTasks was read by the oracle but absent from fixture cleanup. The versioned harness now owns only its controlled event-task rows. Second reset + image stage + independent status proved A+B active through 2026-08-13T15:07:37.047Z, Nova exact active tickets TKT-cc7f973d-f97b-471a-9559-7dde22e12086 and TKT-e5230543-0bd6-4c03-9375-b271e32bd9a5, counters2/2, controls0/0 and zero lifecycle/outbox/notification/recompute residue. Only the same three pages were reloaded; read-only DOM proved Casey/Nova/Riley identities and Ticket counters0/2/0.</t>
+• Clean delta replay READY: the first reset revealed that scheduledMessageTasks was read by the oracle but absent from fixture cleanup. The versioned harness now owns only its controlled event-task rows. Second reset + image stage + independent status proved A+B active through 2026-08-13T15:07:37.047Z, Nova exact active tickets TKT-cc7f973d-f97b-471a-9559-7dde22e12086 and TKT-e5230543-0bd6-4c03-9375-b271e32bd9a5, counters2/2, controls0/0 and zero lifecycle/outbox/notification/recompute residue. Only the same three pages were reloaded; read-only DOM proved Casey/Nova/Riley identities and Ticket counters0/2/0.
+• Removal replay PASS: Casey sent one A Unpublish at 12:14:59 and confirmed the immediately reopened menu showed Publish. Nova's already-open popup used Java POST /api/assets/tickets/sync at 12:15:24 and reached B-only/header1/red Ticket1 without reload; later no-op sync retained it. Oracle proved A DR + exact A ticket D, B exact ticket unchanged A and Nova1/1. Nova/Riley notification badges independently became1.
+• Insertion replay PASS/CLOSED: Casey Published only A at 12:18:36 and confirmed the immediately reopened menu showed Unpublish. Nova's open popup used Java POST /api/assets/tickets/sync at 12:18:54 and reached A+B/header2/red Ticket2 without reload or loss of B. Oracle proved new active A 6a7d99fce90c0afb4dd44fdb / TKT-d5034907-9acd-42b3-bfec-4707fb2e700a, original A stayed D, B exact TKT-e5230543-0bd6-4c03-9375-b271e32bd9a5 stayed A, and Nova2/2. Nova notification2/Riley1 passed.</t>
   </si>
   <si>
     <t>EVENT-TICKET-009</t>
@@ -2621,19 +2617,27 @@
     <t>X; check-in is a direct request path</t>
   </si>
   <si>
-    <t>Nova's persisted session routes from / into the cached app and displays the same cached ticket/QR; anonymous landing may remain available offline; Casey's online phone scans successfully once; repeat is already-used; Nova reconnect creates no replacement or duplicate</t>
-  </si>
-  <si>
-    <t>DEFECT FIXED; HOT-DEPLOY BUILD PASS; MANUAL RETEST PENDING</t>
-  </si>
-  <si>
-    <t>Offline cache/local repository coverage plus session/cache regressions added; frontend hot-deploy build PASS; persisted server-side check-in oracle required</t>
-  </si>
-  <si>
-    <t>Warm the new bundle and Nova Ticket/QR online; apply target-scoped Offline and reload; prove session and QR survive; keep backend and Casey phone online; scan twice; restore No throttling/online and reload; compare canonical ticket</t>
-  </si>
-  <si>
-    <t>Initial offline reload exposed landing fallback instead of persisted-session restoration. Root/session/warmed-demo-cache fix is hot-deployed. Firebase existing local auth may resume offline, but new login/token refresh is outside the promise. Keep this separate from online warning aggregation.</t>
+    <t>• Automatic warm: with Ticket closed, the authenticated side-menu realtime response writes the bounded Upcoming offlineTicketSnapshot; online SmartList continues through its own page/delta APIs and Past is not auto-warmed.
+• Offline reload: authenticated Nova shell uses a distinct dark-gray Offline background/status; only the menu visibility header is gray with an Offline badge. Preferences/filter/history and every member domain action except Ticket are disabled without recoloring their palettes; profile pencil and both notification launchers are absent without notification mutation.
+• Cached holder: the same exact unused B card and complete QR remain available without a server response.
+• Online scanner: Casey succeeds once, repeat is already-used, and Nova reconnect creates no replacement/duplicate.</t>
+  </si>
+  <si>
+    <t>OFFLINE SHELL + AUTO-WARM + SNAPSHOT B QR PASS / FIRST PHYSICAL SCAN PENDING</t>
+  </si>
+  <si>
+    <t>• Dev-only checkpoint PWA switch is ignored in production; held target cleanup restores online.
+• Existing watcher synced the home repair at 12:55:38 and final side-menu chunk at 13:04:29; no parallel build.
+• Read oracle: navigator false, activated controlling worker, game-page-status-offline, gray visibility header + Offline badge, three home controls/all non-Ticket domain items disabled, Ticket active, pencil/header-notification/FAB absent.
+• Existing watchers built Java + users.service-3VAB3CS6.js by 13:20:03. With Ticket never opened after reload, the side-menu poll advanced Upcoming cache 10:46:45Z -&gt; 11:22:56Z and retained A+B with scanCode; B remains A/unused: TKT-e5230543-0bd6-4c03-9375-b271e32bd9a5.
+• First offline B QR visual result is retracted: app-sw returned a cached GET /api/assets/tickets and the local timestamp changed despite no nginx request. The watcher synced the fix at 13:37:19 and the waiting worker was activated.
+• Corrected replay PASS: offline B full QR opened with cache timestamp unchanged at 11:40:47.443Z, no ticket API request and persisted B A/unused. Its visible medium.webp was a CacheStorage hit; this proves an already-cached card image, while automatic unseen-image prefetch is not yet claimed.</t>
+  </si>
+  <si>
+    <t>Keep Nova's offline B QR visible; Casey scans once; prove exact use/actor; repeat once as already-used no-op; restore Nova online and compare exact B/no duplicates</t>
+  </si>
+  <si>
+    <t>A's earlier online scan remains setup-only. The detached one-shot and service-worker-ticket-cache results are retracted; the no-worker ERR_INTERNET_DISCONNECTED attempt remains historical dev-config FAIL. Repaired Offline shell, no-popup Upcoming warm and corrected snapshot-source B QR branches pass. Physical scan/replay/reconnect remain.</t>
   </si>
   <si>
     <t>EVENT-TICKET-010</t>
@@ -8574,132 +8578,132 @@
       </c>
     </row>
     <row r="89" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A89" s="137" t="s">
+      <c r="A89" s="135" t="s">
         <v>811</v>
       </c>
-      <c r="B89" s="137" t="s">
+      <c r="B89" s="135" t="s">
         <v>443</v>
       </c>
-      <c r="C89" s="137" t="s">
+      <c r="C89" s="135" t="s">
         <v>812</v>
       </c>
-      <c r="D89" s="137" t="s">
+      <c r="D89" s="135" t="s">
         <v>813</v>
       </c>
-      <c r="E89" s="137" t="s">
+      <c r="E89" s="135" t="s">
         <v>814</v>
       </c>
-      <c r="F89" s="137" t="s">
+      <c r="F89" s="135" t="s">
         <v>815</v>
       </c>
-      <c r="G89" s="137" t="s">
+      <c r="G89" s="135" t="s">
         <v>816</v>
       </c>
-      <c r="H89" s="137" t="s">
+      <c r="H89" s="135" t="s">
         <v>817</v>
       </c>
-      <c r="I89" s="137" t="s">
+      <c r="I89" s="135" t="s">
         <v>818</v>
       </c>
-      <c r="J89" s="137" t="s">
+      <c r="J89" s="135" t="s">
+        <v>482</v>
+      </c>
+      <c r="K89" s="135" t="s">
+        <v>483</v>
+      </c>
+      <c r="L89" s="135" t="s">
         <v>819</v>
       </c>
-      <c r="K89" s="137" t="s">
+      <c r="M89" s="135" t="s">
+        <v>820</v>
+      </c>
+      <c r="N89" s="135" t="s">
+        <v>47</v>
+      </c>
+      <c r="O89" s="135" t="s">
+        <v>821</v>
+      </c>
+      <c r="P89" s="135" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A90" s="136" t="s">
+        <v>822</v>
+      </c>
+      <c r="B90" s="136" t="s">
+        <v>443</v>
+      </c>
+      <c r="C90" s="136" t="s">
+        <v>823</v>
+      </c>
+      <c r="D90" s="136" t="s">
+        <v>824</v>
+      </c>
+      <c r="E90" s="136" t="s">
+        <v>4</v>
+      </c>
+      <c r="F90" s="136" t="s">
+        <v>825</v>
+      </c>
+      <c r="G90" s="136" t="s">
+        <v>4</v>
+      </c>
+      <c r="H90" s="136" t="s">
+        <v>826</v>
+      </c>
+      <c r="I90" s="136" t="s">
+        <v>827</v>
+      </c>
+      <c r="J90" s="136" t="s">
+        <v>828</v>
+      </c>
+      <c r="K90" s="136" t="s">
         <v>483</v>
       </c>
-      <c r="L89" s="137" t="s">
-        <v>820</v>
-      </c>
-      <c r="M89" s="137" t="s">
-        <v>821</v>
-      </c>
-      <c r="N89" s="137" t="s">
-        <v>822</v>
-      </c>
-      <c r="O89" s="137" t="s">
-        <v>823</v>
-      </c>
-      <c r="P89" s="137" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="146" t="s">
-        <v>824</v>
-      </c>
-      <c r="B90" s="146" t="s">
-        <v>443</v>
-      </c>
-      <c r="C90" s="146" t="s">
-        <v>825</v>
-      </c>
-      <c r="D90" s="146" t="s">
-        <v>826</v>
-      </c>
-      <c r="E90" s="146" t="s">
-        <v>4</v>
-      </c>
-      <c r="F90" s="146" t="s">
-        <v>827</v>
-      </c>
-      <c r="G90" s="146" t="s">
-        <v>4</v>
-      </c>
-      <c r="H90" s="146" t="s">
-        <v>828</v>
-      </c>
-      <c r="I90" s="146" t="s">
+      <c r="L90" s="136" t="s">
         <v>829</v>
       </c>
-      <c r="J90" s="146" t="s">
+      <c r="M90" s="136" t="s">
         <v>830</v>
       </c>
-      <c r="K90" s="146" t="s">
-        <v>738</v>
-      </c>
-      <c r="L90" s="146" t="s">
+      <c r="N90" s="136" t="s">
+        <v>439</v>
+      </c>
+      <c r="O90" s="136" t="s">
         <v>831</v>
       </c>
-      <c r="M90" s="146" t="s">
-        <v>832</v>
-      </c>
-      <c r="N90" s="146" t="s">
-        <v>1</v>
-      </c>
-      <c r="O90" s="146" t="s">
-        <v>833</v>
-      </c>
-      <c r="P90" s="146" t="s">
+      <c r="P90" s="136" t="s">
         <v>429</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="135" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
       <c r="B91" s="135" t="s">
         <v>443</v>
       </c>
       <c r="C91" s="135" t="s">
+        <v>833</v>
+      </c>
+      <c r="D91" s="135" t="s">
+        <v>834</v>
+      </c>
+      <c r="E91" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="F91" s="135" t="s">
         <v>835</v>
       </c>
-      <c r="D91" s="135" t="s">
+      <c r="G91" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="H91" s="135" t="s">
         <v>836</v>
       </c>
-      <c r="E91" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="F91" s="135" t="s">
+      <c r="I91" s="135" t="s">
         <v>837</v>
-      </c>
-      <c r="G91" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="H91" s="135" t="s">
-        <v>838</v>
-      </c>
-      <c r="I91" s="135" t="s">
-        <v>839</v>
       </c>
       <c r="J91" s="135" t="s">
         <v>482</v>
@@ -8708,16 +8712,16 @@
         <v>738</v>
       </c>
       <c r="L91" s="135" t="s">
-        <v>840</v>
+        <v>838</v>
       </c>
       <c r="M91" s="135" t="s">
-        <v>841</v>
+        <v>839</v>
       </c>
       <c r="N91" s="135" t="s">
         <v>47</v>
       </c>
       <c r="O91" s="135" t="s">
-        <v>842</v>
+        <v>840</v>
       </c>
       <c r="P91" s="135" t="s">
         <v>429</v>
@@ -8725,49 +8729,49 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="146" t="s">
+        <v>841</v>
+      </c>
+      <c r="B92" s="146" t="s">
+        <v>842</v>
+      </c>
+      <c r="C92" s="146" t="s">
         <v>843</v>
       </c>
-      <c r="B92" s="146" t="s">
+      <c r="D92" s="146" t="s">
         <v>844</v>
       </c>
-      <c r="C92" s="146" t="s">
+      <c r="E92" s="146" t="s">
         <v>845</v>
       </c>
-      <c r="D92" s="146" t="s">
+      <c r="F92" s="146" t="s">
         <v>846</v>
       </c>
-      <c r="E92" s="146" t="s">
+      <c r="G92" s="146" t="s">
         <v>847</v>
       </c>
-      <c r="F92" s="146" t="s">
+      <c r="H92" s="146" t="s">
         <v>848</v>
       </c>
-      <c r="G92" s="146" t="s">
+      <c r="I92" s="146" t="s">
         <v>849</v>
       </c>
-      <c r="H92" s="146" t="s">
+      <c r="J92" s="146" t="s">
         <v>850</v>
-      </c>
-      <c r="I92" s="146" t="s">
-        <v>851</v>
-      </c>
-      <c r="J92" s="146" t="s">
-        <v>852</v>
       </c>
       <c r="K92" s="146" t="s">
         <v>738</v>
       </c>
       <c r="L92" s="146" t="s">
-        <v>853</v>
+        <v>851</v>
       </c>
       <c r="M92" s="146" t="s">
-        <v>854</v>
+        <v>852</v>
       </c>
       <c r="N92" s="146" t="s">
         <v>16</v>
       </c>
       <c r="O92" s="146" t="s">
-        <v>855</v>
+        <v>853</v>
       </c>
       <c r="P92" s="146" t="s">
         <v>429</v>
@@ -8775,31 +8779,31 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="135" t="s">
-        <v>856</v>
+        <v>854</v>
       </c>
       <c r="B93" s="135" t="s">
         <v>443</v>
       </c>
       <c r="C93" s="135" t="s">
+        <v>855</v>
+      </c>
+      <c r="D93" s="135" t="s">
+        <v>856</v>
+      </c>
+      <c r="E93" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="F93" s="135" t="s">
         <v>857</v>
       </c>
-      <c r="D93" s="135" t="s">
+      <c r="G93" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="H93" s="135" t="s">
         <v>858</v>
       </c>
-      <c r="E93" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="F93" s="135" t="s">
+      <c r="I93" s="135" t="s">
         <v>859</v>
-      </c>
-      <c r="G93" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="H93" s="135" t="s">
-        <v>860</v>
-      </c>
-      <c r="I93" s="135" t="s">
-        <v>861</v>
       </c>
       <c r="J93" s="135" t="s">
         <v>482</v>
@@ -8808,16 +8812,16 @@
         <v>738</v>
       </c>
       <c r="L93" s="135" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="M93" s="135" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
       <c r="N93" s="135" t="s">
         <v>47</v>
       </c>
       <c r="O93" s="135" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="P93" s="135" t="s">
         <v>429</v>
@@ -8825,49 +8829,49 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="136" t="s">
+        <v>863</v>
+      </c>
+      <c r="B94" s="136" t="s">
+        <v>864</v>
+      </c>
+      <c r="C94" s="136" t="s">
         <v>865</v>
       </c>
-      <c r="B94" s="136" t="s">
+      <c r="D94" s="136" t="s">
         <v>866</v>
       </c>
-      <c r="C94" s="136" t="s">
+      <c r="E94" s="136" t="s">
+        <v>4</v>
+      </c>
+      <c r="F94" s="136" t="s">
         <v>867</v>
       </c>
-      <c r="D94" s="136" t="s">
+      <c r="G94" s="136" t="s">
+        <v>4</v>
+      </c>
+      <c r="H94" s="136" t="s">
         <v>868</v>
       </c>
-      <c r="E94" s="136" t="s">
-        <v>4</v>
-      </c>
-      <c r="F94" s="136" t="s">
+      <c r="I94" s="136" t="s">
         <v>869</v>
       </c>
-      <c r="G94" s="136" t="s">
-        <v>4</v>
-      </c>
-      <c r="H94" s="136" t="s">
+      <c r="J94" s="136" t="s">
         <v>870</v>
-      </c>
-      <c r="I94" s="136" t="s">
-        <v>871</v>
-      </c>
-      <c r="J94" s="136" t="s">
-        <v>872</v>
       </c>
       <c r="K94" s="136" t="s">
         <v>738</v>
       </c>
       <c r="L94" s="136" t="s">
+        <v>871</v>
+      </c>
+      <c r="M94" s="136" t="s">
+        <v>872</v>
+      </c>
+      <c r="N94" s="136" t="s">
         <v>873</v>
       </c>
-      <c r="M94" s="136" t="s">
+      <c r="O94" s="136" t="s">
         <v>874</v>
-      </c>
-      <c r="N94" s="136" t="s">
-        <v>875</v>
-      </c>
-      <c r="O94" s="136" t="s">
-        <v>876</v>
       </c>
       <c r="P94" s="136" t="s">
         <v>429</v>
@@ -8875,31 +8879,31 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="146" t="s">
+        <v>875</v>
+      </c>
+      <c r="B95" s="146" t="s">
+        <v>864</v>
+      </c>
+      <c r="C95" s="146" t="s">
+        <v>876</v>
+      </c>
+      <c r="D95" s="146" t="s">
         <v>877</v>
       </c>
-      <c r="B95" s="146" t="s">
-        <v>866</v>
-      </c>
-      <c r="C95" s="146" t="s">
+      <c r="E95" s="146" t="s">
+        <v>4</v>
+      </c>
+      <c r="F95" s="146" t="s">
         <v>878</v>
       </c>
-      <c r="D95" s="146" t="s">
+      <c r="G95" s="146" t="s">
+        <v>4</v>
+      </c>
+      <c r="H95" s="146" t="s">
         <v>879</v>
       </c>
-      <c r="E95" s="146" t="s">
-        <v>4</v>
-      </c>
-      <c r="F95" s="146" t="s">
+      <c r="I95" s="146" t="s">
         <v>880</v>
-      </c>
-      <c r="G95" s="146" t="s">
-        <v>4</v>
-      </c>
-      <c r="H95" s="146" t="s">
-        <v>881</v>
-      </c>
-      <c r="I95" s="146" t="s">
-        <v>882</v>
       </c>
       <c r="J95" s="146" t="s">
         <v>47</v>
@@ -8908,16 +8912,16 @@
         <v>738</v>
       </c>
       <c r="L95" s="146" t="s">
-        <v>883</v>
+        <v>881</v>
       </c>
       <c r="M95" s="146" t="s">
-        <v>884</v>
+        <v>882</v>
       </c>
       <c r="N95" s="146" t="s">
         <v>482</v>
       </c>
       <c r="O95" s="146" t="s">
-        <v>885</v>
+        <v>883</v>
       </c>
       <c r="P95" s="146" t="s">
         <v>429</v>
@@ -8925,49 +8929,49 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="138" t="s">
+        <v>884</v>
+      </c>
+      <c r="B96" s="138" t="s">
+        <v>885</v>
+      </c>
+      <c r="C96" s="138" t="s">
         <v>886</v>
       </c>
-      <c r="B96" s="138" t="s">
+      <c r="D96" s="138" t="s">
         <v>887</v>
       </c>
-      <c r="C96" s="138" t="s">
+      <c r="E96" s="138" t="s">
         <v>888</v>
       </c>
-      <c r="D96" s="138" t="s">
+      <c r="F96" s="138" t="s">
         <v>889</v>
       </c>
-      <c r="E96" s="138" t="s">
+      <c r="G96" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="H96" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="I96" s="138" t="s">
         <v>890</v>
       </c>
-      <c r="F96" s="138" t="s">
+      <c r="J96" s="138" t="s">
         <v>891</v>
       </c>
-      <c r="G96" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="H96" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="I96" s="138" t="s">
+      <c r="K96" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="L96" s="138" t="s">
         <v>892</v>
       </c>
-      <c r="J96" s="138" t="s">
+      <c r="M96" s="138" t="s">
         <v>893</v>
       </c>
-      <c r="K96" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="L96" s="138" t="s">
+      <c r="N96" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O96" s="138" t="s">
         <v>894</v>
-      </c>
-      <c r="M96" s="138" t="s">
-        <v>895</v>
-      </c>
-      <c r="N96" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O96" s="138" t="s">
-        <v>896</v>
       </c>
       <c r="P96" s="138" t="s">
         <v>429</v>
@@ -8975,49 +8979,49 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="138" t="s">
+        <v>895</v>
+      </c>
+      <c r="B97" s="138" t="s">
+        <v>885</v>
+      </c>
+      <c r="C97" s="138" t="s">
+        <v>896</v>
+      </c>
+      <c r="D97" s="138" t="s">
         <v>897</v>
       </c>
-      <c r="B97" s="138" t="s">
-        <v>887</v>
-      </c>
-      <c r="C97" s="138" t="s">
+      <c r="E97" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="F97" s="138" t="s">
         <v>898</v>
       </c>
-      <c r="D97" s="138" t="s">
+      <c r="G97" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="H97" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="I97" s="138" t="s">
         <v>899</v>
       </c>
-      <c r="E97" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="F97" s="138" t="s">
+      <c r="J97" s="138" t="s">
+        <v>891</v>
+      </c>
+      <c r="K97" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="L97" s="138" t="s">
         <v>900</v>
       </c>
-      <c r="G97" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="H97" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="I97" s="138" t="s">
+      <c r="M97" s="138" t="s">
         <v>901</v>
       </c>
-      <c r="J97" s="138" t="s">
-        <v>893</v>
-      </c>
-      <c r="K97" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="L97" s="138" t="s">
+      <c r="N97" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O97" s="138" t="s">
         <v>902</v>
-      </c>
-      <c r="M97" s="138" t="s">
-        <v>903</v>
-      </c>
-      <c r="N97" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O97" s="138" t="s">
-        <v>904</v>
       </c>
       <c r="P97" s="138" t="s">
         <v>429</v>
@@ -9025,31 +9029,31 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="138" t="s">
-        <v>905</v>
+        <v>903</v>
       </c>
       <c r="B98" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C98" s="138" t="s">
+        <v>904</v>
+      </c>
+      <c r="D98" s="138" t="s">
+        <v>905</v>
+      </c>
+      <c r="E98" s="138" t="s">
         <v>906</v>
       </c>
-      <c r="D98" s="138" t="s">
+      <c r="F98" s="138" t="s">
         <v>907</v>
-      </c>
-      <c r="E98" s="138" t="s">
-        <v>908</v>
-      </c>
-      <c r="F98" s="138" t="s">
-        <v>909</v>
       </c>
       <c r="G98" s="138" t="s">
         <v>772</v>
       </c>
       <c r="H98" s="138" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="I98" s="138" t="s">
-        <v>911</v>
+        <v>909</v>
       </c>
       <c r="J98" s="138" t="s">
         <v>54</v>
@@ -9061,13 +9065,13 @@
         <v>551</v>
       </c>
       <c r="M98" s="138" t="s">
-        <v>912</v>
+        <v>910</v>
       </c>
       <c r="N98" s="138" t="s">
         <v>1</v>
       </c>
       <c r="O98" s="138" t="s">
-        <v>913</v>
+        <v>911</v>
       </c>
       <c r="P98" s="138" t="s">
         <v>143</v>
@@ -9075,31 +9079,31 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="138" t="s">
-        <v>914</v>
+        <v>912</v>
       </c>
       <c r="B99" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C99" s="138" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
       <c r="D99" s="138" t="s">
-        <v>915</v>
+        <v>913</v>
       </c>
       <c r="E99" s="138" t="s">
         <v>503</v>
       </c>
       <c r="F99" s="138" t="s">
+        <v>914</v>
+      </c>
+      <c r="G99" s="138" t="s">
+        <v>915</v>
+      </c>
+      <c r="H99" s="138" t="s">
         <v>916</v>
       </c>
-      <c r="G99" s="138" t="s">
+      <c r="I99" s="138" t="s">
         <v>917</v>
-      </c>
-      <c r="H99" s="138" t="s">
-        <v>918</v>
-      </c>
-      <c r="I99" s="138" t="s">
-        <v>919</v>
       </c>
       <c r="J99" s="138" t="s">
         <v>54</v>
@@ -9108,16 +9112,16 @@
         <v>1</v>
       </c>
       <c r="L99" s="138" t="s">
+        <v>918</v>
+      </c>
+      <c r="M99" s="138" t="s">
+        <v>919</v>
+      </c>
+      <c r="N99" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O99" s="138" t="s">
         <v>920</v>
-      </c>
-      <c r="M99" s="138" t="s">
-        <v>921</v>
-      </c>
-      <c r="N99" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O99" s="138" t="s">
-        <v>922</v>
       </c>
       <c r="P99" s="138" t="s">
         <v>223</v>
@@ -9125,31 +9129,31 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="138" t="s">
-        <v>923</v>
+        <v>921</v>
       </c>
       <c r="B100" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C100" s="138" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
       <c r="D100" s="138" t="s">
+        <v>922</v>
+      </c>
+      <c r="E100" s="138" t="s">
+        <v>923</v>
+      </c>
+      <c r="F100" s="138" t="s">
         <v>924</v>
       </c>
-      <c r="E100" s="138" t="s">
+      <c r="G100" s="138" t="s">
         <v>925</v>
       </c>
-      <c r="F100" s="138" t="s">
+      <c r="H100" s="138" t="s">
         <v>926</v>
       </c>
-      <c r="G100" s="138" t="s">
+      <c r="I100" s="138" t="s">
         <v>927</v>
-      </c>
-      <c r="H100" s="138" t="s">
-        <v>928</v>
-      </c>
-      <c r="I100" s="138" t="s">
-        <v>929</v>
       </c>
       <c r="J100" s="138" t="s">
         <v>54</v>
@@ -9158,16 +9162,16 @@
         <v>1</v>
       </c>
       <c r="L100" s="138" t="s">
+        <v>928</v>
+      </c>
+      <c r="M100" s="138" t="s">
+        <v>929</v>
+      </c>
+      <c r="N100" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O100" s="138" t="s">
         <v>930</v>
-      </c>
-      <c r="M100" s="138" t="s">
-        <v>931</v>
-      </c>
-      <c r="N100" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O100" s="138" t="s">
-        <v>932</v>
       </c>
       <c r="P100" s="138" t="s">
         <v>388</v>
@@ -9175,22 +9179,22 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="138" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
       <c r="B101" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C101" s="138" t="s">
+        <v>932</v>
+      </c>
+      <c r="D101" s="138" t="s">
+        <v>933</v>
+      </c>
+      <c r="E101" s="138" t="s">
         <v>934</v>
       </c>
-      <c r="D101" s="138" t="s">
+      <c r="F101" s="138" t="s">
         <v>935</v>
-      </c>
-      <c r="E101" s="138" t="s">
-        <v>936</v>
-      </c>
-      <c r="F101" s="138" t="s">
-        <v>937</v>
       </c>
       <c r="G101" s="138" t="s">
         <v>4</v>
@@ -9199,7 +9203,7 @@
         <v>615</v>
       </c>
       <c r="I101" s="138" t="s">
-        <v>938</v>
+        <v>936</v>
       </c>
       <c r="J101" s="138" t="s">
         <v>54</v>
@@ -9208,16 +9212,16 @@
         <v>1</v>
       </c>
       <c r="L101" s="138" t="s">
+        <v>937</v>
+      </c>
+      <c r="M101" s="138" t="s">
+        <v>938</v>
+      </c>
+      <c r="N101" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O101" s="138" t="s">
         <v>939</v>
-      </c>
-      <c r="M101" s="138" t="s">
-        <v>940</v>
-      </c>
-      <c r="N101" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O101" s="138" t="s">
-        <v>941</v>
       </c>
       <c r="P101" s="138" t="s">
         <v>143</v>
@@ -9225,31 +9229,31 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="138" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
       <c r="B102" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C102" s="138" t="s">
+        <v>932</v>
+      </c>
+      <c r="D102" s="138" t="s">
+        <v>941</v>
+      </c>
+      <c r="E102" s="138" t="s">
         <v>934</v>
       </c>
-      <c r="D102" s="138" t="s">
+      <c r="F102" s="138" t="s">
+        <v>942</v>
+      </c>
+      <c r="G102" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="H102" s="138" t="s">
         <v>943</v>
       </c>
-      <c r="E102" s="138" t="s">
-        <v>936</v>
-      </c>
-      <c r="F102" s="138" t="s">
+      <c r="I102" s="138" t="s">
         <v>944</v>
-      </c>
-      <c r="G102" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="H102" s="138" t="s">
-        <v>945</v>
-      </c>
-      <c r="I102" s="138" t="s">
-        <v>946</v>
       </c>
       <c r="J102" s="138" t="s">
         <v>54</v>
@@ -9258,16 +9262,16 @@
         <v>1</v>
       </c>
       <c r="L102" s="138" t="s">
+        <v>945</v>
+      </c>
+      <c r="M102" s="138" t="s">
+        <v>946</v>
+      </c>
+      <c r="N102" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O102" s="138" t="s">
         <v>947</v>
-      </c>
-      <c r="M102" s="138" t="s">
-        <v>948</v>
-      </c>
-      <c r="N102" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O102" s="138" t="s">
-        <v>949</v>
       </c>
       <c r="P102" s="138" t="s">
         <v>166</v>
@@ -9275,31 +9279,31 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="138" t="s">
-        <v>950</v>
+        <v>948</v>
       </c>
       <c r="B103" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C103" s="138" t="s">
+        <v>949</v>
+      </c>
+      <c r="D103" s="138" t="s">
+        <v>950</v>
+      </c>
+      <c r="E103" s="138" t="s">
         <v>951</v>
       </c>
-      <c r="D103" s="138" t="s">
+      <c r="F103" s="138" t="s">
         <v>952</v>
       </c>
-      <c r="E103" s="138" t="s">
+      <c r="G103" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="H103" s="138" t="s">
         <v>953</v>
       </c>
-      <c r="F103" s="138" t="s">
+      <c r="I103" s="138" t="s">
         <v>954</v>
-      </c>
-      <c r="G103" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="H103" s="138" t="s">
-        <v>955</v>
-      </c>
-      <c r="I103" s="138" t="s">
-        <v>956</v>
       </c>
       <c r="J103" s="138" t="s">
         <v>54</v>
@@ -9308,16 +9312,16 @@
         <v>1</v>
       </c>
       <c r="L103" s="138" t="s">
+        <v>955</v>
+      </c>
+      <c r="M103" s="138" t="s">
+        <v>956</v>
+      </c>
+      <c r="N103" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O103" s="138" t="s">
         <v>957</v>
-      </c>
-      <c r="M103" s="138" t="s">
-        <v>958</v>
-      </c>
-      <c r="N103" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O103" s="138" t="s">
-        <v>959</v>
       </c>
       <c r="P103" s="138" t="s">
         <v>166</v>
@@ -9325,31 +9329,31 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="138" t="s">
-        <v>960</v>
+        <v>958</v>
       </c>
       <c r="B104" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C104" s="138" t="s">
+        <v>959</v>
+      </c>
+      <c r="D104" s="138" t="s">
+        <v>960</v>
+      </c>
+      <c r="E104" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="F104" s="138" t="s">
         <v>961</v>
       </c>
-      <c r="D104" s="138" t="s">
+      <c r="G104" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="H104" s="138" t="s">
         <v>962</v>
       </c>
-      <c r="E104" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="F104" s="138" t="s">
+      <c r="I104" s="138" t="s">
         <v>963</v>
-      </c>
-      <c r="G104" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="H104" s="138" t="s">
-        <v>964</v>
-      </c>
-      <c r="I104" s="138" t="s">
-        <v>965</v>
       </c>
       <c r="J104" s="138" t="s">
         <v>54</v>
@@ -9358,16 +9362,16 @@
         <v>1</v>
       </c>
       <c r="L104" s="138" t="s">
+        <v>964</v>
+      </c>
+      <c r="M104" s="138" t="s">
+        <v>965</v>
+      </c>
+      <c r="N104" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O104" s="138" t="s">
         <v>966</v>
-      </c>
-      <c r="M104" s="138" t="s">
-        <v>967</v>
-      </c>
-      <c r="N104" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O104" s="138" t="s">
-        <v>968</v>
       </c>
       <c r="P104" s="138" t="s">
         <v>429</v>
@@ -9375,49 +9379,49 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="146" t="s">
+        <v>967</v>
+      </c>
+      <c r="B105" s="146" t="s">
+        <v>885</v>
+      </c>
+      <c r="C105" s="146" t="s">
+        <v>968</v>
+      </c>
+      <c r="D105" s="146" t="s">
         <v>969</v>
       </c>
-      <c r="B105" s="146" t="s">
-        <v>887</v>
-      </c>
-      <c r="C105" s="146" t="s">
+      <c r="E105" s="146" t="s">
+        <v>4</v>
+      </c>
+      <c r="F105" s="146" t="s">
         <v>970</v>
       </c>
-      <c r="D105" s="146" t="s">
+      <c r="G105" s="146" t="s">
+        <v>4</v>
+      </c>
+      <c r="H105" s="146" t="s">
         <v>971</v>
       </c>
-      <c r="E105" s="146" t="s">
-        <v>4</v>
-      </c>
-      <c r="F105" s="146" t="s">
+      <c r="I105" s="146" t="s">
         <v>972</v>
       </c>
-      <c r="G105" s="146" t="s">
-        <v>4</v>
-      </c>
-      <c r="H105" s="146" t="s">
+      <c r="J105" s="146" t="s">
         <v>973</v>
       </c>
-      <c r="I105" s="146" t="s">
+      <c r="K105" s="146" t="s">
+        <v>1</v>
+      </c>
+      <c r="L105" s="146" t="s">
         <v>974</v>
       </c>
-      <c r="J105" s="146" t="s">
+      <c r="M105" s="146" t="s">
         <v>975</v>
       </c>
-      <c r="K105" s="146" t="s">
-        <v>1</v>
-      </c>
-      <c r="L105" s="146" t="s">
+      <c r="N105" s="146" t="s">
+        <v>1</v>
+      </c>
+      <c r="O105" s="146" t="s">
         <v>976</v>
-      </c>
-      <c r="M105" s="146" t="s">
-        <v>977</v>
-      </c>
-      <c r="N105" s="146" t="s">
-        <v>1</v>
-      </c>
-      <c r="O105" s="146" t="s">
-        <v>978</v>
       </c>
       <c r="P105" s="146" t="s">
         <v>429</v>
@@ -9425,49 +9429,49 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="146" t="s">
+        <v>977</v>
+      </c>
+      <c r="B106" s="146" t="s">
+        <v>885</v>
+      </c>
+      <c r="C106" s="146" t="s">
+        <v>978</v>
+      </c>
+      <c r="D106" s="146" t="s">
         <v>979</v>
       </c>
-      <c r="B106" s="146" t="s">
-        <v>887</v>
-      </c>
-      <c r="C106" s="146" t="s">
+      <c r="E106" s="146" t="s">
+        <v>4</v>
+      </c>
+      <c r="F106" s="146" t="s">
         <v>980</v>
       </c>
-      <c r="D106" s="146" t="s">
+      <c r="G106" s="146" t="s">
+        <v>4</v>
+      </c>
+      <c r="H106" s="146" t="s">
+        <v>4</v>
+      </c>
+      <c r="I106" s="146" t="s">
         <v>981</v>
       </c>
-      <c r="E106" s="146" t="s">
-        <v>4</v>
-      </c>
-      <c r="F106" s="146" t="s">
+      <c r="J106" s="146" t="s">
+        <v>973</v>
+      </c>
+      <c r="K106" s="146" t="s">
+        <v>1</v>
+      </c>
+      <c r="L106" s="146" t="s">
         <v>982</v>
       </c>
-      <c r="G106" s="146" t="s">
-        <v>4</v>
-      </c>
-      <c r="H106" s="146" t="s">
-        <v>4</v>
-      </c>
-      <c r="I106" s="146" t="s">
+      <c r="M106" s="146" t="s">
         <v>983</v>
       </c>
-      <c r="J106" s="146" t="s">
-        <v>975</v>
-      </c>
-      <c r="K106" s="146" t="s">
-        <v>1</v>
-      </c>
-      <c r="L106" s="146" t="s">
+      <c r="N106" s="146" t="s">
+        <v>1</v>
+      </c>
+      <c r="O106" s="146" t="s">
         <v>984</v>
-      </c>
-      <c r="M106" s="146" t="s">
-        <v>985</v>
-      </c>
-      <c r="N106" s="146" t="s">
-        <v>1</v>
-      </c>
-      <c r="O106" s="146" t="s">
-        <v>986</v>
       </c>
       <c r="P106" s="146" t="s">
         <v>429</v>
@@ -9475,31 +9479,31 @@
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="138" t="s">
-        <v>987</v>
+        <v>985</v>
       </c>
       <c r="B107" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C107" s="138" t="s">
+        <v>986</v>
+      </c>
+      <c r="D107" s="138" t="s">
+        <v>987</v>
+      </c>
+      <c r="E107" s="138" t="s">
         <v>988</v>
       </c>
-      <c r="D107" s="138" t="s">
+      <c r="F107" s="138" t="s">
         <v>989</v>
-      </c>
-      <c r="E107" s="138" t="s">
-        <v>990</v>
-      </c>
-      <c r="F107" s="138" t="s">
-        <v>991</v>
       </c>
       <c r="G107" s="138" t="s">
         <v>772</v>
       </c>
       <c r="H107" s="138" t="s">
-        <v>992</v>
+        <v>990</v>
       </c>
       <c r="I107" s="138" t="s">
-        <v>993</v>
+        <v>991</v>
       </c>
       <c r="J107" s="138" t="s">
         <v>54</v>
@@ -9508,16 +9512,16 @@
         <v>1</v>
       </c>
       <c r="L107" s="138" t="s">
+        <v>992</v>
+      </c>
+      <c r="M107" s="138" t="s">
+        <v>993</v>
+      </c>
+      <c r="N107" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O107" s="138" t="s">
         <v>994</v>
-      </c>
-      <c r="M107" s="138" t="s">
-        <v>995</v>
-      </c>
-      <c r="N107" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O107" s="138" t="s">
-        <v>996</v>
       </c>
       <c r="P107" s="138" t="s">
         <v>166</v>
@@ -9525,31 +9529,31 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="138" t="s">
-        <v>997</v>
+        <v>995</v>
       </c>
       <c r="B108" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C108" s="138" t="s">
+        <v>996</v>
+      </c>
+      <c r="D108" s="138" t="s">
+        <v>997</v>
+      </c>
+      <c r="E108" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="F108" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="G108" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="H108" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="I108" s="138" t="s">
         <v>998</v>
-      </c>
-      <c r="D108" s="138" t="s">
-        <v>999</v>
-      </c>
-      <c r="E108" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="F108" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="G108" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="H108" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="I108" s="138" t="s">
-        <v>1000</v>
       </c>
       <c r="J108" s="138" t="s">
         <v>54</v>
@@ -9558,16 +9562,16 @@
         <v>1</v>
       </c>
       <c r="L108" s="138" t="s">
+        <v>999</v>
+      </c>
+      <c r="M108" s="138" t="s">
+        <v>1000</v>
+      </c>
+      <c r="N108" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O108" s="138" t="s">
         <v>1001</v>
-      </c>
-      <c r="M108" s="138" t="s">
-        <v>1002</v>
-      </c>
-      <c r="N108" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O108" s="138" t="s">
-        <v>1003</v>
       </c>
       <c r="P108" s="138" t="s">
         <v>223</v>
@@ -9575,31 +9579,31 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="138" t="s">
-        <v>1004</v>
+        <v>1002</v>
       </c>
       <c r="B109" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C109" s="138" t="s">
+        <v>1003</v>
+      </c>
+      <c r="D109" s="138" t="s">
+        <v>1004</v>
+      </c>
+      <c r="E109" s="138" t="s">
         <v>1005</v>
       </c>
-      <c r="D109" s="138" t="s">
+      <c r="F109" s="138" t="s">
         <v>1006</v>
-      </c>
-      <c r="E109" s="138" t="s">
-        <v>1007</v>
-      </c>
-      <c r="F109" s="138" t="s">
-        <v>1008</v>
       </c>
       <c r="G109" s="138" t="s">
         <v>448</v>
       </c>
       <c r="H109" s="138" t="s">
-        <v>1009</v>
+        <v>1007</v>
       </c>
       <c r="I109" s="138" t="s">
-        <v>1010</v>
+        <v>1008</v>
       </c>
       <c r="J109" s="138" t="s">
         <v>54</v>
@@ -9608,16 +9612,16 @@
         <v>1</v>
       </c>
       <c r="L109" s="138" t="s">
+        <v>1009</v>
+      </c>
+      <c r="M109" s="138" t="s">
+        <v>1010</v>
+      </c>
+      <c r="N109" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O109" s="138" t="s">
         <v>1011</v>
-      </c>
-      <c r="M109" s="138" t="s">
-        <v>1012</v>
-      </c>
-      <c r="N109" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O109" s="138" t="s">
-        <v>1013</v>
       </c>
       <c r="P109" s="138" t="s">
         <v>388</v>
@@ -9625,31 +9629,31 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="138" t="s">
-        <v>1014</v>
+        <v>1012</v>
       </c>
       <c r="B110" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C110" s="138" t="s">
+        <v>1013</v>
+      </c>
+      <c r="D110" s="138" t="s">
+        <v>1014</v>
+      </c>
+      <c r="E110" s="138" t="s">
         <v>1015</v>
       </c>
-      <c r="D110" s="138" t="s">
+      <c r="F110" s="138" t="s">
         <v>1016</v>
-      </c>
-      <c r="E110" s="138" t="s">
-        <v>1017</v>
-      </c>
-      <c r="F110" s="138" t="s">
-        <v>1018</v>
       </c>
       <c r="G110" s="138" t="s">
         <v>448</v>
       </c>
       <c r="H110" s="138" t="s">
-        <v>1019</v>
+        <v>1017</v>
       </c>
       <c r="I110" s="138" t="s">
-        <v>1020</v>
+        <v>1018</v>
       </c>
       <c r="J110" s="138" t="s">
         <v>54</v>
@@ -9658,16 +9662,16 @@
         <v>1</v>
       </c>
       <c r="L110" s="138" t="s">
+        <v>1019</v>
+      </c>
+      <c r="M110" s="138" t="s">
+        <v>1020</v>
+      </c>
+      <c r="N110" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O110" s="138" t="s">
         <v>1021</v>
-      </c>
-      <c r="M110" s="138" t="s">
-        <v>1022</v>
-      </c>
-      <c r="N110" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O110" s="138" t="s">
-        <v>1023</v>
       </c>
       <c r="P110" s="138" t="s">
         <v>388</v>
@@ -9675,49 +9679,49 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="135" t="s">
-        <v>1024</v>
+        <v>1022</v>
       </c>
       <c r="B111" s="135" t="s">
-        <v>1025</v>
+        <v>1023</v>
       </c>
       <c r="C111" s="135" t="s">
         <v>444</v>
       </c>
       <c r="D111" s="135" t="s">
+        <v>1024</v>
+      </c>
+      <c r="E111" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="F111" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="G111" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="H111" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="I111" s="135" t="s">
+        <v>1025</v>
+      </c>
+      <c r="J111" s="135" t="s">
         <v>1026</v>
-      </c>
-      <c r="E111" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="F111" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="G111" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="H111" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="I111" s="135" t="s">
-        <v>1027</v>
-      </c>
-      <c r="J111" s="135" t="s">
-        <v>1028</v>
       </c>
       <c r="K111" s="135" t="s">
         <v>88</v>
       </c>
       <c r="L111" s="135" t="s">
-        <v>1029</v>
+        <v>1027</v>
       </c>
       <c r="M111" s="135" t="s">
-        <v>1030</v>
+        <v>1028</v>
       </c>
       <c r="N111" s="135" t="s">
         <v>47</v>
       </c>
       <c r="O111" s="135" t="s">
-        <v>1031</v>
+        <v>1029</v>
       </c>
       <c r="P111" s="135" t="s">
         <v>223</v>
@@ -9725,31 +9729,31 @@
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="135" t="s">
-        <v>1032</v>
+        <v>1030</v>
       </c>
       <c r="B112" s="135" t="s">
         <v>443</v>
       </c>
       <c r="C112" s="135" t="s">
+        <v>1031</v>
+      </c>
+      <c r="D112" s="135" t="s">
+        <v>1032</v>
+      </c>
+      <c r="E112" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="F112" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="G112" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="H112" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="I112" s="135" t="s">
         <v>1033</v>
-      </c>
-      <c r="D112" s="135" t="s">
-        <v>1034</v>
-      </c>
-      <c r="E112" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="F112" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="G112" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="H112" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="I112" s="135" t="s">
-        <v>1035</v>
       </c>
       <c r="J112" s="135" t="s">
         <v>43</v>
@@ -9758,16 +9762,16 @@
         <v>88</v>
       </c>
       <c r="L112" s="135" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="M112" s="135" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
       <c r="N112" s="135" t="s">
         <v>47</v>
       </c>
       <c r="O112" s="135" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
       <c r="P112" s="135" t="s">
         <v>166</v>
@@ -9775,31 +9779,31 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="135" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
       <c r="B113" s="135" t="s">
         <v>443</v>
       </c>
       <c r="C113" s="135" t="s">
+        <v>1038</v>
+      </c>
+      <c r="D113" s="135" t="s">
+        <v>1039</v>
+      </c>
+      <c r="E113" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="F113" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="G113" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="H113" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="I113" s="135" t="s">
         <v>1040</v>
-      </c>
-      <c r="D113" s="135" t="s">
-        <v>1041</v>
-      </c>
-      <c r="E113" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="F113" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="G113" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="H113" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="I113" s="135" t="s">
-        <v>1042</v>
       </c>
       <c r="J113" s="135" t="s">
         <v>43</v>
@@ -9808,16 +9812,16 @@
         <v>88</v>
       </c>
       <c r="L113" s="135" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
       <c r="M113" s="135" t="s">
-        <v>1044</v>
+        <v>1042</v>
       </c>
       <c r="N113" s="135" t="s">
         <v>47</v>
       </c>
       <c r="O113" s="135" t="s">
-        <v>1045</v>
+        <v>1043</v>
       </c>
       <c r="P113" s="135" t="s">
         <v>153</v>
@@ -9825,49 +9829,49 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="136" t="s">
+        <v>1044</v>
+      </c>
+      <c r="B114" s="136" t="s">
+        <v>1045</v>
+      </c>
+      <c r="C114" s="136" t="s">
         <v>1046</v>
       </c>
-      <c r="B114" s="136" t="s">
+      <c r="D114" s="136" t="s">
         <v>1047</v>
       </c>
-      <c r="C114" s="136" t="s">
+      <c r="E114" s="136" t="s">
+        <v>4</v>
+      </c>
+      <c r="F114" s="136" t="s">
+        <v>4</v>
+      </c>
+      <c r="G114" s="136" t="s">
+        <v>4</v>
+      </c>
+      <c r="H114" s="136" t="s">
+        <v>4</v>
+      </c>
+      <c r="I114" s="136" t="s">
         <v>1048</v>
       </c>
-      <c r="D114" s="136" t="s">
+      <c r="J114" s="136" t="s">
         <v>1049</v>
-      </c>
-      <c r="E114" s="136" t="s">
-        <v>4</v>
-      </c>
-      <c r="F114" s="136" t="s">
-        <v>4</v>
-      </c>
-      <c r="G114" s="136" t="s">
-        <v>4</v>
-      </c>
-      <c r="H114" s="136" t="s">
-        <v>4</v>
-      </c>
-      <c r="I114" s="136" t="s">
-        <v>1050</v>
-      </c>
-      <c r="J114" s="136" t="s">
-        <v>1051</v>
       </c>
       <c r="K114" s="136" t="s">
         <v>44</v>
       </c>
       <c r="L114" s="136" t="s">
+        <v>1050</v>
+      </c>
+      <c r="M114" s="136" t="s">
+        <v>1051</v>
+      </c>
+      <c r="N114" s="136" t="s">
         <v>1052</v>
       </c>
-      <c r="M114" s="136" t="s">
+      <c r="O114" s="136" t="s">
         <v>1053</v>
-      </c>
-      <c r="N114" s="136" t="s">
-        <v>1054</v>
-      </c>
-      <c r="O114" s="136" t="s">
-        <v>1055</v>
       </c>
       <c r="P114" s="136" t="s">
         <v>239</v>

</xml_diff>

<commit_message>
bucket fix - backup
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1824" uniqueCount="1051">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1824" uniqueCount="1049">
   <si>
     <t>EFFECT MARKERS</t>
   </si>
@@ -43,7 +43,7 @@
     <t>Done</t>
   </si>
   <si>
-    <t>38</t>
+    <t>39</t>
   </si>
   <si>
     <t>DELTA</t>
@@ -55,7 +55,7 @@
     <t>Pending</t>
   </si>
   <si>
-    <t>18</t>
+    <t>17</t>
   </si>
   <si>
     <t>INDIRECT</t>
@@ -85,7 +85,7 @@
     <t>Complete</t>
   </si>
   <si>
-    <t>36%</t>
+    <t>37%</t>
   </si>
   <si>
     <t>QA TEST CASES</t>
@@ -1526,22 +1526,22 @@
     <t>DELTA normal publish recompute; scheduler X</t>
   </si>
   <si>
-    <t>Casey gains exactly one empty event-chat row with unread 0 while top Chats / Chat All / Event attention counters remain unchanged; Publish creates no automatic chat system message and no Casey notification; My Events remains 1 while Drafts changes 1 to 0; reload agrees with backend; Nova and Riley chat rows and counters remain unchanged; active card is 1 / 8 with pending badge 2; acceptance notification X</t>
-  </si>
-  <si>
-    <t>IMPLEMENTATION UPDATED; CLEAN MANUAL RETEST REQUIRED</t>
-  </si>
-  <si>
-    <t>Running hot-deploy frontend/backend builds green; focused local frontend suites 12/12; backend unit rerun stopped under memory pressure and remains pending</t>
-  </si>
-  <si>
-    <t>Publish once from Casey Drafts. Require unchanged Casey chat attention counters, exactly one empty Casey event chat with unread 0, no automatic system message or Casey notification, My Events still 1, the same counters after reload, no Nova/Riley chat change and no invitation-accepted notification.</t>
-  </si>
-  <si>
-    <t>CLEAN RETEST REQUIRED / INVALID SYSTEM-MESSAGE RUN RETAINED</t>
-  </si>
-  <si>
-    <t>Historical failure first omitted the Admin event chat, then the materialized chat used an automatic Event published system message to create attention and leaked a Casey notification. Publish now materializes an empty channel without changing chat attention counters or creating an automatic message; the periodic poll reconciles concurrent changes. A deterministic Draft can be restaged as manual-qa-checkpoint:v1:event-domain:event with zero chats and zero action deltas.</t>
+    <t>Casey gains exactly one empty event-chat row with unread 0 while top Chats / Chat All / Event attention counters remain unchanged; Publish creates no automatic chat system message and no Casey notification; My Events remains 1 while Drafts changes 1 to 0 from either Publish surface; reload agrees with backend; Nova and Riley chat rows and counters remain unchanged; active card is 1 / 8 with pending badge 2; acceptance notification X</t>
+  </si>
+  <si>
+    <t>FIX HOT-DEPLOYED / CLEAN REPLAY STAGED</t>
+  </si>
+  <si>
+    <t>Pre-Publish UI/persisted baseline passed. Draft Publish then exposed a stale my-events query total overwriting the inclusive counter until click/load; Publish from My Events appeared correct. Fix rejects list totals whose query scope is not current; shared SmartList unchanged; watcher rebuilt/hot-synced green. Contaminated fixture reset, verified not-staged and staged clean at 13:34:21Z: DR, Casey My Events1/Drafts1, zero chats/lifecycle artifacts/action deltas. Exactly three fresh sessions load the new bundle; Casey DOM shows My Events1</t>
+  </si>
+  <si>
+    <t>Replay only Draft Publish first: confirm My Events1/Drafts1, Publish once from Drafts, do not click My Events or reload, and require Drafts0 while My Events remains visibly1. Capture immediate persisted oracle before any second branch</t>
+  </si>
+  <si>
+    <t>FAIL / FIX READY FOR REPLAY</t>
+  </si>
+  <si>
+    <t>Historical failures omitted the Admin chat, then created an automatic system message/attention and Casey notification. Current chat producer appears correct, but the Draft producer exposed a stale-scope counter overwrite. Three policy regressions cover matching scope, stale previous scope and non-authoritative loading/calendar states. Clean replay remains required.</t>
   </si>
   <si>
     <t>EVENT-EDITOR-003</t>
@@ -2748,19 +2748,13 @@
     <t>With Nova chat open, Casey Unpublish yields one short bundle-resolved under-review notification within one interval; Casey Republish yields one green available-again row the same way; both titles are only the compact event name with no Manual/changed; Casey receives neither; stable rows are preserved; closing chat resumes deferred ordinary side-menu reconciliation</t>
   </si>
   <si>
-    <t>FIX HOT-DEPLOYED; MANUAL RETEST PENDING</t>
-  </si>
-  <si>
-    <t>Backend lifecycle scheduling plus Mongo/frontend en+hu i18n key mapping; shared UiPollCoordinator independent notification-lane regressions; existing backend/frontend hot-deploy green</t>
-  </si>
-  <si>
-    <t>Restage/reload, keep Nova chat open; Casey Unpublish then Publish; capture notification count/attention and concise rows without reload, then close chat and prove normal side-menu poll resumes</t>
-  </si>
-  <si>
-    <t>OPEN / FIX READY</t>
-  </si>
-  <si>
-    <t>Lifecycle messages are semantic bundle keys, not hard-coded UI strings. Notification template title is exactly @event_title; the event-domain QA fixture uses the compact QA prefix. All three Mongo i18n JSON seeds are generator-synchronized and audited; notification polling stays in its independent lane.</t>
+    <t>Detailed pack retained the completed retest: Nova left Activities -&gt; Chats open; Casey Unpublish added compact Under review within one 30-second foreground poll and Republish removed it without reload/close. The independently serialized notification lane delivered the concise lifecycle row throughout</t>
+  </si>
+  <si>
+    <t>Closed; repeat only after lifecycle notification scheduling/i18n, UiPollCoordinator notification-lane isolation, ordinary chat-list header delta polling or popup ownership changes</t>
+  </si>
+  <si>
+    <t>Lifecycle messages remain semantic bundle keys. Notification title is exactly @event_title. Chat-list header delta and notification polling are independent read-only lanes; stable rows are patched, not rebuilt. Matrix status reconciled to the already-recorded detailed PASS evidence on 2026-08-13.</t>
   </si>
   <si>
     <t>EVENT-CHAT-LIFECYCLE-001</t>
@@ -6953,7 +6947,7 @@
         <v>495</v>
       </c>
       <c r="K56" s="137" t="s">
-        <v>44</v>
+        <v>483</v>
       </c>
       <c r="L56" s="137" t="s">
         <v>496</v>
@@ -8822,82 +8816,82 @@
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="136" t="s">
+      <c r="A94" s="135" t="s">
         <v>861</v>
       </c>
-      <c r="B94" s="136" t="s">
+      <c r="B94" s="135" t="s">
         <v>841</v>
       </c>
-      <c r="C94" s="136" t="s">
+      <c r="C94" s="135" t="s">
         <v>862</v>
       </c>
-      <c r="D94" s="136" t="s">
+      <c r="D94" s="135" t="s">
         <v>863</v>
       </c>
-      <c r="E94" s="136" t="s">
-        <v>4</v>
-      </c>
-      <c r="F94" s="136" t="s">
+      <c r="E94" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="F94" s="135" t="s">
         <v>864</v>
       </c>
-      <c r="G94" s="136" t="s">
-        <v>4</v>
-      </c>
-      <c r="H94" s="136" t="s">
+      <c r="G94" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="H94" s="135" t="s">
         <v>865</v>
       </c>
-      <c r="I94" s="136" t="s">
+      <c r="I94" s="135" t="s">
         <v>866</v>
       </c>
-      <c r="J94" s="136" t="s">
+      <c r="J94" s="135" t="s">
+        <v>482</v>
+      </c>
+      <c r="K94" s="135" t="s">
+        <v>738</v>
+      </c>
+      <c r="L94" s="135" t="s">
         <v>867</v>
       </c>
-      <c r="K94" s="136" t="s">
-        <v>738</v>
-      </c>
-      <c r="L94" s="136" t="s">
+      <c r="M94" s="135" t="s">
         <v>868</v>
       </c>
-      <c r="M94" s="136" t="s">
+      <c r="N94" s="135" t="s">
+        <v>47</v>
+      </c>
+      <c r="O94" s="135" t="s">
         <v>869</v>
       </c>
-      <c r="N94" s="136" t="s">
-        <v>870</v>
-      </c>
-      <c r="O94" s="136" t="s">
-        <v>871</v>
-      </c>
-      <c r="P94" s="136" t="s">
+      <c r="P94" s="135" t="s">
         <v>429</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="146" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
       <c r="B95" s="146" t="s">
         <v>841</v>
       </c>
       <c r="C95" s="146" t="s">
+        <v>871</v>
+      </c>
+      <c r="D95" s="146" t="s">
+        <v>872</v>
+      </c>
+      <c r="E95" s="146" t="s">
+        <v>4</v>
+      </c>
+      <c r="F95" s="146" t="s">
         <v>873</v>
       </c>
-      <c r="D95" s="146" t="s">
+      <c r="G95" s="146" t="s">
+        <v>4</v>
+      </c>
+      <c r="H95" s="146" t="s">
         <v>874</v>
       </c>
-      <c r="E95" s="146" t="s">
-        <v>4</v>
-      </c>
-      <c r="F95" s="146" t="s">
+      <c r="I95" s="146" t="s">
         <v>875</v>
-      </c>
-      <c r="G95" s="146" t="s">
-        <v>4</v>
-      </c>
-      <c r="H95" s="146" t="s">
-        <v>876</v>
-      </c>
-      <c r="I95" s="146" t="s">
-        <v>877</v>
       </c>
       <c r="J95" s="146" t="s">
         <v>47</v>
@@ -8906,16 +8900,16 @@
         <v>738</v>
       </c>
       <c r="L95" s="146" t="s">
-        <v>878</v>
+        <v>876</v>
       </c>
       <c r="M95" s="146" t="s">
-        <v>879</v>
+        <v>877</v>
       </c>
       <c r="N95" s="146" t="s">
         <v>482</v>
       </c>
       <c r="O95" s="146" t="s">
-        <v>880</v>
+        <v>878</v>
       </c>
       <c r="P95" s="146" t="s">
         <v>429</v>
@@ -8923,49 +8917,49 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="138" t="s">
+        <v>879</v>
+      </c>
+      <c r="B96" s="138" t="s">
+        <v>880</v>
+      </c>
+      <c r="C96" s="138" t="s">
         <v>881</v>
       </c>
-      <c r="B96" s="138" t="s">
+      <c r="D96" s="138" t="s">
         <v>882</v>
       </c>
-      <c r="C96" s="138" t="s">
+      <c r="E96" s="138" t="s">
         <v>883</v>
       </c>
-      <c r="D96" s="138" t="s">
+      <c r="F96" s="138" t="s">
         <v>884</v>
       </c>
-      <c r="E96" s="138" t="s">
+      <c r="G96" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="H96" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="I96" s="138" t="s">
         <v>885</v>
       </c>
-      <c r="F96" s="138" t="s">
+      <c r="J96" s="138" t="s">
         <v>886</v>
       </c>
-      <c r="G96" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="H96" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="I96" s="138" t="s">
+      <c r="K96" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="L96" s="138" t="s">
         <v>887</v>
       </c>
-      <c r="J96" s="138" t="s">
+      <c r="M96" s="138" t="s">
         <v>888</v>
       </c>
-      <c r="K96" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="L96" s="138" t="s">
+      <c r="N96" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O96" s="138" t="s">
         <v>889</v>
-      </c>
-      <c r="M96" s="138" t="s">
-        <v>890</v>
-      </c>
-      <c r="N96" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O96" s="138" t="s">
-        <v>891</v>
       </c>
       <c r="P96" s="138" t="s">
         <v>429</v>
@@ -8973,49 +8967,49 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="138" t="s">
+        <v>890</v>
+      </c>
+      <c r="B97" s="138" t="s">
+        <v>880</v>
+      </c>
+      <c r="C97" s="138" t="s">
+        <v>891</v>
+      </c>
+      <c r="D97" s="138" t="s">
         <v>892</v>
       </c>
-      <c r="B97" s="138" t="s">
-        <v>882</v>
-      </c>
-      <c r="C97" s="138" t="s">
+      <c r="E97" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="F97" s="138" t="s">
         <v>893</v>
       </c>
-      <c r="D97" s="138" t="s">
+      <c r="G97" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="H97" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="I97" s="138" t="s">
         <v>894</v>
       </c>
-      <c r="E97" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="F97" s="138" t="s">
+      <c r="J97" s="138" t="s">
+        <v>886</v>
+      </c>
+      <c r="K97" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="L97" s="138" t="s">
         <v>895</v>
       </c>
-      <c r="G97" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="H97" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="I97" s="138" t="s">
+      <c r="M97" s="138" t="s">
         <v>896</v>
       </c>
-      <c r="J97" s="138" t="s">
-        <v>888</v>
-      </c>
-      <c r="K97" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="L97" s="138" t="s">
+      <c r="N97" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O97" s="138" t="s">
         <v>897</v>
-      </c>
-      <c r="M97" s="138" t="s">
-        <v>898</v>
-      </c>
-      <c r="N97" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O97" s="138" t="s">
-        <v>899</v>
       </c>
       <c r="P97" s="138" t="s">
         <v>429</v>
@@ -9023,31 +9017,31 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="138" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
       <c r="B98" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C98" s="138" t="s">
+        <v>899</v>
+      </c>
+      <c r="D98" s="138" t="s">
+        <v>900</v>
+      </c>
+      <c r="E98" s="138" t="s">
         <v>901</v>
       </c>
-      <c r="D98" s="138" t="s">
+      <c r="F98" s="138" t="s">
         <v>902</v>
-      </c>
-      <c r="E98" s="138" t="s">
-        <v>903</v>
-      </c>
-      <c r="F98" s="138" t="s">
-        <v>904</v>
       </c>
       <c r="G98" s="138" t="s">
         <v>772</v>
       </c>
       <c r="H98" s="138" t="s">
-        <v>905</v>
+        <v>903</v>
       </c>
       <c r="I98" s="138" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
       <c r="J98" s="138" t="s">
         <v>54</v>
@@ -9059,13 +9053,13 @@
         <v>551</v>
       </c>
       <c r="M98" s="138" t="s">
-        <v>907</v>
+        <v>905</v>
       </c>
       <c r="N98" s="138" t="s">
         <v>1</v>
       </c>
       <c r="O98" s="138" t="s">
-        <v>908</v>
+        <v>906</v>
       </c>
       <c r="P98" s="138" t="s">
         <v>143</v>
@@ -9073,31 +9067,31 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="138" t="s">
-        <v>909</v>
+        <v>907</v>
       </c>
       <c r="B99" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C99" s="138" t="s">
-        <v>901</v>
+        <v>899</v>
       </c>
       <c r="D99" s="138" t="s">
-        <v>910</v>
+        <v>908</v>
       </c>
       <c r="E99" s="138" t="s">
         <v>503</v>
       </c>
       <c r="F99" s="138" t="s">
+        <v>909</v>
+      </c>
+      <c r="G99" s="138" t="s">
+        <v>910</v>
+      </c>
+      <c r="H99" s="138" t="s">
         <v>911</v>
       </c>
-      <c r="G99" s="138" t="s">
+      <c r="I99" s="138" t="s">
         <v>912</v>
-      </c>
-      <c r="H99" s="138" t="s">
-        <v>913</v>
-      </c>
-      <c r="I99" s="138" t="s">
-        <v>914</v>
       </c>
       <c r="J99" s="138" t="s">
         <v>54</v>
@@ -9106,16 +9100,16 @@
         <v>1</v>
       </c>
       <c r="L99" s="138" t="s">
+        <v>913</v>
+      </c>
+      <c r="M99" s="138" t="s">
+        <v>914</v>
+      </c>
+      <c r="N99" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O99" s="138" t="s">
         <v>915</v>
-      </c>
-      <c r="M99" s="138" t="s">
-        <v>916</v>
-      </c>
-      <c r="N99" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O99" s="138" t="s">
-        <v>917</v>
       </c>
       <c r="P99" s="138" t="s">
         <v>223</v>
@@ -9123,31 +9117,31 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="138" t="s">
-        <v>918</v>
+        <v>916</v>
       </c>
       <c r="B100" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C100" s="138" t="s">
-        <v>901</v>
+        <v>899</v>
       </c>
       <c r="D100" s="138" t="s">
+        <v>917</v>
+      </c>
+      <c r="E100" s="138" t="s">
+        <v>918</v>
+      </c>
+      <c r="F100" s="138" t="s">
         <v>919</v>
       </c>
-      <c r="E100" s="138" t="s">
+      <c r="G100" s="138" t="s">
         <v>920</v>
       </c>
-      <c r="F100" s="138" t="s">
+      <c r="H100" s="138" t="s">
         <v>921</v>
       </c>
-      <c r="G100" s="138" t="s">
+      <c r="I100" s="138" t="s">
         <v>922</v>
-      </c>
-      <c r="H100" s="138" t="s">
-        <v>923</v>
-      </c>
-      <c r="I100" s="138" t="s">
-        <v>924</v>
       </c>
       <c r="J100" s="138" t="s">
         <v>54</v>
@@ -9156,16 +9150,16 @@
         <v>1</v>
       </c>
       <c r="L100" s="138" t="s">
+        <v>923</v>
+      </c>
+      <c r="M100" s="138" t="s">
+        <v>924</v>
+      </c>
+      <c r="N100" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O100" s="138" t="s">
         <v>925</v>
-      </c>
-      <c r="M100" s="138" t="s">
-        <v>926</v>
-      </c>
-      <c r="N100" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O100" s="138" t="s">
-        <v>927</v>
       </c>
       <c r="P100" s="138" t="s">
         <v>388</v>
@@ -9173,22 +9167,22 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="138" t="s">
-        <v>928</v>
+        <v>926</v>
       </c>
       <c r="B101" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C101" s="138" t="s">
+        <v>927</v>
+      </c>
+      <c r="D101" s="138" t="s">
+        <v>928</v>
+      </c>
+      <c r="E101" s="138" t="s">
         <v>929</v>
       </c>
-      <c r="D101" s="138" t="s">
+      <c r="F101" s="138" t="s">
         <v>930</v>
-      </c>
-      <c r="E101" s="138" t="s">
-        <v>931</v>
-      </c>
-      <c r="F101" s="138" t="s">
-        <v>932</v>
       </c>
       <c r="G101" s="138" t="s">
         <v>4</v>
@@ -9197,7 +9191,7 @@
         <v>615</v>
       </c>
       <c r="I101" s="138" t="s">
-        <v>933</v>
+        <v>931</v>
       </c>
       <c r="J101" s="138" t="s">
         <v>54</v>
@@ -9206,16 +9200,16 @@
         <v>1</v>
       </c>
       <c r="L101" s="138" t="s">
+        <v>932</v>
+      </c>
+      <c r="M101" s="138" t="s">
+        <v>933</v>
+      </c>
+      <c r="N101" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O101" s="138" t="s">
         <v>934</v>
-      </c>
-      <c r="M101" s="138" t="s">
-        <v>935</v>
-      </c>
-      <c r="N101" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O101" s="138" t="s">
-        <v>936</v>
       </c>
       <c r="P101" s="138" t="s">
         <v>143</v>
@@ -9223,31 +9217,31 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="138" t="s">
-        <v>937</v>
+        <v>935</v>
       </c>
       <c r="B102" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C102" s="138" t="s">
+        <v>927</v>
+      </c>
+      <c r="D102" s="138" t="s">
+        <v>936</v>
+      </c>
+      <c r="E102" s="138" t="s">
         <v>929</v>
       </c>
-      <c r="D102" s="138" t="s">
+      <c r="F102" s="138" t="s">
+        <v>937</v>
+      </c>
+      <c r="G102" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="H102" s="138" t="s">
         <v>938</v>
       </c>
-      <c r="E102" s="138" t="s">
-        <v>931</v>
-      </c>
-      <c r="F102" s="138" t="s">
+      <c r="I102" s="138" t="s">
         <v>939</v>
-      </c>
-      <c r="G102" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="H102" s="138" t="s">
-        <v>940</v>
-      </c>
-      <c r="I102" s="138" t="s">
-        <v>941</v>
       </c>
       <c r="J102" s="138" t="s">
         <v>54</v>
@@ -9256,16 +9250,16 @@
         <v>1</v>
       </c>
       <c r="L102" s="138" t="s">
+        <v>940</v>
+      </c>
+      <c r="M102" s="138" t="s">
+        <v>941</v>
+      </c>
+      <c r="N102" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O102" s="138" t="s">
         <v>942</v>
-      </c>
-      <c r="M102" s="138" t="s">
-        <v>943</v>
-      </c>
-      <c r="N102" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O102" s="138" t="s">
-        <v>944</v>
       </c>
       <c r="P102" s="138" t="s">
         <v>166</v>
@@ -9273,31 +9267,31 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="138" t="s">
-        <v>945</v>
+        <v>943</v>
       </c>
       <c r="B103" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C103" s="138" t="s">
+        <v>944</v>
+      </c>
+      <c r="D103" s="138" t="s">
+        <v>945</v>
+      </c>
+      <c r="E103" s="138" t="s">
         <v>946</v>
       </c>
-      <c r="D103" s="138" t="s">
+      <c r="F103" s="138" t="s">
         <v>947</v>
       </c>
-      <c r="E103" s="138" t="s">
+      <c r="G103" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="H103" s="138" t="s">
         <v>948</v>
       </c>
-      <c r="F103" s="138" t="s">
+      <c r="I103" s="138" t="s">
         <v>949</v>
-      </c>
-      <c r="G103" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="H103" s="138" t="s">
-        <v>950</v>
-      </c>
-      <c r="I103" s="138" t="s">
-        <v>951</v>
       </c>
       <c r="J103" s="138" t="s">
         <v>54</v>
@@ -9306,16 +9300,16 @@
         <v>1</v>
       </c>
       <c r="L103" s="138" t="s">
+        <v>950</v>
+      </c>
+      <c r="M103" s="138" t="s">
+        <v>951</v>
+      </c>
+      <c r="N103" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O103" s="138" t="s">
         <v>952</v>
-      </c>
-      <c r="M103" s="138" t="s">
-        <v>953</v>
-      </c>
-      <c r="N103" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O103" s="138" t="s">
-        <v>954</v>
       </c>
       <c r="P103" s="138" t="s">
         <v>166</v>
@@ -9323,31 +9317,31 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="138" t="s">
-        <v>955</v>
+        <v>953</v>
       </c>
       <c r="B104" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C104" s="138" t="s">
+        <v>954</v>
+      </c>
+      <c r="D104" s="138" t="s">
+        <v>955</v>
+      </c>
+      <c r="E104" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="F104" s="138" t="s">
         <v>956</v>
       </c>
-      <c r="D104" s="138" t="s">
+      <c r="G104" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="H104" s="138" t="s">
         <v>957</v>
       </c>
-      <c r="E104" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="F104" s="138" t="s">
+      <c r="I104" s="138" t="s">
         <v>958</v>
-      </c>
-      <c r="G104" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="H104" s="138" t="s">
-        <v>959</v>
-      </c>
-      <c r="I104" s="138" t="s">
-        <v>960</v>
       </c>
       <c r="J104" s="138" t="s">
         <v>54</v>
@@ -9356,16 +9350,16 @@
         <v>1</v>
       </c>
       <c r="L104" s="138" t="s">
+        <v>959</v>
+      </c>
+      <c r="M104" s="138" t="s">
+        <v>960</v>
+      </c>
+      <c r="N104" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O104" s="138" t="s">
         <v>961</v>
-      </c>
-      <c r="M104" s="138" t="s">
-        <v>962</v>
-      </c>
-      <c r="N104" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O104" s="138" t="s">
-        <v>963</v>
       </c>
       <c r="P104" s="138" t="s">
         <v>429</v>
@@ -9373,49 +9367,49 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="146" t="s">
+        <v>962</v>
+      </c>
+      <c r="B105" s="146" t="s">
+        <v>880</v>
+      </c>
+      <c r="C105" s="146" t="s">
+        <v>963</v>
+      </c>
+      <c r="D105" s="146" t="s">
         <v>964</v>
       </c>
-      <c r="B105" s="146" t="s">
-        <v>882</v>
-      </c>
-      <c r="C105" s="146" t="s">
+      <c r="E105" s="146" t="s">
+        <v>4</v>
+      </c>
+      <c r="F105" s="146" t="s">
         <v>965</v>
       </c>
-      <c r="D105" s="146" t="s">
+      <c r="G105" s="146" t="s">
+        <v>4</v>
+      </c>
+      <c r="H105" s="146" t="s">
         <v>966</v>
       </c>
-      <c r="E105" s="146" t="s">
-        <v>4</v>
-      </c>
-      <c r="F105" s="146" t="s">
+      <c r="I105" s="146" t="s">
         <v>967</v>
       </c>
-      <c r="G105" s="146" t="s">
-        <v>4</v>
-      </c>
-      <c r="H105" s="146" t="s">
+      <c r="J105" s="146" t="s">
         <v>968</v>
       </c>
-      <c r="I105" s="146" t="s">
+      <c r="K105" s="146" t="s">
+        <v>1</v>
+      </c>
+      <c r="L105" s="146" t="s">
         <v>969</v>
       </c>
-      <c r="J105" s="146" t="s">
+      <c r="M105" s="146" t="s">
         <v>970</v>
       </c>
-      <c r="K105" s="146" t="s">
-        <v>1</v>
-      </c>
-      <c r="L105" s="146" t="s">
+      <c r="N105" s="146" t="s">
+        <v>1</v>
+      </c>
+      <c r="O105" s="146" t="s">
         <v>971</v>
-      </c>
-      <c r="M105" s="146" t="s">
-        <v>972</v>
-      </c>
-      <c r="N105" s="146" t="s">
-        <v>1</v>
-      </c>
-      <c r="O105" s="146" t="s">
-        <v>973</v>
       </c>
       <c r="P105" s="146" t="s">
         <v>429</v>
@@ -9423,49 +9417,49 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="146" t="s">
+        <v>972</v>
+      </c>
+      <c r="B106" s="146" t="s">
+        <v>880</v>
+      </c>
+      <c r="C106" s="146" t="s">
+        <v>973</v>
+      </c>
+      <c r="D106" s="146" t="s">
         <v>974</v>
       </c>
-      <c r="B106" s="146" t="s">
-        <v>882</v>
-      </c>
-      <c r="C106" s="146" t="s">
+      <c r="E106" s="146" t="s">
+        <v>4</v>
+      </c>
+      <c r="F106" s="146" t="s">
         <v>975</v>
       </c>
-      <c r="D106" s="146" t="s">
+      <c r="G106" s="146" t="s">
+        <v>4</v>
+      </c>
+      <c r="H106" s="146" t="s">
+        <v>4</v>
+      </c>
+      <c r="I106" s="146" t="s">
         <v>976</v>
       </c>
-      <c r="E106" s="146" t="s">
-        <v>4</v>
-      </c>
-      <c r="F106" s="146" t="s">
+      <c r="J106" s="146" t="s">
+        <v>968</v>
+      </c>
+      <c r="K106" s="146" t="s">
+        <v>1</v>
+      </c>
+      <c r="L106" s="146" t="s">
         <v>977</v>
       </c>
-      <c r="G106" s="146" t="s">
-        <v>4</v>
-      </c>
-      <c r="H106" s="146" t="s">
-        <v>4</v>
-      </c>
-      <c r="I106" s="146" t="s">
+      <c r="M106" s="146" t="s">
         <v>978</v>
       </c>
-      <c r="J106" s="146" t="s">
-        <v>970</v>
-      </c>
-      <c r="K106" s="146" t="s">
-        <v>1</v>
-      </c>
-      <c r="L106" s="146" t="s">
+      <c r="N106" s="146" t="s">
+        <v>1</v>
+      </c>
+      <c r="O106" s="146" t="s">
         <v>979</v>
-      </c>
-      <c r="M106" s="146" t="s">
-        <v>980</v>
-      </c>
-      <c r="N106" s="146" t="s">
-        <v>1</v>
-      </c>
-      <c r="O106" s="146" t="s">
-        <v>981</v>
       </c>
       <c r="P106" s="146" t="s">
         <v>429</v>
@@ -9473,31 +9467,31 @@
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="138" t="s">
-        <v>982</v>
+        <v>980</v>
       </c>
       <c r="B107" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C107" s="138" t="s">
+        <v>981</v>
+      </c>
+      <c r="D107" s="138" t="s">
+        <v>982</v>
+      </c>
+      <c r="E107" s="138" t="s">
         <v>983</v>
       </c>
-      <c r="D107" s="138" t="s">
+      <c r="F107" s="138" t="s">
         <v>984</v>
-      </c>
-      <c r="E107" s="138" t="s">
-        <v>985</v>
-      </c>
-      <c r="F107" s="138" t="s">
-        <v>986</v>
       </c>
       <c r="G107" s="138" t="s">
         <v>772</v>
       </c>
       <c r="H107" s="138" t="s">
-        <v>987</v>
+        <v>985</v>
       </c>
       <c r="I107" s="138" t="s">
-        <v>988</v>
+        <v>986</v>
       </c>
       <c r="J107" s="138" t="s">
         <v>54</v>
@@ -9506,16 +9500,16 @@
         <v>1</v>
       </c>
       <c r="L107" s="138" t="s">
+        <v>987</v>
+      </c>
+      <c r="M107" s="138" t="s">
+        <v>988</v>
+      </c>
+      <c r="N107" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O107" s="138" t="s">
         <v>989</v>
-      </c>
-      <c r="M107" s="138" t="s">
-        <v>990</v>
-      </c>
-      <c r="N107" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O107" s="138" t="s">
-        <v>991</v>
       </c>
       <c r="P107" s="138" t="s">
         <v>166</v>
@@ -9523,31 +9517,31 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="138" t="s">
-        <v>992</v>
+        <v>990</v>
       </c>
       <c r="B108" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C108" s="138" t="s">
+        <v>991</v>
+      </c>
+      <c r="D108" s="138" t="s">
+        <v>992</v>
+      </c>
+      <c r="E108" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="F108" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="G108" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="H108" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="I108" s="138" t="s">
         <v>993</v>
-      </c>
-      <c r="D108" s="138" t="s">
-        <v>994</v>
-      </c>
-      <c r="E108" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="F108" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="G108" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="H108" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="I108" s="138" t="s">
-        <v>995</v>
       </c>
       <c r="J108" s="138" t="s">
         <v>54</v>
@@ -9556,16 +9550,16 @@
         <v>1</v>
       </c>
       <c r="L108" s="138" t="s">
+        <v>994</v>
+      </c>
+      <c r="M108" s="138" t="s">
+        <v>995</v>
+      </c>
+      <c r="N108" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O108" s="138" t="s">
         <v>996</v>
-      </c>
-      <c r="M108" s="138" t="s">
-        <v>997</v>
-      </c>
-      <c r="N108" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O108" s="138" t="s">
-        <v>998</v>
       </c>
       <c r="P108" s="138" t="s">
         <v>223</v>
@@ -9573,31 +9567,31 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="138" t="s">
-        <v>999</v>
+        <v>997</v>
       </c>
       <c r="B109" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C109" s="138" t="s">
+        <v>998</v>
+      </c>
+      <c r="D109" s="138" t="s">
+        <v>999</v>
+      </c>
+      <c r="E109" s="138" t="s">
         <v>1000</v>
       </c>
-      <c r="D109" s="138" t="s">
+      <c r="F109" s="138" t="s">
         <v>1001</v>
-      </c>
-      <c r="E109" s="138" t="s">
-        <v>1002</v>
-      </c>
-      <c r="F109" s="138" t="s">
-        <v>1003</v>
       </c>
       <c r="G109" s="138" t="s">
         <v>448</v>
       </c>
       <c r="H109" s="138" t="s">
-        <v>1004</v>
+        <v>1002</v>
       </c>
       <c r="I109" s="138" t="s">
-        <v>1005</v>
+        <v>1003</v>
       </c>
       <c r="J109" s="138" t="s">
         <v>54</v>
@@ -9606,16 +9600,16 @@
         <v>1</v>
       </c>
       <c r="L109" s="138" t="s">
+        <v>1004</v>
+      </c>
+      <c r="M109" s="138" t="s">
+        <v>1005</v>
+      </c>
+      <c r="N109" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O109" s="138" t="s">
         <v>1006</v>
-      </c>
-      <c r="M109" s="138" t="s">
-        <v>1007</v>
-      </c>
-      <c r="N109" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O109" s="138" t="s">
-        <v>1008</v>
       </c>
       <c r="P109" s="138" t="s">
         <v>388</v>
@@ -9623,31 +9617,31 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="138" t="s">
-        <v>1009</v>
+        <v>1007</v>
       </c>
       <c r="B110" s="138" t="s">
         <v>443</v>
       </c>
       <c r="C110" s="138" t="s">
+        <v>1008</v>
+      </c>
+      <c r="D110" s="138" t="s">
+        <v>1009</v>
+      </c>
+      <c r="E110" s="138" t="s">
         <v>1010</v>
       </c>
-      <c r="D110" s="138" t="s">
+      <c r="F110" s="138" t="s">
         <v>1011</v>
-      </c>
-      <c r="E110" s="138" t="s">
-        <v>1012</v>
-      </c>
-      <c r="F110" s="138" t="s">
-        <v>1013</v>
       </c>
       <c r="G110" s="138" t="s">
         <v>448</v>
       </c>
       <c r="H110" s="138" t="s">
-        <v>1014</v>
+        <v>1012</v>
       </c>
       <c r="I110" s="138" t="s">
-        <v>1015</v>
+        <v>1013</v>
       </c>
       <c r="J110" s="138" t="s">
         <v>54</v>
@@ -9656,16 +9650,16 @@
         <v>1</v>
       </c>
       <c r="L110" s="138" t="s">
+        <v>1014</v>
+      </c>
+      <c r="M110" s="138" t="s">
+        <v>1015</v>
+      </c>
+      <c r="N110" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O110" s="138" t="s">
         <v>1016</v>
-      </c>
-      <c r="M110" s="138" t="s">
-        <v>1017</v>
-      </c>
-      <c r="N110" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O110" s="138" t="s">
-        <v>1018</v>
       </c>
       <c r="P110" s="138" t="s">
         <v>388</v>
@@ -9673,49 +9667,49 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="135" t="s">
-        <v>1019</v>
+        <v>1017</v>
       </c>
       <c r="B111" s="135" t="s">
-        <v>1020</v>
+        <v>1018</v>
       </c>
       <c r="C111" s="135" t="s">
         <v>444</v>
       </c>
       <c r="D111" s="135" t="s">
+        <v>1019</v>
+      </c>
+      <c r="E111" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="F111" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="G111" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="H111" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="I111" s="135" t="s">
+        <v>1020</v>
+      </c>
+      <c r="J111" s="135" t="s">
         <v>1021</v>
-      </c>
-      <c r="E111" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="F111" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="G111" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="H111" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="I111" s="135" t="s">
-        <v>1022</v>
-      </c>
-      <c r="J111" s="135" t="s">
-        <v>1023</v>
       </c>
       <c r="K111" s="135" t="s">
         <v>88</v>
       </c>
       <c r="L111" s="135" t="s">
-        <v>1024</v>
+        <v>1022</v>
       </c>
       <c r="M111" s="135" t="s">
-        <v>1025</v>
+        <v>1023</v>
       </c>
       <c r="N111" s="135" t="s">
         <v>47</v>
       </c>
       <c r="O111" s="135" t="s">
-        <v>1026</v>
+        <v>1024</v>
       </c>
       <c r="P111" s="135" t="s">
         <v>223</v>
@@ -9723,31 +9717,31 @@
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="135" t="s">
-        <v>1027</v>
+        <v>1025</v>
       </c>
       <c r="B112" s="135" t="s">
         <v>443</v>
       </c>
       <c r="C112" s="135" t="s">
+        <v>1026</v>
+      </c>
+      <c r="D112" s="135" t="s">
+        <v>1027</v>
+      </c>
+      <c r="E112" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="F112" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="G112" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="H112" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="I112" s="135" t="s">
         <v>1028</v>
-      </c>
-      <c r="D112" s="135" t="s">
-        <v>1029</v>
-      </c>
-      <c r="E112" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="F112" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="G112" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="H112" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="I112" s="135" t="s">
-        <v>1030</v>
       </c>
       <c r="J112" s="135" t="s">
         <v>43</v>
@@ -9756,16 +9750,16 @@
         <v>88</v>
       </c>
       <c r="L112" s="135" t="s">
-        <v>1031</v>
+        <v>1029</v>
       </c>
       <c r="M112" s="135" t="s">
-        <v>1032</v>
+        <v>1030</v>
       </c>
       <c r="N112" s="135" t="s">
         <v>47</v>
       </c>
       <c r="O112" s="135" t="s">
-        <v>1033</v>
+        <v>1031</v>
       </c>
       <c r="P112" s="135" t="s">
         <v>166</v>
@@ -9773,31 +9767,31 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="135" t="s">
-        <v>1034</v>
+        <v>1032</v>
       </c>
       <c r="B113" s="135" t="s">
         <v>443</v>
       </c>
       <c r="C113" s="135" t="s">
+        <v>1033</v>
+      </c>
+      <c r="D113" s="135" t="s">
+        <v>1034</v>
+      </c>
+      <c r="E113" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="F113" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="G113" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="H113" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="I113" s="135" t="s">
         <v>1035</v>
-      </c>
-      <c r="D113" s="135" t="s">
-        <v>1036</v>
-      </c>
-      <c r="E113" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="F113" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="G113" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="H113" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="I113" s="135" t="s">
-        <v>1037</v>
       </c>
       <c r="J113" s="135" t="s">
         <v>43</v>
@@ -9806,16 +9800,16 @@
         <v>88</v>
       </c>
       <c r="L113" s="135" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
       <c r="M113" s="135" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
       <c r="N113" s="135" t="s">
         <v>47</v>
       </c>
       <c r="O113" s="135" t="s">
-        <v>1040</v>
+        <v>1038</v>
       </c>
       <c r="P113" s="135" t="s">
         <v>153</v>
@@ -9823,49 +9817,49 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="136" t="s">
+        <v>1039</v>
+      </c>
+      <c r="B114" s="136" t="s">
+        <v>1040</v>
+      </c>
+      <c r="C114" s="136" t="s">
         <v>1041</v>
       </c>
-      <c r="B114" s="136" t="s">
+      <c r="D114" s="136" t="s">
         <v>1042</v>
       </c>
-      <c r="C114" s="136" t="s">
+      <c r="E114" s="136" t="s">
+        <v>4</v>
+      </c>
+      <c r="F114" s="136" t="s">
+        <v>4</v>
+      </c>
+      <c r="G114" s="136" t="s">
+        <v>4</v>
+      </c>
+      <c r="H114" s="136" t="s">
+        <v>4</v>
+      </c>
+      <c r="I114" s="136" t="s">
         <v>1043</v>
       </c>
-      <c r="D114" s="136" t="s">
+      <c r="J114" s="136" t="s">
         <v>1044</v>
-      </c>
-      <c r="E114" s="136" t="s">
-        <v>4</v>
-      </c>
-      <c r="F114" s="136" t="s">
-        <v>4</v>
-      </c>
-      <c r="G114" s="136" t="s">
-        <v>4</v>
-      </c>
-      <c r="H114" s="136" t="s">
-        <v>4</v>
-      </c>
-      <c r="I114" s="136" t="s">
-        <v>1045</v>
-      </c>
-      <c r="J114" s="136" t="s">
-        <v>1046</v>
       </c>
       <c r="K114" s="136" t="s">
         <v>44</v>
       </c>
       <c r="L114" s="136" t="s">
+        <v>1045</v>
+      </c>
+      <c r="M114" s="136" t="s">
+        <v>1046</v>
+      </c>
+      <c r="N114" s="136" t="s">
         <v>1047</v>
       </c>
-      <c r="M114" s="136" t="s">
+      <c r="O114" s="136" t="s">
         <v>1048</v>
-      </c>
-      <c r="N114" s="136" t="s">
-        <v>1049</v>
-      </c>
-      <c r="O114" s="136" t="s">
-        <v>1050</v>
       </c>
       <c r="P114" s="136" t="s">
         <v>239</v>

</xml_diff>

<commit_message>
qa fix - activity events - counter
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -1790,10 +1790,10 @@
     <t>MANUAL UI / IN PROGRESS</t>
   </si>
   <si>
-    <t>Versioned fixture counter/creator-occupancy projection repairs; organizer-vs-participant Trash counter regression source; list-adapter error/empty regressions; guarded lifecycle baseline + terminal Trash verifier; existing dev frontend/backend owner builds PASS</t>
-  </si>
-  <si>
-    <t>Casey opens Events &gt; Trash and proves one organizer row; Nova then opens Notifications New and proves one unread event-deleted row without opening it; finally reconstruct both ownership results from a fresh read</t>
+    <t>Versioned fixture counter/creator-occupancy projection repairs; organizer-vs-participant Trash counter regression source; list-adapter error/empty regressions; full stored event-counter snapshot HTTP/store regression sources; guarded lifecycle baseline + terminal Trash verifier; existing dev frontend/backend owner builds PASS</t>
+  </si>
+  <si>
+    <t>Nova proves the unread event-deleted row without opening it; then use a fresh bundle/read and EVENT-LIFE-003 Restore as the inverse foreground full-snapshot counter replay without repeating Delete</t>
   </si>
   <si>
     <t>• Baseline staged 2026-08-13T19:44:57.209Z: public active QA EVENT-LIFE-002, Casey accepted Admin/owner, Nova accepted Member, canonical occupancy 2/8.
@@ -1810,7 +1810,10 @@
 • Focused recovery PASS: after restarting only the existing backend owner, Casey and Nova endpoints returned 200 with the same A/public 2/8 event; both already-open lists and badges recovered through normal poll without reload or interaction. The captured action baseline remained current.
 • Real producer PASS: Casey confirmed Delete Event once. Without reload, Casey My Events and Nova Active Events removed the card and active/hosting badges became zero. The user did not observe whether Casey Trash +1 came from the action delta or a later poll, so that timing branch is NOT EXECUTED and the producer is not replayed.
 • Terminal verifier PASS at 2026-08-13T20:46:09.146Z: T/statusBeforeSuppression=A/post-baseline trashedAtIso; unchanged Casey Admin + Nova Member 2/8 audit rows; Casey Hosting/All/Trash=0/0/1; Nova Events/Active/All/Trash=0/0/0/0.
-• Exactly one completed Nova-only deleted lifecycle task, one unread event-deleted Notification Center row, one matching dev-mode pending Firebase outbox and one terminal EVENT_CHANGED recompute were attributable to the saved action baseline. Oracle now exposes canonical lifecycle flags/timestamp and the guarded verify-lifecycle-trash command.</t>
+• Exactly one completed Nova-only deleted lifecycle task, one unread event-deleted Notification Center row, one matching dev-mode pending Firebase outbox and one terminal EVENT_CHANGED recompute were attributable to the saved action baseline. Oracle now exposes canonical lifecycle flags/timestamp and the guarded verify-lifecycle-trash command.
+• Casey's later Trash load PASS: exactly one QA EVENT-LIFE-002 card. The missed immediate Trash +1 timing remains NOT EXECUTED.
+• Nova's untouched Active foreground poll removed the card, but FAIL: inclusive All stayed 1 until switching to All returned no card and corrected the menu to 0. Persisted Active/All were already 0/0.
+• Proper-scope fix transports the complete stored write-side event snapshot on Java list pages through HTTP and frontend-local routes and applies it atomically; SmartList is unchanged. Runtime read oracle gives Nova All total0/full zeros and Casey Trash total1/trash1; both owner builds PASS. Fresh-bundle inverse runtime replay is pending.</t>
   </si>
   <si>
     <t>EVENT-LIFE-003</t>

</xml_diff>

<commit_message>
qa fix - no place available
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -31,7 +31,7 @@
     <t>Done</t>
   </si>
   <si>
-    <t>50 (38%)</t>
+    <t>52 (39%)</t>
   </si>
   <si>
     <t>X</t>
@@ -43,7 +43,7 @@
     <t>Pending</t>
   </si>
   <si>
-    <t>18</t>
+    <t>17</t>
   </si>
   <si>
     <t>DELTA</t>
@@ -55,7 +55,7 @@
     <t>Not started</t>
   </si>
   <si>
-    <t>65</t>
+    <t>64</t>
   </si>
   <si>
     <t>INDIRECT</t>
@@ -2076,13 +2076,13 @@
     <t>No duplicate member, overbooking, stale bell or rejected-user chat access</t>
   </si>
   <si>
-    <t>IN PROGRESS; BRANCH B FRONTEND REPLAY REQUIRED</t>
-  </si>
-  <si>
-    <t>Versioned invitation-full fixture, three fresh managed browser documents and independent Mongo/read oracle</t>
-  </si>
-  <si>
-    <t>Reset and replay only Casey Delete invitation; capture the event-card pending badge before poll, then continue independent capacity/idempotence branches</t>
+    <t>MANUAL UI + FUNCTIONAL PASS; FIX VERIFIED; CLOSED</t>
+  </si>
+  <si>
+    <t>Versioned invitation-full fixture, three fresh managed browser documents, exact demo-identity server replay and independent Mongo/read oracle</t>
+  </si>
+  <si>
+    <t>Closed; never repeat branches A-D unless invitation capacity or idempotence contracts change</t>
   </si>
   <si>
     <t>• Branch A first attempt is NOT EXECUTED because the fixture staged capacity1 around Casey+Nova accepted plus Riley's reserved invite.
@@ -2097,10 +2097,31 @@
 • FAIL: zero EVENT_MEMBERS_CHANGED tasks were stored although cancelling the pending invite released its reserved final seat; the same path also skipped waitlist promotion.
 • Java write repair now routes the released seat through the waitlist and otherwise refreshes dependent slot/event projections plus recompute, while preserving zero ticket/chat. Main source compiled through the existing watcher; two focused regression tests were authored but no separate Gradle process was started because swap was full.
 • Repair replay baseline staged at 16:01:33.676Z and proved again by read-only status: capacity3, accepted/pending2/1, Riley final-seat invite, chats0 and zero tasks/artifacts. Same three managed documents reloaded and match Casey My Events1, Nova Events1, Riley Invitations1, all Chats0.
+• Branch C independent baseline staged at 17:27:14.493Z; post-stage Casey/Nova/Riley hard reloads and a later oracle prove capacity3, accepted/pending2/1 with Riley reserving the final seat and zero tasks/artifacts.
+• Casey read-only candidate query returned multiple selectable non-members; a repeated Mongo oracle proved the query itself performed no write. The actual picker shows Riley selected and Farkas Anna as the visible new candidate.
+• Branch C first write at 19:48:43+02:00 is server/write PASS but UX FAIL: Farkas Anna was rejected with unchanged capacity3 accepted/pending2/1 and zero tasks/artifacts, yet the picker closed silently.
+• Repair requires one shared HTTP/local invite outcome, frontend-local capacity parity, the existing confirmation dialog in actionless information mode, and matching versioned en/hu local plus Mongo translations.
+• Branch C repair hot-deployed: Java returns committed members plus typed invited/rejected outcomes; shared HTTP/local handling enforces reserved-seat capacity parity; the existing dialog has an actionless notice mode. Frontend watcher built20:05:23+02:00/synced20:05:26; live Mongo API returned en.55 and hu.55 with the expected capacity/generic keys. Regression tests authored but not separately run because the dev pipeline owns compilation and swap is full.
+• Branch C repaired replay READY: reset-&gt;not-staged then one stage at18:11:43.640Z; repeated statuses prove capacity3 accepted/pending2/1, Riley final-seat reservation and zero artifacts. Same documents hard-reloaded after bundle sync at Casey18:13:10.693Z, Nova18:13:13.525Z, Riley18:13:16.460Z; initial My Events/Events/Invitations are1 and all Chats0.
+• First repaired display content/write PASS but close-control FAIL: correct capacity title/message, no action row and unchanged zero-write oracle, but standard top-right close was missing. Shared dialog now reuses existing .popup-close only for notice mode; watcher built20:21:31/synced20:21:33 and Casey alone reloaded18:22:14.622Z. Replay only this no-write display without reset.
+• Standard-close replay write PASS but visual proof pending: exact capacity3 accepted/pending2/1 and all artifacts0, but the dialog was closed by the 18:23:40.879Z DOM inspection. Accept explicit user confirmation that the visible X closed it, otherwise repeat only the no-write display and leave it open; no reset.
+• Branch C terminal PASS/CLOSED: user explicitly confirmed the visible standard top-right X closed the notice; combined screenshot proves exact message/no footer actions, and terminal oracle proves capacity3 accepted/pending2/1 with every artifact0. Never repeat Branch C.
+• Branch D next: fresh reset/stage, Riley accepts once through UI, snapshot exact membership/chat/task/notification effects, then replay the identical authenticated join once and require changed=false with every count unchanged.
+• Branch D READY: staged18:31:33.042Z; two statuses prove capacity3 accepted/pending2/1 and zero chats/tasks/acceptance artifacts/payments. Same documents reloaded Casey18:32:11.813Z, Nova18:32:15.329Z, Riley18:32:19.418Z; initial My Events/Events/Invitations1 and Chats0.
+• Branch D first UI Accept PASS at18:35:47.091901466Z: exact Casey+Nova+Riley accepted3/pending0, Riley Events1/Chats1/card3/3, unchanged Casey/Nova documents each Chats1. Fingerprint chat projections3, member-joined1, task1 id6a7f6003ae56910e99a48529, acceptance notifications2/outbox1, payments/basket0.
+• Raw replay18:38:34.950Z NOT IDEMPOTENCE EXECUTION / orchestration error: missing X-App-Session-Kind and X-Demo-User-Id authenticated the configured default member bf057de7c586eede7e84bdc7, creating that different actor's waitlist row. Preserve prior UI PASS, reset contamination, replay server pair with exact Riley headers; no user repeat.
+• Clean Riley server pair: first18:43:38.889Z recreated fingerprint; identical second18:44:10.885Z changed no persisted field/count but response incorrectly changed=true with counterDelta null. Common Java mapper now uses mutationApplied; regressions authored, watcher BUILD SUCCESSFUL/restarted20:45:47.587. Replay only response without reset.
+• Post-fix no-op18:47:37.568Z PASS: HTTP200 accepted changed=false counterDelta null; accepted3/pending0, Riley timestamp18:43:38.772815972Z, chat3/message1/task1 same id/availability, notifications2/outbox1, payments/basket0. Only terminal original-task read remains; no more joins.
+• Terminal worker PASS/CLOSED: task6a7f61daae56910e99a48530 done18:49:15.677199764Z attempt1/error-empty, pendingCount0; final membership/chat/notification/payment fingerprint unchanged. EVENT-INV-005 all branches PASS/CLOSED.
 • Java repair replay at 16:06:13.505868724Z PASS: one EVENT_MEMBERS_CHANGED task, completed 16:12:08.607775317Z attempt1/error-empty; capacity3, accepted/pending2/0 and every chat/notification control zero.
 • UI FAIL: event-card pending badge did not update from the action signal and only a later poll repaired it. Root cause was the common Activities consumer discarding membership sync while Event Editor was open. The absolute/idempotent sync is now always applied under stacked surfaces; no action-specific or Smart List poll branch was added. Existing frontend watcher built successfully in 7.612s.
 • The 16:13:41.562Z replay lineage is NOT EXECUTED because the reload boundary was not yet proven; no Delete occurred and the fixture was reset.
-• Current baseline staged 16:18:50.026Z and re-proved by read-only status: capacity3, accepted/pending2/1, Riley pending admin invite from Casey, chats0 and zero tasks/artifacts. All three existing documents were hard reloaded with cache/service-worker bypass; new time origins are Casey16:19:57.407Z, Nova16:19:55.167Z and Riley16:19:53.108Z. Replay only Casey Delete once and capture badge before poll.</t>
+• Current baseline staged 16:18:50.026Z and re-proved by read-only status: capacity3, accepted/pending2/1, Riley pending admin invite from Casey, chats0 and zero tasks/artifacts. All three existing documents were hard reloaded with cache/service-worker bypass; new time origins are Casey16:19:57.407Z, Nova16:19:55.167Z and Riley16:19:53.108Z.
+• Hard-reloaded replay at 16:54:18.515456561Z UI FAIL: Members/write succeeded but the event-card pending badge remained1 about ten seconds after Delete. Terminal Java oracle still PASS: one task done 16:59:28.940091047Z attempt1/error-empty, capacity3 accepted/pending2/0 and zero chat/notification controls.
+• Live Angular proof: membership signal already had pendingMembers0, but the common Activities consumer looked only in an empty EventsService cache and silently returned the stale row; the server-backed Smart List source held the complete capacity3 DTO. The consumer now resolves and re-caches that source, preserves known capacity and has a direct card fallback. No Delete-specific or poll/query branch changed. Existing watcher built/synced at 17:06:56Z; focused regression tests authored but not separately run with full swap.
+• Source-fallback replay baseline staged17:09:30.775Z and second status proves capacity3 accepted/pending2/1, Riley pending admin invite, chats0 and zero tasks/artifacts. Same three documents hard reloaded with repaired bundle at time origins Casey17:10:01.546Z, Nova17:10:01.160Z, Riley17:10:01.022Z; initial counters My Events1/Events1/Invitations1 and Chats0.
+• Final action17:17:47.400237969Z immediate UI/write PASS: Casey same document (origin17:17:39.954Z before action) has action-time signal pending0, row/source pending0 and capacity3, DOM 2/3 without red pending number; Riley unchanged document Invitations0 and Nova unchanged Events1. Oracle capacity3 accepted/pending2/0, Riley deleted, zero chat/notification controls, exactly one task.
+• Branch B worker terminal PASS/CLOSED at17:23:40.030663919Z: task done attempt1/error-empty, worker pendingCount0, capacity/members and every zero-artifact control unchanged. Never repeat Casey Delete; reset before independent capacity branch.</t>
   </si>
   <si>
     <t>EVENT-INV-006</t>
@@ -2121,13 +2142,13 @@
     <t>Open notifies Admin plus visible pending control; Blind notifies Admin only; actor never receives own acceptance; each chat has one join row and zero system-derived chat notifications</t>
   </si>
   <si>
-    <t>Backend and local Open/Blind recipient tests added; system-chat notification regression added</t>
-  </si>
-  <si>
-    <t>Compare Casey, Nova and Riley Notification Center rows by printed eventId and blindMode, then count member-joined rows and chat-message notification artifacts</t>
-  </si>
-  <si>
-    <t>Independent privacy boundary; do not infer it from chat authorization</t>
+    <t>Backend and local Open/Blind recipient tests added; system-chat notification regression added; backend dev-profile hot reload PASS with 2s member-change debounce while production remains 5m</t>
+  </si>
+  <si>
+    <t>Closed; repeat only after acceptance recipient visibility, Blind member visibility, join-system-message notification suppression or affinity task scheduling changes</t>
+  </si>
+  <si>
+    <t>• Open: Riley accepted; Casey and visible pending Nova alone received the acceptance row; Riley received none.\n• Blind used a role-equivalent actor/control swap: Nova accepted; Casey alone received the row; actor Nova and hidden pending Riley received none.\n• UI and oracle agreed; both event chats contain one member-joined row and zero chat-message notifications.\n• Both event-scoped recompute tasks completed exactly once with empty error and unchanged accepted2/pending1 fingerprints.\n• Dev member-change debounce is now 2s to avoid the production five-minute wait during manual QA.</t>
   </si>
   <si>
     <t>CHAT-AUTH-001</t>
@@ -6518,7 +6539,7 @@
       </c>
       <c r="E1" s="149" t="str">
         <f>COUNTIFS(Q10:Q198,"Done",R10:R198,"Core")&amp;" ("&amp;IF(COUNTIF(R10:R198,"Core")=0,"0%",TEXT(COUNTIFS(Q10:Q198,"Done",R10:R198,"Core")/COUNTIF(R10:R198,"Core"),"0%"))&amp;")"</f>
-        <v>50 (38%)</v>
+        <v>52 (39%)</v>
       </c>
       <c r="F1" s="146" t="s">
         <v>1</v>
@@ -6569,7 +6590,7 @@
       </c>
       <c r="E2" s="159">
         <f>COUNTIFS(Q10:Q198,"Pending",R10:R198,"Core")</f>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F2" s="146" t="s">
         <v>1</v>
@@ -6620,7 +6641,7 @@
       </c>
       <c r="E3" s="175">
         <f>COUNTIFS(Q10:Q198,"Not started",R10:R198,"Core")</f>
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F3" s="146" t="s">
         <v>1</v>
@@ -10615,57 +10636,57 @@
       </c>
     </row>
     <row r="73" customFormat="false" ht="180" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A73" s="146" t="s">
+      <c r="A73" s="135" t="s">
         <v>653</v>
       </c>
-      <c r="B73" s="146" t="s">
+      <c r="B73" s="135" t="s">
         <v>447</v>
       </c>
-      <c r="C73" s="146" t="s">
+      <c r="C73" s="135" t="s">
         <v>654</v>
       </c>
-      <c r="D73" s="146" t="s">
+      <c r="D73" s="135" t="s">
         <v>655</v>
       </c>
-      <c r="E73" s="146" t="s">
+      <c r="E73" s="135" t="s">
         <v>656</v>
       </c>
-      <c r="F73" s="146" t="s">
+      <c r="F73" s="135" t="s">
         <v>657</v>
       </c>
-      <c r="G73" s="146" t="s">
+      <c r="G73" s="135" t="s">
         <v>656</v>
       </c>
-      <c r="H73" s="146" t="s">
+      <c r="H73" s="135" t="s">
         <v>658</v>
       </c>
-      <c r="I73" s="146" t="s">
+      <c r="I73" s="135" t="s">
         <v>659</v>
       </c>
-      <c r="J73" s="146" t="s">
+      <c r="J73" s="135" t="s">
         <v>660</v>
       </c>
-      <c r="K73" s="146" t="s">
+      <c r="K73" s="135" t="s">
         <v>591</v>
       </c>
-      <c r="L73" s="146" t="s">
+      <c r="L73" s="135" t="s">
         <v>661</v>
       </c>
-      <c r="M73" s="146" t="s">
+      <c r="M73" s="135" t="s">
         <v>662</v>
       </c>
-      <c r="N73" s="146" t="s">
-        <v>1</v>
-      </c>
-      <c r="O73" s="146" t="s">
+      <c r="N73" s="135" t="s">
+        <v>51</v>
+      </c>
+      <c r="O73" s="135" t="s">
         <v>663</v>
       </c>
-      <c r="P73" s="146" t="s">
+      <c r="P73" s="135" t="s">
         <v>392</v>
       </c>
       <c r="Q73" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",J73&amp;" "&amp;N73)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",J73&amp;" "&amp;N73))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",J73&amp;" "&amp;N73)),ISNUMBER(SEARCH("NOT IMPLEMENTED",J73&amp;" "&amp;N73))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",J73&amp;" "&amp;N73)),ISNUMBER(SEARCH("PENDING",J73&amp;" "&amp;N73)),ISNUMBER(SEARCH("IN PROGRESS",J73&amp;" "&amp;N73)),ISNUMBER(SEARCH("OPEN",J73&amp;" "&amp;N73)),ISNUMBER(SEARCH("RETEST REQUIRED",J73&amp;" "&amp;N73)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",J73&amp;" "&amp;N73)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",J73&amp;" "&amp;N73))),"Pending",IF(OR(N73="PASS",ISNUMBER(SEARCH("PASS",J73&amp;" "&amp;N73))),"Done","Pending"))))</f>
-        <v>Pending</v>
+        <v>Done</v>
       </c>
       <c r="R73" s="146" t="str">
         <f>IF(OR(LEFT(A73,9)="OPERATOR-",LEFT(A73,8)="PAYMENT-",LEFT(A73,7)="DEPLOY-"),"External","Core")</f>
@@ -10673,57 +10694,57 @@
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="138" t="s">
+      <c r="A74" s="135" t="s">
         <v>664</v>
       </c>
-      <c r="B74" s="138" t="s">
+      <c r="B74" s="135" t="s">
         <v>447</v>
       </c>
-      <c r="C74" s="138" t="s">
+      <c r="C74" s="135" t="s">
         <v>665</v>
       </c>
-      <c r="D74" s="138" t="s">
+      <c r="D74" s="135" t="s">
         <v>666</v>
       </c>
-      <c r="E74" s="138" t="s">
+      <c r="E74" s="135" t="s">
         <v>667</v>
       </c>
-      <c r="F74" s="138" t="s">
+      <c r="F74" s="135" t="s">
         <v>668</v>
       </c>
-      <c r="G74" s="138" t="s">
+      <c r="G74" s="135" t="s">
         <v>618</v>
       </c>
-      <c r="H74" s="138" t="s">
+      <c r="H74" s="135" t="s">
         <v>637</v>
       </c>
-      <c r="I74" s="138" t="s">
+      <c r="I74" s="135" t="s">
         <v>669</v>
       </c>
-      <c r="J74" s="138" t="s">
-        <v>58</v>
-      </c>
-      <c r="K74" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="L74" s="138" t="s">
+      <c r="J74" s="135" t="s">
+        <v>486</v>
+      </c>
+      <c r="K74" s="135" t="s">
+        <v>591</v>
+      </c>
+      <c r="L74" s="135" t="s">
         <v>670</v>
       </c>
-      <c r="M74" s="138" t="s">
+      <c r="M74" s="135" t="s">
         <v>671</v>
       </c>
-      <c r="N74" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O74" s="138" t="s">
+      <c r="N74" s="135" t="s">
+        <v>51</v>
+      </c>
+      <c r="O74" s="135" t="s">
         <v>672</v>
       </c>
-      <c r="P74" s="138" t="s">
+      <c r="P74" s="135" t="s">
         <v>433</v>
       </c>
       <c r="Q74" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",J74&amp;" "&amp;N74)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",J74&amp;" "&amp;N74))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",J74&amp;" "&amp;N74)),ISNUMBER(SEARCH("NOT IMPLEMENTED",J74&amp;" "&amp;N74))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",J74&amp;" "&amp;N74)),ISNUMBER(SEARCH("PENDING",J74&amp;" "&amp;N74)),ISNUMBER(SEARCH("IN PROGRESS",J74&amp;" "&amp;N74)),ISNUMBER(SEARCH("OPEN",J74&amp;" "&amp;N74)),ISNUMBER(SEARCH("RETEST REQUIRED",J74&amp;" "&amp;N74)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",J74&amp;" "&amp;N74)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",J74&amp;" "&amp;N74))),"Pending",IF(OR(N74="PASS",ISNUMBER(SEARCH("PASS",J74&amp;" "&amp;N74))),"Done","Pending"))))</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="R74" s="146" t="str">
         <f>IF(OR(LEFT(A74,9)="OPERATOR-",LEFT(A74,8)="PAYMENT-",LEFT(A74,7)="DEPLOY-"),"External","Core")</f>

</xml_diff>

<commit_message>
qa fix - tournament
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -31,7 +31,7 @@
     <t>Done</t>
   </si>
   <si>
-    <t>53 (40%)</t>
+    <t>54 (41%)</t>
   </si>
   <si>
     <t>X</t>
@@ -43,7 +43,7 @@
     <t>Pending</t>
   </si>
   <si>
-    <t>19</t>
+    <t>18</t>
   </si>
   <si>
     <t>DELTA</t>
@@ -55,7 +55,7 @@
     <t>Not started</t>
   </si>
   <si>
-    <t>61</t>
+    <t>60</t>
   </si>
   <si>
     <t>INDIRECT</t>
@@ -67,7 +67,7 @@
     <t>Failed</t>
   </si>
   <si>
-    <t>0</t>
+    <t>1</t>
   </si>
   <si>
     <t>GAP</t>
@@ -2982,46 +2982,46 @@
     <t>Parent, stages, capacities, sequence and initial counts agree</t>
   </si>
   <si>
+    <t>Shared Java and frontend-local group-count policy coverage; tournament service coverage partial</t>
+  </si>
+  <si>
+    <t>Reset cleanly, then stage TOURNAMENT-002 and capture the real grouping identities</t>
+  </si>
+  <si>
+    <t>Published runtime repair replay showed Qualifiers Groups: 2 × 1–2 members with A–B and Final Groups: 1 × 1–2 members with A only. The separate draft editor screenshots 13-16-22/05/10 proved Tournament, parent 1–8, Qualifiers 60/0, per-group 1–2, Score, advance 1 and estimate 1–4; Final 45/0, per-group 1–2, Score, advance 0 and estimate 1–2. The final oracle retained DR/published=false, three exact accepted identities and zero runtime/group/leaderboard/task/outbox writes. Published locking is respected: the checkpoint no longer asks for Unpublish merely to reach Edit Event.</t>
+  </si>
+  <si>
+    <t>TOURNAMENT-002</t>
+  </si>
+  <si>
+    <t>Run real grouping and inspect group membership</t>
+  </si>
+  <si>
+    <t>DELTA group/member/chat materialization</t>
+  </si>
+  <si>
+    <t>INDIRECT after membership changes</t>
+  </si>
+  <si>
+    <t>DELTA named real grouping path</t>
+  </si>
+  <si>
+    <t>Each accepted user occurs once in the correct group and group chat</t>
+  </si>
+  <si>
     <t>IN PROGRESS</t>
   </si>
   <si>
-    <t>Shared Java and frontend-local group-count policy coverage; tournament service coverage partial</t>
-  </si>
-  <si>
-    <t>Inspect the explicit draft Event Editor definition without saving, then compare it with the persisted oracle</t>
-  </si>
-  <si>
-    <t>PARTIAL PASS</t>
-  </si>
-  <si>
-    <t>Runtime branch repaired and replayed: Qualifiers now shows Groups: 2 × 1–2 members with A–B; Final shows Groups: 1 × 1–2 members with only A. Post-view oracle retained the exact 3/8 identities and zero runtime group, leaderboard, task and outbox writes. The checkpoint incorrectly assumed Manage Event was reachable from the published card; because published details are locked, the final editor branch now uses a separate explicit draft fixture and never asks for an Unpublish mutation.</t>
-  </si>
-  <si>
-    <t>TOURNAMENT-002</t>
-  </si>
-  <si>
-    <t>Run real grouping and inspect group membership</t>
-  </si>
-  <si>
-    <t>DELTA group/member/chat materialization</t>
-  </si>
-  <si>
-    <t>INDIRECT after membership changes</t>
-  </si>
-  <si>
-    <t>DELTA named real grouping path</t>
-  </si>
-  <si>
-    <t>Each accepted user occurs once in the correct group and group chat</t>
-  </si>
-  <si>
-    <t>Random grouping fixture/service coverage</t>
-  </si>
-  <si>
-    <t>Match parent, stage, group, member and chat identities</t>
-  </si>
-  <si>
-    <t>Pending invites are not accepted group members</t>
+    <t>Random grouping fixture/service coverage; versioned activity-counter and stage-time oracle added</t>
+  </si>
+  <si>
+    <t>Replay Start Stage once, then match parent, stage, group, member, chat and counter identities</t>
+  </si>
+  <si>
+    <t>FAIL / REPLAY REQUIRED</t>
+  </si>
+  <si>
+    <t>Initial fixture omitted actor event counters and physical subEvents startAt/endAt. Counters are now snapshotted/synchronized. First Start returned unchanged RS and the UI correctly showed Stage action was not applied; post-action oracle proved zero partial writes. Root cause: UI could derive visible stage time while the backend guard requires the persisted stage instant. Fixture now materializes production-shaped stage times; clean replay required.</t>
   </si>
   <si>
     <t>TOURNAMENT-003</t>
@@ -6568,7 +6568,7 @@
       </c>
       <c r="E1" s="149" t="str">
         <f>COUNTIFS(Q10:Q198,"Done",R10:R198,"Core")&amp;" ("&amp;IF(COUNTIF(R10:R198,"Core")=0,"0%",TEXT(COUNTIFS(Q10:Q198,"Done",R10:R198,"Core")/COUNTIF(R10:R198,"Core"),"0%"))&amp;")"</f>
-        <v>53 (40%)</v>
+        <v>54 (41%)</v>
       </c>
       <c r="F1" s="146" t="s">
         <v>1</v>
@@ -6619,7 +6619,7 @@
       </c>
       <c r="E2" s="159">
         <f>COUNTIFS(Q10:Q198,"Pending",R10:R198,"Core")</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F2" s="146" t="s">
         <v>1</v>
@@ -6670,7 +6670,7 @@
       </c>
       <c r="E3" s="175">
         <f>COUNTIFS(Q10:Q198,"Not started",R10:R198,"Core")</f>
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F3" s="146" t="s">
         <v>1</v>
@@ -6721,7 +6721,7 @@
       </c>
       <c r="E4" s="167">
         <f>COUNTIFS(Q10:Q198,"Failed",R10:R198,"Core")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" s="146" t="s">
         <v>1</v>
@@ -12173,57 +12173,57 @@
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="136" t="s">
+      <c r="A99" s="135" t="s">
         <v>904</v>
       </c>
-      <c r="B99" s="136" t="s">
+      <c r="B99" s="135" t="s">
         <v>447</v>
       </c>
-      <c r="C99" s="136" t="s">
+      <c r="C99" s="135" t="s">
         <v>905</v>
       </c>
-      <c r="D99" s="136" t="s">
+      <c r="D99" s="135" t="s">
         <v>906</v>
       </c>
-      <c r="E99" s="136" t="s">
+      <c r="E99" s="135" t="s">
         <v>907</v>
       </c>
-      <c r="F99" s="136" t="s">
+      <c r="F99" s="135" t="s">
         <v>908</v>
       </c>
-      <c r="G99" s="136" t="s">
+      <c r="G99" s="135" t="s">
         <v>777</v>
       </c>
-      <c r="H99" s="136" t="s">
+      <c r="H99" s="135" t="s">
         <v>909</v>
       </c>
-      <c r="I99" s="136" t="s">
+      <c r="I99" s="135" t="s">
         <v>910</v>
       </c>
-      <c r="J99" s="136" t="s">
+      <c r="J99" s="135" t="s">
+        <v>47</v>
+      </c>
+      <c r="K99" s="135" t="s">
+        <v>900</v>
+      </c>
+      <c r="L99" s="135" t="s">
         <v>911</v>
       </c>
-      <c r="K99" s="136" t="s">
-        <v>900</v>
-      </c>
-      <c r="L99" s="136" t="s">
+      <c r="M99" s="135" t="s">
         <v>912</v>
       </c>
-      <c r="M99" s="136" t="s">
+      <c r="N99" s="135" t="s">
+        <v>51</v>
+      </c>
+      <c r="O99" s="135" t="s">
         <v>913</v>
       </c>
-      <c r="N99" s="136" t="s">
-        <v>914</v>
-      </c>
-      <c r="O99" s="136" t="s">
-        <v>915</v>
-      </c>
-      <c r="P99" s="136" t="s">
+      <c r="P99" s="135" t="s">
         <v>147</v>
       </c>
       <c r="Q99" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",J99&amp;" "&amp;N99)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",J99&amp;" "&amp;N99))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",J99&amp;" "&amp;N99)),ISNUMBER(SEARCH("NOT IMPLEMENTED",J99&amp;" "&amp;N99))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",J99&amp;" "&amp;N99)),ISNUMBER(SEARCH("PENDING",J99&amp;" "&amp;N99)),ISNUMBER(SEARCH("IN PROGRESS",J99&amp;" "&amp;N99)),ISNUMBER(SEARCH("OPEN",J99&amp;" "&amp;N99)),ISNUMBER(SEARCH("RETEST REQUIRED",J99&amp;" "&amp;N99)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",J99&amp;" "&amp;N99)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",J99&amp;" "&amp;N99))),"Pending",IF(OR(N99="PASS",ISNUMBER(SEARCH("PASS",J99&amp;" "&amp;N99))),"Done","Pending"))))</f>
-        <v>Pending</v>
+        <v>Done</v>
       </c>
       <c r="R99" s="146" t="str">
         <f>IF(OR(LEFT(A99,9)="OPERATOR-",LEFT(A99,8)="PAYMENT-",LEFT(A99,7)="DEPLOY-"),"External","Core")</f>
@@ -12231,57 +12231,57 @@
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="138" t="s">
+      <c r="A100" s="137" t="s">
+        <v>914</v>
+      </c>
+      <c r="B100" s="137" t="s">
+        <v>447</v>
+      </c>
+      <c r="C100" s="137" t="s">
+        <v>905</v>
+      </c>
+      <c r="D100" s="137" t="s">
+        <v>915</v>
+      </c>
+      <c r="E100" s="137" t="s">
+        <v>506</v>
+      </c>
+      <c r="F100" s="137" t="s">
         <v>916</v>
       </c>
-      <c r="B100" s="138" t="s">
-        <v>447</v>
-      </c>
-      <c r="C100" s="138" t="s">
-        <v>905</v>
-      </c>
-      <c r="D100" s="138" t="s">
+      <c r="G100" s="137" t="s">
         <v>917</v>
       </c>
-      <c r="E100" s="138" t="s">
-        <v>506</v>
-      </c>
-      <c r="F100" s="138" t="s">
+      <c r="H100" s="137" t="s">
         <v>918</v>
       </c>
-      <c r="G100" s="138" t="s">
+      <c r="I100" s="137" t="s">
         <v>919</v>
       </c>
-      <c r="H100" s="138" t="s">
+      <c r="J100" s="137" t="s">
         <v>920</v>
       </c>
-      <c r="I100" s="138" t="s">
+      <c r="K100" s="137" t="s">
+        <v>900</v>
+      </c>
+      <c r="L100" s="137" t="s">
         <v>921</v>
       </c>
-      <c r="J100" s="138" t="s">
-        <v>58</v>
-      </c>
-      <c r="K100" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="L100" s="138" t="s">
+      <c r="M100" s="137" t="s">
         <v>922</v>
       </c>
-      <c r="M100" s="138" t="s">
+      <c r="N100" s="137" t="s">
         <v>923</v>
       </c>
-      <c r="N100" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O100" s="138" t="s">
+      <c r="O100" s="137" t="s">
         <v>924</v>
       </c>
-      <c r="P100" s="138" t="s">
+      <c r="P100" s="137" t="s">
         <v>227</v>
       </c>
       <c r="Q100" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",J100&amp;" "&amp;N100)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",J100&amp;" "&amp;N100))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",J100&amp;" "&amp;N100)),ISNUMBER(SEARCH("NOT IMPLEMENTED",J100&amp;" "&amp;N100))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",J100&amp;" "&amp;N100)),ISNUMBER(SEARCH("PENDING",J100&amp;" "&amp;N100)),ISNUMBER(SEARCH("IN PROGRESS",J100&amp;" "&amp;N100)),ISNUMBER(SEARCH("OPEN",J100&amp;" "&amp;N100)),ISNUMBER(SEARCH("RETEST REQUIRED",J100&amp;" "&amp;N100)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",J100&amp;" "&amp;N100)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",J100&amp;" "&amp;N100))),"Pending",IF(OR(N100="PASS",ISNUMBER(SEARCH("PASS",J100&amp;" "&amp;N100))),"Done","Pending"))))</f>
-        <v>Not started</v>
+        <v>Failed</v>
       </c>
       <c r="R100" s="146" t="str">
         <f>IF(OR(LEFT(A100,9)="OPERATOR-",LEFT(A100,8)="PAYMENT-",LEFT(A100,7)="DEPLOY-"),"External","Core")</f>

</xml_diff>

<commit_message>
qa fix - tournament fix
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -31,7 +31,7 @@
     <t>Done</t>
   </si>
   <si>
-    <t>61 (39%)</t>
+    <t>62 (39%)</t>
   </si>
   <si>
     <t>X</t>
@@ -55,7 +55,7 @@
     <t>Not started</t>
   </si>
   <si>
-    <t>79</t>
+    <t>78</t>
   </si>
   <si>
     <t>INDIRECT</t>
@@ -202,7 +202,7 @@
     <t>10</t>
   </si>
   <si>
-    <t>8 passed / 9 total (89%)</t>
+    <t>9 passed / 9 total (100%)</t>
   </si>
   <si>
     <t>Client platform</t>
@@ -2666,13 +2666,13 @@
     <t>No ordinary Reopen after a dependent stage is active/closed; a future explicit rollback workflow is separate</t>
   </si>
   <si>
-    <t>Backend, frontend-local and UI guards now reject a correction after dependent play; watcher compilation passed, manual fixture replay is pending</t>
-  </si>
-  <si>
-    <t>Prove pre-start allow and post-start atomic rejection</t>
-  </si>
-  <si>
-    <t>Do not silently rewrite memberships or results already consumed by a later stage.</t>
+    <t>Backend/frontend-local guard implementation; replayable dependent-stage fixture; authenticated Java HTTP rejection; full related-record snapshot oracle</t>
+  </si>
+  <si>
+    <t>Closed; repeat only after Reopen eligibility or stage progression semantics change</t>
+  </si>
+  <si>
+    <t>The already-PASS pre-start Reopen branch remained untouched. With Final active, Casey's reloaded Qualifiers menu omitted Reopen Scores. One authenticated forbidden Java request returned unchanged F/revision 2; exact 9/14/7 scores, Nova+Riley Final membership, current-stage state and every related event/member/runtime/group/chat/notification/task/counter record remained byte-identical. No lifecycle producer was replayed; frontend-local runtime was not executed.</t>
   </si>
   <si>
     <t>CHAT-AUTH-001</t>
@@ -8324,7 +8324,7 @@
       </c>
       <c r="E1" s="476" t="str">
         <f>COUNTIFS(T18:T231,"Done",U18:U231,"Core")&amp;" ("&amp;IF(COUNTIF(U18:U231,"Core")=0,"0%",TEXT(COUNTIFS(T18:T231,"Done",U18:U231,"Core")/COUNTIF(U18:U231,"Core"),"0%"))&amp;")"</f>
-        <v>61 (39%)</v>
+        <v>62 (39%)</v>
       </c>
       <c r="F1" s="146" t="s">
         <v>1</v>
@@ -8444,7 +8444,7 @@
       </c>
       <c r="E3" s="502">
         <f>COUNTIFS(T18:T231,"Not started",U18:U231,"Core")</f>
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F3" s="146" t="s">
         <v>1</v>
@@ -9043,11 +9043,11 @@
       <c r="C13" s="257" t="s">
         <v>59</v>
       </c>
-      <c r="D13" s="450" t="str">
+      <c r="D13" s="135" t="str">
         <f>COUNTIFS($C$18:$C$231,A13,$T$18:$T$231,"Done")&amp;" passed / "&amp;COUNTIF($C$18:$C$231,A13)&amp;" total ("&amp;IF(COUNTIF($C$18:$C$231,A13)=0,"0%",TEXT(COUNTIFS($C$18:$C$231,A13,$T$18:$T$231,"Done")/COUNTIF($C$18:$C$231,A13),"0%"))&amp;")"</f>
-        <v>8 passed / 9 total (89%)</v>
-      </c>
-      <c r="E13" s="462" t="s">
+        <v>9 passed / 9 total (100%)</v>
+      </c>
+      <c r="E13" s="151" t="s">
         <v>1</v>
       </c>
       <c r="F13" s="357" t="s">
@@ -14023,66 +14023,66 @@
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="138" t="s">
+      <c r="A88" s="135" t="s">
         <v>792</v>
       </c>
-      <c r="B88" s="138" t="s">
+      <c r="B88" s="135" t="s">
         <v>741</v>
       </c>
       <c r="C88" s="257" t="s">
         <v>58</v>
       </c>
-      <c r="D88" s="138" t="s">
+      <c r="D88" s="135" t="s">
         <v>793</v>
       </c>
-      <c r="E88" s="138" t="s">
+      <c r="E88" s="135" t="s">
         <v>794</v>
       </c>
-      <c r="F88" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="G88" s="138" t="s">
+      <c r="F88" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="G88" s="135" t="s">
         <v>795</v>
       </c>
-      <c r="H88" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="I88" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="J88" s="138" t="s">
+      <c r="H88" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="I88" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="J88" s="135" t="s">
         <v>796</v>
       </c>
-      <c r="K88" s="138" t="s">
-        <v>135</v>
-      </c>
-      <c r="L88" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="M88" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="N88" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O88" s="138" t="s">
+      <c r="K88" s="135" t="s">
+        <v>158</v>
+      </c>
+      <c r="L88" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="M88" s="135" t="s">
+        <v>777</v>
+      </c>
+      <c r="N88" s="135" t="s">
+        <v>778</v>
+      </c>
+      <c r="O88" s="135" t="s">
         <v>797</v>
       </c>
-      <c r="P88" s="138" t="s">
+      <c r="P88" s="135" t="s">
         <v>798</v>
       </c>
-      <c r="Q88" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="R88" s="138" t="s">
+      <c r="Q88" s="135" t="s">
+        <v>128</v>
+      </c>
+      <c r="R88" s="135" t="s">
         <v>799</v>
       </c>
-      <c r="S88" s="138" t="s">
+      <c r="S88" s="135" t="s">
         <v>104</v>
       </c>
       <c r="T88" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",K88&amp;" "&amp;Q88)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K88&amp;" "&amp;Q88))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K88&amp;" "&amp;Q88)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K88&amp;" "&amp;Q88))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K88&amp;" "&amp;Q88)),ISNUMBER(SEARCH("PENDING",K88&amp;" "&amp;Q88)),ISNUMBER(SEARCH("IN PROGRESS",K88&amp;" "&amp;Q88)),ISNUMBER(SEARCH("OPEN",K88&amp;" "&amp;Q88)),ISNUMBER(SEARCH("RETEST REQUIRED",K88&amp;" "&amp;Q88)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K88&amp;" "&amp;Q88)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K88&amp;" "&amp;Q88))),"Pending",IF(OR(Q88="PASS",ISNUMBER(SEARCH("PASS",K88&amp;" "&amp;Q88))),"Done","Pending"))))</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="U88" s="146" t="str">
         <f>IF(OR(LEFT(A88,9)="OPERATOR-",LEFT(A88,8)="PAYMENT-",LEFT(A88,7)="DEPLOY-"),"External","Core")</f>

</xml_diff>

<commit_message>
[MSC-77] Qualify borrowing, availability ranges and HTTP request behavior
Consolidate resource/member and asset borrowing corrections, date-range
handling, duplicate HTTP-call fixes and the corresponding automated/manual
QA evidence.

Original-snapshot: 3bd7fcd051277039b28fd6f8537700ae088a889a

Tasks: fssrepository/myscoutee-roadmap#77
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2360" uniqueCount="1139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2380" uniqueCount="1149">
   <si>
     <t>EFFECT / SCOPE MARKERS</t>
   </si>
@@ -31,7 +31,7 @@
     <t>Done</t>
   </si>
   <si>
-    <t>88 (85%)</t>
+    <t>89 (86%)</t>
   </si>
   <si>
     <t>X</t>
@@ -79,7 +79,7 @@
     <t>Total</t>
   </si>
   <si>
-    <t>103</t>
+    <t>104</t>
   </si>
   <si>
     <t>DOMAIN PRIORITY</t>
@@ -109,7 +109,7 @@
     <t>9</t>
   </si>
   <si>
-    <t>4 passed / 6 total (67%) · 255/605</t>
+    <t>5 passed / 7 total (71%) · 135/320</t>
   </si>
   <si>
     <t>Identity &amp; access</t>
@@ -139,7 +139,7 @@
     <t>Notifications</t>
   </si>
   <si>
-    <t>0 passed / 6 total (0%) · 410/995</t>
+    <t>0 passed / 6 total (0%) · 425/1025</t>
   </si>
   <si>
     <t>Tournament</t>
@@ -3030,43 +3030,46 @@
     <t>User-approved flexible closure from the accumulated 2026-09-03 run instead of another ordered 46-step replay. The run covered distinct Invite/Join pending states, resolution and rejection, contextual pending counters, recipient Notifications, standard Service chat/Ask Organizer, ordinary-member restrictions, owner/delegated Manager grant and revoke rules, live/reload card role and menu changes, removal, Event-role isolation, and both Manager-first and no-manager Take Over branches. The final correction replay produced Casey Leave 3-&gt;2, Nova Take Over 2-&gt;2, Riley removal 2-&gt;1 and Nova final Leave 1-&gt;absent through the live UI. The terminal read-only Mongo oracle proved Riley's canonical Asset member row was deleted, activityResources was D with no Asset assignment, the generated-group runtime resource map was empty, and no notification was created after Nova's final Leave. The corrections use canonical write-side status and existing signal propagation, with no read projection or frontend-only hide; the retained terminal fixture was not silently reset after the user's verdict.</t>
   </si>
   <si>
-    <t>ASSET-BORROW-LIFECYCLE-001</t>
-  </si>
-  <si>
-    <t>Borrow, timeframe, capacity and Statistics lifecycle</t>
-  </si>
-  <si>
-    <t>Request one asset for the exact event/stage/group range, accept it, reject a control, create overlapping finite-capacity requests, move one outside overlap and verify the exact Asset Statistics delta</t>
-  </si>
-  <si>
-    <t>INDIRECT pending/accepted asset request counts; INDIRECT available quantity/order; Asset activity and asset-request delta</t>
-  </si>
-  <si>
-    <t>DELTA one request/payment-session reference per branch and exact availability quantity; DELTA booking quantities and availability projection only; Assets queue/flow delta</t>
-  </si>
-  <si>
-    <t>CONDITIONAL provider/outbox work only when the staged asset policy requires it; X unless the configured booking policy explicitly produces provider work; Affinity recompute may run</t>
-  </si>
-  <si>
-    <t>Requester and owner see the same request state; accepted borrower becomes assignment-eligible only for the exact generated-group booking scope; reject/cancel clean up once and the sibling group stays unchanged; Explore availability and assignment eligibility never exceed quantity/capacity; moving one timeframe restores exactly its released capacity in place and after reload; Asset request state correct</t>
-  </si>
-  <si>
-    <t>PREPARED / DEFERRED / NOT STAGED</t>
-  </si>
-  <si>
-    <t>Consolidates ASSET-BORROW-001, ASSET-AVAIL-001, STAT-013. Its isolated fixture, guide and browser-session definition were prepared and the baseline was staged/read-only verified, then reset through the versioned snapshot without starting browser QA because the payment-facing interface will be rewritten</t>
-  </si>
-  <si>
-    <t>Deferred until the payment interface rewrite is complete; then restage through the isolated Borrow harness and prove its read-only baseline before opening browsers</t>
-  </si>
-  <si>
-    <t>Source status: ASSET-BORROW-001=DESIGN CAPTURED / NOT RUN; ASSET-AVAIL-001=DESIGN CAPTURED / NOT RUN; STAT-013=NOT RUN. No Borrow browser action or manual verdict exists. Borrow permission is not Asset Manager membership and never promotes an Event or Tournament-group role. Use seconds/minutes fixture spacing; no real-time waiting is required.</t>
-  </si>
-  <si>
-    <t>P2 58</t>
-  </si>
-  <si>
-    <t>105/250</t>
+    <t>ASSET-BORROW-001</t>
+  </si>
+  <si>
+    <t>One-unit free and paid Borrow, timeframe, capacity and exact-scope Organizer-only lifecycle</t>
+  </si>
+  <si>
+    <t>Against three free and one paid Public Transport control, cancel one request, reject one, accept one, submit the same paid Borrow twice as separate requests, compare overlapping/non-overlapping capacity and fine-tune Organizer-only at Event, Stage, Group and Asset scope</t>
+  </si>
+  <si>
+    <t>INDIRECT pending/accepted Asset request counts; INDIRECT available quantity/order; exact-scope participant counter delta; Asset activity and request delta</t>
+  </si>
+  <si>
+    <t>DELTA one request identity per one-unit submission; separate paid payment/approval/card per repeated Borrow; exact availability and date range; no request merging</t>
+  </si>
+  <si>
+    <t>Normal Asset request notification/outbox and affinity-task effects; Barion once per paid submission; schedulers X</t>
+  </si>
+  <si>
+    <t>Every Borrow quantity is read-only 1; source Explore Asset appears once without Payment summary; repeated assigned request cards remain separate with #1/#2, date ranges and paid summaries; Organizer-only changes only the selected scope counter without role or membership cascade; reload retains the exact projection</t>
+  </si>
+  <si>
+    <t>STAGED / BASELINE READY / BROWSER RELAUNCH REQUIRED</t>
+  </si>
+  <si>
+    <t>2026-09-08</t>
+  </si>
+  <si>
+    <t>Revised concise guide and six guarded cancel/reject/accepted/paid-organizer/terminal oracles are implemented. Fixture restaged at 2026-09-08T09:24:00.778Z; read-only status proves all ten baseline checks, four Transport controls, Lina's retained Group B Quantity 2 control, Nova's Barion 4444 card and zero basket/payment state. Running backend and frontend watcher builds passed</t>
+  </si>
+  <si>
+    <t>Run read-only status; if baseline-ready, prepare and launch the configured Casey/Nova/Riley sessions once, then user starts step 1 without restaging</t>
+  </si>
+  <si>
+    <t>ASSET-CHECKOUT-001 is PASS/CLOSED and retains 3DS/refund/Take Over/Leave/Remove coverage. Direct Assign/Edit/Unassign remains owned by ASSET-ASSIGNMENT-LIFECYCLE-001. No Borrow browser verdict exists yet.</t>
+  </si>
+  <si>
+    <t>P2 72</t>
+  </si>
+  <si>
+    <t>70/165</t>
   </si>
   <si>
     <t>ASSET-CHECKOUT-001</t>
@@ -3093,22 +3096,52 @@
     <t>Fresh paid: Borrow -&gt; Confirm borrow; saved draft: Borrow Basket/Continue request; payment-ready: Barion card/Pay plus neutral Back and red Cancel; paid pending: Payment summary and one owner Pending row; accepted: same read-only summary and exact scoped resource; free uses Send borrow request and unavailable is absent from availability-filtered Explore; no freeze or duplicate payment/request/reservation</t>
   </si>
   <si>
-    <t>IN PROGRESS — TAKEOVER PASS THROUGH STEP 79</t>
-  </si>
-  <si>
-    <t>2026-09-07</t>
-  </si>
-  <si>
-    <t>Asset Explore checkout/session, pricing, request, availability and scoped-resource sources have automated coverage in parts; the complete HTTP browser Barion payment/action/destination journey has not run</t>
-  </si>
-  <si>
-    <t>Continue at step 80 with runtime Remove; then verify service chat, policy refund and last-manager Leave</t>
-  </si>
-  <si>
-    <t>Steps 1-68 reached the core terminal PASS on 2026-09-07: one approved target payment, one declined control, one expired control and one cancelled Adjacent audit. Stored target quantity remains 3, selected-window availability remains 2, and sibling/Riley isolation passed. The manager-left oracle passed through step 73. The paid Take Over oracle then passed through step 79: Riley is the Captured/Joined successor and scoped Manager, Nova's Captured predecessor has a separate full-refund transaction, payer-swap finance totals changed exactly once, and Nova received only the refund-result notification. Accepted, cancelled-control, manager-left and takeover-complete savepoints are retained.</t>
-  </si>
-  <si>
-    <t>150/355</t>
+    <t>Complete user-driven steps 1-98; guarded core, request-destination, acceptance, manager-left, paid Take Over, refund, last-Leave and mixed-status Remove Mongo oracles; running backend/frontend watcher builds passed during defect repairs</t>
+  </si>
+  <si>
+    <t>Closed; continue with the restaged one-unit free/paid ASSET-BORROW-001 baseline</t>
+  </si>
+  <si>
+    <t>Steps 1-68 proved one approved, one declined and one expired payment plus one cancelled basket with quantity and sibling isolation. Steps 69-89 proved manager Leave, paid Take Over, runtime Remove, exact Asset-owner service chat and one separate 50% refund request/approval with pending counter 0-&gt;1-&gt;0. The last-manager Leave oracle passed at 2026-09-08T03:42:02.224Z. The final mixed-status Remove oracle passed at 2026-09-08T03:48:22.239Z: accepted Nova and pending Riley requests/projections were retired, runtime metrics disappeared, Casey's global Asset and all payment histories remained unchanged, availability returned to 3 and no automatic refund or Take Over notification appeared. The observed missing refund action was fixture policy/window drift and is corrected for future guarded replays without restaging this completed run.</t>
+  </si>
+  <si>
+    <t>ASSET-PRICING-001</t>
+  </si>
+  <si>
+    <t>Interactive journey</t>
+  </si>
+  <si>
+    <t>Interactive pricing configuration and payment-time snapshots</t>
+  </si>
+  <si>
+    <t>On one Public Transport Asset repeatedly change fixed/variable/audience/refund pricing, observe every open Borrow projection on the fly, then capture active-policy, no-policy and passed-cutoff payments on three Event stages</t>
+  </si>
+  <si>
+    <t>X before payment; indirect Asset visibility and Borrow price projection changes</t>
+  </si>
+  <si>
+    <t>DELTA one Asset pricing config per user Save; then exactly three primary captured payments with distinct immutable effective-row and cancellation-policy snapshots</t>
+  </si>
+  <si>
+    <t>Barion provider runs exactly once per payment; no scheduler; normal Asset request/outbox and affinity effects only</t>
+  </si>
+  <si>
+    <t>Fixed per-booking duration, per-item quantity/demand/time/min-max/rounding, member/public/audience contract, Confirm/Payment disclosure and historical Payment summaries all agree with the pricing version active at each capture; later live edits never rewrite earlier payments</t>
+  </si>
+  <si>
+    <t>HARNESS PREPARED / NOT STAGED</t>
+  </si>
+  <si>
+    <t>Interactive guide, dedicated asset-pricing stage/status/phase/final/reset harness and browser-session definition prepared. Hard pre-stage development gate records that Asset editor currently hides Audience Pricing and Asset Borrow has no VIP identity or promo application route; payment already stores effective rows and cancellation-policy snapshot, while full disclosure UI remains incomplete</t>
+  </si>
+  <si>
+    <t>Finish and reset Borrow; first implement/define Asset member/VIP/invite/promo pricing and promo entry, then implement refund-policy disclosure/snapshot projection; only afterward stage ASSET-PRICING-001</t>
+  </si>
+  <si>
+    <t>Refund policy is one Pricing field group, not a standalone testcase. The journey uses one repeatedly edited Asset rather than pre-baked item controls. Do not stage against the current implementation: the next session starts with the missing Asset audience/VIP/promo and refund-disclosure development, without inventing a VIP fixture.</t>
+  </si>
+  <si>
+    <t>65/155</t>
   </si>
   <si>
     <t>ASSET-ASSIGNMENT-LIFECYCLE-001</t>
@@ -3402,34 +3435,34 @@
     <t>Admin Jobs + Chat</t>
   </si>
   <si>
-    <t>Compare pointer, scroll and input frame pacing across idle UI, Admin process list, Job Detail and Chat during periodic/live updates</t>
+    <t>Compare pointer, scroll and input frame pacing across idle UI, Admin process list, Job Detail and Chat during periodic/live updates; in the same run attribute unexpected logout across two intended sessions, CDP attachment and normal browser close</t>
   </si>
   <si>
     <t>Job Detail must stay responsive during SmartList refresh; unchanged polls must not mutate rows; only the selected changed rule may reach the detail signal</t>
   </si>
   <si>
-    <t>Chat must stay responsive during WebSocket and user-realtime updates</t>
+    <t>Chat must stay responsive during WebSocket and user-realtime updates; read-only CDP attach creates no server session/context, and browser-close evidence is captured before intentional launcher cleanup</t>
   </si>
   <si>
     <t>ADMIN JOB MANUAL VISUAL PASS; PERFORMANCE TRACE + CHAT RETEST PENDING</t>
   </si>
   <si>
-    <t>Focused component tests pass 6/6 for SmartList loading, keyed equality, row patching, detail isolation and local patch routing; running hot-deploy build manually showed no prior Job Detail stutter; browser frame-time trace not captured</t>
-  </si>
-  <si>
-    <t>Capture 20–30 second Performance + Network traces for idle/list/detail/chat; prove unchanged Job polls preserve DOM rows and non-selected updates do not re-render detail; correlate Chat hitches independently</t>
+    <t>Focused component tests pass 6/6 for SmartList loading, keyed equality, row patching, detail isolation and local patch routing; running hot-deploy build manually showed no prior Job Detail stutter; browser frame-time trace and session-retention attribution not captured</t>
+  </si>
+  <si>
+    <t>Capture Performance + Network traces for idle/list/detail/chat, then run the supplemental two-session attribution block: compare server sessions/audits, context/profile and auth-carrier presence before/after read-only CDP attach and immediately after user browser close, before any launcher cleanup</t>
   </si>
   <si>
     <t>OPEN / PARTIAL PASS</t>
   </si>
   <si>
-    <t>Admin Jobs now uses SmartList-owned five-second polling, cancellation, keyed equality, visible-row patching and re-sorting with OnPush. Job Detail receives only its selected changed rule through a separate signal; the complete list is not pushed into detail. The full center remains the table data source. The 2026-08-04 hot-deployed build no longer showed the reported stutter during manual use, but no Performance trace was captured. Chat remains a separate reported symptom using OnPush, WebSocket live events and a 30-second global user realtime poll, shortened to 10 seconds in demo; its root cause remains unconfirmed. Both checkpoints must pass before closure.</t>
+    <t>Admin Jobs now uses SmartList-owned five-second polling, cancellation, keyed equality, visible-row patching and re-sorting with OnPush. Job Detail receives only its selected changed rule through a separate signal; the complete list is not pushed into detail. The full center remains the table data source. The 2026-08-04 hot-deployed build no longer showed the reported stutter during manual use, but no Performance trace was captured. Chat remains a separate reported symptom using OnPush, WebSocket live events and a 30-second global user realtime poll, shortened to 10 seconds in demo; its root cause remains unconfirmed. The added block is diagnostic coverage inside this open testcase, not a new row or an Identity retest; it must distinguish CDP-created context/session, browser storage loss, ordinary-close revocation and intentional prepare-browser/launcher cleanup without recording secrets.</t>
   </si>
   <si>
     <t>P1 65</t>
   </si>
   <si>
-    <t>45/115</t>
+    <t>60/145</t>
   </si>
   <si>
     <t>BASE-STAT</t>
@@ -3526,9 +3559,6 @@
   </si>
   <si>
     <t>P2 52</t>
-  </si>
-  <si>
-    <t>60/145</t>
   </si>
   <si>
     <t>ADMIN-PARAMETERS-001</t>
@@ -5560,7 +5590,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:W118"/>
+  <dimension ref="A1:W119"/>
   <sheetFormatPr defaultColWidth="11.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="14" hidden="false" customWidth="true"/>
@@ -5602,8 +5632,8 @@
         <v>2</v>
       </c>
       <c r="E1" s="476" t="str">
-        <f>COUNTIF(U16:U118,"Done")&amp;" ("&amp;IF(COUNTA(A16:A118)=0,"0%",TEXT(COUNTIF(U16:U118,"Done")/COUNTA(A16:A118),"0%"))&amp;")"</f>
-        <v>88 (85%)</v>
+        <f>COUNTIF(U16:U119,"Done")&amp;" ("&amp;IF(COUNTA(A16:A119)=0,"0%",TEXT(COUNTIF(U16:U119,"Done")/COUNTA(A16:A119),"0%"))&amp;")"</f>
+        <v>89 (86%)</v>
       </c>
       <c r="F1" s="146" t="s">
         <v>1</v>
@@ -5665,7 +5695,7 @@
         <v>6</v>
       </c>
       <c r="E2" s="486">
-        <f>COUNTIF(U16:U118,"Pending")</f>
+        <f>COUNTIF(U16:U119,"Pending")</f>
         <v>7</v>
       </c>
       <c r="F2" s="146" t="s">
@@ -5728,7 +5758,7 @@
         <v>10</v>
       </c>
       <c r="E3" s="502">
-        <f>COUNTIF(U16:U118,"Not started")</f>
+        <f>COUNTIF(U16:U119,"Not started")</f>
         <v>8</v>
       </c>
       <c r="F3" s="146" t="s">
@@ -5791,7 +5821,7 @@
         <v>14</v>
       </c>
       <c r="E4" s="494">
-        <f>COUNTIF(U16:U118,"Failed")</f>
+        <f>COUNTIF(U16:U119,"Failed")</f>
         <v>0</v>
       </c>
       <c r="F4" s="146" t="s">
@@ -5854,8 +5884,8 @@
         <v>18</v>
       </c>
       <c r="E5" s="513">
-        <f>COUNTA(A16:A118)</f>
-        <v>103</v>
+        <f>COUNTA(A16:A119)</f>
+        <v>104</v>
       </c>
       <c r="F5" s="146" t="s">
         <v>1</v>
@@ -6038,7 +6068,7 @@
         <v>25</v>
       </c>
       <c r="D8" s="135" t="str">
-        <f>COUNTIFS($C$16:$C$118,A8,$U$16:$U$118,"Done")&amp;" passed / "&amp;COUNTIF($C$16:$C$118,A8)&amp;" total ("&amp;IF(COUNTIF($C$16:$C$118,A8)=0,"0%",TEXT(COUNTIFS($C$16:$C$118,A8,$U$16:$U$118,"Done")/COUNTIF($C$16:$C$118,A8),"0%"))&amp;") · "&amp;SUMIFS($V$16:$V$118,$C$16:$C$118,A8,$U$16:$U$118,"&lt;&gt;Done")&amp;"/"&amp;SUMIFS($W$16:$W$118,$C$16:$C$118,A8,$U$16:$U$118,"&lt;&gt;Done")</f>
+        <f>COUNTIFS($C$16:$C$119,A8,$U$16:$U$119,"Done")&amp;" passed / "&amp;COUNTIF($C$16:$C$119,A8)&amp;" total ("&amp;IF(COUNTIF($C$16:$C$119,A8)=0,"0%",TEXT(COUNTIFS($C$16:$C$119,A8,$U$16:$U$119,"Done")/COUNTIF($C$16:$C$119,A8),"0%"))&amp;") · "&amp;SUMIFS($V$16:$V$119,$C$16:$C$119,A8,$U$16:$U$119,"&lt;&gt;Done")&amp;"/"&amp;SUMIFS($W$16:$W$119,$C$16:$C$119,A8,$U$16:$U$119,"&lt;&gt;Done")</f>
         <v>2 passed / 2 total (100%) · 0/0</v>
       </c>
       <c r="E8" s="151" t="s">
@@ -6054,8 +6084,8 @@
         <v>28</v>
       </c>
       <c r="I8" s="136" t="str">
-        <f>COUNTIFS($C$16:$C$118,F8,$U$16:$U$118,"Done")&amp;" passed / "&amp;COUNTIF($C$16:$C$118,F8)&amp;" total ("&amp;IF(COUNTIF($C$16:$C$118,F8)=0,"0%",TEXT(COUNTIFS($C$16:$C$118,F8,$U$16:$U$118,"Done")/COUNTIF($C$16:$C$118,F8),"0%"))&amp;") · "&amp;SUMIFS($V$16:$V$118,$C$16:$C$118,F8,$U$16:$U$118,"&lt;&gt;Done")&amp;"/"&amp;SUMIFS($W$16:$W$118,$C$16:$C$118,F8,$U$16:$U$118,"&lt;&gt;Done")</f>
-        <v>4 passed / 6 total (67%) · 255/605</v>
+        <f>COUNTIFS($C$16:$C$119,F8,$U$16:$U$119,"Done")&amp;" passed / "&amp;COUNTIF($C$16:$C$119,F8)&amp;" total ("&amp;IF(COUNTIF($C$16:$C$119,F8)=0,"0%",TEXT(COUNTIFS($C$16:$C$119,F8,$U$16:$U$119,"Done")/COUNTIF($C$16:$C$119,F8),"0%"))&amp;") · "&amp;SUMIFS($V$16:$V$119,$C$16:$C$119,F8,$U$16:$U$119,"&lt;&gt;Done")&amp;"/"&amp;SUMIFS($W$16:$W$119,$C$16:$C$119,F8,$U$16:$U$119,"&lt;&gt;Done")</f>
+        <v>5 passed / 7 total (71%) · 135/320</v>
       </c>
       <c r="J8" s="159" t="s">
         <v>1</v>
@@ -6102,7 +6132,7 @@
         <v>31</v>
       </c>
       <c r="D9" s="135" t="str">
-        <f>COUNTIFS($C$16:$C$118,A9,$U$16:$U$118,"Done")&amp;" passed / "&amp;COUNTIF($C$16:$C$118,A9)&amp;" total ("&amp;IF(COUNTIF($C$16:$C$118,A9)=0,"0%",TEXT(COUNTIFS($C$16:$C$118,A9,$U$16:$U$118,"Done")/COUNTIF($C$16:$C$118,A9),"0%"))&amp;") · "&amp;SUMIFS($V$16:$V$118,$C$16:$C$118,A9,$U$16:$U$118,"&lt;&gt;Done")&amp;"/"&amp;SUMIFS($W$16:$W$118,$C$16:$C$118,A9,$U$16:$U$118,"&lt;&gt;Done")</f>
+        <f>COUNTIFS($C$16:$C$119,A9,$U$16:$U$119,"Done")&amp;" passed / "&amp;COUNTIF($C$16:$C$119,A9)&amp;" total ("&amp;IF(COUNTIF($C$16:$C$119,A9)=0,"0%",TEXT(COUNTIFS($C$16:$C$119,A9,$U$16:$U$119,"Done")/COUNTIF($C$16:$C$119,A9),"0%"))&amp;") · "&amp;SUMIFS($V$16:$V$119,$C$16:$C$119,A9,$U$16:$U$119,"&lt;&gt;Done")&amp;"/"&amp;SUMIFS($W$16:$W$119,$C$16:$C$119,A9,$U$16:$U$119,"&lt;&gt;Done")</f>
         <v>8 passed / 8 total (100%) · 0/0</v>
       </c>
       <c r="E9" s="151" t="s">
@@ -6118,7 +6148,7 @@
         <v>11</v>
       </c>
       <c r="I9" s="135" t="str">
-        <f>COUNTIFS($C$16:$C$118,F9,$U$16:$U$118,"Done")&amp;" passed / "&amp;COUNTIF($C$16:$C$118,F9)&amp;" total ("&amp;IF(COUNTIF($C$16:$C$118,F9)=0,"0%",TEXT(COUNTIFS($C$16:$C$118,F9,$U$16:$U$118,"Done")/COUNTIF($C$16:$C$118,F9),"0%"))&amp;") · "&amp;SUMIFS($V$16:$V$118,$C$16:$C$118,F9,$U$16:$U$118,"&lt;&gt;Done")&amp;"/"&amp;SUMIFS($W$16:$W$118,$C$16:$C$118,F9,$U$16:$U$118,"&lt;&gt;Done")</f>
+        <f>COUNTIFS($C$16:$C$119,F9,$U$16:$U$119,"Done")&amp;" passed / "&amp;COUNTIF($C$16:$C$119,F9)&amp;" total ("&amp;IF(COUNTIF($C$16:$C$119,F9)=0,"0%",TEXT(COUNTIFS($C$16:$C$119,F9,$U$16:$U$119,"Done")/COUNTIF($C$16:$C$119,F9),"0%"))&amp;") · "&amp;SUMIFS($V$16:$V$119,$C$16:$C$119,F9,$U$16:$U$119,"&lt;&gt;Done")&amp;"/"&amp;SUMIFS($W$16:$W$119,$C$16:$C$119,F9,$U$16:$U$119,"&lt;&gt;Done")</f>
         <v>3 passed / 3 total (100%) · 0/0</v>
       </c>
       <c r="J9" s="151" t="s">
@@ -6166,7 +6196,7 @@
         <v>36</v>
       </c>
       <c r="D10" s="135" t="str">
-        <f>COUNTIFS($C$16:$C$118,A10,$U$16:$U$118,"Done")&amp;" passed / "&amp;COUNTIF($C$16:$C$118,A10)&amp;" total ("&amp;IF(COUNTIF($C$16:$C$118,A10)=0,"0%",TEXT(COUNTIFS($C$16:$C$118,A10,$U$16:$U$118,"Done")/COUNTIF($C$16:$C$118,A10),"0%"))&amp;") · "&amp;SUMIFS($V$16:$V$118,$C$16:$C$118,A10,$U$16:$U$118,"&lt;&gt;Done")&amp;"/"&amp;SUMIFS($W$16:$W$118,$C$16:$C$118,A10,$U$16:$U$118,"&lt;&gt;Done")</f>
+        <f>COUNTIFS($C$16:$C$119,A10,$U$16:$U$119,"Done")&amp;" passed / "&amp;COUNTIF($C$16:$C$119,A10)&amp;" total ("&amp;IF(COUNTIF($C$16:$C$119,A10)=0,"0%",TEXT(COUNTIFS($C$16:$C$119,A10,$U$16:$U$119,"Done")/COUNTIF($C$16:$C$119,A10),"0%"))&amp;") · "&amp;SUMIFS($V$16:$V$119,$C$16:$C$119,A10,$U$16:$U$119,"&lt;&gt;Done")&amp;"/"&amp;SUMIFS($W$16:$W$119,$C$16:$C$119,A10,$U$16:$U$119,"&lt;&gt;Done")</f>
         <v>49 passed / 49 total (100%) · 0/0</v>
       </c>
       <c r="E10" s="151" t="s">
@@ -6182,8 +6212,8 @@
         <v>7</v>
       </c>
       <c r="I10" s="138" t="str">
-        <f>COUNTIFS($C$16:$C$118,F10,$U$16:$U$118,"Done")&amp;" passed / "&amp;COUNTIF($C$16:$C$118,F10)&amp;" total ("&amp;IF(COUNTIF($C$16:$C$118,F10)=0,"0%",TEXT(COUNTIFS($C$16:$C$118,F10,$U$16:$U$118,"Done")/COUNTIF($C$16:$C$118,F10),"0%"))&amp;") · "&amp;SUMIFS($V$16:$V$118,$C$16:$C$118,F10,$U$16:$U$118,"&lt;&gt;Done")&amp;"/"&amp;SUMIFS($W$16:$W$118,$C$16:$C$118,F10,$U$16:$U$118,"&lt;&gt;Done")</f>
-        <v>0 passed / 6 total (0%) · 410/995</v>
+        <f>COUNTIFS($C$16:$C$119,F10,$U$16:$U$119,"Done")&amp;" passed / "&amp;COUNTIF($C$16:$C$119,F10)&amp;" total ("&amp;IF(COUNTIF($C$16:$C$119,F10)=0,"0%",TEXT(COUNTIFS($C$16:$C$119,F10,$U$16:$U$119,"Done")/COUNTIF($C$16:$C$119,F10),"0%"))&amp;") · "&amp;SUMIFS($V$16:$V$119,$C$16:$C$119,F10,$U$16:$U$119,"&lt;&gt;Done")&amp;"/"&amp;SUMIFS($W$16:$W$119,$C$16:$C$119,F10,$U$16:$U$119,"&lt;&gt;Done")</f>
+        <v>0 passed / 6 total (0%) · 425/1025</v>
       </c>
       <c r="J10" s="175" t="s">
         <v>1</v>
@@ -6230,7 +6260,7 @@
         <v>41</v>
       </c>
       <c r="D11" s="135" t="str">
-        <f>COUNTIFS($C$16:$C$118,A11,$U$16:$U$118,"Done")&amp;" passed / "&amp;COUNTIF($C$16:$C$118,A11)&amp;" total ("&amp;IF(COUNTIF($C$16:$C$118,A11)=0,"0%",TEXT(COUNTIFS($C$16:$C$118,A11,$U$16:$U$118,"Done")/COUNTIF($C$16:$C$118,A11),"0%"))&amp;") · "&amp;SUMIFS($V$16:$V$118,$C$16:$C$118,A11,$U$16:$U$118,"&lt;&gt;Done")&amp;"/"&amp;SUMIFS($W$16:$W$118,$C$16:$C$118,A11,$U$16:$U$118,"&lt;&gt;Done")</f>
+        <f>COUNTIFS($C$16:$C$119,A11,$U$16:$U$119,"Done")&amp;" passed / "&amp;COUNTIF($C$16:$C$119,A11)&amp;" total ("&amp;IF(COUNTIF($C$16:$C$119,A11)=0,"0%",TEXT(COUNTIFS($C$16:$C$119,A11,$U$16:$U$119,"Done")/COUNTIF($C$16:$C$119,A11),"0%"))&amp;") · "&amp;SUMIFS($V$16:$V$119,$C$16:$C$119,A11,$U$16:$U$119,"&lt;&gt;Done")&amp;"/"&amp;SUMIFS($W$16:$W$119,$C$16:$C$119,A11,$U$16:$U$119,"&lt;&gt;Done")</f>
         <v>15 passed / 15 total (100%) · 0/0</v>
       </c>
       <c r="E11" s="151" t="s">
@@ -6246,7 +6276,7 @@
         <v>44</v>
       </c>
       <c r="I11" s="451" t="str">
-        <f>COUNTIFS($C$16:$C$118,F11,$U$16:$U$118,"Done")&amp;" passed / "&amp;COUNTIF($C$16:$C$118,F11)&amp;" total ("&amp;IF(COUNTIF($C$16:$C$118,F11)=0,"0%",TEXT(COUNTIFS($C$16:$C$118,F11,$U$16:$U$118,"Done")/COUNTIF($C$16:$C$118,F11),"0%"))&amp;") · "&amp;SUMIFS($V$16:$V$118,$C$16:$C$118,F11,$U$16:$U$118,"&lt;&gt;Done")&amp;"/"&amp;SUMIFS($W$16:$W$118,$C$16:$C$118,F11,$U$16:$U$118,"&lt;&gt;Done")</f>
+        <f>COUNTIFS($C$16:$C$119,F11,$U$16:$U$119,"Done")&amp;" passed / "&amp;COUNTIF($C$16:$C$119,F11)&amp;" total ("&amp;IF(COUNTIF($C$16:$C$119,F11)=0,"0%",TEXT(COUNTIFS($C$16:$C$119,F11,$U$16:$U$119,"Done")/COUNTIF($C$16:$C$119,F11),"0%"))&amp;") · "&amp;SUMIFS($V$16:$V$119,$C$16:$C$119,F11,$U$16:$U$119,"&lt;&gt;Done")&amp;"/"&amp;SUMIFS($W$16:$W$119,$C$16:$C$119,F11,$U$16:$U$119,"&lt;&gt;Done")</f>
         <v>1 passed / 4 total (25%) · 265/635</v>
       </c>
       <c r="J11" s="470" t="s">
@@ -6294,7 +6324,7 @@
         <v>47</v>
       </c>
       <c r="D12" s="153" t="str">
-        <f>COUNTIFS($C$16:$C$118,A12,$U$16:$U$118,"Done")&amp;" passed / "&amp;COUNTIF($C$16:$C$118,A12)&amp;" total ("&amp;IF(COUNTIF($C$16:$C$118,A12)=0,"0%",TEXT(COUNTIFS($C$16:$C$118,A12,$U$16:$U$118,"Done")/COUNTIF($C$16:$C$118,A12),"0%"))&amp;") · "&amp;SUMIFS($V$16:$V$118,$C$16:$C$118,A12,$U$16:$U$118,"&lt;&gt;Done")&amp;"/"&amp;SUMIFS($W$16:$W$118,$C$16:$C$118,A12,$U$16:$U$118,"&lt;&gt;Done")</f>
+        <f>COUNTIFS($C$16:$C$119,A12,$U$16:$U$119,"Done")&amp;" passed / "&amp;COUNTIF($C$16:$C$119,A12)&amp;" total ("&amp;IF(COUNTIF($C$16:$C$119,A12)=0,"0%",TEXT(COUNTIFS($C$16:$C$119,A12,$U$16:$U$119,"Done")/COUNTIF($C$16:$C$119,A12),"0%"))&amp;") · "&amp;SUMIFS($V$16:$V$119,$C$16:$C$119,A12,$U$16:$U$119,"&lt;&gt;Done")&amp;"/"&amp;SUMIFS($W$16:$W$119,$C$16:$C$119,A12,$U$16:$U$119,"&lt;&gt;Done")</f>
         <v>6 passed / 6 total (100%) · 0/0</v>
       </c>
       <c r="E12" s="154" t="s">
@@ -6310,7 +6340,7 @@
         <v>50</v>
       </c>
       <c r="I12" s="177" t="str">
-        <f>COUNTIFS($C$16:$C$118,F12,$U$16:$U$118,"Done")&amp;" passed / "&amp;COUNTIF($C$16:$C$118,F12)&amp;" total ("&amp;IF(COUNTIF($C$16:$C$118,F12)=0,"0%",TEXT(COUNTIFS($C$16:$C$118,F12,$U$16:$U$118,"Done")/COUNTIF($C$16:$C$118,F12),"0%"))&amp;") · "&amp;SUMIFS($V$16:$V$118,$C$16:$C$118,F12,$U$16:$U$118,"&lt;&gt;Done")&amp;"/"&amp;SUMIFS($W$16:$W$118,$C$16:$C$118,F12,$U$16:$U$118,"&lt;&gt;Done")</f>
+        <f>COUNTIFS($C$16:$C$119,F12,$U$16:$U$119,"Done")&amp;" passed / "&amp;COUNTIF($C$16:$C$119,F12)&amp;" total ("&amp;IF(COUNTIF($C$16:$C$119,F12)=0,"0%",TEXT(COUNTIFS($C$16:$C$119,F12,$U$16:$U$119,"Done")/COUNTIF($C$16:$C$119,F12),"0%"))&amp;") · "&amp;SUMIFS($V$16:$V$119,$C$16:$C$119,F12,$U$16:$U$119,"&lt;&gt;Done")&amp;"/"&amp;SUMIFS($W$16:$W$119,$C$16:$C$119,F12,$U$16:$U$119,"&lt;&gt;Done")</f>
         <v>0 passed / 4 total (0%) · 195/485</v>
       </c>
       <c r="J12" s="178" t="s">
@@ -12716,25 +12746,25 @@
         <v>1</v>
       </c>
       <c r="N99" s="136" t="s">
-        <v>894</v>
+        <v>927</v>
       </c>
       <c r="O99" s="136" t="s">
-        <v>927</v>
+        <v>928</v>
       </c>
       <c r="P99" s="136" t="s">
-        <v>928</v>
+        <v>929</v>
       </c>
       <c r="Q99" s="136" t="s">
         <v>1</v>
       </c>
       <c r="R99" s="136" t="s">
-        <v>929</v>
+        <v>930</v>
       </c>
       <c r="S99" s="136" t="s">
-        <v>930</v>
+        <v>931</v>
       </c>
       <c r="T99" s="136" t="s">
-        <v>931</v>
+        <v>932</v>
       </c>
       <c r="U99" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",K99&amp;" "&amp;Q99)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K99&amp;" "&amp;Q99))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K99&amp;" "&amp;Q99)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K99&amp;" "&amp;Q99))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K99&amp;" "&amp;Q99)),ISNUMBER(SEARCH("PENDING",K99&amp;" "&amp;Q99)),ISNUMBER(SEARCH("IN PROGRESS",K99&amp;" "&amp;Q99)),ISNUMBER(SEARCH("OPEN",K99&amp;" "&amp;Q99)),ISNUMBER(SEARCH("RETEST REQUIRED",K99&amp;" "&amp;Q99)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K99&amp;" "&amp;Q99)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K99&amp;" "&amp;Q99))),"Pending",IF(OR(Q99="PASS",ISNUMBER(SEARCH("PASS",K99&amp;" "&amp;Q99))),"Done","Pending"))))</f>
@@ -12742,159 +12772,159 @@
       </c>
       <c r="V99" s="146">
         <f>IF(T99="","",VALUE(LEFT(T99,SEARCH("/",T99)-1)))</f>
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="W99" s="146">
         <f>IF(T99="","",VALUE(MID(T99,SEARCH("/",T99)+1,LEN(T99))))</f>
-        <v>250</v>
+        <v>165</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="136" t="s">
-        <v>932</v>
-      </c>
-      <c r="B100" s="136" t="s">
+      <c r="A100" s="135" t="s">
+        <v>933</v>
+      </c>
+      <c r="B100" s="135" t="s">
         <v>180</v>
       </c>
       <c r="C100" s="259" t="s">
         <v>27</v>
       </c>
-      <c r="D100" s="136" t="s">
-        <v>933</v>
-      </c>
-      <c r="E100" s="136" t="s">
+      <c r="D100" s="135" t="s">
         <v>934</v>
       </c>
-      <c r="F100" s="136" t="s">
+      <c r="E100" s="135" t="s">
         <v>935</v>
       </c>
-      <c r="G100" s="136" t="s">
+      <c r="F100" s="135" t="s">
         <v>936</v>
       </c>
-      <c r="H100" s="136" t="s">
+      <c r="G100" s="135" t="s">
         <v>937</v>
       </c>
-      <c r="I100" s="136" t="s">
+      <c r="H100" s="135" t="s">
         <v>938</v>
       </c>
-      <c r="J100" s="136" t="s">
+      <c r="I100" s="135" t="s">
         <v>939</v>
       </c>
-      <c r="K100" s="136" t="s">
+      <c r="J100" s="135" t="s">
         <v>940</v>
       </c>
-      <c r="L100" s="136" t="s">
-        <v>1</v>
-      </c>
-      <c r="M100" s="136" t="s">
-        <v>1</v>
-      </c>
-      <c r="N100" s="136" t="s">
+      <c r="K100" s="135" t="s">
+        <v>82</v>
+      </c>
+      <c r="L100" s="135" t="s">
+        <v>1</v>
+      </c>
+      <c r="M100" s="135" t="s">
+        <v>1</v>
+      </c>
+      <c r="N100" s="135" t="s">
+        <v>927</v>
+      </c>
+      <c r="O100" s="135" t="s">
         <v>941</v>
       </c>
-      <c r="O100" s="136" t="s">
+      <c r="P100" s="135" t="s">
         <v>942</v>
       </c>
-      <c r="P100" s="136" t="s">
+      <c r="Q100" s="135" t="s">
+        <v>86</v>
+      </c>
+      <c r="R100" s="135" t="s">
         <v>943</v>
       </c>
-      <c r="Q100" s="136" t="s">
-        <v>1</v>
-      </c>
-      <c r="R100" s="136" t="s">
-        <v>944</v>
-      </c>
-      <c r="S100" s="136" t="s">
+      <c r="S100" s="135" t="s">
         <v>88</v>
       </c>
-      <c r="T100" s="136" t="s">
-        <v>945</v>
+      <c r="T100" s="135" t="s">
+        <v>1</v>
       </c>
       <c r="U100" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",K100&amp;" "&amp;Q100)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K100&amp;" "&amp;Q100))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K100&amp;" "&amp;Q100)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K100&amp;" "&amp;Q100))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K100&amp;" "&amp;Q100)),ISNUMBER(SEARCH("PENDING",K100&amp;" "&amp;Q100)),ISNUMBER(SEARCH("IN PROGRESS",K100&amp;" "&amp;Q100)),ISNUMBER(SEARCH("OPEN",K100&amp;" "&amp;Q100)),ISNUMBER(SEARCH("RETEST REQUIRED",K100&amp;" "&amp;Q100)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K100&amp;" "&amp;Q100)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K100&amp;" "&amp;Q100))),"Pending",IF(OR(Q100="PASS",ISNUMBER(SEARCH("PASS",K100&amp;" "&amp;Q100))),"Done","Pending"))))</f>
-        <v>Pending</v>
+        <v>Done</v>
       </c>
       <c r="V100" s="146">
         <f>IF(T100="","",VALUE(LEFT(T100,SEARCH("/",T100)-1)))</f>
-        <v>150</v>
+        <v/>
       </c>
       <c r="W100" s="146">
         <f>IF(T100="","",VALUE(MID(T100,SEARCH("/",T100)+1,LEN(T100))))</f>
-        <v>355</v>
+        <v/>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="135" t="s">
-        <v>946</v>
-      </c>
-      <c r="B101" s="135" t="s">
-        <v>155</v>
+      <c r="A101" s="136" t="s">
+        <v>944</v>
+      </c>
+      <c r="B101" s="136" t="s">
+        <v>945</v>
       </c>
       <c r="C101" s="259" t="s">
         <v>27</v>
       </c>
-      <c r="D101" s="135" t="s">
+      <c r="D101" s="136" t="s">
+        <v>946</v>
+      </c>
+      <c r="E101" s="136" t="s">
         <v>947</v>
       </c>
-      <c r="E101" s="135" t="s">
+      <c r="F101" s="136" t="s">
         <v>948</v>
       </c>
-      <c r="F101" s="135" t="s">
+      <c r="G101" s="136" t="s">
         <v>949</v>
       </c>
-      <c r="G101" s="135" t="s">
+      <c r="H101" s="136" t="s">
+        <v>4</v>
+      </c>
+      <c r="I101" s="136" t="s">
         <v>950</v>
       </c>
-      <c r="H101" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="I101" s="135" t="s">
+      <c r="J101" s="136" t="s">
         <v>951</v>
       </c>
-      <c r="J101" s="135" t="s">
+      <c r="K101" s="136" t="s">
         <v>952</v>
       </c>
-      <c r="K101" s="135" t="s">
-        <v>82</v>
-      </c>
-      <c r="L101" s="135" t="s">
-        <v>86</v>
-      </c>
-      <c r="M101" s="135" t="s">
-        <v>86</v>
-      </c>
-      <c r="N101" s="135" t="s">
+      <c r="L101" s="136" t="s">
+        <v>1</v>
+      </c>
+      <c r="M101" s="136" t="s">
+        <v>1</v>
+      </c>
+      <c r="N101" s="136" t="s">
+        <v>927</v>
+      </c>
+      <c r="O101" s="136" t="s">
         <v>953</v>
       </c>
-      <c r="O101" s="135" t="s">
+      <c r="P101" s="136" t="s">
         <v>954</v>
       </c>
-      <c r="P101" s="135" t="s">
+      <c r="Q101" s="136" t="s">
+        <v>1</v>
+      </c>
+      <c r="R101" s="136" t="s">
         <v>955</v>
       </c>
-      <c r="Q101" s="135" t="s">
-        <v>86</v>
-      </c>
-      <c r="R101" s="135" t="s">
+      <c r="S101" s="136" t="s">
+        <v>111</v>
+      </c>
+      <c r="T101" s="136" t="s">
         <v>956</v>
-      </c>
-      <c r="S101" s="135" t="s">
-        <v>248</v>
-      </c>
-      <c r="T101" s="135" t="s">
-        <v>1</v>
       </c>
       <c r="U101" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",K101&amp;" "&amp;Q101)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K101&amp;" "&amp;Q101))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K101&amp;" "&amp;Q101)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K101&amp;" "&amp;Q101))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K101&amp;" "&amp;Q101)),ISNUMBER(SEARCH("PENDING",K101&amp;" "&amp;Q101)),ISNUMBER(SEARCH("IN PROGRESS",K101&amp;" "&amp;Q101)),ISNUMBER(SEARCH("OPEN",K101&amp;" "&amp;Q101)),ISNUMBER(SEARCH("RETEST REQUIRED",K101&amp;" "&amp;Q101)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K101&amp;" "&amp;Q101)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K101&amp;" "&amp;Q101))),"Pending",IF(OR(Q101="PASS",ISNUMBER(SEARCH("PASS",K101&amp;" "&amp;Q101))),"Done","Pending"))))</f>
-        <v>Done</v>
+        <v>Pending</v>
       </c>
       <c r="V101" s="146">
         <f>IF(T101="","",VALUE(LEFT(T101,SEARCH("/",T101)-1)))</f>
-        <v/>
+        <v>65</v>
       </c>
       <c r="W101" s="146">
         <f>IF(T101="","",VALUE(MID(T101,SEARCH("/",T101)+1,LEN(T101))))</f>
-        <v/>
+        <v>155</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12902,10 +12932,10 @@
         <v>957</v>
       </c>
       <c r="B102" s="135" t="s">
-        <v>180</v>
-      </c>
-      <c r="C102" s="261" t="s">
-        <v>33</v>
+        <v>155</v>
+      </c>
+      <c r="C102" s="259" t="s">
+        <v>27</v>
       </c>
       <c r="D102" s="135" t="s">
         <v>958</v>
@@ -12914,43 +12944,43 @@
         <v>959</v>
       </c>
       <c r="F102" s="135" t="s">
-        <v>4</v>
+        <v>960</v>
       </c>
       <c r="G102" s="135" t="s">
-        <v>4</v>
+        <v>961</v>
       </c>
       <c r="H102" s="135" t="s">
         <v>4</v>
       </c>
       <c r="I102" s="135" t="s">
-        <v>4</v>
+        <v>962</v>
       </c>
       <c r="J102" s="135" t="s">
-        <v>960</v>
+        <v>963</v>
       </c>
       <c r="K102" s="135" t="s">
-        <v>685</v>
+        <v>82</v>
       </c>
       <c r="L102" s="135" t="s">
-        <v>1</v>
+        <v>86</v>
       </c>
       <c r="M102" s="135" t="s">
-        <v>1</v>
+        <v>86</v>
       </c>
       <c r="N102" s="135" t="s">
-        <v>423</v>
+        <v>964</v>
       </c>
       <c r="O102" s="135" t="s">
-        <v>961</v>
+        <v>965</v>
       </c>
       <c r="P102" s="135" t="s">
-        <v>962</v>
+        <v>966</v>
       </c>
       <c r="Q102" s="135" t="s">
         <v>86</v>
       </c>
       <c r="R102" s="135" t="s">
-        <v>963</v>
+        <v>967</v>
       </c>
       <c r="S102" s="135" t="s">
         <v>248</v>
@@ -12973,7 +13003,7 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="135" t="s">
-        <v>964</v>
+        <v>968</v>
       </c>
       <c r="B103" s="135" t="s">
         <v>180</v>
@@ -12982,10 +13012,10 @@
         <v>33</v>
       </c>
       <c r="D103" s="135" t="s">
-        <v>965</v>
+        <v>969</v>
       </c>
       <c r="E103" s="135" t="s">
-        <v>966</v>
+        <v>970</v>
       </c>
       <c r="F103" s="135" t="s">
         <v>4</v>
@@ -13000,7 +13030,7 @@
         <v>4</v>
       </c>
       <c r="J103" s="135" t="s">
-        <v>967</v>
+        <v>971</v>
       </c>
       <c r="K103" s="135" t="s">
         <v>685</v>
@@ -13015,19 +13045,19 @@
         <v>423</v>
       </c>
       <c r="O103" s="135" t="s">
-        <v>968</v>
+        <v>972</v>
       </c>
       <c r="P103" s="135" t="s">
-        <v>969</v>
+        <v>973</v>
       </c>
       <c r="Q103" s="135" t="s">
         <v>86</v>
       </c>
       <c r="R103" s="135" t="s">
-        <v>970</v>
+        <v>974</v>
       </c>
       <c r="S103" s="135" t="s">
-        <v>317</v>
+        <v>248</v>
       </c>
       <c r="T103" s="135" t="s">
         <v>1</v>
@@ -13047,25 +13077,25 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="135" t="s">
-        <v>971</v>
+        <v>975</v>
       </c>
       <c r="B104" s="135" t="s">
-        <v>155</v>
+        <v>180</v>
       </c>
       <c r="C104" s="261" t="s">
         <v>33</v>
       </c>
       <c r="D104" s="135" t="s">
-        <v>972</v>
+        <v>976</v>
       </c>
       <c r="E104" s="135" t="s">
-        <v>973</v>
+        <v>977</v>
       </c>
       <c r="F104" s="135" t="s">
-        <v>974</v>
+        <v>4</v>
       </c>
       <c r="G104" s="135" t="s">
-        <v>975</v>
+        <v>4</v>
       </c>
       <c r="H104" s="135" t="s">
         <v>4</v>
@@ -13074,34 +13104,34 @@
         <v>4</v>
       </c>
       <c r="J104" s="135" t="s">
-        <v>976</v>
+        <v>978</v>
       </c>
       <c r="K104" s="135" t="s">
-        <v>82</v>
+        <v>685</v>
       </c>
       <c r="L104" s="135" t="s">
-        <v>86</v>
+        <v>1</v>
       </c>
       <c r="M104" s="135" t="s">
-        <v>86</v>
+        <v>1</v>
       </c>
       <c r="N104" s="135" t="s">
-        <v>953</v>
+        <v>423</v>
       </c>
       <c r="O104" s="135" t="s">
-        <v>977</v>
+        <v>979</v>
       </c>
       <c r="P104" s="135" t="s">
-        <v>978</v>
+        <v>980</v>
       </c>
       <c r="Q104" s="135" t="s">
         <v>86</v>
       </c>
       <c r="R104" s="135" t="s">
-        <v>979</v>
+        <v>981</v>
       </c>
       <c r="S104" s="135" t="s">
-        <v>980</v>
+        <v>317</v>
       </c>
       <c r="T104" s="135" t="s">
         <v>1</v>
@@ -13120,180 +13150,180 @@
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="138" t="s">
-        <v>981</v>
-      </c>
-      <c r="B105" s="138" t="s">
+      <c r="A105" s="135" t="s">
+        <v>982</v>
+      </c>
+      <c r="B105" s="135" t="s">
         <v>155</v>
       </c>
-      <c r="C105" s="255" t="s">
-        <v>38</v>
-      </c>
-      <c r="D105" s="138" t="s">
-        <v>982</v>
-      </c>
-      <c r="E105" s="138" t="s">
+      <c r="C105" s="261" t="s">
+        <v>33</v>
+      </c>
+      <c r="D105" s="135" t="s">
         <v>983</v>
       </c>
-      <c r="F105" s="138" t="s">
+      <c r="E105" s="135" t="s">
         <v>984</v>
       </c>
-      <c r="G105" s="138" t="s">
+      <c r="F105" s="135" t="s">
         <v>985</v>
       </c>
-      <c r="H105" s="138" t="s">
+      <c r="G105" s="135" t="s">
+        <v>986</v>
+      </c>
+      <c r="H105" s="135" t="s">
         <v>4</v>
       </c>
-      <c r="I105" s="138" t="s">
-        <v>986</v>
-      </c>
-      <c r="J105" s="138" t="s">
+      <c r="I105" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="J105" s="135" t="s">
         <v>987</v>
       </c>
-      <c r="K105" s="138" t="s">
+      <c r="K105" s="135" t="s">
+        <v>82</v>
+      </c>
+      <c r="L105" s="135" t="s">
+        <v>86</v>
+      </c>
+      <c r="M105" s="135" t="s">
+        <v>86</v>
+      </c>
+      <c r="N105" s="135" t="s">
+        <v>964</v>
+      </c>
+      <c r="O105" s="135" t="s">
         <v>988</v>
       </c>
-      <c r="L105" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="M105" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="N105" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O105" s="138" t="s">
+      <c r="P105" s="135" t="s">
         <v>989</v>
       </c>
-      <c r="P105" s="138" t="s">
+      <c r="Q105" s="135" t="s">
+        <v>86</v>
+      </c>
+      <c r="R105" s="135" t="s">
         <v>990</v>
       </c>
-      <c r="Q105" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="R105" s="138" t="s">
+      <c r="S105" s="135" t="s">
         <v>991</v>
       </c>
-      <c r="S105" s="138" t="s">
-        <v>111</v>
-      </c>
-      <c r="T105" s="138" t="s">
-        <v>992</v>
+      <c r="T105" s="135" t="s">
+        <v>1</v>
       </c>
       <c r="U105" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",K105&amp;" "&amp;Q105)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K105&amp;" "&amp;Q105))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K105&amp;" "&amp;Q105)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K105&amp;" "&amp;Q105))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K105&amp;" "&amp;Q105)),ISNUMBER(SEARCH("PENDING",K105&amp;" "&amp;Q105)),ISNUMBER(SEARCH("IN PROGRESS",K105&amp;" "&amp;Q105)),ISNUMBER(SEARCH("OPEN",K105&amp;" "&amp;Q105)),ISNUMBER(SEARCH("RETEST REQUIRED",K105&amp;" "&amp;Q105)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K105&amp;" "&amp;Q105)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K105&amp;" "&amp;Q105))),"Pending",IF(OR(Q105="PASS",ISNUMBER(SEARCH("PASS",K105&amp;" "&amp;Q105))),"Done","Pending"))))</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="V105" s="146">
         <f>IF(T105="","",VALUE(LEFT(T105,SEARCH("/",T105)-1)))</f>
-        <v>100</v>
+        <v/>
       </c>
       <c r="W105" s="146">
         <f>IF(T105="","",VALUE(MID(T105,SEARCH("/",T105)+1,LEN(T105))))</f>
-        <v>235</v>
+        <v/>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="136" t="s">
-        <v>993</v>
-      </c>
-      <c r="B106" s="136" t="s">
+      <c r="A106" s="138" t="s">
+        <v>992</v>
+      </c>
+      <c r="B106" s="138" t="s">
         <v>155</v>
       </c>
       <c r="C106" s="255" t="s">
         <v>38</v>
       </c>
-      <c r="D106" s="136" t="s">
+      <c r="D106" s="138" t="s">
+        <v>993</v>
+      </c>
+      <c r="E106" s="138" t="s">
         <v>994</v>
       </c>
-      <c r="E106" s="136" t="s">
+      <c r="F106" s="138" t="s">
         <v>995</v>
       </c>
-      <c r="F106" s="136" t="s">
+      <c r="G106" s="138" t="s">
         <v>996</v>
       </c>
-      <c r="G106" s="136" t="s">
+      <c r="H106" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="I106" s="138" t="s">
         <v>997</v>
       </c>
-      <c r="H106" s="136" t="s">
+      <c r="J106" s="138" t="s">
         <v>998</v>
       </c>
-      <c r="I106" s="136" t="s">
+      <c r="K106" s="138" t="s">
         <v>999</v>
       </c>
-      <c r="J106" s="136" t="s">
+      <c r="L106" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="M106" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="N106" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O106" s="138" t="s">
         <v>1000</v>
       </c>
-      <c r="K106" s="136" t="s">
+      <c r="P106" s="138" t="s">
         <v>1001</v>
       </c>
-      <c r="L106" s="136" t="s">
-        <v>1</v>
-      </c>
-      <c r="M106" s="136" t="s">
-        <v>1</v>
-      </c>
-      <c r="N106" s="136" t="s">
-        <v>189</v>
-      </c>
-      <c r="O106" s="136" t="s">
+      <c r="Q106" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="R106" s="138" t="s">
         <v>1002</v>
       </c>
-      <c r="P106" s="136" t="s">
+      <c r="S106" s="138" t="s">
+        <v>111</v>
+      </c>
+      <c r="T106" s="138" t="s">
         <v>1003</v>
-      </c>
-      <c r="Q106" s="136" t="s">
-        <v>1004</v>
-      </c>
-      <c r="R106" s="136" t="s">
-        <v>1005</v>
-      </c>
-      <c r="S106" s="136" t="s">
-        <v>260</v>
-      </c>
-      <c r="T106" s="136" t="s">
-        <v>1006</v>
       </c>
       <c r="U106" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",K106&amp;" "&amp;Q106)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K106&amp;" "&amp;Q106))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K106&amp;" "&amp;Q106)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K106&amp;" "&amp;Q106))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K106&amp;" "&amp;Q106)),ISNUMBER(SEARCH("PENDING",K106&amp;" "&amp;Q106)),ISNUMBER(SEARCH("IN PROGRESS",K106&amp;" "&amp;Q106)),ISNUMBER(SEARCH("OPEN",K106&amp;" "&amp;Q106)),ISNUMBER(SEARCH("RETEST REQUIRED",K106&amp;" "&amp;Q106)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K106&amp;" "&amp;Q106)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K106&amp;" "&amp;Q106))),"Pending",IF(OR(Q106="PASS",ISNUMBER(SEARCH("PASS",K106&amp;" "&amp;Q106))),"Done","Pending"))))</f>
-        <v>Pending</v>
+        <v>Not started</v>
       </c>
       <c r="V106" s="146">
         <f>IF(T106="","",VALUE(LEFT(T106,SEARCH("/",T106)-1)))</f>
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="W106" s="146">
         <f>IF(T106="","",VALUE(MID(T106,SEARCH("/",T106)+1,LEN(T106))))</f>
-        <v>130</v>
+        <v>235</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="136" t="s">
-        <v>1007</v>
+        <v>1004</v>
       </c>
       <c r="B107" s="136" t="s">
-        <v>169</v>
+        <v>155</v>
       </c>
       <c r="C107" s="255" t="s">
         <v>38</v>
       </c>
       <c r="D107" s="136" t="s">
+        <v>1005</v>
+      </c>
+      <c r="E107" s="136" t="s">
+        <v>1006</v>
+      </c>
+      <c r="F107" s="136" t="s">
+        <v>1007</v>
+      </c>
+      <c r="G107" s="136" t="s">
         <v>1008</v>
       </c>
-      <c r="E107" s="136" t="s">
+      <c r="H107" s="136" t="s">
         <v>1009</v>
       </c>
-      <c r="F107" s="136" t="s">
-        <v>4</v>
-      </c>
-      <c r="G107" s="136" t="s">
+      <c r="I107" s="136" t="s">
         <v>1010</v>
-      </c>
-      <c r="H107" s="136" t="s">
-        <v>4</v>
-      </c>
-      <c r="I107" s="136" t="s">
-        <v>8</v>
       </c>
       <c r="J107" s="136" t="s">
         <v>1011</v>
@@ -13308,22 +13338,22 @@
         <v>1</v>
       </c>
       <c r="N107" s="136" t="s">
+        <v>189</v>
+      </c>
+      <c r="O107" s="136" t="s">
         <v>1013</v>
       </c>
-      <c r="O107" s="136" t="s">
+      <c r="P107" s="136" t="s">
         <v>1014</v>
       </c>
-      <c r="P107" s="136" t="s">
+      <c r="Q107" s="136" t="s">
         <v>1015</v>
-      </c>
-      <c r="Q107" s="136" t="s">
-        <v>1004</v>
       </c>
       <c r="R107" s="136" t="s">
         <v>1016</v>
       </c>
       <c r="S107" s="136" t="s">
-        <v>827</v>
+        <v>260</v>
       </c>
       <c r="T107" s="136" t="s">
         <v>1017</v>
@@ -13334,11 +13364,11 @@
       </c>
       <c r="V107" s="146">
         <f>IF(T107="","",VALUE(LEFT(T107,SEARCH("/",T107)-1)))</f>
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="W107" s="146">
         <f>IF(T107="","",VALUE(MID(T107,SEARCH("/",T107)+1,LEN(T107))))</f>
-        <v>65</v>
+        <v>130</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13346,7 +13376,7 @@
         <v>1018</v>
       </c>
       <c r="B108" s="136" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
       <c r="C108" s="255" t="s">
         <v>38</v>
@@ -13358,31 +13388,31 @@
         <v>1020</v>
       </c>
       <c r="F108" s="136" t="s">
+        <v>4</v>
+      </c>
+      <c r="G108" s="136" t="s">
         <v>1021</v>
-      </c>
-      <c r="G108" s="136" t="s">
-        <v>1022</v>
       </c>
       <c r="H108" s="136" t="s">
         <v>4</v>
       </c>
       <c r="I108" s="136" t="s">
+        <v>8</v>
+      </c>
+      <c r="J108" s="136" t="s">
+        <v>1022</v>
+      </c>
+      <c r="K108" s="136" t="s">
         <v>1023</v>
       </c>
-      <c r="J108" s="136" t="s">
+      <c r="L108" s="136" t="s">
+        <v>1</v>
+      </c>
+      <c r="M108" s="136" t="s">
+        <v>1</v>
+      </c>
+      <c r="N108" s="136" t="s">
         <v>1024</v>
-      </c>
-      <c r="K108" s="136" t="s">
-        <v>1001</v>
-      </c>
-      <c r="L108" s="136" t="s">
-        <v>1</v>
-      </c>
-      <c r="M108" s="136" t="s">
-        <v>1</v>
-      </c>
-      <c r="N108" s="136" t="s">
-        <v>189</v>
       </c>
       <c r="O108" s="136" t="s">
         <v>1025</v>
@@ -13391,13 +13421,13 @@
         <v>1026</v>
       </c>
       <c r="Q108" s="136" t="s">
-        <v>1004</v>
+        <v>1015</v>
       </c>
       <c r="R108" s="136" t="s">
         <v>1027</v>
       </c>
       <c r="S108" s="136" t="s">
-        <v>328</v>
+        <v>827</v>
       </c>
       <c r="T108" s="136" t="s">
         <v>1028</v>
@@ -13408,517 +13438,517 @@
       </c>
       <c r="V108" s="146">
         <f>IF(T108="","",VALUE(LEFT(T108,SEARCH("/",T108)-1)))</f>
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="W108" s="146">
         <f>IF(T108="","",VALUE(MID(T108,SEARCH("/",T108)+1,LEN(T108))))</f>
-        <v>190</v>
+        <v>65</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="138" t="s">
+      <c r="A109" s="136" t="s">
         <v>1029</v>
       </c>
-      <c r="B109" s="138" t="s">
+      <c r="B109" s="136" t="s">
         <v>155</v>
       </c>
       <c r="C109" s="255" t="s">
         <v>38</v>
       </c>
-      <c r="D109" s="138" t="s">
+      <c r="D109" s="136" t="s">
         <v>1030</v>
       </c>
-      <c r="E109" s="138" t="s">
+      <c r="E109" s="136" t="s">
         <v>1031</v>
       </c>
-      <c r="F109" s="138" t="s">
+      <c r="F109" s="136" t="s">
         <v>1032</v>
       </c>
-      <c r="G109" s="138" t="s">
+      <c r="G109" s="136" t="s">
         <v>1033</v>
       </c>
-      <c r="H109" s="138" t="s">
+      <c r="H109" s="136" t="s">
         <v>4</v>
       </c>
-      <c r="I109" s="138" t="s">
+      <c r="I109" s="136" t="s">
         <v>1034</v>
       </c>
-      <c r="J109" s="138" t="s">
+      <c r="J109" s="136" t="s">
         <v>1035</v>
       </c>
-      <c r="K109" s="138" t="s">
-        <v>988</v>
-      </c>
-      <c r="L109" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="M109" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="N109" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O109" s="138" t="s">
+      <c r="K109" s="136" t="s">
+        <v>1012</v>
+      </c>
+      <c r="L109" s="136" t="s">
+        <v>1</v>
+      </c>
+      <c r="M109" s="136" t="s">
+        <v>1</v>
+      </c>
+      <c r="N109" s="136" t="s">
+        <v>189</v>
+      </c>
+      <c r="O109" s="136" t="s">
         <v>1036</v>
       </c>
-      <c r="P109" s="138" t="s">
+      <c r="P109" s="136" t="s">
         <v>1037</v>
       </c>
-      <c r="Q109" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="R109" s="138" t="s">
+      <c r="Q109" s="136" t="s">
+        <v>1015</v>
+      </c>
+      <c r="R109" s="136" t="s">
         <v>1038</v>
       </c>
-      <c r="S109" s="138" t="s">
-        <v>88</v>
-      </c>
-      <c r="T109" s="138" t="s">
+      <c r="S109" s="136" t="s">
+        <v>328</v>
+      </c>
+      <c r="T109" s="136" t="s">
         <v>1039</v>
       </c>
       <c r="U109" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",K109&amp;" "&amp;Q109)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K109&amp;" "&amp;Q109))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K109&amp;" "&amp;Q109)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K109&amp;" "&amp;Q109))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K109&amp;" "&amp;Q109)),ISNUMBER(SEARCH("PENDING",K109&amp;" "&amp;Q109)),ISNUMBER(SEARCH("IN PROGRESS",K109&amp;" "&amp;Q109)),ISNUMBER(SEARCH("OPEN",K109&amp;" "&amp;Q109)),ISNUMBER(SEARCH("RETEST REQUIRED",K109&amp;" "&amp;Q109)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K109&amp;" "&amp;Q109)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K109&amp;" "&amp;Q109))),"Pending",IF(OR(Q109="PASS",ISNUMBER(SEARCH("PASS",K109&amp;" "&amp;Q109))),"Done","Pending"))))</f>
-        <v>Not started</v>
+        <v>Pending</v>
       </c>
       <c r="V109" s="146">
         <f>IF(T109="","",VALUE(LEFT(T109,SEARCH("/",T109)-1)))</f>
-        <v>110</v>
+        <v>80</v>
       </c>
       <c r="W109" s="146">
         <f>IF(T109="","",VALUE(MID(T109,SEARCH("/",T109)+1,LEN(T109))))</f>
-        <v>260</v>
+        <v>190</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="136" t="s">
+      <c r="A110" s="138" t="s">
         <v>1040</v>
       </c>
-      <c r="B110" s="136" t="s">
-        <v>1041</v>
+      <c r="B110" s="138" t="s">
+        <v>155</v>
       </c>
       <c r="C110" s="255" t="s">
         <v>38</v>
       </c>
-      <c r="D110" s="136" t="s">
+      <c r="D110" s="138" t="s">
+        <v>1041</v>
+      </c>
+      <c r="E110" s="138" t="s">
         <v>1042</v>
       </c>
-      <c r="E110" s="136" t="s">
+      <c r="F110" s="138" t="s">
         <v>1043</v>
       </c>
-      <c r="F110" s="136" t="s">
+      <c r="G110" s="138" t="s">
+        <v>1044</v>
+      </c>
+      <c r="H110" s="138" t="s">
         <v>4</v>
       </c>
-      <c r="G110" s="136" t="s">
-        <v>4</v>
-      </c>
-      <c r="H110" s="136" t="s">
-        <v>4</v>
-      </c>
-      <c r="I110" s="136" t="s">
-        <v>1044</v>
-      </c>
-      <c r="J110" s="136" t="s">
+      <c r="I110" s="138" t="s">
         <v>1045</v>
       </c>
-      <c r="K110" s="136" t="s">
+      <c r="J110" s="138" t="s">
         <v>1046</v>
       </c>
-      <c r="L110" s="136" t="s">
-        <v>1</v>
-      </c>
-      <c r="M110" s="136" t="s">
-        <v>1</v>
-      </c>
-      <c r="N110" s="136" t="s">
-        <v>189</v>
-      </c>
-      <c r="O110" s="136" t="s">
+      <c r="K110" s="138" t="s">
+        <v>999</v>
+      </c>
+      <c r="L110" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="M110" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="N110" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O110" s="138" t="s">
         <v>1047</v>
       </c>
-      <c r="P110" s="136" t="s">
+      <c r="P110" s="138" t="s">
         <v>1048</v>
       </c>
-      <c r="Q110" s="136" t="s">
+      <c r="Q110" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="R110" s="138" t="s">
         <v>1049</v>
       </c>
-      <c r="R110" s="136" t="s">
+      <c r="S110" s="138" t="s">
+        <v>88</v>
+      </c>
+      <c r="T110" s="138" t="s">
         <v>1050</v>
-      </c>
-      <c r="S110" s="136" t="s">
-        <v>1051</v>
-      </c>
-      <c r="T110" s="136" t="s">
-        <v>1052</v>
       </c>
       <c r="U110" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",K110&amp;" "&amp;Q110)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K110&amp;" "&amp;Q110))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K110&amp;" "&amp;Q110)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K110&amp;" "&amp;Q110))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K110&amp;" "&amp;Q110)),ISNUMBER(SEARCH("PENDING",K110&amp;" "&amp;Q110)),ISNUMBER(SEARCH("IN PROGRESS",K110&amp;" "&amp;Q110)),ISNUMBER(SEARCH("OPEN",K110&amp;" "&amp;Q110)),ISNUMBER(SEARCH("RETEST REQUIRED",K110&amp;" "&amp;Q110)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K110&amp;" "&amp;Q110)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K110&amp;" "&amp;Q110))),"Pending",IF(OR(Q110="PASS",ISNUMBER(SEARCH("PASS",K110&amp;" "&amp;Q110))),"Done","Pending"))))</f>
-        <v>Pending</v>
+        <v>Not started</v>
       </c>
       <c r="V110" s="146">
         <f>IF(T110="","",VALUE(LEFT(T110,SEARCH("/",T110)-1)))</f>
-        <v>45</v>
+        <v>110</v>
       </c>
       <c r="W110" s="146">
         <f>IF(T110="","",VALUE(MID(T110,SEARCH("/",T110)+1,LEN(T110))))</f>
-        <v>115</v>
+        <v>260</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="135" t="s">
+      <c r="A111" s="136" t="s">
+        <v>1051</v>
+      </c>
+      <c r="B111" s="136" t="s">
+        <v>1052</v>
+      </c>
+      <c r="C111" s="255" t="s">
+        <v>38</v>
+      </c>
+      <c r="D111" s="136" t="s">
         <v>1053</v>
       </c>
-      <c r="B111" s="135" t="s">
+      <c r="E111" s="136" t="s">
         <v>1054</v>
       </c>
-      <c r="C111" s="263" t="s">
-        <v>43</v>
-      </c>
-      <c r="D111" s="135" t="s">
-        <v>58</v>
-      </c>
-      <c r="E111" s="135" t="s">
+      <c r="F111" s="136" t="s">
+        <v>4</v>
+      </c>
+      <c r="G111" s="136" t="s">
+        <v>4</v>
+      </c>
+      <c r="H111" s="136" t="s">
+        <v>4</v>
+      </c>
+      <c r="I111" s="136" t="s">
         <v>1055</v>
       </c>
-      <c r="F111" s="135" t="s">
+      <c r="J111" s="136" t="s">
         <v>1056</v>
       </c>
-      <c r="G111" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="H111" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="I111" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="J111" s="135" t="s">
-        <v>4</v>
-      </c>
-      <c r="K111" s="135" t="s">
-        <v>685</v>
-      </c>
-      <c r="L111" s="135" t="s">
-        <v>1</v>
-      </c>
-      <c r="M111" s="135" t="s">
-        <v>1</v>
-      </c>
-      <c r="N111" s="135" t="s">
+      <c r="K111" s="136" t="s">
+        <v>1057</v>
+      </c>
+      <c r="L111" s="136" t="s">
+        <v>1</v>
+      </c>
+      <c r="M111" s="136" t="s">
+        <v>1</v>
+      </c>
+      <c r="N111" s="136" t="s">
         <v>189</v>
       </c>
-      <c r="O111" s="135" t="s">
-        <v>1057</v>
-      </c>
-      <c r="P111" s="135" t="s">
+      <c r="O111" s="136" t="s">
         <v>1058</v>
       </c>
-      <c r="Q111" s="135" t="s">
-        <v>86</v>
-      </c>
-      <c r="R111" s="135" t="s">
+      <c r="P111" s="136" t="s">
         <v>1059</v>
       </c>
-      <c r="S111" s="135" t="s">
+      <c r="Q111" s="136" t="s">
         <v>1060</v>
       </c>
-      <c r="T111" s="135" t="s">
-        <v>1</v>
+      <c r="R111" s="136" t="s">
+        <v>1061</v>
+      </c>
+      <c r="S111" s="136" t="s">
+        <v>1062</v>
+      </c>
+      <c r="T111" s="136" t="s">
+        <v>1063</v>
       </c>
       <c r="U111" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",K111&amp;" "&amp;Q111)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K111&amp;" "&amp;Q111))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K111&amp;" "&amp;Q111)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K111&amp;" "&amp;Q111))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K111&amp;" "&amp;Q111)),ISNUMBER(SEARCH("PENDING",K111&amp;" "&amp;Q111)),ISNUMBER(SEARCH("IN PROGRESS",K111&amp;" "&amp;Q111)),ISNUMBER(SEARCH("OPEN",K111&amp;" "&amp;Q111)),ISNUMBER(SEARCH("RETEST REQUIRED",K111&amp;" "&amp;Q111)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K111&amp;" "&amp;Q111)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K111&amp;" "&amp;Q111))),"Pending",IF(OR(Q111="PASS",ISNUMBER(SEARCH("PASS",K111&amp;" "&amp;Q111))),"Done","Pending"))))</f>
-        <v>Done</v>
+        <v>Pending</v>
       </c>
       <c r="V111" s="146">
         <f>IF(T111="","",VALUE(LEFT(T111,SEARCH("/",T111)-1)))</f>
-        <v/>
+        <v>60</v>
       </c>
       <c r="W111" s="146">
         <f>IF(T111="","",VALUE(MID(T111,SEARCH("/",T111)+1,LEN(T111))))</f>
-        <v/>
+        <v>145</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="138" t="s">
-        <v>1061</v>
-      </c>
-      <c r="B112" s="138" t="s">
-        <v>155</v>
+      <c r="A112" s="135" t="s">
+        <v>1064</v>
+      </c>
+      <c r="B112" s="135" t="s">
+        <v>1065</v>
       </c>
       <c r="C112" s="263" t="s">
         <v>43</v>
       </c>
-      <c r="D112" s="138" t="s">
-        <v>1062</v>
-      </c>
-      <c r="E112" s="138" t="s">
-        <v>1063</v>
-      </c>
-      <c r="F112" s="138" t="s">
-        <v>1064</v>
-      </c>
-      <c r="G112" s="138" t="s">
-        <v>1065</v>
-      </c>
-      <c r="H112" s="138" t="s">
+      <c r="D112" s="135" t="s">
+        <v>58</v>
+      </c>
+      <c r="E112" s="135" t="s">
         <v>1066</v>
       </c>
-      <c r="I112" s="138" t="s">
+      <c r="F112" s="135" t="s">
         <v>1067</v>
       </c>
-      <c r="J112" s="138" t="s">
+      <c r="G112" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="H112" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="I112" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="J112" s="135" t="s">
+        <v>4</v>
+      </c>
+      <c r="K112" s="135" t="s">
+        <v>685</v>
+      </c>
+      <c r="L112" s="135" t="s">
+        <v>1</v>
+      </c>
+      <c r="M112" s="135" t="s">
+        <v>1</v>
+      </c>
+      <c r="N112" s="135" t="s">
+        <v>189</v>
+      </c>
+      <c r="O112" s="135" t="s">
         <v>1068</v>
       </c>
-      <c r="K112" s="138" t="s">
-        <v>988</v>
-      </c>
-      <c r="L112" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="M112" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="N112" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O112" s="138" t="s">
+      <c r="P112" s="135" t="s">
         <v>1069</v>
       </c>
-      <c r="P112" s="138" t="s">
+      <c r="Q112" s="135" t="s">
+        <v>86</v>
+      </c>
+      <c r="R112" s="135" t="s">
         <v>1070</v>
       </c>
-      <c r="Q112" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="R112" s="138" t="s">
+      <c r="S112" s="135" t="s">
         <v>1071</v>
       </c>
-      <c r="S112" s="138" t="s">
-        <v>248</v>
-      </c>
-      <c r="T112" s="138" t="s">
-        <v>1072</v>
+      <c r="T112" s="135" t="s">
+        <v>1</v>
       </c>
       <c r="U112" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",K112&amp;" "&amp;Q112)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K112&amp;" "&amp;Q112))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K112&amp;" "&amp;Q112)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K112&amp;" "&amp;Q112))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K112&amp;" "&amp;Q112)),ISNUMBER(SEARCH("PENDING",K112&amp;" "&amp;Q112)),ISNUMBER(SEARCH("IN PROGRESS",K112&amp;" "&amp;Q112)),ISNUMBER(SEARCH("OPEN",K112&amp;" "&amp;Q112)),ISNUMBER(SEARCH("RETEST REQUIRED",K112&amp;" "&amp;Q112)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K112&amp;" "&amp;Q112)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K112&amp;" "&amp;Q112))),"Pending",IF(OR(Q112="PASS",ISNUMBER(SEARCH("PASS",K112&amp;" "&amp;Q112))),"Done","Pending"))))</f>
-        <v>Not started</v>
+        <v>Done</v>
       </c>
       <c r="V112" s="146">
         <f>IF(T112="","",VALUE(LEFT(T112,SEARCH("/",T112)-1)))</f>
-        <v>75</v>
+        <v/>
       </c>
       <c r="W112" s="146">
         <f>IF(T112="","",VALUE(MID(T112,SEARCH("/",T112)+1,LEN(T112))))</f>
-        <v>180</v>
+        <v/>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="136" t="s">
-        <v>1073</v>
-      </c>
-      <c r="B113" s="136" t="s">
+      <c r="A113" s="138" t="s">
+        <v>1072</v>
+      </c>
+      <c r="B113" s="138" t="s">
         <v>155</v>
       </c>
       <c r="C113" s="263" t="s">
         <v>43</v>
       </c>
-      <c r="D113" s="136" t="s">
+      <c r="D113" s="138" t="s">
+        <v>1073</v>
+      </c>
+      <c r="E113" s="138" t="s">
         <v>1074</v>
       </c>
-      <c r="E113" s="136" t="s">
+      <c r="F113" s="138" t="s">
         <v>1075</v>
       </c>
-      <c r="F113" s="136" t="s">
+      <c r="G113" s="138" t="s">
         <v>1076</v>
       </c>
-      <c r="G113" s="136" t="s">
+      <c r="H113" s="138" t="s">
         <v>1077</v>
       </c>
-      <c r="H113" s="136" t="s">
+      <c r="I113" s="138" t="s">
         <v>1078</v>
       </c>
-      <c r="I113" s="136" t="s">
+      <c r="J113" s="138" t="s">
         <v>1079</v>
       </c>
-      <c r="J113" s="136" t="s">
+      <c r="K113" s="138" t="s">
+        <v>999</v>
+      </c>
+      <c r="L113" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="M113" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="N113" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O113" s="138" t="s">
         <v>1080</v>
       </c>
-      <c r="K113" s="136" t="s">
-        <v>1001</v>
-      </c>
-      <c r="L113" s="136" t="s">
-        <v>1</v>
-      </c>
-      <c r="M113" s="136" t="s">
-        <v>1</v>
-      </c>
-      <c r="N113" s="136" t="s">
-        <v>189</v>
-      </c>
-      <c r="O113" s="136" t="s">
+      <c r="P113" s="138" t="s">
         <v>1081</v>
       </c>
-      <c r="P113" s="136" t="s">
+      <c r="Q113" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="R113" s="138" t="s">
         <v>1082</v>
       </c>
-      <c r="Q113" s="136" t="s">
-        <v>1004</v>
-      </c>
-      <c r="R113" s="136" t="s">
+      <c r="S113" s="138" t="s">
+        <v>248</v>
+      </c>
+      <c r="T113" s="138" t="s">
         <v>1083</v>
-      </c>
-      <c r="S113" s="136" t="s">
-        <v>1084</v>
-      </c>
-      <c r="T113" s="136" t="s">
-        <v>1085</v>
       </c>
       <c r="U113" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",K113&amp;" "&amp;Q113)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K113&amp;" "&amp;Q113))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K113&amp;" "&amp;Q113)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K113&amp;" "&amp;Q113))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K113&amp;" "&amp;Q113)),ISNUMBER(SEARCH("PENDING",K113&amp;" "&amp;Q113)),ISNUMBER(SEARCH("IN PROGRESS",K113&amp;" "&amp;Q113)),ISNUMBER(SEARCH("OPEN",K113&amp;" "&amp;Q113)),ISNUMBER(SEARCH("RETEST REQUIRED",K113&amp;" "&amp;Q113)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K113&amp;" "&amp;Q113)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K113&amp;" "&amp;Q113))),"Pending",IF(OR(Q113="PASS",ISNUMBER(SEARCH("PASS",K113&amp;" "&amp;Q113))),"Done","Pending"))))</f>
-        <v>Pending</v>
+        <v>Not started</v>
       </c>
       <c r="V113" s="146">
         <f>IF(T113="","",VALUE(LEFT(T113,SEARCH("/",T113)-1)))</f>
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="W113" s="146">
         <f>IF(T113="","",VALUE(MID(T113,SEARCH("/",T113)+1,LEN(T113))))</f>
-        <v>145</v>
+        <v>180</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="138" t="s">
-        <v>1086</v>
-      </c>
-      <c r="B114" s="138" t="s">
+      <c r="A114" s="136" t="s">
+        <v>1084</v>
+      </c>
+      <c r="B114" s="136" t="s">
         <v>155</v>
       </c>
       <c r="C114" s="263" t="s">
         <v>43</v>
       </c>
-      <c r="D114" s="138" t="s">
+      <c r="D114" s="136" t="s">
+        <v>1085</v>
+      </c>
+      <c r="E114" s="136" t="s">
+        <v>1086</v>
+      </c>
+      <c r="F114" s="136" t="s">
         <v>1087</v>
       </c>
-      <c r="E114" s="138" t="s">
+      <c r="G114" s="136" t="s">
         <v>1088</v>
       </c>
-      <c r="F114" s="138" t="s">
+      <c r="H114" s="136" t="s">
         <v>1089</v>
       </c>
-      <c r="G114" s="138" t="s">
+      <c r="I114" s="136" t="s">
         <v>1090</v>
       </c>
-      <c r="H114" s="138" t="s">
+      <c r="J114" s="136" t="s">
         <v>1091</v>
       </c>
-      <c r="I114" s="138" t="s">
+      <c r="K114" s="136" t="s">
+        <v>1012</v>
+      </c>
+      <c r="L114" s="136" t="s">
+        <v>1</v>
+      </c>
+      <c r="M114" s="136" t="s">
+        <v>1</v>
+      </c>
+      <c r="N114" s="136" t="s">
+        <v>189</v>
+      </c>
+      <c r="O114" s="136" t="s">
         <v>1092</v>
       </c>
-      <c r="J114" s="138" t="s">
+      <c r="P114" s="136" t="s">
         <v>1093</v>
       </c>
-      <c r="K114" s="138" t="s">
-        <v>988</v>
-      </c>
-      <c r="L114" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="M114" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="N114" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O114" s="138" t="s">
+      <c r="Q114" s="136" t="s">
+        <v>1015</v>
+      </c>
+      <c r="R114" s="136" t="s">
         <v>1094</v>
       </c>
-      <c r="P114" s="138" t="s">
+      <c r="S114" s="136" t="s">
         <v>1095</v>
       </c>
-      <c r="Q114" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="R114" s="138" t="s">
-        <v>1096</v>
-      </c>
-      <c r="S114" s="138" t="s">
-        <v>1097</v>
-      </c>
-      <c r="T114" s="138" t="s">
-        <v>1098</v>
+      <c r="T114" s="136" t="s">
+        <v>1063</v>
       </c>
       <c r="U114" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",K114&amp;" "&amp;Q114)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K114&amp;" "&amp;Q114))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K114&amp;" "&amp;Q114)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K114&amp;" "&amp;Q114))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K114&amp;" "&amp;Q114)),ISNUMBER(SEARCH("PENDING",K114&amp;" "&amp;Q114)),ISNUMBER(SEARCH("IN PROGRESS",K114&amp;" "&amp;Q114)),ISNUMBER(SEARCH("OPEN",K114&amp;" "&amp;Q114)),ISNUMBER(SEARCH("RETEST REQUIRED",K114&amp;" "&amp;Q114)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K114&amp;" "&amp;Q114)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K114&amp;" "&amp;Q114))),"Pending",IF(OR(Q114="PASS",ISNUMBER(SEARCH("PASS",K114&amp;" "&amp;Q114))),"Done","Pending"))))</f>
-        <v>Not started</v>
+        <v>Pending</v>
       </c>
       <c r="V114" s="146">
         <f>IF(T114="","",VALUE(LEFT(T114,SEARCH("/",T114)-1)))</f>
-        <v>130</v>
+        <v>60</v>
       </c>
       <c r="W114" s="146">
         <f>IF(T114="","",VALUE(MID(T114,SEARCH("/",T114)+1,LEN(T114))))</f>
-        <v>310</v>
+        <v>145</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="138" t="s">
-        <v>1099</v>
+        <v>1096</v>
       </c>
       <c r="B115" s="138" t="s">
         <v>155</v>
       </c>
-      <c r="C115" s="243" t="s">
-        <v>49</v>
+      <c r="C115" s="263" t="s">
+        <v>43</v>
       </c>
       <c r="D115" s="138" t="s">
+        <v>1097</v>
+      </c>
+      <c r="E115" s="138" t="s">
+        <v>1098</v>
+      </c>
+      <c r="F115" s="138" t="s">
+        <v>1099</v>
+      </c>
+      <c r="G115" s="138" t="s">
         <v>1100</v>
       </c>
-      <c r="E115" s="138" t="s">
+      <c r="H115" s="138" t="s">
         <v>1101</v>
       </c>
-      <c r="F115" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="G115" s="138" t="s">
+      <c r="I115" s="138" t="s">
         <v>1102</v>
       </c>
-      <c r="H115" s="138" t="s">
-        <v>4</v>
-      </c>
-      <c r="I115" s="138" t="s">
+      <c r="J115" s="138" t="s">
         <v>1103</v>
       </c>
-      <c r="J115" s="138" t="s">
+      <c r="K115" s="138" t="s">
+        <v>999</v>
+      </c>
+      <c r="L115" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="M115" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="N115" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O115" s="138" t="s">
         <v>1104</v>
       </c>
-      <c r="K115" s="138" t="s">
-        <v>988</v>
-      </c>
-      <c r="L115" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="M115" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="N115" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O115" s="138" t="s">
+      <c r="P115" s="138" t="s">
         <v>1105</v>
       </c>
-      <c r="P115" s="138" t="s">
+      <c r="Q115" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="R115" s="138" t="s">
         <v>1106</v>
       </c>
-      <c r="Q115" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="R115" s="138" t="s">
+      <c r="S115" s="138" t="s">
         <v>1107</v>
       </c>
-      <c r="S115" s="138" t="s">
-        <v>88</v>
-      </c>
       <c r="T115" s="138" t="s">
-        <v>1085</v>
+        <v>1108</v>
       </c>
       <c r="U115" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K115&amp;" "&amp;Q115))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K115&amp;" "&amp;Q115))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("PENDING",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("IN PROGRESS",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("OPEN",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("RETEST REQUIRED",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K115&amp;" "&amp;Q115))),"Pending",IF(OR(Q115="PASS",ISNUMBER(SEARCH("PASS",K115&amp;" "&amp;Q115))),"Done","Pending"))))</f>
@@ -13926,16 +13956,16 @@
       </c>
       <c r="V115" s="146">
         <f>IF(T115="","",VALUE(LEFT(T115,SEARCH("/",T115)-1)))</f>
-        <v>60</v>
+        <v>130</v>
       </c>
       <c r="W115" s="146">
         <f>IF(T115="","",VALUE(MID(T115,SEARCH("/",T115)+1,LEN(T115))))</f>
-        <v>145</v>
+        <v>310</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="138" t="s">
-        <v>1108</v>
+        <v>1109</v>
       </c>
       <c r="B116" s="138" t="s">
         <v>155</v>
@@ -13944,55 +13974,55 @@
         <v>49</v>
       </c>
       <c r="D116" s="138" t="s">
-        <v>1109</v>
+        <v>1110</v>
       </c>
       <c r="E116" s="138" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="F116" s="138" t="s">
-        <v>1111</v>
+        <v>4</v>
       </c>
       <c r="G116" s="138" t="s">
         <v>1112</v>
       </c>
       <c r="H116" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="I116" s="138" t="s">
         <v>1113</v>
       </c>
-      <c r="I116" s="138" t="s">
+      <c r="J116" s="138" t="s">
         <v>1114</v>
       </c>
-      <c r="J116" s="138" t="s">
+      <c r="K116" s="138" t="s">
+        <v>999</v>
+      </c>
+      <c r="L116" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="M116" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="N116" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O116" s="138" t="s">
         <v>1115</v>
       </c>
-      <c r="K116" s="138" t="s">
-        <v>988</v>
-      </c>
-      <c r="L116" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="M116" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="N116" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O116" s="138" t="s">
+      <c r="P116" s="138" t="s">
         <v>1116</v>
       </c>
-      <c r="P116" s="138" t="s">
+      <c r="Q116" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="R116" s="138" t="s">
         <v>1117</v>
-      </c>
-      <c r="Q116" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="R116" s="138" t="s">
-        <v>1118</v>
       </c>
       <c r="S116" s="138" t="s">
         <v>88</v>
       </c>
       <c r="T116" s="138" t="s">
-        <v>1072</v>
+        <v>1063</v>
       </c>
       <c r="U116" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K116&amp;" "&amp;Q116))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K116&amp;" "&amp;Q116))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("PENDING",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("IN PROGRESS",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("OPEN",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("RETEST REQUIRED",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K116&amp;" "&amp;Q116))),"Pending",IF(OR(Q116="PASS",ISNUMBER(SEARCH("PASS",K116&amp;" "&amp;Q116))),"Done","Pending"))))</f>
@@ -14000,16 +14030,16 @@
       </c>
       <c r="V116" s="146">
         <f>IF(T116="","",VALUE(LEFT(T116,SEARCH("/",T116)-1)))</f>
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="W116" s="146">
         <f>IF(T116="","",VALUE(MID(T116,SEARCH("/",T116)+1,LEN(T116))))</f>
-        <v>180</v>
+        <v>145</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="138" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="B117" s="138" t="s">
         <v>155</v>
@@ -14018,28 +14048,28 @@
         <v>49</v>
       </c>
       <c r="D117" s="138" t="s">
+        <v>1119</v>
+      </c>
+      <c r="E117" s="138" t="s">
         <v>1120</v>
       </c>
-      <c r="E117" s="138" t="s">
+      <c r="F117" s="138" t="s">
         <v>1121</v>
-      </c>
-      <c r="F117" s="138" t="s">
-        <v>4</v>
       </c>
       <c r="G117" s="138" t="s">
         <v>1122</v>
       </c>
       <c r="H117" s="138" t="s">
-        <v>4</v>
+        <v>1123</v>
       </c>
       <c r="I117" s="138" t="s">
-        <v>1123</v>
+        <v>1124</v>
       </c>
       <c r="J117" s="138" t="s">
-        <v>1124</v>
+        <v>1125</v>
       </c>
       <c r="K117" s="138" t="s">
-        <v>988</v>
+        <v>999</v>
       </c>
       <c r="L117" s="138" t="s">
         <v>1</v>
@@ -14051,22 +14081,22 @@
         <v>1</v>
       </c>
       <c r="O117" s="138" t="s">
-        <v>1125</v>
+        <v>1126</v>
       </c>
       <c r="P117" s="138" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="Q117" s="138" t="s">
         <v>1</v>
       </c>
       <c r="R117" s="138" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="S117" s="138" t="s">
-        <v>111</v>
+        <v>88</v>
       </c>
       <c r="T117" s="138" t="s">
-        <v>1128</v>
+        <v>1083</v>
       </c>
       <c r="U117" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",K117&amp;" "&amp;Q117)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K117&amp;" "&amp;Q117))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K117&amp;" "&amp;Q117)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K117&amp;" "&amp;Q117))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K117&amp;" "&amp;Q117)),ISNUMBER(SEARCH("PENDING",K117&amp;" "&amp;Q117)),ISNUMBER(SEARCH("IN PROGRESS",K117&amp;" "&amp;Q117)),ISNUMBER(SEARCH("OPEN",K117&amp;" "&amp;Q117)),ISNUMBER(SEARCH("RETEST REQUIRED",K117&amp;" "&amp;Q117)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K117&amp;" "&amp;Q117)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K117&amp;" "&amp;Q117))),"Pending",IF(OR(Q117="PASS",ISNUMBER(SEARCH("PASS",K117&amp;" "&amp;Q117))),"Done","Pending"))))</f>
@@ -14074,11 +14104,11 @@
       </c>
       <c r="V117" s="146">
         <f>IF(T117="","",VALUE(LEFT(T117,SEARCH("/",T117)-1)))</f>
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="W117" s="146">
         <f>IF(T117="","",VALUE(MID(T117,SEARCH("/",T117)+1,LEN(T117))))</f>
-        <v>80</v>
+        <v>180</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14098,49 +14128,49 @@
         <v>1131</v>
       </c>
       <c r="F118" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="G118" s="138" t="s">
         <v>1132</v>
-      </c>
-      <c r="G118" s="138" t="s">
-        <v>1133</v>
       </c>
       <c r="H118" s="138" t="s">
         <v>4</v>
       </c>
       <c r="I118" s="138" t="s">
+        <v>1133</v>
+      </c>
+      <c r="J118" s="138" t="s">
         <v>1134</v>
       </c>
-      <c r="J118" s="138" t="s">
+      <c r="K118" s="138" t="s">
+        <v>999</v>
+      </c>
+      <c r="L118" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="M118" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="N118" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O118" s="138" t="s">
         <v>1135</v>
       </c>
-      <c r="K118" s="138" t="s">
-        <v>988</v>
-      </c>
-      <c r="L118" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="M118" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="N118" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="O118" s="138" t="s">
+      <c r="P118" s="138" t="s">
         <v>1136</v>
       </c>
-      <c r="P118" s="138" t="s">
+      <c r="Q118" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="R118" s="138" t="s">
         <v>1137</v>
       </c>
-      <c r="Q118" s="138" t="s">
-        <v>1</v>
-      </c>
-      <c r="R118" s="138" t="s">
+      <c r="S118" s="138" t="s">
+        <v>111</v>
+      </c>
+      <c r="T118" s="138" t="s">
         <v>1138</v>
-      </c>
-      <c r="S118" s="138" t="s">
-        <v>980</v>
-      </c>
-      <c r="T118" s="138" t="s">
-        <v>1128</v>
       </c>
       <c r="U118" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",K118&amp;" "&amp;Q118)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K118&amp;" "&amp;Q118))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K118&amp;" "&amp;Q118)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K118&amp;" "&amp;Q118))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K118&amp;" "&amp;Q118)),ISNUMBER(SEARCH("PENDING",K118&amp;" "&amp;Q118)),ISNUMBER(SEARCH("IN PROGRESS",K118&amp;" "&amp;Q118)),ISNUMBER(SEARCH("OPEN",K118&amp;" "&amp;Q118)),ISNUMBER(SEARCH("RETEST REQUIRED",K118&amp;" "&amp;Q118)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K118&amp;" "&amp;Q118)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K118&amp;" "&amp;Q118))),"Pending",IF(OR(Q118="PASS",ISNUMBER(SEARCH("PASS",K118&amp;" "&amp;Q118))),"Done","Pending"))))</f>
@@ -14152,6 +14182,80 @@
       </c>
       <c r="W118" s="146">
         <f>IF(T118="","",VALUE(MID(T118,SEARCH("/",T118)+1,LEN(T118))))</f>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="138" t="s">
+        <v>1139</v>
+      </c>
+      <c r="B119" s="138" t="s">
+        <v>155</v>
+      </c>
+      <c r="C119" s="243" t="s">
+        <v>49</v>
+      </c>
+      <c r="D119" s="138" t="s">
+        <v>1140</v>
+      </c>
+      <c r="E119" s="138" t="s">
+        <v>1141</v>
+      </c>
+      <c r="F119" s="138" t="s">
+        <v>1142</v>
+      </c>
+      <c r="G119" s="138" t="s">
+        <v>1143</v>
+      </c>
+      <c r="H119" s="138" t="s">
+        <v>4</v>
+      </c>
+      <c r="I119" s="138" t="s">
+        <v>1144</v>
+      </c>
+      <c r="J119" s="138" t="s">
+        <v>1145</v>
+      </c>
+      <c r="K119" s="138" t="s">
+        <v>999</v>
+      </c>
+      <c r="L119" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="M119" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="N119" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="O119" s="138" t="s">
+        <v>1146</v>
+      </c>
+      <c r="P119" s="138" t="s">
+        <v>1147</v>
+      </c>
+      <c r="Q119" s="138" t="s">
+        <v>1</v>
+      </c>
+      <c r="R119" s="138" t="s">
+        <v>1148</v>
+      </c>
+      <c r="S119" s="138" t="s">
+        <v>991</v>
+      </c>
+      <c r="T119" s="138" t="s">
+        <v>1138</v>
+      </c>
+      <c r="U119" s="146" t="str">
+        <f>IF(OR(ISNUMBER(SEARCH("FAIL",K119&amp;" "&amp;Q119)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K119&amp;" "&amp;Q119))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K119&amp;" "&amp;Q119)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K119&amp;" "&amp;Q119))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K119&amp;" "&amp;Q119)),ISNUMBER(SEARCH("PENDING",K119&amp;" "&amp;Q119)),ISNUMBER(SEARCH("IN PROGRESS",K119&amp;" "&amp;Q119)),ISNUMBER(SEARCH("OPEN",K119&amp;" "&amp;Q119)),ISNUMBER(SEARCH("RETEST REQUIRED",K119&amp;" "&amp;Q119)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K119&amp;" "&amp;Q119)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K119&amp;" "&amp;Q119))),"Pending",IF(OR(Q119="PASS",ISNUMBER(SEARCH("PASS",K119&amp;" "&amp;Q119))),"Done","Pending"))))</f>
+        <v>Not started</v>
+      </c>
+      <c r="V119" s="146">
+        <f>IF(T119="","",VALUE(LEFT(T119,SEARCH("/",T119)-1)))</f>
+        <v>30</v>
+      </c>
+      <c r="W119" s="146">
+        <f>IF(T119="","",VALUE(MID(T119,SEARCH("/",T119)+1,LEN(T119))))</f>
         <v>80</v>
       </c>
     </row>

</xml_diff>

<commit_message>
pair qa - webview fix
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -3420,16 +3420,16 @@
     <t>2026-09-14</t>
   </si>
   <si>
-    <t>Physical Android: coherent old/candidate upgrade; native clipboard approval and exact paste; Chrome resident resume; own Ticket/QR and empty Nova Notifications; cached Nova QR under verified transport loss and online restore. No separate build/test process run. Opt-in demo fallback: watcher-output regression checks cover identity/security gates, storage restoration, write/editor guards, cold start and account switch. Phone API-outage/local-save/repeated-outage passed; reconnect preserves the local page. API-only and network-emulated offline icons, polling recovery without reload, drag/dismiss and mute-control recovery verified. Continuation: fixture media public/negative boundary checks passed; standalone Java QA removed. Physical offline cold-start avatar, own cached Ticket/QR and reconnect without reload passed on lifecycle-3.</t>
-  </si>
-  <si>
-    <t>Complete remaining lifecycle/media branches and cleanup; analyze live member versus completed-event friendship contracts before changing read models. Real Firebase image success/revocation and Friends only image authorization unproven.</t>
+    <t>Physical Android: coherent old/candidate upgrade; native clipboard approval and exact paste; Chrome resident resume; own Ticket/QR and empty Nova Notifications; cached Nova QR under verified transport loss and online restore. No separate build/test process run. Opt-in demo fallback: watcher-output regression checks cover identity/security gates, storage restoration, write/editor guards, cold start and account switch. Phone API-outage/local-save/repeated-outage passed; reconnect preserves the local page. API-only and network-emulated offline icons, polling recovery without reload, drag/dismiss and mute-control recovery verified. Continuation: fixture media public/negative boundary checks passed; standalone Java QA removed. Physical offline cold-start avatar, own cached Ticket/QR and reconnect without reload passed on lifecycle-3. Shared setup: seven compiled workflow contract groups passed on desktop and physical PWA with native/provider doubles; 340/341 px panels, equal 224 px switches, no overflow, notification toggle both ways, location locked and Update right-aligned. Existing watcher build/sync passed.</t>
+  </si>
+  <si>
+    <t>Rerun affected ordinary frontend-local UI/reload and deployed-demo outage without URL switches; then actual Firebase entry/media/logout and Push activation/delivery. External phone page+worker transport fixture only; do not disable radios/tethering.</t>
   </si>
   <si>
     <t>PARTIAL</t>
   </si>
   <si>
-    <t>See DOMAIN_LIFECYCLE_MANUAL_QA_PACK.md, Mobile WebView physical-device execution 2026-09-14. Old 4be4a1c596e2-20260905140310 -&gt; mobile-webview-20260914-icon-fix. Initial mixed dev/old fixture caused font HTML responses; coherent old shell fixed them. Candidate Preview badge hidden offline. Riley offline Ticket/profile keys retained after ordinary logout. Chrome open list reconciled one new row, counter 2 -&gt; 3. Settings observation recreated page. Paste exact, editor width stable; notification trigger covered Remove link. Real offline Nova QR rendered; uncached Game showed misleading empty result. Native Chrome SIGTRAP captured; seamless offline cold-start not proven. Owned fixture and server session snapshot restored; original nginx route restored. No FCM test. Later authorized localhost/dev-only offline-demo trial implemented: phone HTTP Anna -&gt; local u1 passed; reconnect stays local without reload, next explicit opening prefers HTTP; saved local edit survives another outage, cancelled draft does not; Mongo confirms neither marker reached live user. Full internet-offline cold start remains unproven. See the added opt-in trial evidence. Floating cloud_off appears at zero unread, remains movable/dismissible; menu/list icons track connection and preserve mute preference. Continuation evidence supersedes the earlier cache-purge/cold-start failures: Riley logout purged private cache, Nova isolated Ticket/QR remained usable after offline cold-start; reconnect retained timeOrigin. Fixture currently staged, Nova logged in, transport online, lifecycle-3 route retained. Existing hash-based Friends only is not the clarified completed-event friendship rule; unfinished replacement removed pending member-screen analysis.</t>
+    <t>See DOMAIN_LIFECYCLE_MANUAL_QA_PACK.md, Mobile WebView physical-device execution 2026-09-14. Old 4be4a1c596e2-20260905140310 -&gt; mobile-webview-20260914-icon-fix. Initial mixed dev/old fixture caused font HTML responses; coherent old shell fixed them. Candidate Preview badge hidden offline. Riley offline Ticket/profile keys retained after ordinary logout. Chrome open list reconciled one new row, counter 2 -&gt; 3. Settings observation recreated page. Paste exact, editor width stable; notification trigger covered Remove link. Real offline Nova QR rendered; uncached Game showed misleading empty result. Native Chrome SIGTRAP captured; seamless offline cold-start not proven. Owned fixture and server session snapshot restored; original nginx route restored. No FCM test. Later authorized localhost/dev-only offline-demo trial implemented: phone HTTP Anna -&gt; local u1 passed; reconnect stays local without reload, next explicit opening prefers HTTP; saved local edit survives another outage, cancelled draft does not; Mongo confirms neither marker reached live user. Full internet-offline cold start remains unproven. See the added opt-in trial evidence. Floating cloud_off appears at zero unread, remains movable/dismissible; menu/list icons track connection and preserve mute preference. Continuation evidence supersedes the earlier cache-purge/cold-start failures: Riley logout purged private cache, Nova isolated Ticket/QR remained usable after offline cold-start; reconnect retained timeOrigin. Fixture currently staged, Nova logged in, transport online, lifecycle-3 route retained. Existing hash-based Friends only is not the clarified completed-event friendship rule; unfinished replacement removed pending member-screen analysis. Latest continuation supersedes stale friendship and actor notes: real completed-event/media policy proof is in the QA pack; Riley phone and Casey managed desktop remain staged, Nova logged out. lifecycle-16 build mobile-webview-lifecycle-1789393814593, shared-setup screenshots/results retained. No real FCM activation/delivery or external Firebase entry proof; PARTIAL remains. 2026-09-14 correction: application query/storage test switches removed; six local device persistence checks and seven popup contracts on desktop/phone passed; external page+worker outage and same-page reconnect passed lifecycle-17. Extra offline labels removed; latest candidate lifecycle-19. Full local UI and real provider tests remain open.</t>
   </si>
   <si>
     <t>110/260</t>

</xml_diff>

<commit_message>
[MSC-100] Qualify community group membership and profile switching
Consolidate group mapping, membership notifications,
profile/location/counter services and fixtures, with the recorded lifecycle
QA evidence.

Original-snapshot: 04f4f056ccdea44206c8642c07139f6eafa5e525

Tasks: fssrepository/myscoutee-roadmap#100
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2680" uniqueCount="1281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2680" uniqueCount="1284">
   <si>
     <t>EFFECT / SCOPE MARKERS</t>
   </si>
@@ -421,10 +421,10 @@
     <t>15 focused backend tests PASS (2026-09-24): filter defaults/preservation and shared invitation claim plus community admission/replay. Does not prove this full UI/HTTP journey. Profile selection correction: 21 focused Java tests PASS (2026-09-25); profile-load parameter, read-only restore, accepted-membership authority, failed-load non-commit, invite activation and removal. Added frontend HTTP parameter/retry unit cases; not executed separately from the running build watcher.</t>
   </si>
   <si>
-    <t>Prepare/verify versioned fixture baseline and managed launcher, then execute the stable checklist; record local/HTTP evidence separately. | NOT RUN additions: API and UI external invitation URLs preserve affiliate attribution through registration and target participation; per-participant API claim versus reusable UI link; repeat/existing-user attribution; group active workspace; event admission gates; cash exclusion from affiliate totals. See Affiliate and external-link additions in the existing checklist.</t>
-  </si>
-  <si>
-    <t>guides/qa/checklists/integration/INTEGRATION-API-GROUP-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=5/4/4/4/4; effort actions/extra actors/oracles/boundaries/restore/external=26/2/4/3/1/1. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed.</t>
+    <t>Prepare/verify versioned fixture baseline and managed launcher, then execute the stable checklist; record local/HTTP evidence separately. | NOT RUN additions: API and UI external invitation URLs preserve affiliate attribution through registration and target participation; per-participant API claim versus reusable UI link; repeat/existing-user attribution; group active workspace; event admission gates; cash exclusion from affiliate totals. See Affiliate and external-link additions in the existing checklist. | Block 7: MCP discovery, API authority, anonymous shared help, client packages/logo and remote connections. These unexecuted micros moved from closed INTEGRATION-API-001; no inherited PASS.</t>
+  </si>
+  <si>
+    <t>guides/qa/checklists/integration/INTEGRATION-API-GROUP-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=5/4/4/4/4; effort actions/extra actors/oracles/boundaries/restore/external=26/2/4/3/1/1. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | NOT RUN blocks 2-3: fresh registration versus existing pre-registered demo recipient; real entry UI, cancelled/retried Setup retains invitation, first active-group load and reload/login. No session injection to skip entry gates.</t>
   </si>
   <si>
     <t>P0 85</t>
@@ -3540,34 +3540,43 @@
     <t>DELTA community membership, workspace profile and stored policy; accepted/pending lists and counters match canonical records.</t>
   </si>
   <si>
+    <t>IN PROGRESS</t>
+  </si>
+  <si>
+    <t>2026-09-26</t>
+  </si>
+  <si>
+    <t>31 focused backend moderation/chat/counter tests PASS (2026-09-25): separate scope settings, authority/foreign IDs, persisted pending count and idempotence, worker, Group support access/filter/unread. Earlier 15 filter/invitation tests PASS (2026-09-24). Frontend/backend dev watchers compiled. Full local/UI/HTTP journey NOT RUN. Profile selection correction: 21 focused Java tests PASS (2026-09-25); profile-load parameter, read-only restore, accepted-membership authority, failed-load non-commit, invite activation and removal. Added frontend HTTP parameter/retry unit cases; not executed separately from the running build watcher. | 2026-09-26: 105 focused backend tests PASS and 47 frontend tests PASS, covering explore boundaries, Base-only asset API key, contact repository account resolution and ticket account aggregation. These unit results do not close the manual local/HTTP journey. | My Tools follow-up (2026-09-26): 40 focused frontend tests PASS; 1 backend stored menu-counter test PASS. Account ownership/store/counters and stale-poll checks covered; browser journey NOT RUN. | Scope follow-up (2026-09-26): 195 backend and 32 frontend focused tests PASS. Payment payer/recipient query identity, account contacts, group event authorization and ticket scanner covered; manual local/HTTP journey NOT RUN. | Overlay navigation (2026-09-26): 27 focused frontend tests PASS; no real-device/Router/Firebase journey claimed. MCP Go race tests and image 1.3.0 initialization/discovery PASS; six generated schemas match OpenAPI. Help source parity PASS. | 2026-09-26: 13 focused frontend checks passed: popup/category/distance (5), local membership/notification lifecycle (5), workspace scopes and stale polls (3). Existing dev watchers compiled frontend/backend; added Java regression cases not run. No full-flow PASS.</t>
+  </si>
+  <si>
+    <t>HTTP block 6 to completion; 5/29 HTTP blocks closed, Local 0/29. Then HTTP 7–29, Local 1–29. Preserve live isolated moderation fixture; no restart for restructuring.</t>
+  </si>
+  <si>
+    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.</t>
+  </si>
+  <si>
+    <t>180/420</t>
+  </si>
+  <si>
+    <t>GROUP-ISOLATION-001</t>
+  </si>
+  <si>
+    <t>Workspace privacy and domain samples</t>
+  </si>
+  <si>
+    <t>Compare Base, Group A and Group B using Asset and Event membership/chat samples plus home ratings/filters, Feed/Following, delayed responses, revoked access, scoped moderation settings/counts/previews/decisions, Group support privacy and intentionally aggregated notifications.; direct-chat consent Requests/Contacts buckets and live pending-only badge</t>
+  </si>
+  <si>
+    <t>DELTA only the owning workspace; no cross-workspace private detail/write, relationship, card exclusion or counter leak. Group-admin moderation is scoped to its group.</t>
+  </si>
+  <si>
     <t>31 focused backend moderation/chat/counter tests PASS (2026-09-25): separate scope settings, authority/foreign IDs, persisted pending count and idempotence, worker, Group support access/filter/unread. Earlier 15 filter/invitation tests PASS (2026-09-24). Frontend/backend dev watchers compiled. Full local/UI/HTTP journey NOT RUN. Profile selection correction: 21 focused Java tests PASS (2026-09-25); profile-load parameter, read-only restore, accepted-membership authority, failed-load non-commit, invite activation and removal. Added frontend HTTP parameter/retry unit cases; not executed separately from the running build watcher.</t>
   </si>
   <si>
-    <t>Prepare/verify versioned fixture baseline and managed launcher, then execute the stable checklist; record local/HTTP evidence separately. | NOT RUN additions: external-link popup with Profile Affiliate copy look and feel; one share menu/no legacy raw-token dialog; mixed basket additions/removals in one confirmation; separate message per item; old-page deletion; partial retry and stale replies; cash receipt/member/note/notification/no commission; contacts/direct chat/filter/member picker. See the 12 numbered sharing-batch microchecks in the existing checklist. Contact-chat invite: only the inviting actor’s saved contacts, excluding existing members; empty stays empty. Reject non-contact / foreign-workspace / support-channel add-member commands. Verify own-store update and recipients’ contact chat unread/read counters. Existing chat popup stacks above the still-open contact list; closing restores its search/window. Member and share pickers stay above the chat; returned members update SmartList without reopening or reloading.</t>
-  </si>
-  <si>
-    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed.</t>
-  </si>
-  <si>
-    <t>180/420</t>
-  </si>
-  <si>
-    <t>GROUP-ISOLATION-001</t>
-  </si>
-  <si>
-    <t>Workspace privacy and domain samples</t>
-  </si>
-  <si>
-    <t>Compare Base, Group A and Group B using Asset and Event membership/chat samples plus home ratings/filters, Feed/Following, delayed responses, revoked access, scoped moderation settings/counts/previews/decisions, Group support privacy and intentionally aggregated notifications.</t>
-  </si>
-  <si>
-    <t>DELTA only the owning workspace; no cross-workspace private detail/write, relationship, card exclusion or counter leak. Group-admin moderation is scoped to its group.</t>
-  </si>
-  <si>
     <t>Prepare/verify versioned fixture baseline and managed launcher, then execute the stable checklist; record local/HTTP evidence separately. | NOT RUN additions beyond the new feature batch: re-test existing eventless App support and Group support chats, persisted participants/header member popup, two-way messages/unread/filter, cross-workspace access, old messages and late-response isolation. Compare new contact chats separately; preserve support authority. Contact-chat invite: only the inviting actor’s saved contacts, excluding existing members; empty stays empty. Reject non-contact / foreign-workspace / support-channel add-member commands. Verify own-store update and recipients’ contact chat unread/read counters.</t>
   </si>
   <si>
-    <t>guides/qa/checklists/group/GROUP-ISOLATION-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=5/5/4/4/5; effort actions/extra actors/oracles/boundaries/restore/external=40/2/5/5/1/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed.</t>
+    <t>guides/qa/checklists/group/GROUP-ISOLATION-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=5/5/4/4/5; effort actions/extra actors/oracles/boundaries/restore/external=40/2/5/5/1/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed.; 2026-09-26 NOT RUN micros: separate direct-chat request/approve/reject; recipient-only notifications; approval saves public contact; write-side pending counter vs saved-contact count; search-row icon+label menu on mobile; SmartList live remove/insert; blurred confirmation; retry, stale version and workspace isolation. See existing GROUP-ISOLATION-001 checklist.</t>
   </si>
   <si>
     <t>165/395</t>
@@ -14340,34 +14349,34 @@
         <v>1088</v>
       </c>
       <c r="K115" s="138" t="s">
-        <v>130</v>
+        <v>1089</v>
       </c>
       <c r="L115" s="138" t="s">
-        <v>96</v>
+        <v>1089</v>
       </c>
       <c r="M115" s="138" t="s">
         <v>96</v>
       </c>
       <c r="N115" s="138" t="s">
-        <v>1</v>
+        <v>1090</v>
       </c>
       <c r="O115" s="138" t="s">
-        <v>1089</v>
+        <v>1091</v>
       </c>
       <c r="P115" s="138" t="s">
-        <v>1090</v>
+        <v>1092</v>
       </c>
       <c r="Q115" s="138" t="s">
         <v>96</v>
       </c>
       <c r="R115" s="138" t="s">
-        <v>1091</v>
+        <v>1093</v>
       </c>
       <c r="S115" s="138" t="s">
         <v>459</v>
       </c>
       <c r="T115" s="138" t="s">
-        <v>1092</v>
+        <v>1094</v>
       </c>
       <c r="U115" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K115&amp;" "&amp;Q115))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K115&amp;" "&amp;Q115))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("PENDING",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("IN PROGRESS",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("OPEN",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("RETEST REQUIRED",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K115&amp;" "&amp;Q115))),"Pending",IF(OR(Q115="PASS",ISNUMBER(SEARCH("PASS",K115&amp;" "&amp;Q115))),"Done","Pending"))))</f>
@@ -14384,7 +14393,7 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="138" t="s">
-        <v>1093</v>
+        <v>1095</v>
       </c>
       <c r="B116" s="138" t="s">
         <v>122</v>
@@ -14393,10 +14402,10 @@
         <v>32</v>
       </c>
       <c r="D116" s="138" t="s">
-        <v>1094</v>
+        <v>1096</v>
       </c>
       <c r="E116" s="138" t="s">
-        <v>1095</v>
+        <v>1097</v>
       </c>
       <c r="F116" s="138" t="s">
         <v>125</v>
@@ -14411,7 +14420,7 @@
         <v>128</v>
       </c>
       <c r="J116" s="138" t="s">
-        <v>1096</v>
+        <v>1098</v>
       </c>
       <c r="K116" s="138" t="s">
         <v>130</v>
@@ -14426,22 +14435,22 @@
         <v>1</v>
       </c>
       <c r="O116" s="138" t="s">
-        <v>1089</v>
+        <v>1099</v>
       </c>
       <c r="P116" s="138" t="s">
-        <v>1097</v>
+        <v>1100</v>
       </c>
       <c r="Q116" s="138" t="s">
         <v>96</v>
       </c>
       <c r="R116" s="138" t="s">
-        <v>1098</v>
+        <v>1101</v>
       </c>
       <c r="S116" s="138" t="s">
         <v>420</v>
       </c>
       <c r="T116" s="138" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="U116" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K116&amp;" "&amp;Q116))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K116&amp;" "&amp;Q116))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("PENDING",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("IN PROGRESS",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("OPEN",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("RETEST REQUIRED",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K116&amp;" "&amp;Q116))),"Pending",IF(OR(Q116="PASS",ISNUMBER(SEARCH("PASS",K116&amp;" "&amp;Q116))),"Done","Pending"))))</f>
@@ -14458,7 +14467,7 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="135" t="s">
-        <v>1100</v>
+        <v>1103</v>
       </c>
       <c r="B117" s="135" t="s">
         <v>284</v>
@@ -14467,10 +14476,10 @@
         <v>38</v>
       </c>
       <c r="D117" s="135" t="s">
-        <v>1101</v>
+        <v>1104</v>
       </c>
       <c r="E117" s="135" t="s">
-        <v>1102</v>
+        <v>1105</v>
       </c>
       <c r="F117" s="135" t="s">
         <v>4</v>
@@ -14485,7 +14494,7 @@
         <v>4</v>
       </c>
       <c r="J117" s="135" t="s">
-        <v>1103</v>
+        <v>1106</v>
       </c>
       <c r="K117" s="135" t="s">
         <v>806</v>
@@ -14500,16 +14509,16 @@
         <v>526</v>
       </c>
       <c r="O117" s="135" t="s">
-        <v>1104</v>
+        <v>1107</v>
       </c>
       <c r="P117" s="135" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="Q117" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R117" s="135" t="s">
-        <v>1106</v>
+        <v>1109</v>
       </c>
       <c r="S117" s="135" t="s">
         <v>352</v>
@@ -14532,7 +14541,7 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="135" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="B118" s="135" t="s">
         <v>284</v>
@@ -14541,10 +14550,10 @@
         <v>38</v>
       </c>
       <c r="D118" s="135" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="E118" s="135" t="s">
-        <v>1109</v>
+        <v>1112</v>
       </c>
       <c r="F118" s="135" t="s">
         <v>4</v>
@@ -14559,7 +14568,7 @@
         <v>4</v>
       </c>
       <c r="J118" s="135" t="s">
-        <v>1110</v>
+        <v>1113</v>
       </c>
       <c r="K118" s="135" t="s">
         <v>806</v>
@@ -14574,16 +14583,16 @@
         <v>526</v>
       </c>
       <c r="O118" s="135" t="s">
-        <v>1111</v>
+        <v>1114</v>
       </c>
       <c r="P118" s="135" t="s">
-        <v>1112</v>
+        <v>1115</v>
       </c>
       <c r="Q118" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R118" s="135" t="s">
-        <v>1113</v>
+        <v>1116</v>
       </c>
       <c r="S118" s="135" t="s">
         <v>420</v>
@@ -14606,7 +14615,7 @@
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="135" t="s">
-        <v>1114</v>
+        <v>1117</v>
       </c>
       <c r="B119" s="135" t="s">
         <v>217</v>
@@ -14615,16 +14624,16 @@
         <v>38</v>
       </c>
       <c r="D119" s="135" t="s">
-        <v>1115</v>
+        <v>1118</v>
       </c>
       <c r="E119" s="135" t="s">
-        <v>1116</v>
+        <v>1119</v>
       </c>
       <c r="F119" s="135" t="s">
-        <v>1117</v>
+        <v>1120</v>
       </c>
       <c r="G119" s="135" t="s">
-        <v>1118</v>
+        <v>1121</v>
       </c>
       <c r="H119" s="135" t="s">
         <v>4</v>
@@ -14633,7 +14642,7 @@
         <v>4</v>
       </c>
       <c r="J119" s="135" t="s">
-        <v>1119</v>
+        <v>1122</v>
       </c>
       <c r="K119" s="135" t="s">
         <v>146</v>
@@ -14648,19 +14657,19 @@
         <v>1081</v>
       </c>
       <c r="O119" s="135" t="s">
-        <v>1120</v>
+        <v>1123</v>
       </c>
       <c r="P119" s="135" t="s">
-        <v>1121</v>
+        <v>1124</v>
       </c>
       <c r="Q119" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R119" s="135" t="s">
-        <v>1122</v>
+        <v>1125</v>
       </c>
       <c r="S119" s="135" t="s">
-        <v>1123</v>
+        <v>1126</v>
       </c>
       <c r="T119" s="135" t="s">
         <v>1</v>
@@ -14680,7 +14689,7 @@
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="135" t="s">
-        <v>1124</v>
+        <v>1127</v>
       </c>
       <c r="B120" s="135" t="s">
         <v>217</v>
@@ -14689,28 +14698,28 @@
         <v>44</v>
       </c>
       <c r="D120" s="135" t="s">
-        <v>1125</v>
+        <v>1128</v>
       </c>
       <c r="E120" s="135" t="s">
-        <v>1126</v>
+        <v>1129</v>
       </c>
       <c r="F120" s="135" t="s">
-        <v>1127</v>
+        <v>1130</v>
       </c>
       <c r="G120" s="135" t="s">
-        <v>1128</v>
+        <v>1131</v>
       </c>
       <c r="H120" s="135" t="s">
         <v>4</v>
       </c>
       <c r="I120" s="135" t="s">
-        <v>1129</v>
+        <v>1132</v>
       </c>
       <c r="J120" s="135" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="K120" s="135" t="s">
-        <v>1131</v>
+        <v>1134</v>
       </c>
       <c r="L120" s="135" t="s">
         <v>1</v>
@@ -14719,19 +14728,19 @@
         <v>1</v>
       </c>
       <c r="N120" s="135" t="s">
-        <v>1132</v>
+        <v>1135</v>
       </c>
       <c r="O120" s="135" t="s">
-        <v>1133</v>
+        <v>1136</v>
       </c>
       <c r="P120" s="135" t="s">
-        <v>1134</v>
+        <v>1137</v>
       </c>
       <c r="Q120" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R120" s="135" t="s">
-        <v>1135</v>
+        <v>1138</v>
       </c>
       <c r="S120" s="135" t="s">
         <v>173</v>
@@ -14754,7 +14763,7 @@
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="135" t="s">
-        <v>1136</v>
+        <v>1139</v>
       </c>
       <c r="B121" s="135" t="s">
         <v>217</v>
@@ -14763,25 +14772,25 @@
         <v>44</v>
       </c>
       <c r="D121" s="135" t="s">
-        <v>1137</v>
+        <v>1140</v>
       </c>
       <c r="E121" s="135" t="s">
-        <v>1138</v>
+        <v>1141</v>
       </c>
       <c r="F121" s="135" t="s">
-        <v>1139</v>
+        <v>1142</v>
       </c>
       <c r="G121" s="135" t="s">
-        <v>1140</v>
+        <v>1143</v>
       </c>
       <c r="H121" s="135" t="s">
-        <v>1141</v>
+        <v>1144</v>
       </c>
       <c r="I121" s="135" t="s">
-        <v>1142</v>
+        <v>1145</v>
       </c>
       <c r="J121" s="135" t="s">
-        <v>1143</v>
+        <v>1146</v>
       </c>
       <c r="K121" s="135" t="s">
         <v>85</v>
@@ -14793,19 +14802,19 @@
         <v>1</v>
       </c>
       <c r="N121" s="135" t="s">
-        <v>1132</v>
+        <v>1135</v>
       </c>
       <c r="O121" s="135" t="s">
-        <v>1144</v>
+        <v>1147</v>
       </c>
       <c r="P121" s="135" t="s">
-        <v>1145</v>
+        <v>1148</v>
       </c>
       <c r="Q121" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R121" s="135" t="s">
-        <v>1146</v>
+        <v>1149</v>
       </c>
       <c r="S121" s="135" t="s">
         <v>364</v>
@@ -14828,7 +14837,7 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="135" t="s">
-        <v>1147</v>
+        <v>1150</v>
       </c>
       <c r="B122" s="135" t="s">
         <v>231</v>
@@ -14837,16 +14846,16 @@
         <v>44</v>
       </c>
       <c r="D122" s="135" t="s">
-        <v>1148</v>
+        <v>1151</v>
       </c>
       <c r="E122" s="135" t="s">
-        <v>1149</v>
+        <v>1152</v>
       </c>
       <c r="F122" s="135" t="s">
         <v>4</v>
       </c>
       <c r="G122" s="135" t="s">
-        <v>1150</v>
+        <v>1153</v>
       </c>
       <c r="H122" s="135" t="s">
         <v>4</v>
@@ -14855,7 +14864,7 @@
         <v>8</v>
       </c>
       <c r="J122" s="135" t="s">
-        <v>1151</v>
+        <v>1154</v>
       </c>
       <c r="K122" s="135" t="s">
         <v>85</v>
@@ -14867,19 +14876,19 @@
         <v>1</v>
       </c>
       <c r="N122" s="135" t="s">
-        <v>1132</v>
+        <v>1135</v>
       </c>
       <c r="O122" s="135" t="s">
-        <v>1152</v>
+        <v>1155</v>
       </c>
       <c r="P122" s="135" t="s">
-        <v>1153</v>
+        <v>1156</v>
       </c>
       <c r="Q122" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R122" s="135" t="s">
-        <v>1154</v>
+        <v>1157</v>
       </c>
       <c r="S122" s="135" t="s">
         <v>120</v>
@@ -14902,7 +14911,7 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="135" t="s">
-        <v>1155</v>
+        <v>1158</v>
       </c>
       <c r="B123" s="135" t="s">
         <v>217</v>
@@ -14911,25 +14920,25 @@
         <v>44</v>
       </c>
       <c r="D123" s="135" t="s">
-        <v>1156</v>
+        <v>1159</v>
       </c>
       <c r="E123" s="135" t="s">
-        <v>1157</v>
+        <v>1160</v>
       </c>
       <c r="F123" s="135" t="s">
-        <v>1158</v>
+        <v>1161</v>
       </c>
       <c r="G123" s="135" t="s">
-        <v>1159</v>
+        <v>1162</v>
       </c>
       <c r="H123" s="135" t="s">
         <v>4</v>
       </c>
       <c r="I123" s="135" t="s">
-        <v>1160</v>
+        <v>1163</v>
       </c>
       <c r="J123" s="135" t="s">
-        <v>1161</v>
+        <v>1164</v>
       </c>
       <c r="K123" s="135" t="s">
         <v>85</v>
@@ -14941,19 +14950,19 @@
         <v>1</v>
       </c>
       <c r="N123" s="135" t="s">
-        <v>1132</v>
+        <v>1135</v>
       </c>
       <c r="O123" s="135" t="s">
-        <v>1162</v>
+        <v>1165</v>
       </c>
       <c r="P123" s="135" t="s">
-        <v>1163</v>
+        <v>1166</v>
       </c>
       <c r="Q123" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R123" s="135" t="s">
-        <v>1164</v>
+        <v>1167</v>
       </c>
       <c r="S123" s="135" t="s">
         <v>431</v>
@@ -14976,7 +14985,7 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="135" t="s">
-        <v>1165</v>
+        <v>1168</v>
       </c>
       <c r="B124" s="135" t="s">
         <v>217</v>
@@ -14985,28 +14994,28 @@
         <v>44</v>
       </c>
       <c r="D124" s="135" t="s">
-        <v>1166</v>
+        <v>1169</v>
       </c>
       <c r="E124" s="135" t="s">
-        <v>1167</v>
+        <v>1170</v>
       </c>
       <c r="F124" s="135" t="s">
-        <v>1168</v>
+        <v>1171</v>
       </c>
       <c r="G124" s="135" t="s">
-        <v>1169</v>
+        <v>1172</v>
       </c>
       <c r="H124" s="135" t="s">
         <v>4</v>
       </c>
       <c r="I124" s="135" t="s">
-        <v>1170</v>
+        <v>1173</v>
       </c>
       <c r="J124" s="135" t="s">
-        <v>1171</v>
+        <v>1174</v>
       </c>
       <c r="K124" s="135" t="s">
-        <v>1172</v>
+        <v>1175</v>
       </c>
       <c r="L124" s="135" t="s">
         <v>1</v>
@@ -15015,19 +15024,19 @@
         <v>1</v>
       </c>
       <c r="N124" s="135" t="s">
-        <v>1132</v>
+        <v>1135</v>
       </c>
       <c r="O124" s="135" t="s">
-        <v>1173</v>
+        <v>1176</v>
       </c>
       <c r="P124" s="135" t="s">
-        <v>1174</v>
+        <v>1177</v>
       </c>
       <c r="Q124" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R124" s="135" t="s">
-        <v>1175</v>
+        <v>1178</v>
       </c>
       <c r="S124" s="135" t="s">
         <v>90</v>
@@ -15050,19 +15059,19 @@
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="135" t="s">
-        <v>1176</v>
+        <v>1179</v>
       </c>
       <c r="B125" s="135" t="s">
-        <v>1177</v>
+        <v>1180</v>
       </c>
       <c r="C125" s="255" t="s">
         <v>44</v>
       </c>
       <c r="D125" s="135" t="s">
-        <v>1178</v>
+        <v>1181</v>
       </c>
       <c r="E125" s="135" t="s">
-        <v>1179</v>
+        <v>1182</v>
       </c>
       <c r="F125" s="135" t="s">
         <v>4</v>
@@ -15074,13 +15083,13 @@
         <v>4</v>
       </c>
       <c r="I125" s="135" t="s">
-        <v>1180</v>
+        <v>1183</v>
       </c>
       <c r="J125" s="135" t="s">
-        <v>1181</v>
+        <v>1184</v>
       </c>
       <c r="K125" s="135" t="s">
-        <v>1182</v>
+        <v>1185</v>
       </c>
       <c r="L125" s="135" t="s">
         <v>1</v>
@@ -15089,22 +15098,22 @@
         <v>1</v>
       </c>
       <c r="N125" s="135" t="s">
-        <v>1183</v>
+        <v>1186</v>
       </c>
       <c r="O125" s="135" t="s">
-        <v>1184</v>
+        <v>1187</v>
       </c>
       <c r="P125" s="135" t="s">
-        <v>1185</v>
+        <v>1188</v>
       </c>
       <c r="Q125" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R125" s="135" t="s">
-        <v>1186</v>
+        <v>1189</v>
       </c>
       <c r="S125" s="135" t="s">
-        <v>1187</v>
+        <v>1190</v>
       </c>
       <c r="T125" s="135" t="s">
         <v>1</v>
@@ -15124,10 +15133,10 @@
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="135" t="s">
-        <v>1188</v>
+        <v>1191</v>
       </c>
       <c r="B126" s="135" t="s">
-        <v>1189</v>
+        <v>1192</v>
       </c>
       <c r="C126" s="263" t="s">
         <v>50</v>
@@ -15136,10 +15145,10 @@
         <v>63</v>
       </c>
       <c r="E126" s="135" t="s">
-        <v>1190</v>
+        <v>1193</v>
       </c>
       <c r="F126" s="135" t="s">
-        <v>1191</v>
+        <v>1194</v>
       </c>
       <c r="G126" s="135" t="s">
         <v>4</v>
@@ -15166,19 +15175,19 @@
         <v>293</v>
       </c>
       <c r="O126" s="135" t="s">
-        <v>1192</v>
+        <v>1195</v>
       </c>
       <c r="P126" s="135" t="s">
-        <v>1193</v>
+        <v>1196</v>
       </c>
       <c r="Q126" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R126" s="135" t="s">
-        <v>1194</v>
+        <v>1197</v>
       </c>
       <c r="S126" s="135" t="s">
-        <v>1195</v>
+        <v>1198</v>
       </c>
       <c r="T126" s="135" t="s">
         <v>1</v>
@@ -15198,7 +15207,7 @@
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="135" t="s">
-        <v>1196</v>
+        <v>1199</v>
       </c>
       <c r="B127" s="135" t="s">
         <v>217</v>
@@ -15207,25 +15216,25 @@
         <v>50</v>
       </c>
       <c r="D127" s="135" t="s">
-        <v>1197</v>
+        <v>1200</v>
       </c>
       <c r="E127" s="135" t="s">
-        <v>1198</v>
+        <v>1201</v>
       </c>
       <c r="F127" s="135" t="s">
-        <v>1199</v>
+        <v>1202</v>
       </c>
       <c r="G127" s="135" t="s">
-        <v>1200</v>
+        <v>1203</v>
       </c>
       <c r="H127" s="135" t="s">
-        <v>1201</v>
+        <v>1204</v>
       </c>
       <c r="I127" s="135" t="s">
-        <v>1202</v>
+        <v>1205</v>
       </c>
       <c r="J127" s="135" t="s">
-        <v>1203</v>
+        <v>1206</v>
       </c>
       <c r="K127" s="135" t="s">
         <v>146</v>
@@ -15237,19 +15246,19 @@
         <v>1</v>
       </c>
       <c r="N127" s="135" t="s">
-        <v>1204</v>
+        <v>1207</v>
       </c>
       <c r="O127" s="135" t="s">
-        <v>1205</v>
+        <v>1208</v>
       </c>
       <c r="P127" s="135" t="s">
-        <v>1206</v>
+        <v>1209</v>
       </c>
       <c r="Q127" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R127" s="135" t="s">
-        <v>1207</v>
+        <v>1210</v>
       </c>
       <c r="S127" s="135" t="s">
         <v>352</v>
@@ -15272,7 +15281,7 @@
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="135" t="s">
-        <v>1208</v>
+        <v>1211</v>
       </c>
       <c r="B128" s="135" t="s">
         <v>217</v>
@@ -15281,25 +15290,25 @@
         <v>50</v>
       </c>
       <c r="D128" s="135" t="s">
-        <v>1209</v>
+        <v>1212</v>
       </c>
       <c r="E128" s="135" t="s">
-        <v>1210</v>
+        <v>1213</v>
       </c>
       <c r="F128" s="135" t="s">
-        <v>1211</v>
+        <v>1214</v>
       </c>
       <c r="G128" s="135" t="s">
-        <v>1212</v>
+        <v>1215</v>
       </c>
       <c r="H128" s="135" t="s">
-        <v>1213</v>
+        <v>1216</v>
       </c>
       <c r="I128" s="135" t="s">
-        <v>1214</v>
+        <v>1217</v>
       </c>
       <c r="J128" s="135" t="s">
-        <v>1215</v>
+        <v>1218</v>
       </c>
       <c r="K128" s="135" t="s">
         <v>146</v>
@@ -15311,22 +15320,22 @@
         <v>1</v>
       </c>
       <c r="N128" s="135" t="s">
-        <v>1204</v>
+        <v>1207</v>
       </c>
       <c r="O128" s="135" t="s">
-        <v>1216</v>
+        <v>1219</v>
       </c>
       <c r="P128" s="135" t="s">
-        <v>1217</v>
+        <v>1220</v>
       </c>
       <c r="Q128" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R128" s="135" t="s">
-        <v>1218</v>
+        <v>1221</v>
       </c>
       <c r="S128" s="135" t="s">
-        <v>1219</v>
+        <v>1222</v>
       </c>
       <c r="T128" s="135" t="s">
         <v>1</v>
@@ -15346,7 +15355,7 @@
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="135" t="s">
-        <v>1220</v>
+        <v>1223</v>
       </c>
       <c r="B129" s="135" t="s">
         <v>217</v>
@@ -15355,25 +15364,25 @@
         <v>50</v>
       </c>
       <c r="D129" s="135" t="s">
-        <v>1221</v>
+        <v>1224</v>
       </c>
       <c r="E129" s="135" t="s">
-        <v>1222</v>
+        <v>1225</v>
       </c>
       <c r="F129" s="135" t="s">
-        <v>1223</v>
+        <v>1226</v>
       </c>
       <c r="G129" s="135" t="s">
-        <v>1224</v>
+        <v>1227</v>
       </c>
       <c r="H129" s="135" t="s">
-        <v>1225</v>
+        <v>1228</v>
       </c>
       <c r="I129" s="135" t="s">
-        <v>1226</v>
+        <v>1229</v>
       </c>
       <c r="J129" s="135" t="s">
-        <v>1227</v>
+        <v>1230</v>
       </c>
       <c r="K129" s="135" t="s">
         <v>85</v>
@@ -15385,22 +15394,22 @@
         <v>1</v>
       </c>
       <c r="N129" s="135" t="s">
-        <v>1204</v>
+        <v>1207</v>
       </c>
       <c r="O129" s="135" t="s">
-        <v>1228</v>
+        <v>1231</v>
       </c>
       <c r="P129" s="135" t="s">
-        <v>1229</v>
+        <v>1232</v>
       </c>
       <c r="Q129" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R129" s="135" t="s">
-        <v>1230</v>
+        <v>1233</v>
       </c>
       <c r="S129" s="135" t="s">
-        <v>1231</v>
+        <v>1234</v>
       </c>
       <c r="T129" s="135" t="s">
         <v>1</v>
@@ -15420,7 +15429,7 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="135" t="s">
-        <v>1232</v>
+        <v>1235</v>
       </c>
       <c r="B130" s="135" t="s">
         <v>217</v>
@@ -15429,25 +15438,25 @@
         <v>55</v>
       </c>
       <c r="D130" s="135" t="s">
-        <v>1233</v>
+        <v>1236</v>
       </c>
       <c r="E130" s="135" t="s">
-        <v>1234</v>
+        <v>1237</v>
       </c>
       <c r="F130" s="135" t="s">
         <v>4</v>
       </c>
       <c r="G130" s="135" t="s">
-        <v>1235</v>
+        <v>1238</v>
       </c>
       <c r="H130" s="135" t="s">
         <v>4</v>
       </c>
       <c r="I130" s="135" t="s">
-        <v>1236</v>
+        <v>1239</v>
       </c>
       <c r="J130" s="135" t="s">
-        <v>1237</v>
+        <v>1240</v>
       </c>
       <c r="K130" s="135" t="s">
         <v>146</v>
@@ -15459,19 +15468,19 @@
         <v>1</v>
       </c>
       <c r="N130" s="135" t="s">
-        <v>1204</v>
+        <v>1207</v>
       </c>
       <c r="O130" s="135" t="s">
-        <v>1238</v>
+        <v>1241</v>
       </c>
       <c r="P130" s="135" t="s">
-        <v>1239</v>
+        <v>1242</v>
       </c>
       <c r="Q130" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R130" s="135" t="s">
-        <v>1240</v>
+        <v>1243</v>
       </c>
       <c r="S130" s="135" t="s">
         <v>90</v>
@@ -15494,7 +15503,7 @@
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="135" t="s">
-        <v>1241</v>
+        <v>1244</v>
       </c>
       <c r="B131" s="135" t="s">
         <v>217</v>
@@ -15503,25 +15512,25 @@
         <v>55</v>
       </c>
       <c r="D131" s="135" t="s">
-        <v>1242</v>
+        <v>1245</v>
       </c>
       <c r="E131" s="135" t="s">
-        <v>1243</v>
+        <v>1246</v>
       </c>
       <c r="F131" s="135" t="s">
-        <v>1244</v>
+        <v>1247</v>
       </c>
       <c r="G131" s="135" t="s">
-        <v>1245</v>
+        <v>1248</v>
       </c>
       <c r="H131" s="135" t="s">
-        <v>1246</v>
+        <v>1249</v>
       </c>
       <c r="I131" s="135" t="s">
-        <v>1247</v>
+        <v>1250</v>
       </c>
       <c r="J131" s="135" t="s">
-        <v>1248</v>
+        <v>1251</v>
       </c>
       <c r="K131" s="135" t="s">
         <v>85</v>
@@ -15533,19 +15542,19 @@
         <v>1</v>
       </c>
       <c r="N131" s="135" t="s">
-        <v>1204</v>
+        <v>1207</v>
       </c>
       <c r="O131" s="135" t="s">
-        <v>1249</v>
+        <v>1252</v>
       </c>
       <c r="P131" s="135" t="s">
-        <v>1250</v>
+        <v>1253</v>
       </c>
       <c r="Q131" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R131" s="135" t="s">
-        <v>1251</v>
+        <v>1254</v>
       </c>
       <c r="S131" s="135" t="s">
         <v>90</v>
@@ -15568,7 +15577,7 @@
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="135" t="s">
-        <v>1252</v>
+        <v>1255</v>
       </c>
       <c r="B132" s="135" t="s">
         <v>217</v>
@@ -15577,25 +15586,25 @@
         <v>55</v>
       </c>
       <c r="D132" s="135" t="s">
-        <v>1253</v>
+        <v>1256</v>
       </c>
       <c r="E132" s="135" t="s">
-        <v>1254</v>
+        <v>1257</v>
       </c>
       <c r="F132" s="135" t="s">
         <v>4</v>
       </c>
       <c r="G132" s="135" t="s">
-        <v>1255</v>
+        <v>1258</v>
       </c>
       <c r="H132" s="135" t="s">
         <v>4</v>
       </c>
       <c r="I132" s="135" t="s">
-        <v>1256</v>
+        <v>1259</v>
       </c>
       <c r="J132" s="135" t="s">
-        <v>1257</v>
+        <v>1260</v>
       </c>
       <c r="K132" s="135" t="s">
         <v>146</v>
@@ -15607,19 +15616,19 @@
         <v>1</v>
       </c>
       <c r="N132" s="135" t="s">
-        <v>1204</v>
+        <v>1207</v>
       </c>
       <c r="O132" s="135" t="s">
-        <v>1258</v>
+        <v>1261</v>
       </c>
       <c r="P132" s="135" t="s">
-        <v>1259</v>
+        <v>1262</v>
       </c>
       <c r="Q132" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R132" s="135" t="s">
-        <v>1260</v>
+        <v>1263</v>
       </c>
       <c r="S132" s="135" t="s">
         <v>173</v>
@@ -15642,7 +15651,7 @@
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="135" t="s">
-        <v>1261</v>
+        <v>1264</v>
       </c>
       <c r="B133" s="135" t="s">
         <v>217</v>
@@ -15651,25 +15660,25 @@
         <v>55</v>
       </c>
       <c r="D133" s="135" t="s">
-        <v>1262</v>
+        <v>1265</v>
       </c>
       <c r="E133" s="135" t="s">
-        <v>1263</v>
+        <v>1266</v>
       </c>
       <c r="F133" s="135" t="s">
-        <v>1264</v>
+        <v>1267</v>
       </c>
       <c r="G133" s="135" t="s">
-        <v>1265</v>
+        <v>1268</v>
       </c>
       <c r="H133" s="135" t="s">
         <v>4</v>
       </c>
       <c r="I133" s="135" t="s">
-        <v>1266</v>
+        <v>1269</v>
       </c>
       <c r="J133" s="135" t="s">
-        <v>1267</v>
+        <v>1270</v>
       </c>
       <c r="K133" s="135" t="s">
         <v>85</v>
@@ -15681,22 +15690,22 @@
         <v>1</v>
       </c>
       <c r="N133" s="135" t="s">
-        <v>1204</v>
+        <v>1207</v>
       </c>
       <c r="O133" s="135" t="s">
-        <v>1268</v>
+        <v>1271</v>
       </c>
       <c r="P133" s="135" t="s">
-        <v>1269</v>
+        <v>1272</v>
       </c>
       <c r="Q133" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R133" s="135" t="s">
-        <v>1270</v>
+        <v>1273</v>
       </c>
       <c r="S133" s="135" t="s">
-        <v>1123</v>
+        <v>1126</v>
       </c>
       <c r="T133" s="135" t="s">
         <v>1</v>
@@ -15716,7 +15725,7 @@
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="135" t="s">
-        <v>1271</v>
+        <v>1274</v>
       </c>
       <c r="B134" s="135" t="s">
         <v>101</v>
@@ -15725,25 +15734,25 @@
         <v>55</v>
       </c>
       <c r="D134" s="135" t="s">
-        <v>1272</v>
+        <v>1275</v>
       </c>
       <c r="E134" s="135" t="s">
-        <v>1273</v>
+        <v>1276</v>
       </c>
       <c r="F134" s="135" t="s">
         <v>4</v>
       </c>
       <c r="G134" s="135" t="s">
-        <v>1274</v>
+        <v>1277</v>
       </c>
       <c r="H134" s="135" t="s">
         <v>4</v>
       </c>
       <c r="I134" s="135" t="s">
-        <v>1275</v>
+        <v>1278</v>
       </c>
       <c r="J134" s="135" t="s">
-        <v>1276</v>
+        <v>1279</v>
       </c>
       <c r="K134" s="135" t="s">
         <v>85</v>
@@ -15758,19 +15767,19 @@
         <v>106</v>
       </c>
       <c r="O134" s="135" t="s">
-        <v>1277</v>
+        <v>1280</v>
       </c>
       <c r="P134" s="135" t="s">
-        <v>1278</v>
+        <v>1281</v>
       </c>
       <c r="Q134" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R134" s="135" t="s">
-        <v>1279</v>
+        <v>1282</v>
       </c>
       <c r="S134" s="135" t="s">
-        <v>1280</v>
+        <v>1283</v>
       </c>
       <c r="T134" s="135" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
group fix - chat
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -3298,10 +3298,10 @@
     <t>31 focused backend moderation/chat/counter tests PASS (2026-09-25): separate scope settings, authority/foreign IDs, persisted pending count and idempotence, worker, Group support access/filter/unread. Earlier 15 filter/invitation tests PASS (2026-09-24). Frontend/backend dev watchers compiled. Full local/UI/HTTP journey NOT RUN. Profile selection correction: 21 focused Java tests PASS (2026-09-25); profile-load parameter, read-only restore, accepted-membership authority, failed-load non-commit, invite activation and removal. Added frontend HTTP parameter/retry unit cases; not executed separately from the running build watcher. | 2026-09-26: 105 focused backend tests PASS and 47 frontend tests PASS, covering explore boundaries, Base-only asset API key, contact repository account resolution and ticket account aggregation. These unit results do not close the manual local/HTTP journey. | My Tools follow-up (2026-09-26): 40 focused frontend tests PASS; 1 backend stored menu-counter test PASS. Account ownership/store/counters and stale-poll checks covered; browser journey NOT RUN. | Scope follow-up (2026-09-26): 195 backend and 32 frontend focused tests PASS. Payment payer/recipient query identity, account contacts, group event authorization and ticket scanner covered; manual local/HTTP journey NOT RUN. | Overlay navigation (2026-09-26): 27 focused frontend tests PASS; no real-device/Router/Firebase journey claimed. MCP Go race tests and image 1.3.0 initialization/discovery PASS; six generated schemas match OpenAPI. Help source parity PASS. | 2026-09-26: 13 focused frontend checks passed: popup/category/distance (5), local membership/notification lifecycle (5), workspace scopes and stale polls (3). Existing dev watchers compiled frontend/backend; added Java regression cases not run. No full-flow PASS.</t>
   </si>
   <si>
-    <t>HTTP8/29 closed (8/48 Group campaign); block9 Chat sharing basket/message changes current. Local0/29, Isolation and API NOT RUN. Keep only required browser actors open.</t>
-  </si>
-  <si>
-    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7.</t>
+    <t>HTTP8/29 closed (8/48 Group campaign); block9 remaining off-page share, baseline failure, pending-context, mobile and exact cleanup. Alex/Maya only. Local NOT RUN.</t>
+  </si>
+  <si>
+    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure.</t>
   </si>
   <si>
     <t>180/420</t>

</xml_diff>

<commit_message>
group fix - payment
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -3298,10 +3298,10 @@
     <t>31 focused backend moderation/chat/counter tests PASS (2026-09-25): separate scope settings, authority/foreign IDs, persisted pending count and idempotence, worker, Group support access/filter/unread. Earlier 15 filter/invitation tests PASS (2026-09-24). Frontend/backend dev watchers compiled. Full local/UI/HTTP journey NOT RUN. Profile selection correction: 21 focused Java tests PASS (2026-09-25); profile-load parameter, read-only restore, accepted-membership authority, failed-load non-commit, invite activation and removal. Added frontend HTTP parameter/retry unit cases; not executed separately from the running build watcher. | 2026-09-26: 105 focused backend tests PASS and 47 frontend tests PASS, covering explore boundaries, Base-only asset API key, contact repository account resolution and ticket account aggregation. These unit results do not close the manual local/HTTP journey. | My Tools follow-up (2026-09-26): 40 focused frontend tests PASS; 1 backend stored menu-counter test PASS. Account ownership/store/counters and stale-poll checks covered; browser journey NOT RUN. | Scope follow-up (2026-09-26): 195 backend and 32 frontend focused tests PASS. Payment payer/recipient query identity, account contacts, group event authorization and ticket scanner covered; manual local/HTTP journey NOT RUN. | Overlay navigation (2026-09-26): 27 focused frontend tests PASS; no real-device/Router/Firebase journey claimed. MCP Go race tests and image 1.3.0 initialization/discovery PASS; six generated schemas match OpenAPI. Help source parity PASS. | 2026-09-26: 13 focused frontend checks passed: popup/category/distance (5), local membership/notification lifecycle (5), workspace scopes and stale polls (3). Existing dev watchers compiled frontend/backend; added Java regression cases not run. No full-flow PASS.</t>
   </si>
   <si>
-    <t>HTTP9/29 closed (9/48 Group campaign); block10 cash history and affiliate exclusion current. Local NOT RUN. Versioned snapshot preparation before UI.</t>
-  </si>
-  <si>
-    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS.</t>
+    <t>HTTP10/48 closed; Lifecycle10/29. Block11 Contacts and existing chat popup current. Versioned prerequisite snapshot before UI. Local NOT RUN.</t>
+  </si>
+  <si>
+    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup.</t>
   </si>
   <si>
     <t>180/420</t>

</xml_diff>

<commit_message>
group fix  - contact
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2680" uniqueCount="1284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2680" uniqueCount="1285">
   <si>
     <t>EFFECT / SCOPE MARKERS</t>
   </si>
@@ -3292,16 +3292,19 @@
     <t>IN PROGRESS</t>
   </si>
   <si>
+    <t>IN PROGRESS: HTTP Lifecycle11/29 closed; Group overall11/48 (22.92%). Current block12.</t>
+  </si>
+  <si>
     <t>2026-09-27</t>
   </si>
   <si>
     <t>31 focused backend moderation/chat/counter tests PASS (2026-09-25): separate scope settings, authority/foreign IDs, persisted pending count and idempotence, worker, Group support access/filter/unread. Earlier 15 filter/invitation tests PASS (2026-09-24). Frontend/backend dev watchers compiled. Full local/UI/HTTP journey NOT RUN. Profile selection correction: 21 focused Java tests PASS (2026-09-25); profile-load parameter, read-only restore, accepted-membership authority, failed-load non-commit, invite activation and removal. Added frontend HTTP parameter/retry unit cases; not executed separately from the running build watcher. | 2026-09-26: 105 focused backend tests PASS and 47 frontend tests PASS, covering explore boundaries, Base-only asset API key, contact repository account resolution and ticket account aggregation. These unit results do not close the manual local/HTTP journey. | My Tools follow-up (2026-09-26): 40 focused frontend tests PASS; 1 backend stored menu-counter test PASS. Account ownership/store/counters and stale-poll checks covered; browser journey NOT RUN. | Scope follow-up (2026-09-26): 195 backend and 32 frontend focused tests PASS. Payment payer/recipient query identity, account contacts, group event authorization and ticket scanner covered; manual local/HTTP journey NOT RUN. | Overlay navigation (2026-09-26): 27 focused frontend tests PASS; no real-device/Router/Firebase journey claimed. MCP Go race tests and image 1.3.0 initialization/discovery PASS; six generated schemas match OpenAPI. Help source parity PASS. | 2026-09-26: 13 focused frontend checks passed: popup/category/distance (5), local membership/notification lifecycle (5), workspace scopes and stale polls (3). Existing dev watchers compiled frontend/backend; added Java regression cases not run. No full-flow PASS.</t>
   </si>
   <si>
-    <t>HTTP10/48 closed; Lifecycle10/29. Block11 Contacts and existing chat popup current. Versioned prerequisite snapshot before UI. Local NOT RUN.</t>
-  </si>
-  <si>
-    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup.</t>
+    <t>HTTP block12: configured selection limits and direct-chat contact-request controls. Preserve closed blocks1–11; Local NOT RUN.</t>
+  </si>
+  <si>
+    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup. | 2026-09-27 block11 CLOSED: approved-only contact invitations/denials, retained overlays, recipient messages/unread reset, phone/share nesting, EN desktop/HU mobile; exact fixture restore PASS; after-contacts savepoint resume12. Evidence GROUP-LIFECYCLE-001-block11-contacts-20260927.json.</t>
   </si>
   <si>
     <t>180/420</t>
@@ -14101,31 +14104,31 @@
         <v>1089</v>
       </c>
       <c r="L115" s="138" t="s">
-        <v>1089</v>
+        <v>1090</v>
       </c>
       <c r="M115" s="138" t="s">
         <v>96</v>
       </c>
       <c r="N115" s="138" t="s">
-        <v>1090</v>
+        <v>1091</v>
       </c>
       <c r="O115" s="138" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="P115" s="138" t="s">
-        <v>1092</v>
+        <v>1093</v>
       </c>
       <c r="Q115" s="138" t="s">
         <v>96</v>
       </c>
       <c r="R115" s="138" t="s">
-        <v>1093</v>
+        <v>1094</v>
       </c>
       <c r="S115" s="138" t="s">
         <v>459</v>
       </c>
       <c r="T115" s="138" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="U115" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K115&amp;" "&amp;Q115))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K115&amp;" "&amp;Q115))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("PENDING",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("IN PROGRESS",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("OPEN",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("RETEST REQUIRED",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K115&amp;" "&amp;Q115)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K115&amp;" "&amp;Q115))),"Pending",IF(OR(Q115="PASS",ISNUMBER(SEARCH("PASS",K115&amp;" "&amp;Q115))),"Done","Pending"))))</f>
@@ -14142,7 +14145,7 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="138" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="B116" s="138" t="s">
         <v>122</v>
@@ -14151,10 +14154,10 @@
         <v>32</v>
       </c>
       <c r="D116" s="138" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="E116" s="138" t="s">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="F116" s="138" t="s">
         <v>125</v>
@@ -14169,7 +14172,7 @@
         <v>128</v>
       </c>
       <c r="J116" s="138" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="K116" s="138" t="s">
         <v>130</v>
@@ -14184,22 +14187,22 @@
         <v>1</v>
       </c>
       <c r="O116" s="138" t="s">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="P116" s="138" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="Q116" s="138" t="s">
         <v>96</v>
       </c>
       <c r="R116" s="138" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="S116" s="138" t="s">
         <v>420</v>
       </c>
       <c r="T116" s="138" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="U116" s="146" t="str">
         <f>IF(OR(ISNUMBER(SEARCH("FAIL",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("CLEAN RETEST REQUIRED",K116&amp;" "&amp;Q116))),"Failed",IF(OR(ISNUMBER(SEARCH("NOT RUN",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("NOT IMPLEMENTED",K116&amp;" "&amp;Q116))),"Not started",IF(OR(ISNUMBER(SEARCH("PARTIAL",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("PENDING",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("IN PROGRESS",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("OPEN",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("RETEST REQUIRED",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("IMPLEMENTATION UPDATED",K116&amp;" "&amp;Q116)),ISNUMBER(SEARCH("REQUIRED EVERY SESSION",K116&amp;" "&amp;Q116))),"Pending",IF(OR(Q116="PASS",ISNUMBER(SEARCH("PASS",K116&amp;" "&amp;Q116))),"Done","Pending"))))</f>
@@ -14216,7 +14219,7 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="135" t="s">
-        <v>1103</v>
+        <v>1104</v>
       </c>
       <c r="B117" s="135" t="s">
         <v>284</v>
@@ -14225,10 +14228,10 @@
         <v>38</v>
       </c>
       <c r="D117" s="135" t="s">
-        <v>1104</v>
+        <v>1105</v>
       </c>
       <c r="E117" s="135" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="F117" s="135" t="s">
         <v>4</v>
@@ -14243,7 +14246,7 @@
         <v>4</v>
       </c>
       <c r="J117" s="135" t="s">
-        <v>1106</v>
+        <v>1107</v>
       </c>
       <c r="K117" s="135" t="s">
         <v>806</v>
@@ -14258,16 +14261,16 @@
         <v>526</v>
       </c>
       <c r="O117" s="135" t="s">
-        <v>1107</v>
+        <v>1108</v>
       </c>
       <c r="P117" s="135" t="s">
-        <v>1108</v>
+        <v>1109</v>
       </c>
       <c r="Q117" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R117" s="135" t="s">
-        <v>1109</v>
+        <v>1110</v>
       </c>
       <c r="S117" s="135" t="s">
         <v>352</v>
@@ -14290,7 +14293,7 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="135" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="B118" s="135" t="s">
         <v>284</v>
@@ -14299,10 +14302,10 @@
         <v>38</v>
       </c>
       <c r="D118" s="135" t="s">
-        <v>1111</v>
+        <v>1112</v>
       </c>
       <c r="E118" s="135" t="s">
-        <v>1112</v>
+        <v>1113</v>
       </c>
       <c r="F118" s="135" t="s">
         <v>4</v>
@@ -14317,7 +14320,7 @@
         <v>4</v>
       </c>
       <c r="J118" s="135" t="s">
-        <v>1113</v>
+        <v>1114</v>
       </c>
       <c r="K118" s="135" t="s">
         <v>806</v>
@@ -14332,16 +14335,16 @@
         <v>526</v>
       </c>
       <c r="O118" s="135" t="s">
-        <v>1114</v>
+        <v>1115</v>
       </c>
       <c r="P118" s="135" t="s">
-        <v>1115</v>
+        <v>1116</v>
       </c>
       <c r="Q118" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R118" s="135" t="s">
-        <v>1116</v>
+        <v>1117</v>
       </c>
       <c r="S118" s="135" t="s">
         <v>420</v>
@@ -14364,7 +14367,7 @@
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="135" t="s">
-        <v>1117</v>
+        <v>1118</v>
       </c>
       <c r="B119" s="135" t="s">
         <v>217</v>
@@ -14373,16 +14376,16 @@
         <v>38</v>
       </c>
       <c r="D119" s="135" t="s">
-        <v>1118</v>
+        <v>1119</v>
       </c>
       <c r="E119" s="135" t="s">
-        <v>1119</v>
+        <v>1120</v>
       </c>
       <c r="F119" s="135" t="s">
-        <v>1120</v>
+        <v>1121</v>
       </c>
       <c r="G119" s="135" t="s">
-        <v>1121</v>
+        <v>1122</v>
       </c>
       <c r="H119" s="135" t="s">
         <v>4</v>
@@ -14391,7 +14394,7 @@
         <v>4</v>
       </c>
       <c r="J119" s="135" t="s">
-        <v>1122</v>
+        <v>1123</v>
       </c>
       <c r="K119" s="135" t="s">
         <v>146</v>
@@ -14406,19 +14409,19 @@
         <v>1081</v>
       </c>
       <c r="O119" s="135" t="s">
-        <v>1123</v>
+        <v>1124</v>
       </c>
       <c r="P119" s="135" t="s">
-        <v>1124</v>
+        <v>1125</v>
       </c>
       <c r="Q119" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R119" s="135" t="s">
-        <v>1125</v>
+        <v>1126</v>
       </c>
       <c r="S119" s="135" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="T119" s="135" t="s">
         <v>1</v>
@@ -14438,7 +14441,7 @@
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="135" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="B120" s="135" t="s">
         <v>217</v>
@@ -14447,28 +14450,28 @@
         <v>44</v>
       </c>
       <c r="D120" s="135" t="s">
-        <v>1128</v>
+        <v>1129</v>
       </c>
       <c r="E120" s="135" t="s">
-        <v>1129</v>
+        <v>1130</v>
       </c>
       <c r="F120" s="135" t="s">
-        <v>1130</v>
+        <v>1131</v>
       </c>
       <c r="G120" s="135" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
       <c r="H120" s="135" t="s">
         <v>4</v>
       </c>
       <c r="I120" s="135" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="J120" s="135" t="s">
-        <v>1133</v>
+        <v>1134</v>
       </c>
       <c r="K120" s="135" t="s">
-        <v>1134</v>
+        <v>1135</v>
       </c>
       <c r="L120" s="135" t="s">
         <v>1</v>
@@ -14477,19 +14480,19 @@
         <v>1</v>
       </c>
       <c r="N120" s="135" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
       <c r="O120" s="135" t="s">
-        <v>1136</v>
+        <v>1137</v>
       </c>
       <c r="P120" s="135" t="s">
-        <v>1137</v>
+        <v>1138</v>
       </c>
       <c r="Q120" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R120" s="135" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="S120" s="135" t="s">
         <v>173</v>
@@ -14512,7 +14515,7 @@
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="135" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="B121" s="135" t="s">
         <v>217</v>
@@ -14521,25 +14524,25 @@
         <v>44</v>
       </c>
       <c r="D121" s="135" t="s">
-        <v>1140</v>
+        <v>1141</v>
       </c>
       <c r="E121" s="135" t="s">
-        <v>1141</v>
+        <v>1142</v>
       </c>
       <c r="F121" s="135" t="s">
-        <v>1142</v>
+        <v>1143</v>
       </c>
       <c r="G121" s="135" t="s">
-        <v>1143</v>
+        <v>1144</v>
       </c>
       <c r="H121" s="135" t="s">
-        <v>1144</v>
+        <v>1145</v>
       </c>
       <c r="I121" s="135" t="s">
-        <v>1145</v>
+        <v>1146</v>
       </c>
       <c r="J121" s="135" t="s">
-        <v>1146</v>
+        <v>1147</v>
       </c>
       <c r="K121" s="135" t="s">
         <v>85</v>
@@ -14551,19 +14554,19 @@
         <v>1</v>
       </c>
       <c r="N121" s="135" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
       <c r="O121" s="135" t="s">
-        <v>1147</v>
+        <v>1148</v>
       </c>
       <c r="P121" s="135" t="s">
-        <v>1148</v>
+        <v>1149</v>
       </c>
       <c r="Q121" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R121" s="135" t="s">
-        <v>1149</v>
+        <v>1150</v>
       </c>
       <c r="S121" s="135" t="s">
         <v>364</v>
@@ -14586,7 +14589,7 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="135" t="s">
-        <v>1150</v>
+        <v>1151</v>
       </c>
       <c r="B122" s="135" t="s">
         <v>231</v>
@@ -14595,16 +14598,16 @@
         <v>44</v>
       </c>
       <c r="D122" s="135" t="s">
-        <v>1151</v>
+        <v>1152</v>
       </c>
       <c r="E122" s="135" t="s">
-        <v>1152</v>
+        <v>1153</v>
       </c>
       <c r="F122" s="135" t="s">
         <v>4</v>
       </c>
       <c r="G122" s="135" t="s">
-        <v>1153</v>
+        <v>1154</v>
       </c>
       <c r="H122" s="135" t="s">
         <v>4</v>
@@ -14613,7 +14616,7 @@
         <v>8</v>
       </c>
       <c r="J122" s="135" t="s">
-        <v>1154</v>
+        <v>1155</v>
       </c>
       <c r="K122" s="135" t="s">
         <v>85</v>
@@ -14625,19 +14628,19 @@
         <v>1</v>
       </c>
       <c r="N122" s="135" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
       <c r="O122" s="135" t="s">
-        <v>1155</v>
+        <v>1156</v>
       </c>
       <c r="P122" s="135" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="Q122" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R122" s="135" t="s">
-        <v>1157</v>
+        <v>1158</v>
       </c>
       <c r="S122" s="135" t="s">
         <v>120</v>
@@ -14660,7 +14663,7 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="135" t="s">
-        <v>1158</v>
+        <v>1159</v>
       </c>
       <c r="B123" s="135" t="s">
         <v>217</v>
@@ -14669,25 +14672,25 @@
         <v>44</v>
       </c>
       <c r="D123" s="135" t="s">
-        <v>1159</v>
+        <v>1160</v>
       </c>
       <c r="E123" s="135" t="s">
-        <v>1160</v>
+        <v>1161</v>
       </c>
       <c r="F123" s="135" t="s">
-        <v>1161</v>
+        <v>1162</v>
       </c>
       <c r="G123" s="135" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="H123" s="135" t="s">
         <v>4</v>
       </c>
       <c r="I123" s="135" t="s">
-        <v>1163</v>
+        <v>1164</v>
       </c>
       <c r="J123" s="135" t="s">
-        <v>1164</v>
+        <v>1165</v>
       </c>
       <c r="K123" s="135" t="s">
         <v>85</v>
@@ -14699,19 +14702,19 @@
         <v>1</v>
       </c>
       <c r="N123" s="135" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
       <c r="O123" s="135" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="P123" s="135" t="s">
-        <v>1166</v>
+        <v>1167</v>
       </c>
       <c r="Q123" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R123" s="135" t="s">
-        <v>1167</v>
+        <v>1168</v>
       </c>
       <c r="S123" s="135" t="s">
         <v>431</v>
@@ -14734,7 +14737,7 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="135" t="s">
-        <v>1168</v>
+        <v>1169</v>
       </c>
       <c r="B124" s="135" t="s">
         <v>217</v>
@@ -14743,28 +14746,28 @@
         <v>44</v>
       </c>
       <c r="D124" s="135" t="s">
-        <v>1169</v>
+        <v>1170</v>
       </c>
       <c r="E124" s="135" t="s">
-        <v>1170</v>
+        <v>1171</v>
       </c>
       <c r="F124" s="135" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="G124" s="135" t="s">
-        <v>1172</v>
+        <v>1173</v>
       </c>
       <c r="H124" s="135" t="s">
         <v>4</v>
       </c>
       <c r="I124" s="135" t="s">
-        <v>1173</v>
+        <v>1174</v>
       </c>
       <c r="J124" s="135" t="s">
-        <v>1174</v>
+        <v>1175</v>
       </c>
       <c r="K124" s="135" t="s">
-        <v>1175</v>
+        <v>1176</v>
       </c>
       <c r="L124" s="135" t="s">
         <v>1</v>
@@ -14773,19 +14776,19 @@
         <v>1</v>
       </c>
       <c r="N124" s="135" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
       <c r="O124" s="135" t="s">
-        <v>1176</v>
+        <v>1177</v>
       </c>
       <c r="P124" s="135" t="s">
-        <v>1177</v>
+        <v>1178</v>
       </c>
       <c r="Q124" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R124" s="135" t="s">
-        <v>1178</v>
+        <v>1179</v>
       </c>
       <c r="S124" s="135" t="s">
         <v>90</v>
@@ -14808,19 +14811,19 @@
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="135" t="s">
-        <v>1179</v>
+        <v>1180</v>
       </c>
       <c r="B125" s="135" t="s">
-        <v>1180</v>
+        <v>1181</v>
       </c>
       <c r="C125" s="255" t="s">
         <v>44</v>
       </c>
       <c r="D125" s="135" t="s">
-        <v>1181</v>
+        <v>1182</v>
       </c>
       <c r="E125" s="135" t="s">
-        <v>1182</v>
+        <v>1183</v>
       </c>
       <c r="F125" s="135" t="s">
         <v>4</v>
@@ -14832,13 +14835,13 @@
         <v>4</v>
       </c>
       <c r="I125" s="135" t="s">
-        <v>1183</v>
+        <v>1184</v>
       </c>
       <c r="J125" s="135" t="s">
-        <v>1184</v>
+        <v>1185</v>
       </c>
       <c r="K125" s="135" t="s">
-        <v>1185</v>
+        <v>1186</v>
       </c>
       <c r="L125" s="135" t="s">
         <v>1</v>
@@ -14847,22 +14850,22 @@
         <v>1</v>
       </c>
       <c r="N125" s="135" t="s">
-        <v>1186</v>
+        <v>1187</v>
       </c>
       <c r="O125" s="135" t="s">
-        <v>1187</v>
+        <v>1188</v>
       </c>
       <c r="P125" s="135" t="s">
-        <v>1188</v>
+        <v>1189</v>
       </c>
       <c r="Q125" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R125" s="135" t="s">
-        <v>1189</v>
+        <v>1190</v>
       </c>
       <c r="S125" s="135" t="s">
-        <v>1190</v>
+        <v>1191</v>
       </c>
       <c r="T125" s="135" t="s">
         <v>1</v>
@@ -14882,10 +14885,10 @@
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="135" t="s">
-        <v>1191</v>
+        <v>1192</v>
       </c>
       <c r="B126" s="135" t="s">
-        <v>1192</v>
+        <v>1193</v>
       </c>
       <c r="C126" s="263" t="s">
         <v>50</v>
@@ -14894,10 +14897,10 @@
         <v>63</v>
       </c>
       <c r="E126" s="135" t="s">
-        <v>1193</v>
+        <v>1194</v>
       </c>
       <c r="F126" s="135" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="G126" s="135" t="s">
         <v>4</v>
@@ -14924,19 +14927,19 @@
         <v>293</v>
       </c>
       <c r="O126" s="135" t="s">
-        <v>1195</v>
+        <v>1196</v>
       </c>
       <c r="P126" s="135" t="s">
-        <v>1196</v>
+        <v>1197</v>
       </c>
       <c r="Q126" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R126" s="135" t="s">
-        <v>1197</v>
+        <v>1198</v>
       </c>
       <c r="S126" s="135" t="s">
-        <v>1198</v>
+        <v>1199</v>
       </c>
       <c r="T126" s="135" t="s">
         <v>1</v>
@@ -14956,7 +14959,7 @@
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="135" t="s">
-        <v>1199</v>
+        <v>1200</v>
       </c>
       <c r="B127" s="135" t="s">
         <v>217</v>
@@ -14965,25 +14968,25 @@
         <v>50</v>
       </c>
       <c r="D127" s="135" t="s">
-        <v>1200</v>
+        <v>1201</v>
       </c>
       <c r="E127" s="135" t="s">
-        <v>1201</v>
+        <v>1202</v>
       </c>
       <c r="F127" s="135" t="s">
-        <v>1202</v>
+        <v>1203</v>
       </c>
       <c r="G127" s="135" t="s">
-        <v>1203</v>
+        <v>1204</v>
       </c>
       <c r="H127" s="135" t="s">
-        <v>1204</v>
+        <v>1205</v>
       </c>
       <c r="I127" s="135" t="s">
-        <v>1205</v>
+        <v>1206</v>
       </c>
       <c r="J127" s="135" t="s">
-        <v>1206</v>
+        <v>1207</v>
       </c>
       <c r="K127" s="135" t="s">
         <v>146</v>
@@ -14995,19 +14998,19 @@
         <v>1</v>
       </c>
       <c r="N127" s="135" t="s">
-        <v>1207</v>
+        <v>1208</v>
       </c>
       <c r="O127" s="135" t="s">
-        <v>1208</v>
+        <v>1209</v>
       </c>
       <c r="P127" s="135" t="s">
-        <v>1209</v>
+        <v>1210</v>
       </c>
       <c r="Q127" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R127" s="135" t="s">
-        <v>1210</v>
+        <v>1211</v>
       </c>
       <c r="S127" s="135" t="s">
         <v>352</v>
@@ -15030,7 +15033,7 @@
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="135" t="s">
-        <v>1211</v>
+        <v>1212</v>
       </c>
       <c r="B128" s="135" t="s">
         <v>217</v>
@@ -15039,25 +15042,25 @@
         <v>50</v>
       </c>
       <c r="D128" s="135" t="s">
-        <v>1212</v>
+        <v>1213</v>
       </c>
       <c r="E128" s="135" t="s">
-        <v>1213</v>
+        <v>1214</v>
       </c>
       <c r="F128" s="135" t="s">
-        <v>1214</v>
+        <v>1215</v>
       </c>
       <c r="G128" s="135" t="s">
-        <v>1215</v>
+        <v>1216</v>
       </c>
       <c r="H128" s="135" t="s">
-        <v>1216</v>
+        <v>1217</v>
       </c>
       <c r="I128" s="135" t="s">
-        <v>1217</v>
+        <v>1218</v>
       </c>
       <c r="J128" s="135" t="s">
-        <v>1218</v>
+        <v>1219</v>
       </c>
       <c r="K128" s="135" t="s">
         <v>146</v>
@@ -15069,22 +15072,22 @@
         <v>1</v>
       </c>
       <c r="N128" s="135" t="s">
-        <v>1207</v>
+        <v>1208</v>
       </c>
       <c r="O128" s="135" t="s">
-        <v>1219</v>
+        <v>1220</v>
       </c>
       <c r="P128" s="135" t="s">
-        <v>1220</v>
+        <v>1221</v>
       </c>
       <c r="Q128" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R128" s="135" t="s">
-        <v>1221</v>
+        <v>1222</v>
       </c>
       <c r="S128" s="135" t="s">
-        <v>1222</v>
+        <v>1223</v>
       </c>
       <c r="T128" s="135" t="s">
         <v>1</v>
@@ -15104,7 +15107,7 @@
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="135" t="s">
-        <v>1223</v>
+        <v>1224</v>
       </c>
       <c r="B129" s="135" t="s">
         <v>217</v>
@@ -15113,25 +15116,25 @@
         <v>50</v>
       </c>
       <c r="D129" s="135" t="s">
-        <v>1224</v>
+        <v>1225</v>
       </c>
       <c r="E129" s="135" t="s">
-        <v>1225</v>
+        <v>1226</v>
       </c>
       <c r="F129" s="135" t="s">
-        <v>1226</v>
+        <v>1227</v>
       </c>
       <c r="G129" s="135" t="s">
-        <v>1227</v>
+        <v>1228</v>
       </c>
       <c r="H129" s="135" t="s">
-        <v>1228</v>
+        <v>1229</v>
       </c>
       <c r="I129" s="135" t="s">
-        <v>1229</v>
+        <v>1230</v>
       </c>
       <c r="J129" s="135" t="s">
-        <v>1230</v>
+        <v>1231</v>
       </c>
       <c r="K129" s="135" t="s">
         <v>85</v>
@@ -15143,22 +15146,22 @@
         <v>1</v>
       </c>
       <c r="N129" s="135" t="s">
-        <v>1207</v>
+        <v>1208</v>
       </c>
       <c r="O129" s="135" t="s">
-        <v>1231</v>
+        <v>1232</v>
       </c>
       <c r="P129" s="135" t="s">
-        <v>1232</v>
+        <v>1233</v>
       </c>
       <c r="Q129" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R129" s="135" t="s">
-        <v>1233</v>
+        <v>1234</v>
       </c>
       <c r="S129" s="135" t="s">
-        <v>1234</v>
+        <v>1235</v>
       </c>
       <c r="T129" s="135" t="s">
         <v>1</v>
@@ -15178,7 +15181,7 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="135" t="s">
-        <v>1235</v>
+        <v>1236</v>
       </c>
       <c r="B130" s="135" t="s">
         <v>217</v>
@@ -15187,25 +15190,25 @@
         <v>55</v>
       </c>
       <c r="D130" s="135" t="s">
-        <v>1236</v>
+        <v>1237</v>
       </c>
       <c r="E130" s="135" t="s">
-        <v>1237</v>
+        <v>1238</v>
       </c>
       <c r="F130" s="135" t="s">
         <v>4</v>
       </c>
       <c r="G130" s="135" t="s">
-        <v>1238</v>
+        <v>1239</v>
       </c>
       <c r="H130" s="135" t="s">
         <v>4</v>
       </c>
       <c r="I130" s="135" t="s">
-        <v>1239</v>
+        <v>1240</v>
       </c>
       <c r="J130" s="135" t="s">
-        <v>1240</v>
+        <v>1241</v>
       </c>
       <c r="K130" s="135" t="s">
         <v>146</v>
@@ -15217,19 +15220,19 @@
         <v>1</v>
       </c>
       <c r="N130" s="135" t="s">
-        <v>1207</v>
+        <v>1208</v>
       </c>
       <c r="O130" s="135" t="s">
-        <v>1241</v>
+        <v>1242</v>
       </c>
       <c r="P130" s="135" t="s">
-        <v>1242</v>
+        <v>1243</v>
       </c>
       <c r="Q130" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R130" s="135" t="s">
-        <v>1243</v>
+        <v>1244</v>
       </c>
       <c r="S130" s="135" t="s">
         <v>90</v>
@@ -15252,7 +15255,7 @@
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="135" t="s">
-        <v>1244</v>
+        <v>1245</v>
       </c>
       <c r="B131" s="135" t="s">
         <v>217</v>
@@ -15261,25 +15264,25 @@
         <v>55</v>
       </c>
       <c r="D131" s="135" t="s">
-        <v>1245</v>
+        <v>1246</v>
       </c>
       <c r="E131" s="135" t="s">
-        <v>1246</v>
+        <v>1247</v>
       </c>
       <c r="F131" s="135" t="s">
-        <v>1247</v>
+        <v>1248</v>
       </c>
       <c r="G131" s="135" t="s">
-        <v>1248</v>
+        <v>1249</v>
       </c>
       <c r="H131" s="135" t="s">
-        <v>1249</v>
+        <v>1250</v>
       </c>
       <c r="I131" s="135" t="s">
-        <v>1250</v>
+        <v>1251</v>
       </c>
       <c r="J131" s="135" t="s">
-        <v>1251</v>
+        <v>1252</v>
       </c>
       <c r="K131" s="135" t="s">
         <v>85</v>
@@ -15291,19 +15294,19 @@
         <v>1</v>
       </c>
       <c r="N131" s="135" t="s">
-        <v>1207</v>
+        <v>1208</v>
       </c>
       <c r="O131" s="135" t="s">
-        <v>1252</v>
+        <v>1253</v>
       </c>
       <c r="P131" s="135" t="s">
-        <v>1253</v>
+        <v>1254</v>
       </c>
       <c r="Q131" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R131" s="135" t="s">
-        <v>1254</v>
+        <v>1255</v>
       </c>
       <c r="S131" s="135" t="s">
         <v>90</v>
@@ -15326,7 +15329,7 @@
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="135" t="s">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="B132" s="135" t="s">
         <v>217</v>
@@ -15335,25 +15338,25 @@
         <v>55</v>
       </c>
       <c r="D132" s="135" t="s">
-        <v>1256</v>
+        <v>1257</v>
       </c>
       <c r="E132" s="135" t="s">
-        <v>1257</v>
+        <v>1258</v>
       </c>
       <c r="F132" s="135" t="s">
         <v>4</v>
       </c>
       <c r="G132" s="135" t="s">
-        <v>1258</v>
+        <v>1259</v>
       </c>
       <c r="H132" s="135" t="s">
         <v>4</v>
       </c>
       <c r="I132" s="135" t="s">
-        <v>1259</v>
+        <v>1260</v>
       </c>
       <c r="J132" s="135" t="s">
-        <v>1260</v>
+        <v>1261</v>
       </c>
       <c r="K132" s="135" t="s">
         <v>146</v>
@@ -15365,19 +15368,19 @@
         <v>1</v>
       </c>
       <c r="N132" s="135" t="s">
-        <v>1207</v>
+        <v>1208</v>
       </c>
       <c r="O132" s="135" t="s">
-        <v>1261</v>
+        <v>1262</v>
       </c>
       <c r="P132" s="135" t="s">
-        <v>1262</v>
+        <v>1263</v>
       </c>
       <c r="Q132" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R132" s="135" t="s">
-        <v>1263</v>
+        <v>1264</v>
       </c>
       <c r="S132" s="135" t="s">
         <v>173</v>
@@ -15400,7 +15403,7 @@
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="135" t="s">
-        <v>1264</v>
+        <v>1265</v>
       </c>
       <c r="B133" s="135" t="s">
         <v>217</v>
@@ -15409,25 +15412,25 @@
         <v>55</v>
       </c>
       <c r="D133" s="135" t="s">
-        <v>1265</v>
+        <v>1266</v>
       </c>
       <c r="E133" s="135" t="s">
-        <v>1266</v>
+        <v>1267</v>
       </c>
       <c r="F133" s="135" t="s">
-        <v>1267</v>
+        <v>1268</v>
       </c>
       <c r="G133" s="135" t="s">
-        <v>1268</v>
+        <v>1269</v>
       </c>
       <c r="H133" s="135" t="s">
         <v>4</v>
       </c>
       <c r="I133" s="135" t="s">
-        <v>1269</v>
+        <v>1270</v>
       </c>
       <c r="J133" s="135" t="s">
-        <v>1270</v>
+        <v>1271</v>
       </c>
       <c r="K133" s="135" t="s">
         <v>85</v>
@@ -15439,22 +15442,22 @@
         <v>1</v>
       </c>
       <c r="N133" s="135" t="s">
-        <v>1207</v>
+        <v>1208</v>
       </c>
       <c r="O133" s="135" t="s">
-        <v>1271</v>
+        <v>1272</v>
       </c>
       <c r="P133" s="135" t="s">
-        <v>1272</v>
+        <v>1273</v>
       </c>
       <c r="Q133" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R133" s="135" t="s">
-        <v>1273</v>
+        <v>1274</v>
       </c>
       <c r="S133" s="135" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="T133" s="135" t="s">
         <v>1</v>
@@ -15474,7 +15477,7 @@
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="135" t="s">
-        <v>1274</v>
+        <v>1275</v>
       </c>
       <c r="B134" s="135" t="s">
         <v>101</v>
@@ -15483,25 +15486,25 @@
         <v>55</v>
       </c>
       <c r="D134" s="135" t="s">
-        <v>1275</v>
+        <v>1276</v>
       </c>
       <c r="E134" s="135" t="s">
-        <v>1276</v>
+        <v>1277</v>
       </c>
       <c r="F134" s="135" t="s">
         <v>4</v>
       </c>
       <c r="G134" s="135" t="s">
-        <v>1277</v>
+        <v>1278</v>
       </c>
       <c r="H134" s="135" t="s">
         <v>4</v>
       </c>
       <c r="I134" s="135" t="s">
-        <v>1278</v>
+        <v>1279</v>
       </c>
       <c r="J134" s="135" t="s">
-        <v>1279</v>
+        <v>1280</v>
       </c>
       <c r="K134" s="135" t="s">
         <v>85</v>
@@ -15516,19 +15519,19 @@
         <v>106</v>
       </c>
       <c r="O134" s="135" t="s">
-        <v>1280</v>
+        <v>1281</v>
       </c>
       <c r="P134" s="135" t="s">
-        <v>1281</v>
+        <v>1282</v>
       </c>
       <c r="Q134" s="135" t="s">
         <v>85</v>
       </c>
       <c r="R134" s="135" t="s">
-        <v>1282</v>
+        <v>1283</v>
       </c>
       <c r="S134" s="135" t="s">
-        <v>1283</v>
+        <v>1284</v>
       </c>
       <c r="T134" s="135" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
group fix - mcp
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -3292,7 +3292,7 @@
     <t>IN PROGRESS</t>
   </si>
   <si>
-    <t>IN PROGRESS: HTTP Lifecycle12/29 closed; Group overall12/48 (25%). Current block13.</t>
+    <t>IN PROGRESS: HTTP Lifecycle13/29 closed; Group overall13/48 (27.08%). Block14 partial; blocks15–16 desktop checks retained.</t>
   </si>
   <si>
     <t>2026-09-27</t>
@@ -3301,10 +3301,10 @@
     <t>31 focused backend moderation/chat/counter tests PASS (2026-09-25): separate scope settings, authority/foreign IDs, persisted pending count and idempotence, worker, Group support access/filter/unread. Earlier 15 filter/invitation tests PASS (2026-09-24). Frontend/backend dev watchers compiled. Full local/UI/HTTP journey NOT RUN. Profile selection correction: 21 focused Java tests PASS (2026-09-25); profile-load parameter, read-only restore, accepted-membership authority, failed-load non-commit, invite activation and removal. Added frontend HTTP parameter/retry unit cases; not executed separately from the running build watcher. | 2026-09-26: 105 focused backend tests PASS and 47 frontend tests PASS, covering explore boundaries, Base-only asset API key, contact repository account resolution and ticket account aggregation. These unit results do not close the manual local/HTTP journey. | My Tools follow-up (2026-09-26): 40 focused frontend tests PASS; 1 backend stored menu-counter test PASS. Account ownership/store/counters and stale-poll checks covered; browser journey NOT RUN. | Scope follow-up (2026-09-26): 195 backend and 32 frontend focused tests PASS. Payment payer/recipient query identity, account contacts, group event authorization and ticket scanner covered; manual local/HTTP journey NOT RUN. | Overlay navigation (2026-09-26): 27 focused frontend tests PASS; no real-device/Router/Firebase journey claimed. MCP Go race tests and image 1.3.0 initialization/discovery PASS; six generated schemas match OpenAPI. Help source parity PASS. | 2026-09-26: 13 focused frontend checks passed: popup/category/distance (5), local membership/notification lifecycle (5), workspace scopes and stale polls (3). Existing dev watchers compiled frontend/backend; added Java regression cases not run. No full-flow PASS.</t>
   </si>
   <si>
-    <t>HTTP block13: empty calendar export. Preserve closed blocks1–12; Local NOT RUN.</t>
-  </si>
-  <si>
-    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup. | 2026-09-27 block11 CLOSED: approved-only contact invitations/denials, retained overlays, recipient messages/unread reset, phone/share nesting, EN desktop/HU mobile; exact fixture restore PASS; after-contacts savepoint resume12. Evidence GROUP-LIFECYCLE-001-block11-contacts-20260927.json. | 2026-09-27 block12 CLOSED: selection limits including nested/mobile; contact consent cancellation/failure/retry/decisions, pagination/search, private methods, same chat/persistence and delayed group/account switch PASS. Exact contacts restore and after-contacts verification PASS; after-contact-controls captured resume13. Evidence GROUP-LIFECYCLE-001-block12-controls-20260927.json.</t>
+    <t>Continue block14 remaining children/profile and eligible native registration; blocks15–16 desktop proof retained, external authenticated/device branches pending. No replay blocks1–13.</t>
+  </si>
+  <si>
+    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup. | 2026-09-27 block11 CLOSED: approved-only contact invitations/denials, retained overlays, recipient messages/unread reset, phone/share nesting, EN desktop/HU mobile; exact fixture restore PASS; after-contacts savepoint resume12. Evidence GROUP-LIFECYCLE-001-block11-contacts-20260927.json. | 2026-09-27 block12 CLOSED: selection limits including nested/mobile; contact consent cancellation/failure/retry/decisions, pagination/search, private methods, same chat/persistence and delayed group/account switch PASS. Exact contacts restore and after-contacts verification PASS; after-contact-controls captured resume13. Evidence GROUP-LIFECYCLE-001-block12-controls-20260927.json. | 2026-09-27 block13 CLOSED: empty HU/EN calendar notices retain blurred parent and produce no download; positive ICS download and libical import four events PASS. Desktop calendar UI NOT RUN. Blocks14–16 partial evidence retained in per-block JSON; no replay of completed subchecks.</t>
   </si>
   <si>
     <t>180/420</t>

</xml_diff>

<commit_message>
group fix - mobile sheet
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -427,7 +427,7 @@
     <t>Prepare/verify versioned fixture baseline and managed launcher, then execute the stable checklist; record local/HTTP evidence separately. | NOT RUN additions: API and UI external invitation URLs preserve affiliate attribution through registration and target participation; per-participant API claim versus reusable UI link; repeat/existing-user attribution; group active workspace; event admission gates; cash exclusion from affiliate totals. See Affiliate and external-link additions in the existing checklist. | Block 7: MCP discovery, API authority, anonymous shared help, client packages/logo and remote connections. These unexecuted micros moved from closed INTEGRATION-API-001; no inherited PASS.</t>
   </si>
   <si>
-    <t>guides/qa/checklists/integration/INTEGRATION-API-GROUP-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=5/4/4/4/4; effort actions/extra actors/oracles/boundaries/restore/external=26/2/4/3/1/1. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | NOT RUN blocks 2-3: fresh registration versus existing pre-registered demo recipient; real entry UI, cancelled/retried Setup retains invitation, first active-group load and reload/login. No session injection to skip entry gates.</t>
+    <t>guides/qa/checklists/integration/INTEGRATION-API-GROUP-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=5/4/4/4/4; effort actions/extra actors/oracles/boundaries/restore/external=26/2/4/3/1/1. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | NOT RUN blocks 2-3: fresh registration versus existing pre-registered demo recipient; real entry UI, cancelled/retried Setup retains invitation, first active-group load and reload/login. No session injection to skip entry gates. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase.</t>
   </si>
   <si>
     <t>P0 85</t>
@@ -781,7 +781,7 @@
     <t>Later: configure the isolated Firebase and external-client deployment, then execute the dedicated checklist</t>
   </si>
   <si>
-    <t>User explicitly deferred configuration-dependent checks2026-09-27. Moved from GROUP-LIFECYCLE-00119.2 and INTEGRATION-API-GROUP-0017; retains earlier DEPLOY-FIREBASE-LIFECYCLE-001 invitation-policy assertion. guides/qa/checklists/deployment/DEPLOY-EXTERNAL-CONFIG-001.md. Current firebase-config404; no external-provider PASS. Time range is a planning estimate after prerequisites are configured; includes configured deployment help update/import.</t>
+    <t>User explicitly deferred configuration-dependent checks2026-09-27. Moved from GROUP-LIFECYCLE-00119.2 and INTEGRATION-API-GROUP-0017; retains earlier DEPLOY-FIREBASE-LIFECYCLE-001 invitation-policy assertion. guides/qa/checklists/deployment/DEPLOY-EXTERNAL-CONFIG-001.md. Current firebase-config404; no external-provider PASS. Time range is a planning estimate after prerequisites are configured; includes configured deployment help update/import. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase.</t>
   </si>
   <si>
     <t>P2 60</t>
@@ -3337,16 +3337,16 @@
     <t>IN PROGRESS</t>
   </si>
   <si>
-    <t>IN PROGRESS: HTTP Lifecycle16/29 closed (1–13,17–19); Group overall16/48 (33.33%). Blocks14–16 partial retained;20 active.</t>
+    <t>IN PROGRESS: HTTP Lifecycle17/29 closed (1–13,17–20); Group overall17/48 (35.42%). Blocks14–16 partial retained;21 active.</t>
   </si>
   <si>
     <t>31 focused backend moderation/chat/counter tests PASS (2026-09-25): separate scope settings, authority/foreign IDs, persisted pending count and idempotence, worker, Group support access/filter/unread. Earlier 15 filter/invitation tests PASS (2026-09-24). Frontend/backend dev watchers compiled. Full local/UI/HTTP journey NOT RUN. Profile selection correction: 21 focused Java tests PASS (2026-09-25); profile-load parameter, read-only restore, accepted-membership authority, failed-load non-commit, invite activation and removal. Added frontend HTTP parameter/retry unit cases; not executed separately from the running build watcher. | 2026-09-26: 105 focused backend tests PASS and 47 frontend tests PASS, covering explore boundaries, Base-only asset API key, contact repository account resolution and ticket account aggregation. These unit results do not close the manual local/HTTP journey. | My Tools follow-up (2026-09-26): 40 focused frontend tests PASS; 1 backend stored menu-counter test PASS. Account ownership/store/counters and stale-poll checks covered; browser journey NOT RUN. | Scope follow-up (2026-09-26): 195 backend and 32 frontend focused tests PASS. Payment payer/recipient query identity, account contacts, group event authorization and ticket scanner covered; manual local/HTTP journey NOT RUN. | Overlay navigation (2026-09-26): 27 focused frontend tests PASS; no real-device/Router/Firebase journey claimed. MCP Go race tests and image 1.3.0 initialization/discovery PASS; six generated schemas match OpenAPI. Help source parity PASS. | 2026-09-26: 13 focused frontend checks passed: popup/category/distance (5), local membership/notification lifecycle (5), workspace scopes and stale polls (3). Existing dev watchers compiled frontend/backend; added Java regression cases not run. No full-flow PASS.</t>
   </si>
   <si>
-    <t>Block20 stored location/optional tracking: OFF/save/reopen/ON, &lt;5km and &gt;=5km, unsupported sample retention. Zoe tracking snapshot retained. Firebase/external configuration deferred to DEPLOY-EXTERNAL-CONFIG-001; Local separate.</t>
-  </si>
-  <si>
-    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup. | 2026-09-27 block11 CLOSED: approved-only contact invitations/denials, retained overlays, recipient messages/unread reset, phone/share nesting, EN desktop/HU mobile; exact fixture restore PASS; after-contacts savepoint resume12. Evidence GROUP-LIFECYCLE-001-block11-contacts-20260927.json. | 2026-09-27 block12 CLOSED: selection limits including nested/mobile; contact consent cancellation/failure/retry/decisions, pagination/search, private methods, same chat/persistence and delayed group/account switch PASS. Exact contacts restore and after-contacts verification PASS; after-contact-controls captured resume13. Evidence GROUP-LIFECYCLE-001-block12-controls-20260927.json. | 2026-09-27 block13 CLOSED: empty HU/EN calendar notices retain blurred parent and produce no download; positive ICS download and libical import four events PASS. Desktop calendar UI NOT RUN. Blocks14–16 partial evidence retained in per-block JSON; no replay of completed subchecks. | 2026-09-27 block17 CLOSED for user-agreed HTTP Help/native anonymous MCP scope: current Codex conversation directly invoked MyScoutee topic list/read successfully. MCP connection UI create/reload/secret-hide/revoke also verified. No private OAuth or Local PASS claimed. Block18 X/Back and rapid reopen checks passed; remaining checks continue. | 2026-09-27 block18 CLOSED: physical Android native-Back defect fixed in shared overlay history owner; nested Back, X/Back, rapid reopen, busy refusal, desktop Forward/Router/reload and unchanged rating dock verified. Existing frontend-sync PASS05:46:29Z; unit specs not rerun. Evidence GROUP-LIFECYCLE-001-block18-20260927.json. Normal phone logout, owned browser/tunnel cleanup complete; ENTRY untouched. User requested STOP before19. | 2026-09-27 resumed19: actual demo selector admission, denied/unsupported GPS, isolated Zoe missing/invalid Setup cancel/retry and first profile persistence/reload partially PASS. False Location required race fixed; real stale null poll retest retained accepted point over12.4s. frontend-sync PASS15:24:34Z. One ENTRY-BLOCK19 window, Zoe snapshot retained. Block19 IN PROGRESS; counts unchanged. Evidence GROUP-LIFECYCLE-001-block19-entry-20260927.json. | 2026-09-27 18:22:19.1 HTTP complete incl invitation claim/first target profile/reload/replay and GPS-denied relogin; exact scoped cleanup. Avatar wait/error boundary and Setup disabled action verified.19.2 active:53/53 seed points accepted; Firebase config404 blocks real sign-in; pending-coordinate controls/Local remain. No count change. | User scope change2026-09-27: Firebase and actual external-client/provider-configuration checks moved to DEPLOY-EXTERNAL-CONFIG-001, DEFERRED/NOT RUN. They no longer gate Group19; continue demo pending-coordinate controls. | Block19 HTTP CLOSED in user-approved demo scope:53/53 seed points; two-account real login/profile-ext unsupported pending samples rejected with original points retained and per-account acknowledgement. Earlier failure/retry/claim/cleanup evidence retained.16/48 and16/29 closed;20 active.</t>
+    <t>Block21 mobile sheet close buttons: seven audited surfaces plus profile multiselect/price scope/checkout; HU/EN narrow mobile and desktop controls. Firebase/external configuration deferred; Local separate.</t>
+  </si>
+  <si>
+    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup. | 2026-09-27 block11 CLOSED: approved-only contact invitations/denials, retained overlays, recipient messages/unread reset, phone/share nesting, EN desktop/HU mobile; exact fixture restore PASS; after-contacts savepoint resume12. Evidence GROUP-LIFECYCLE-001-block11-contacts-20260927.json. | 2026-09-27 block12 CLOSED: selection limits including nested/mobile; contact consent cancellation/failure/retry/decisions, pagination/search, private methods, same chat/persistence and delayed group/account switch PASS. Exact contacts restore and after-contacts verification PASS; after-contact-controls captured resume13. Evidence GROUP-LIFECYCLE-001-block12-controls-20260927.json. | 2026-09-27 block13 CLOSED: empty HU/EN calendar notices retain blurred parent and produce no download; positive ICS download and libical import four events PASS. Desktop calendar UI NOT RUN. Blocks14–16 partial evidence retained in per-block JSON; no replay of completed subchecks. | 2026-09-27 block17 CLOSED for user-agreed HTTP Help/native anonymous MCP scope: current Codex conversation directly invoked MyScoutee topic list/read successfully. MCP connection UI create/reload/secret-hide/revoke also verified. No private OAuth or Local PASS claimed. Block18 X/Back and rapid reopen checks passed; remaining checks continue. | 2026-09-27 block18 CLOSED: physical Android native-Back defect fixed in shared overlay history owner; nested Back, X/Back, rapid reopen, busy refusal, desktop Forward/Router/reload and unchanged rating dock verified. Existing frontend-sync PASS05:46:29Z; unit specs not rerun. Evidence GROUP-LIFECYCLE-001-block18-20260927.json. Normal phone logout, owned browser/tunnel cleanup complete; ENTRY untouched. User requested STOP before19. | 2026-09-27 resumed19: actual demo selector admission, denied/unsupported GPS, isolated Zoe missing/invalid Setup cancel/retry and first profile persistence/reload partially PASS. False Location required race fixed; real stale null poll retest retained accepted point over12.4s. frontend-sync PASS15:24:34Z. One ENTRY-BLOCK19 window, Zoe snapshot retained. Block19 IN PROGRESS; counts unchanged. Evidence GROUP-LIFECYCLE-001-block19-entry-20260927.json. | 2026-09-27 18:22:19.1 HTTP complete incl invitation claim/first target profile/reload/replay and GPS-denied relogin; exact scoped cleanup. Avatar wait/error boundary and Setup disabled action verified.19.2 active:53/53 seed points accepted; Firebase config404 blocks real sign-in; pending-coordinate controls/Local remain. No count change. | User scope change2026-09-27: Firebase and actual external-client/provider-configuration checks moved to DEPLOY-EXTERNAL-CONFIG-001, DEFERRED/NOT RUN. They no longer gate Group19; continue demo pending-coordinate controls. | Block19 HTTP CLOSED in user-approved demo scope:53/53 seed points; two-account real login/profile-ext unsupported pending samples rejected with original points retained and per-account acknowledgement. Earlier failure/retry/claim/cleanup evidence retained.16/48 and16/29 closed;20 active. | 2026-09-27 block20 HTTP PASS/CLOSED: stored point with denied GPS and same-session reload; tracking OFF/save/reopen/ON; &lt;5km zero writes, &gt;=5km POST200; unsupported Paris POST403 retains accepted profile/cache/baseline/session and no popup; later eligible movement POST200. Independent Mongo point47.6747/19.0354 verified, normal logout then exact original47.5147/19.0354 restore, location snapshot removed. Evidence: GROUP-LIFECYCLE-001-block20-tracking-20260927.json. HTTP17/48 (35.42%), Lifecycle17/29 closed (1–13,17–20);21 active. Local NOT RUN; older contact/badge snapshots retained. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase.</t>
   </si>
   <si>
     <t>180/420</t>

</xml_diff>

<commit_message>
group fix - tools
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -3337,16 +3337,16 @@
     <t>IN PROGRESS</t>
   </si>
   <si>
-    <t>IN PROGRESS: HTTP Lifecycle17/29 closed (1–13,17–20); Group overall17/48 (35.42%). Blocks14–16 partial retained;21 active.</t>
+    <t>IN PROGRESS: HTTP Lifecycle18/29 closed (1–13,17–21); Group overall18/48 (37.50%). Blocks14–16 partial retained;22 active.</t>
   </si>
   <si>
     <t>31 focused backend moderation/chat/counter tests PASS (2026-09-25): separate scope settings, authority/foreign IDs, persisted pending count and idempotence, worker, Group support access/filter/unread. Earlier 15 filter/invitation tests PASS (2026-09-24). Frontend/backend dev watchers compiled. Full local/UI/HTTP journey NOT RUN. Profile selection correction: 21 focused Java tests PASS (2026-09-25); profile-load parameter, read-only restore, accepted-membership authority, failed-load non-commit, invite activation and removal. Added frontend HTTP parameter/retry unit cases; not executed separately from the running build watcher. | 2026-09-26: 105 focused backend tests PASS and 47 frontend tests PASS, covering explore boundaries, Base-only asset API key, contact repository account resolution and ticket account aggregation. These unit results do not close the manual local/HTTP journey. | My Tools follow-up (2026-09-26): 40 focused frontend tests PASS; 1 backend stored menu-counter test PASS. Account ownership/store/counters and stale-poll checks covered; browser journey NOT RUN. | Scope follow-up (2026-09-26): 195 backend and 32 frontend focused tests PASS. Payment payer/recipient query identity, account contacts, group event authorization and ticket scanner covered; manual local/HTTP journey NOT RUN. | Overlay navigation (2026-09-26): 27 focused frontend tests PASS; no real-device/Router/Firebase journey claimed. MCP Go race tests and image 1.3.0 initialization/discovery PASS; six generated schemas match OpenAPI. Help source parity PASS. | 2026-09-26: 13 focused frontend checks passed: popup/category/distance (5), local membership/notification lifecycle (5), workspace scopes and stale polls (3). Existing dev watchers compiled frontend/backend; added Java regression cases not run. No full-flow PASS.</t>
   </si>
   <si>
-    <t>Finish21 checkout optional-card menu from own valid slot checkpoint; other menu smoke complete. Then22 account-owned assets. Counts unchanged; testcase transfers are closed in source and target runs independently.</t>
-  </si>
-  <si>
-    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup. | 2026-09-27 block11 CLOSED: approved-only contact invitations/denials, retained overlays, recipient messages/unread reset, phone/share nesting, EN desktop/HU mobile; exact fixture restore PASS; after-contacts savepoint resume12. Evidence GROUP-LIFECYCLE-001-block11-contacts-20260927.json. | 2026-09-27 block12 CLOSED: selection limits including nested/mobile; contact consent cancellation/failure/retry/decisions, pagination/search, private methods, same chat/persistence and delayed group/account switch PASS. Exact contacts restore and after-contacts verification PASS; after-contact-controls captured resume13. Evidence GROUP-LIFECYCLE-001-block12-controls-20260927.json. | 2026-09-27 block13 CLOSED: empty HU/EN calendar notices retain blurred parent and produce no download; positive ICS download and libical import four events PASS. Desktop calendar UI NOT RUN. Blocks14–16 partial evidence retained in per-block JSON; no replay of completed subchecks. | 2026-09-27 block17 CLOSED for user-agreed HTTP Help/native anonymous MCP scope: current Codex conversation directly invoked MyScoutee topic list/read successfully. MCP connection UI create/reload/secret-hide/revoke also verified. No private OAuth or Local PASS claimed. Block18 X/Back and rapid reopen checks passed; remaining checks continue. | 2026-09-27 block18 CLOSED: physical Android native-Back defect fixed in shared overlay history owner; nested Back, X/Back, rapid reopen, busy refusal, desktop Forward/Router/reload and unchanged rating dock verified. Existing frontend-sync PASS05:46:29Z; unit specs not rerun. Evidence GROUP-LIFECYCLE-001-block18-20260927.json. Normal phone logout, owned browser/tunnel cleanup complete; ENTRY untouched. User requested STOP before19. | 2026-09-27 resumed19: actual demo selector admission, denied/unsupported GPS, isolated Zoe missing/invalid Setup cancel/retry and first profile persistence/reload partially PASS. False Location required race fixed; real stale null poll retest retained accepted point over12.4s. frontend-sync PASS15:24:34Z. One ENTRY-BLOCK19 window, Zoe snapshot retained. Block19 IN PROGRESS; counts unchanged. Evidence GROUP-LIFECYCLE-001-block19-entry-20260927.json. | 2026-09-27 18:22:19.1 HTTP complete incl invitation claim/first target profile/reload/replay and GPS-denied relogin; exact scoped cleanup. Avatar wait/error boundary and Setup disabled action verified.19.2 active:53/53 seed points accepted; Firebase config404 blocks real sign-in; pending-coordinate controls/Local remain. No count change. | User scope change2026-09-27: Firebase and actual external-client/provider-configuration checks moved to DEPLOY-EXTERNAL-CONFIG-001, DEFERRED/NOT RUN. They no longer gate Group19; continue demo pending-coordinate controls. | Block19 HTTP CLOSED in user-approved demo scope:53/53 seed points; two-account real login/profile-ext unsupported pending samples rejected with original points retained and per-account acknowledgement. Earlier failure/retry/claim/cleanup evidence retained.16/48 and16/29 closed;20 active. | 2026-09-27 block20 HTTP PASS/CLOSED: stored point with denied GPS and same-session reload; tracking OFF/save/reopen/ON; &lt;5km zero writes, &gt;=5km POST200; unsupported Paris POST403 retains accepted profile/cache/baseline/session and no popup; later eligible movement POST200. Independent Mongo point47.6747/19.0354 verified, normal logout then exact original47.5147/19.0354 restore, location snapshot removed. Evidence: GROUP-LIFECYCLE-001-block20-tracking-20260927.json. HTTP17/48 (35.42%), Lifecycle17/29 closed (1–13,17–20);21 active. Local NOT RUN; older contact/badge snapshots retained. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | 2026-09-27 block21 HTTP partial: seven audited menu surfaces, profile multiselect, pricing scope and card menus exercised; HU320/EN360/desktop1100 representative checks. Notification launcher overlap and forced-sheet desktop X repaired and replayed through existing frontend-sync. Assignment basket restaged with own Group fixture and exactly restored, no assignment/share/checkout commit. Checkout optional-item menu remains NOT RUN because selected real event/date combinations returned no available slots; suitable own checkpoint required. Do not mark full21 closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP17/48 and Lifecycle17/29 unchanged.</t>
+    <t>22 account-owned tools and Asset Explore, own scoped checkpoint. At testcase boundary audit remaining NOT RUN external-config checks; transferred source scope closed and independent target requires its own run.</t>
+  </si>
+  <si>
+    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup. | 2026-09-27 block11 CLOSED: approved-only contact invitations/denials, retained overlays, recipient messages/unread reset, phone/share nesting, EN desktop/HU mobile; exact fixture restore PASS; after-contacts savepoint resume12. Evidence GROUP-LIFECYCLE-001-block11-contacts-20260927.json. | 2026-09-27 block12 CLOSED: selection limits including nested/mobile; contact consent cancellation/failure/retry/decisions, pagination/search, private methods, same chat/persistence and delayed group/account switch PASS. Exact contacts restore and after-contacts verification PASS; after-contact-controls captured resume13. Evidence GROUP-LIFECYCLE-001-block12-controls-20260927.json. | 2026-09-27 block13 CLOSED: empty HU/EN calendar notices retain blurred parent and produce no download; positive ICS download and libical import four events PASS. Desktop calendar UI NOT RUN. Blocks14–16 partial evidence retained in per-block JSON; no replay of completed subchecks. | 2026-09-27 block17 CLOSED for user-agreed HTTP Help/native anonymous MCP scope: current Codex conversation directly invoked MyScoutee topic list/read successfully. MCP connection UI create/reload/secret-hide/revoke also verified. No private OAuth or Local PASS claimed. Block18 X/Back and rapid reopen checks passed; remaining checks continue. | 2026-09-27 block18 CLOSED: physical Android native-Back defect fixed in shared overlay history owner; nested Back, X/Back, rapid reopen, busy refusal, desktop Forward/Router/reload and unchanged rating dock verified. Existing frontend-sync PASS05:46:29Z; unit specs not rerun. Evidence GROUP-LIFECYCLE-001-block18-20260927.json. Normal phone logout, owned browser/tunnel cleanup complete; ENTRY untouched. User requested STOP before19. | 2026-09-27 resumed19: actual demo selector admission, denied/unsupported GPS, isolated Zoe missing/invalid Setup cancel/retry and first profile persistence/reload partially PASS. False Location required race fixed; real stale null poll retest retained accepted point over12.4s. frontend-sync PASS15:24:34Z. One ENTRY-BLOCK19 window, Zoe snapshot retained. Block19 IN PROGRESS; counts unchanged. Evidence GROUP-LIFECYCLE-001-block19-entry-20260927.json. | 2026-09-27 18:22:19.1 HTTP complete incl invitation claim/first target profile/reload/replay and GPS-denied relogin; exact scoped cleanup. Avatar wait/error boundary and Setup disabled action verified.19.2 active:53/53 seed points accepted; Firebase config404 blocks real sign-in; pending-coordinate controls/Local remain. No count change. | User scope change2026-09-27: Firebase and actual external-client/provider-configuration checks moved to DEPLOY-EXTERNAL-CONFIG-001, DEFERRED/NOT RUN. They no longer gate Group19; continue demo pending-coordinate controls. | Block19 HTTP CLOSED in user-approved demo scope:53/53 seed points; two-account real login/profile-ext unsupported pending samples rejected with original points retained and per-account acknowledgement. Earlier failure/retry/claim/cleanup evidence retained.16/48 and16/29 closed;20 active. | 2026-09-27 block20 HTTP PASS/CLOSED: stored point with denied GPS and same-session reload; tracking OFF/save/reopen/ON; &lt;5km zero writes, &gt;=5km POST200; unsupported Paris POST403 retains accepted profile/cache/baseline/session and no popup; later eligible movement POST200. Independent Mongo point47.6747/19.0354 verified, normal logout then exact original47.5147/19.0354 restore, location snapshot removed. Evidence: GROUP-LIFECYCLE-001-block20-tracking-20260927.json. HTTP17/48 (35.42%), Lifecycle17/29 closed (1–13,17–20);21 active. Local NOT RUN; older contact/badge snapshots retained. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | 2026-09-27 block21 HTTP partial: seven audited menu surfaces, profile multiselect, pricing scope and card menus exercised; HU320/EN360/desktop1100 representative checks. Notification launcher overlap and forced-sheet desktop X repaired and replayed through existing frontend-sync. Assignment basket restaged with own Group fixture and exactly restored, no assignment/share/checkout commit. Checkout optional-item menu remains NOT RUN because selected real event/date combinations returned no available slots; suitable own checkpoint required. Do not mark full21 closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP17/48 and Lifecycle17/29 unchanged. | 2026-09-27 block21 HTTP PASS/CLOSED: final checkout optional-card control used its own versioned Group slot fixture. Native pointer selected/reverted optional item; mobile X remained reachable and closed only the sheet with parent dialogs/scroll retained; desktop title/no mobile X PASS. No checkout writes; draft discarded. Exact restore-sharing completed and original contact/badge snapshots retained. Together with the recorded seven menu surfaces, profile/price controls and HU/EN smoke,21 is closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP18/48 (37.50%), Lifecycle18/29 (1–13,17–21);22 active. Local NOT RUN.</t>
   </si>
   <si>
     <t>180/420</t>

</xml_diff>

<commit_message>
group fix - profile scope
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -424,10 +424,10 @@
     <t>15 focused backend tests PASS (2026-09-24): filter defaults/preservation and shared invitation claim plus community admission/replay. Does not prove this full UI/HTTP journey. Profile selection correction: 21 focused Java tests PASS (2026-09-25); profile-load parameter, read-only restore, accepted-membership authority, failed-load non-commit, invite activation and removal. Added frontend HTTP parameter/retry unit cases; not executed separately from the running build watcher.</t>
   </si>
   <si>
-    <t>Prepare/verify versioned fixture baseline and managed launcher, then execute the stable checklist; record local/HTTP evidence separately. | NOT RUN additions: API and UI external invitation URLs preserve affiliate attribution through registration and target participation; per-participant API claim versus reusable UI link; repeat/existing-user attribution; group active workspace; event admission gates; cash exclusion from affiliate totals. See Affiliate and external-link additions in the existing checklist. | Block 7: MCP discovery, API authority, anonymous shared help, client packages/logo and remote connections. These unexecuted micros moved from closed INTEGRATION-API-001; no inherited PASS.</t>
-  </si>
-  <si>
-    <t>guides/qa/checklists/integration/INTEGRATION-API-GROUP-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=5/4/4/4/4; effort actions/extra actors/oracles/boundaries/restore/external=26/2/4/3/1/1. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | NOT RUN blocks 2-3: fresh registration versus existing pre-registered demo recipient; real entry UI, cancelled/retried Setup retains invitation, first active-group load and reload/login. No session injection to skip entry gates. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase.</t>
+    <t>Own Group API checkpoint; section7 URL-first MCP flow is NOT IMPLEMENTED: develop in the existing API/MCP owners first, then test URL/Connect/sign-in/profile approval/callback without manual secret copying. Keep own restage and cleanup.</t>
+  </si>
+  <si>
+    <t>guides/qa/checklists/integration/INTEGRATION-API-GROUP-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=5/4/4/4/4; effort actions/extra actors/oracles/boundaries/restore/external=26/2/4/3/1/1. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | NOT RUN blocks 2-3: fresh registration versus existing pre-registered demo recipient; real entry UI, cancelled/retried Setup retains invitation, first active-group load and reload/login. No session injection to skip entry gates. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | User clarification2026-09-27: URL-first MCP connection is API-domain development, NOT IMPLEMENTED. Added to section7: implement first, then execute the independent API checkpoint. Existing manual client registration/consent is partial implementation; ordinary user flow must not require client-secret copying. Tall revoke-card layout included. | Local/dev full-flow requirement: implement a versioned real MCP/OAuth test client and callback receiver so URL discovery -&gt; browser sign-in/consent -&gt; token exchange -&gt; private tool call completes against the running application without fabricated grants/responses or a production dependency.</t>
   </si>
   <si>
     <t>P0 85</t>
@@ -778,10 +778,10 @@
     <t>Supporting shared-path tests only; real provider outcomes NOT RUN</t>
   </si>
   <si>
-    <t>Later: configure the isolated Firebase and external-client deployment, then execute the dedicated checklist</t>
-  </si>
-  <si>
-    <t>User explicitly deferred configuration-dependent checks2026-09-27. Moved from GROUP-LIFECYCLE-00119.2 and INTEGRATION-API-GROUP-0017; retains earlier DEPLOY-FIREBASE-LIFECYCLE-001 invitation-policy assertion. guides/qa/checklists/deployment/DEPLOY-EXTERNAL-CONFIG-001.md. Current firebase-config404; no external-provider PASS. Time range is a planning estimate after prerequisites are configured; includes configured deployment help update/import. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase.</t>
+    <t>Configure the isolated deployment and independently verify Firebase, supported real MCP clients URL/Connect/sign-in/approval/callback, and help initialization/update with own restage/checkpoints.</t>
+  </si>
+  <si>
+    <t>User explicitly deferred configuration-dependent checks2026-09-27. Moved from GROUP-LIFECYCLE-00119.2 and INTEGRATION-API-GROUP-0017; retains earlier DEPLOY-FIREBASE-LIFECYCLE-001 invitation-policy assertion. guides/qa/checklists/deployment/DEPLOY-EXTERNAL-CONFIG-001.md. Current firebase-config404; no external-provider PASS. Time range is a planning estimate after prerequisites are configured; includes configured deployment help update/import. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | User clarification2026-09-27: URL-first ChatGPT/Codex/Claude MCP connection without manual client-secret copying is NOT IMPLEMENTED. Development is required BEFORE deployment QA. Existing manual client registration and consent page do not prove the complete flow; external client initiates Connect. Tall connection cards keep Revoke top right. | Corrected domain2026-09-27: URL-first MCP implementation belongs to API test, not deployment setup. This row retains actual configured external-client interoperability checks only; no cross-case execution dependency or inherited PASS. | Boundary clarified: public HTTPS/external service registration/real ChatGPT-Codex-Claude interoperability belong here when they require configured deployment. Local/dev must still complete the real application protocol with a test client. Each case runs independently; URL-first feature still NOT IMPLEMENTED.</t>
   </si>
   <si>
     <t>P2 60</t>
@@ -3337,16 +3337,16 @@
     <t>IN PROGRESS</t>
   </si>
   <si>
-    <t>IN PROGRESS: HTTP Lifecycle18/29 closed (1–13,17–21); Group overall18/48 (37.50%). Blocks14–16 partial retained;22 active.</t>
+    <t>IN PROGRESS: HTTP Lifecycle19/29 closed (1–13,17–22); Group overall19/48 (39.58%). Blocks14–16 partial retained;23 active.</t>
   </si>
   <si>
     <t>31 focused backend moderation/chat/counter tests PASS (2026-09-25): separate scope settings, authority/foreign IDs, persisted pending count and idempotence, worker, Group support access/filter/unread. Earlier 15 filter/invitation tests PASS (2026-09-24). Frontend/backend dev watchers compiled. Full local/UI/HTTP journey NOT RUN. Profile selection correction: 21 focused Java tests PASS (2026-09-25); profile-load parameter, read-only restore, accepted-membership authority, failed-load non-commit, invite activation and removal. Added frontend HTTP parameter/retry unit cases; not executed separately from the running build watcher. | 2026-09-26: 105 focused backend tests PASS and 47 frontend tests PASS, covering explore boundaries, Base-only asset API key, contact repository account resolution and ticket account aggregation. These unit results do not close the manual local/HTTP journey. | My Tools follow-up (2026-09-26): 40 focused frontend tests PASS; 1 backend stored menu-counter test PASS. Account ownership/store/counters and stale-poll checks covered; browser journey NOT RUN. | Scope follow-up (2026-09-26): 195 backend and 32 frontend focused tests PASS. Payment payer/recipient query identity, account contacts, group event authorization and ticket scanner covered; manual local/HTTP journey NOT RUN. | Overlay navigation (2026-09-26): 27 focused frontend tests PASS; no real-device/Router/Firebase journey claimed. MCP Go race tests and image 1.3.0 initialization/discovery PASS; six generated schemas match OpenAPI. Help source parity PASS. | 2026-09-26: 13 focused frontend checks passed: popup/category/distance (5), local membership/notification lifecycle (5), workspace scopes and stale polls (3). Existing dev watchers compiled frontend/backend; added Java regression cases not run. No full-flow PASS.</t>
   </si>
   <si>
-    <t>22 account-owned tools and Asset Explore, own scoped checkpoint. At testcase boundary audit remaining NOT RUN external-config checks; transferred source scope closed and independent target requires its own run.</t>
-  </si>
-  <si>
-    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup. | 2026-09-27 block11 CLOSED: approved-only contact invitations/denials, retained overlays, recipient messages/unread reset, phone/share nesting, EN desktop/HU mobile; exact fixture restore PASS; after-contacts savepoint resume12. Evidence GROUP-LIFECYCLE-001-block11-contacts-20260927.json. | 2026-09-27 block12 CLOSED: selection limits including nested/mobile; contact consent cancellation/failure/retry/decisions, pagination/search, private methods, same chat/persistence and delayed group/account switch PASS. Exact contacts restore and after-contacts verification PASS; after-contact-controls captured resume13. Evidence GROUP-LIFECYCLE-001-block12-controls-20260927.json. | 2026-09-27 block13 CLOSED: empty HU/EN calendar notices retain blurred parent and produce no download; positive ICS download and libical import four events PASS. Desktop calendar UI NOT RUN. Blocks14–16 partial evidence retained in per-block JSON; no replay of completed subchecks. | 2026-09-27 block17 CLOSED for user-agreed HTTP Help/native anonymous MCP scope: current Codex conversation directly invoked MyScoutee topic list/read successfully. MCP connection UI create/reload/secret-hide/revoke also verified. No private OAuth or Local PASS claimed. Block18 X/Back and rapid reopen checks passed; remaining checks continue. | 2026-09-27 block18 CLOSED: physical Android native-Back defect fixed in shared overlay history owner; nested Back, X/Back, rapid reopen, busy refusal, desktop Forward/Router/reload and unchanged rating dock verified. Existing frontend-sync PASS05:46:29Z; unit specs not rerun. Evidence GROUP-LIFECYCLE-001-block18-20260927.json. Normal phone logout, owned browser/tunnel cleanup complete; ENTRY untouched. User requested STOP before19. | 2026-09-27 resumed19: actual demo selector admission, denied/unsupported GPS, isolated Zoe missing/invalid Setup cancel/retry and first profile persistence/reload partially PASS. False Location required race fixed; real stale null poll retest retained accepted point over12.4s. frontend-sync PASS15:24:34Z. One ENTRY-BLOCK19 window, Zoe snapshot retained. Block19 IN PROGRESS; counts unchanged. Evidence GROUP-LIFECYCLE-001-block19-entry-20260927.json. | 2026-09-27 18:22:19.1 HTTP complete incl invitation claim/first target profile/reload/replay and GPS-denied relogin; exact scoped cleanup. Avatar wait/error boundary and Setup disabled action verified.19.2 active:53/53 seed points accepted; Firebase config404 blocks real sign-in; pending-coordinate controls/Local remain. No count change. | User scope change2026-09-27: Firebase and actual external-client/provider-configuration checks moved to DEPLOY-EXTERNAL-CONFIG-001, DEFERRED/NOT RUN. They no longer gate Group19; continue demo pending-coordinate controls. | Block19 HTTP CLOSED in user-approved demo scope:53/53 seed points; two-account real login/profile-ext unsupported pending samples rejected with original points retained and per-account acknowledgement. Earlier failure/retry/claim/cleanup evidence retained.16/48 and16/29 closed;20 active. | 2026-09-27 block20 HTTP PASS/CLOSED: stored point with denied GPS and same-session reload; tracking OFF/save/reopen/ON; &lt;5km zero writes, &gt;=5km POST200; unsupported Paris POST403 retains accepted profile/cache/baseline/session and no popup; later eligible movement POST200. Independent Mongo point47.6747/19.0354 verified, normal logout then exact original47.5147/19.0354 restore, location snapshot removed. Evidence: GROUP-LIFECYCLE-001-block20-tracking-20260927.json. HTTP17/48 (35.42%), Lifecycle17/29 closed (1–13,17–20);21 active. Local NOT RUN; older contact/badge snapshots retained. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | 2026-09-27 block21 HTTP partial: seven audited menu surfaces, profile multiselect, pricing scope and card menus exercised; HU320/EN360/desktop1100 representative checks. Notification launcher overlap and forced-sheet desktop X repaired and replayed through existing frontend-sync. Assignment basket restaged with own Group fixture and exactly restored, no assignment/share/checkout commit. Checkout optional-item menu remains NOT RUN because selected real event/date combinations returned no available slots; suitable own checkpoint required. Do not mark full21 closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP17/48 and Lifecycle17/29 unchanged. | 2026-09-27 block21 HTTP PASS/CLOSED: final checkout optional-card control used its own versioned Group slot fixture. Native pointer selected/reverted optional item; mobile X remained reachable and closed only the sheet with parent dialogs/scroll retained; desktop title/no mobile X PASS. No checkout writes; draft discarded. Exact restore-sharing completed and original contact/badge snapshots retained. Together with the recorded seven menu surfaces, profile/price controls and HU/EN smoke,21 is closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP18/48 (37.50%), Lifecycle18/29 (1–13,17–21);22 active. Local NOT RUN.</t>
+    <t>23 profile scope and asset payment history. At testcase boundary audit remaining NOT RUN external-config checks; transferred source scope closed and independent target requires its own run.</t>
+  </si>
+  <si>
+    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup. | 2026-09-27 block11 CLOSED: approved-only contact invitations/denials, retained overlays, recipient messages/unread reset, phone/share nesting, EN desktop/HU mobile; exact fixture restore PASS; after-contacts savepoint resume12. Evidence GROUP-LIFECYCLE-001-block11-contacts-20260927.json. | 2026-09-27 block12 CLOSED: selection limits including nested/mobile; contact consent cancellation/failure/retry/decisions, pagination/search, private methods, same chat/persistence and delayed group/account switch PASS. Exact contacts restore and after-contacts verification PASS; after-contact-controls captured resume13. Evidence GROUP-LIFECYCLE-001-block12-controls-20260927.json. | 2026-09-27 block13 CLOSED: empty HU/EN calendar notices retain blurred parent and produce no download; positive ICS download and libical import four events PASS. Desktop calendar UI NOT RUN. Blocks14–16 partial evidence retained in per-block JSON; no replay of completed subchecks. | 2026-09-27 block17 CLOSED for user-agreed HTTP Help/native anonymous MCP scope: current Codex conversation directly invoked MyScoutee topic list/read successfully. MCP connection UI create/reload/secret-hide/revoke also verified. No private OAuth or Local PASS claimed. Block18 X/Back and rapid reopen checks passed; remaining checks continue. | 2026-09-27 block18 CLOSED: physical Android native-Back defect fixed in shared overlay history owner; nested Back, X/Back, rapid reopen, busy refusal, desktop Forward/Router/reload and unchanged rating dock verified. Existing frontend-sync PASS05:46:29Z; unit specs not rerun. Evidence GROUP-LIFECYCLE-001-block18-20260927.json. Normal phone logout, owned browser/tunnel cleanup complete; ENTRY untouched. User requested STOP before19. | 2026-09-27 resumed19: actual demo selector admission, denied/unsupported GPS, isolated Zoe missing/invalid Setup cancel/retry and first profile persistence/reload partially PASS. False Location required race fixed; real stale null poll retest retained accepted point over12.4s. frontend-sync PASS15:24:34Z. One ENTRY-BLOCK19 window, Zoe snapshot retained. Block19 IN PROGRESS; counts unchanged. Evidence GROUP-LIFECYCLE-001-block19-entry-20260927.json. | 2026-09-27 18:22:19.1 HTTP complete incl invitation claim/first target profile/reload/replay and GPS-denied relogin; exact scoped cleanup. Avatar wait/error boundary and Setup disabled action verified.19.2 active:53/53 seed points accepted; Firebase config404 blocks real sign-in; pending-coordinate controls/Local remain. No count change. | User scope change2026-09-27: Firebase and actual external-client/provider-configuration checks moved to DEPLOY-EXTERNAL-CONFIG-001, DEFERRED/NOT RUN. They no longer gate Group19; continue demo pending-coordinate controls. | Block19 HTTP CLOSED in user-approved demo scope:53/53 seed points; two-account real login/profile-ext unsupported pending samples rejected with original points retained and per-account acknowledgement. Earlier failure/retry/claim/cleanup evidence retained.16/48 and16/29 closed;20 active. | 2026-09-27 block20 HTTP PASS/CLOSED: stored point with denied GPS and same-session reload; tracking OFF/save/reopen/ON; &lt;5km zero writes, &gt;=5km POST200; unsupported Paris POST403 retains accepted profile/cache/baseline/session and no popup; later eligible movement POST200. Independent Mongo point47.6747/19.0354 verified, normal logout then exact original47.5147/19.0354 restore, location snapshot removed. Evidence: GROUP-LIFECYCLE-001-block20-tracking-20260927.json. HTTP17/48 (35.42%), Lifecycle17/29 closed (1–13,17–20);21 active. Local NOT RUN; older contact/badge snapshots retained. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | 2026-09-27 block21 HTTP partial: seven audited menu surfaces, profile multiselect, pricing scope and card menus exercised; HU320/EN360/desktop1100 representative checks. Notification launcher overlap and forced-sheet desktop X repaired and replayed through existing frontend-sync. Assignment basket restaged with own Group fixture and exactly restored, no assignment/share/checkout commit. Checkout optional-item menu remains NOT RUN because selected real event/date combinations returned no available slots; suitable own checkpoint required. Do not mark full21 closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP17/48 and Lifecycle17/29 unchanged. | 2026-09-27 block21 HTTP PASS/CLOSED: final checkout optional-card control used its own versioned Group slot fixture. Native pointer selected/reverted optional item; mobile X remained reachable and closed only the sheet with parent dialogs/scroll retained; desktop title/no mobile X PASS. No checkout writes; draft discarded. Exact restore-sharing completed and original contact/badge snapshots retained. Together with the recorded seven menu surfaces, profile/price controls and HU/EN smoke,21 is closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP18/48 (37.50%), Lifecycle18/29 (1–13,17–21);22 active. Local NOT RUN. | 2026-09-27 block22 HTTP PASS/CLOSED: Design Circle UI create/edit/delete persisted Base asset ownership; Main/Design Circle/Seattle Friends inventory and immediate asset counters match, event counters remain separate. Real response-stage delayed long-poll released after deletion did not resurrect count; no page reload. Own scoped fixture public Asset booked to an inaccessible Language Lab event remains in Explore (UI + three-profile authenticated reads); own/private/non-friend controls absent, foreign Event/private Asset details withheld with empty HTTP200. Event Explore UI changes with workspace. Existing Group chat preparation and tools fixtures exactly restored; no chat share submitted. Evidence GROUP-LIFECYCLE-001-block22-tools-20260927.json. HTTP19/48 (39.58%), Lifecycle19/29 (1–13,17–22);23 active. Local NOT RUN.</t>
   </si>
   <si>
     <t>180/420</t>

</xml_diff>

<commit_message>
group fix - asset
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -424,10 +424,10 @@
     <t>15 focused backend tests PASS (2026-09-24): filter defaults/preservation and shared invitation claim plus community admission/replay. Does not prove this full UI/HTTP journey. Profile selection correction: 21 focused Java tests PASS (2026-09-25); profile-load parameter, read-only restore, accepted-membership authority, failed-load non-commit, invite activation and removal. Added frontend HTTP parameter/retry unit cases; not executed separately from the running build watcher.</t>
   </si>
   <si>
-    <t>Own Group API checkpoint; section7 URL-first MCP flow is NOT IMPLEMENTED: develop in the existing API/MCP owners first, then test URL/Connect/sign-in/profile approval/callback without manual secret copying. Keep own restage and cleanup.</t>
-  </si>
-  <si>
-    <t>guides/qa/checklists/integration/INTEGRATION-API-GROUP-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=5/4/4/4/4; effort actions/extra actors/oracles/boundaries/restore/external=26/2/4/3/1/1. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | NOT RUN blocks 2-3: fresh registration versus existing pre-registered demo recipient; real entry UI, cancelled/retried Setup retains invitation, first active-group load and reload/login. No session injection to skip entry gates. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | User clarification2026-09-27: URL-first MCP connection is API-domain development, NOT IMPLEMENTED. Added to section7: implement first, then execute the independent API checkpoint. Existing manual client registration/consent is partial implementation; ordinary user flow must not require client-secret copying. Tall revoke-card layout included. | Local/dev full-flow requirement: implement a versioned real MCP/OAuth test client and callback receiver so URL discovery -&gt; browser sign-in/consent -&gt; token exchange -&gt; private tool call completes against the running application without fabricated grants/responses or a production dependency. | MCP client development target refined: optional browser URL/Connect client in myscoutee-mcp; reuse Inspector/OAuth, real login/callback/private tool result. Full Help Center and API popup question-mark help have separate HU/EN seeds. Feature remains NOT IMPLEMENTED; no runtime UI support claimed.</t>
+    <t>Final NOT RUN block7: develop and test URL/Connect OAuth simulator locally in myscoutee-mcp with real dev endpoints, browser login/consent, callback and authenticated tool calls. No production configuration or external ChatGPT account required. Own baseline/checkpoints/cleanup.</t>
+  </si>
+  <si>
+    <t>guides/qa/checklists/integration/INTEGRATION-API-GROUP-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=5/4/4/4/4; effort actions/extra actors/oracles/boundaries/restore/external=26/2/4/3/1/1. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | NOT RUN blocks 2-3: fresh registration versus existing pre-registered demo recipient; real entry UI, cancelled/retried Setup retains invitation, first active-group load and reload/login. No session injection to skip entry gates. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | User clarification2026-09-27: URL-first MCP connection is API-domain development, NOT IMPLEMENTED. Added to section7: implement first, then execute the independent API checkpoint. Existing manual client registration/consent is partial implementation; ordinary user flow must not require client-secret copying. Tall revoke-card layout included. | Local/dev full-flow requirement: implement a versioned real MCP/OAuth test client and callback receiver so URL discovery -&gt; browser sign-in/consent -&gt; token exchange -&gt; private tool call completes against the running application without fabricated grants/responses or a production dependency. | MCP client development target refined: optional browser URL/Connect client in myscoutee-mcp; reuse Inspector/OAuth, real login/callback/private tool result. Full Help Center and API popup question-mark help have separate HU/EN seeds. Feature remains NOT IMPLEMENTED; no runtime UI support claimed. | 2026-09-27 clarification: local MCP OAuth simulation remains in final API NOT RUN block7; no live deployment config prerequisite. Actual browser-based ChatGPT is a separate user-operated manual deployment test.</t>
   </si>
   <si>
     <t>P0 85</t>
@@ -778,10 +778,10 @@
     <t>Supporting shared-path tests only; real provider outcomes NOT RUN</t>
   </si>
   <si>
-    <t>Configure the isolated deployment and independently verify Firebase, supported real MCP clients URL/Connect/sign-in/approval/callback, and help initialization/update with own restage/checkpoints.</t>
-  </si>
-  <si>
-    <t>User explicitly deferred configuration-dependent checks2026-09-27. Moved from GROUP-LIFECYCLE-00119.2 and INTEGRATION-API-GROUP-0017; retains earlier DEPLOY-FIREBASE-LIFECYCLE-001 invitation-policy assertion. guides/qa/checklists/deployment/DEPLOY-EXTERNAL-CONFIG-001.md. Current firebase-config404; no external-provider PASS. Time range is a planning estimate after prerequisites are configured; includes configured deployment help update/import. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | User clarification2026-09-27: URL-first ChatGPT/Codex/Claude MCP connection without manual client-secret copying is NOT IMPLEMENTED. Development is required BEFORE deployment QA. Existing manual client registration and consent page do not prove the complete flow; external client initiates Connect. Tall connection cards keep Revoke top right. | Corrected domain2026-09-27: URL-first MCP implementation belongs to API test, not deployment setup. This row retains actual configured external-client interoperability checks only; no cross-case execution dependency or inherited PASS. | Boundary clarified: public HTTPS/external service registration/real ChatGPT-Codex-Claude interoperability belong here when they require configured deployment. Local/dev must still complete the real application protocol with a test client. Each case runs independently; URL-first feature still NOT IMPLEMENTED. | External assistant acceptance requires user Connect/login/approval, followed by actual authorized MCP tool discovery and read invocation in that same host/account. Simulator success alone is insufficient. Record actual ChatGPT/Claude conversation result; a supported dev tunnel may supply reachability.</t>
+    <t>Own configured test deployment: Firebase and help checks; user manually connects MyScoutee from the browser-based ChatGPT website, completes login/consent, invokes an allowed tool in that conversation and verifies revocation. Local OAuth simulator is outside deployment scope.</t>
+  </si>
+  <si>
+    <t>User explicitly deferred configuration-dependent checks2026-09-27. Moved from GROUP-LIFECYCLE-00119.2 and INTEGRATION-API-GROUP-0017; retains earlier DEPLOY-FIREBASE-LIFECYCLE-001 invitation-policy assertion. guides/qa/checklists/deployment/DEPLOY-EXTERNAL-CONFIG-001.md. Current firebase-config404; no external-provider PASS. Time range is a planning estimate after prerequisites are configured; includes configured deployment help update/import. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | User clarification2026-09-27: URL-first ChatGPT/Codex/Claude MCP connection without manual client-secret copying is NOT IMPLEMENTED. Development is required BEFORE deployment QA. Existing manual client registration and consent page do not prove the complete flow; external client initiates Connect. Tall connection cards keep Revoke top right. | Corrected domain2026-09-27: URL-first MCP implementation belongs to API test, not deployment setup. This row retains actual configured external-client interoperability checks only; no cross-case execution dependency or inherited PASS. | Boundary clarified: public HTTPS/external service registration/real ChatGPT-Codex-Claude interoperability belong here when they require configured deployment. Local/dev must still complete the real application protocol with a test client. Each case runs independently; URL-first feature still NOT IMPLEMENTED. | External assistant acceptance requires user Connect/login/approval, followed by actual authorized MCP tool discovery and read invocation in that same host/account. Simulator success alone is insufficient. Record actual ChatGPT/Claude conversation result; a supported dev tunnel may supply reachability. | 2026-09-27 clarification: explicit user-operated manual ChatGPT website acceptance added; not Codex-host substitution. Local simulator needs no production config and remains API scope.</t>
   </si>
   <si>
     <t>P2 60</t>
@@ -3337,13 +3337,13 @@
     <t>IN PROGRESS</t>
   </si>
   <si>
-    <t>IN PROGRESS: HTTP Lifecycle19/29 closed (1–13,17–22); Group overall19/48 (39.58%). Blocks14–16 partial retained;23 active.</t>
+    <t>IN PROGRESS: HTTP Lifecycle20/29 closed (1–13,17–23); Group overall20/48 (41.67%). Blocks14–16 partial retained;24 active.</t>
   </si>
   <si>
     <t>31 focused backend moderation/chat/counter tests PASS (2026-09-25): separate scope settings, authority/foreign IDs, persisted pending count and idempotence, worker, Group support access/filter/unread. Earlier 15 filter/invitation tests PASS (2026-09-24). Frontend/backend dev watchers compiled. Full local/UI/HTTP journey NOT RUN. Profile selection correction: 21 focused Java tests PASS (2026-09-25); profile-load parameter, read-only restore, accepted-membership authority, failed-load non-commit, invite activation and removal. Added frontend HTTP parameter/retry unit cases; not executed separately from the running build watcher. | 2026-09-26: 105 focused backend tests PASS and 47 frontend tests PASS, covering explore boundaries, Base-only asset API key, contact repository account resolution and ticket account aggregation. These unit results do not close the manual local/HTTP journey. | My Tools follow-up (2026-09-26): 40 focused frontend tests PASS; 1 backend stored menu-counter test PASS. Account ownership/store/counters and stale-poll checks covered; browser journey NOT RUN. | Scope follow-up (2026-09-26): 195 backend and 32 frontend focused tests PASS. Payment payer/recipient query identity, account contacts, group event authorization and ticket scanner covered; manual local/HTTP journey NOT RUN. | Overlay navigation (2026-09-26): 27 focused frontend tests PASS; no real-device/Router/Firebase journey claimed. MCP Go race tests and image 1.3.0 initialization/discovery PASS; six generated schemas match OpenAPI. Help source parity PASS. | 2026-09-26: 13 focused frontend checks passed: popup/category/distance (5), local membership/notification lifecycle (5), workspace scopes and stale polls (3). Existing dev watchers compiled frontend/backend; added Java regression cases not run. No full-flow PASS.</t>
   </si>
   <si>
-    <t>24 account contacts and event-linked assets. Own staged baseline and checkpoints; at testcase boundary audit remaining NOT RUN external-config checks.</t>
+    <t>24: finish Base/Group B resource denial and account-wide tickets/authenticated scanning; contact request/reject/re-request/approve and Base/Group chat verified, contact fixture restored. Independent24 free resource fixture active.</t>
   </si>
   <si>
     <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup. | 2026-09-27 block11 CLOSED: approved-only contact invitations/denials, retained overlays, recipient messages/unread reset, phone/share nesting, EN desktop/HU mobile; exact fixture restore PASS; after-contacts savepoint resume12. Evidence GROUP-LIFECYCLE-001-block11-contacts-20260927.json. | 2026-09-27 block12 CLOSED: selection limits including nested/mobile; contact consent cancellation/failure/retry/decisions, pagination/search, private methods, same chat/persistence and delayed group/account switch PASS. Exact contacts restore and after-contacts verification PASS; after-contact-controls captured resume13. Evidence GROUP-LIFECYCLE-001-block12-controls-20260927.json. | 2026-09-27 block13 CLOSED: empty HU/EN calendar notices retain blurred parent and produce no download; positive ICS download and libical import four events PASS. Desktop calendar UI NOT RUN. Blocks14–16 partial evidence retained in per-block JSON; no replay of completed subchecks. | 2026-09-27 block17 CLOSED for user-agreed HTTP Help/native anonymous MCP scope: current Codex conversation directly invoked MyScoutee topic list/read successfully. MCP connection UI create/reload/secret-hide/revoke also verified. No private OAuth or Local PASS claimed. Block18 X/Back and rapid reopen checks passed; remaining checks continue. | 2026-09-27 block18 CLOSED: physical Android native-Back defect fixed in shared overlay history owner; nested Back, X/Back, rapid reopen, busy refusal, desktop Forward/Router/reload and unchanged rating dock verified. Existing frontend-sync PASS05:46:29Z; unit specs not rerun. Evidence GROUP-LIFECYCLE-001-block18-20260927.json. Normal phone logout, owned browser/tunnel cleanup complete; ENTRY untouched. User requested STOP before19. | 2026-09-27 resumed19: actual demo selector admission, denied/unsupported GPS, isolated Zoe missing/invalid Setup cancel/retry and first profile persistence/reload partially PASS. False Location required race fixed; real stale null poll retest retained accepted point over12.4s. frontend-sync PASS15:24:34Z. One ENTRY-BLOCK19 window, Zoe snapshot retained. Block19 IN PROGRESS; counts unchanged. Evidence GROUP-LIFECYCLE-001-block19-entry-20260927.json. | 2026-09-27 18:22:19.1 HTTP complete incl invitation claim/first target profile/reload/replay and GPS-denied relogin; exact scoped cleanup. Avatar wait/error boundary and Setup disabled action verified.19.2 active:53/53 seed points accepted; Firebase config404 blocks real sign-in; pending-coordinate controls/Local remain. No count change. | User scope change2026-09-27: Firebase and actual external-client/provider-configuration checks moved to DEPLOY-EXTERNAL-CONFIG-001, DEFERRED/NOT RUN. They no longer gate Group19; continue demo pending-coordinate controls. | Block19 HTTP CLOSED in user-approved demo scope:53/53 seed points; two-account real login/profile-ext unsupported pending samples rejected with original points retained and per-account acknowledgement. Earlier failure/retry/claim/cleanup evidence retained.16/48 and16/29 closed;20 active. | 2026-09-27 block20 HTTP PASS/CLOSED: stored point with denied GPS and same-session reload; tracking OFF/save/reopen/ON; &lt;5km zero writes, &gt;=5km POST200; unsupported Paris POST403 retains accepted profile/cache/baseline/session and no popup; later eligible movement POST200. Independent Mongo point47.6747/19.0354 verified, normal logout then exact original47.5147/19.0354 restore, location snapshot removed. Evidence: GROUP-LIFECYCLE-001-block20-tracking-20260927.json. HTTP17/48 (35.42%), Lifecycle17/29 closed (1–13,17–20);21 active. Local NOT RUN; older contact/badge snapshots retained. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | 2026-09-27 block21 HTTP partial: seven audited menu surfaces, profile multiselect, pricing scope and card menus exercised; HU320/EN360/desktop1100 representative checks. Notification launcher overlap and forced-sheet desktop X repaired and replayed through existing frontend-sync. Assignment basket restaged with own Group fixture and exactly restored, no assignment/share/checkout commit. Checkout optional-item menu remains NOT RUN because selected real event/date combinations returned no available slots; suitable own checkpoint required. Do not mark full21 closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP17/48 and Lifecycle17/29 unchanged. | 2026-09-27 block21 HTTP PASS/CLOSED: final checkout optional-card control used its own versioned Group slot fixture. Native pointer selected/reverted optional item; mobile X remained reachable and closed only the sheet with parent dialogs/scroll retained; desktop title/no mobile X PASS. No checkout writes; draft discarded. Exact restore-sharing completed and original contact/badge snapshots retained. Together with the recorded seven menu surfaces, profile/price controls and HU/EN smoke,21 is closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP18/48 (37.50%), Lifecycle18/29 (1–13,17–21);22 active. Local NOT RUN. | 2026-09-27 block22 HTTP PASS/CLOSED: Design Circle UI create/edit/delete persisted Base asset ownership; Main/Design Circle/Seattle Friends inventory and immediate asset counters match, event counters remain separate. Real response-stage delayed long-poll released after deletion did not resurrect count; no page reload. Own scoped fixture public Asset booked to an inaccessible Language Lab event remains in Explore (UI + three-profile authenticated reads); own/private/non-friend controls absent, foreign Event/private Asset details withheld with empty HTTP200. Event Explore UI changes with workspace. Existing Group chat preparation and tools fixtures exactly restored; no chat share submitted. Evidence GROUP-LIFECYCLE-001-block22-tools-20260927.json. HTTP19/48 (39.58%), Lifecycle19/29 (1–13,17–22);23 active. Local NOT RUN. | 2026-09-27 block23 HTTP PASS/CLOSED: independent Group Asset checkout captured HUF3200 on Design Circle payer; Maya Base reads the same stored payment as income, Base/other Group controls excluded. Real owner acceptance and payer refund request/recipient approval reversed HUF3200 on the same payer/recipient; one capture plus normal refund audit. Initial unknown provider-card fixture caused one failed attempt; repaired via snapshot-protected real provider card registration, not a manufactured payment. Card revoked and restore-sharing exactly verified. Base/Group Profile/Affiliate/API/history and bounded Feed/Impressions/Chats/Ticket scope smoke recorded; empty ticket views supported by account-scope/converter source review, no populated-ticket visual claim or exhaustive nested-screen sweep. Shared booking-row badge overlap fixed and watcher/mobile320/360/desktop1100 verified. Evidence GROUP-LIFECYCLE-001-block23-profile-payments-20260927.json. HTTP20/48 (41.67%), Lifecycle20/29 (1–13,17–23);24 next. Local NOT RUN.</t>

</xml_diff>

<commit_message>
group fix - scope
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -3337,7 +3337,7 @@
     <t>IN PROGRESS</t>
   </si>
   <si>
-    <t>IN PROGRESS: HTTP Lifecycle21/29 closed (1–13,17–24); Group overall21/48 (43.75%).24 authorization repair verified by19 Java tests, E2E excluded by user;25 next.</t>
+    <t>IN PROGRESS: HTTP Lifecycle21/29 closed (1–13,17–24); Group overall21/48 (43.75%).25 active: layout and API key branch PASS; notification account scope/live counters and confirmation wording remain.</t>
   </si>
   <si>
     <t>31 focused backend moderation/chat/counter tests PASS (2026-09-25): separate scope settings, authority/foreign IDs, persisted pending count and idempotence, worker, Group support access/filter/unread. Earlier 15 filter/invitation tests PASS (2026-09-24). Frontend/backend dev watchers compiled. Full local/UI/HTTP journey NOT RUN. Profile selection correction: 21 focused Java tests PASS (2026-09-25); profile-load parameter, read-only restore, accepted-membership authority, failed-load non-commit, invite activation and removal. Added frontend HTTP parameter/retry unit cases; not executed separately from the running build watcher. | 2026-09-26: 105 focused backend tests PASS and 47 frontend tests PASS, covering explore boundaries, Base-only asset API key, contact repository account resolution and ticket account aggregation. These unit results do not close the manual local/HTTP journey. | My Tools follow-up (2026-09-26): 40 focused frontend tests PASS; 1 backend stored menu-counter test PASS. Account ownership/store/counters and stale-poll checks covered; browser journey NOT RUN. | Scope follow-up (2026-09-26): 195 backend and 32 frontend focused tests PASS. Payment payer/recipient query identity, account contacts, group event authorization and ticket scanner covered; manual local/HTTP journey NOT RUN. | Overlay navigation (2026-09-26): 27 focused frontend tests PASS; no real-device/Router/Firebase journey claimed. MCP Go race tests and image 1.3.0 initialization/discovery PASS; six generated schemas match OpenAPI. Help source parity PASS. | 2026-09-26: 13 focused frontend checks passed: popup/category/distance (5), local membership/notification lifecycle (5), workspace scopes and stale polls (3). Existing dev watchers compiled frontend/backend; added Java regression cases not run. No full-flow PASS.</t>
@@ -3346,7 +3346,7 @@
     <t>25 notifications and scoped API keys from own baseline; fixtures restored.24 direct-actor fix passed19 Java tests; no post-fix security E2E per user.</t>
   </si>
   <si>
-    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup. | 2026-09-27 block11 CLOSED: approved-only contact invitations/denials, retained overlays, recipient messages/unread reset, phone/share nesting, EN desktop/HU mobile; exact fixture restore PASS; after-contacts savepoint resume12. Evidence GROUP-LIFECYCLE-001-block11-contacts-20260927.json. | 2026-09-27 block12 CLOSED: selection limits including nested/mobile; contact consent cancellation/failure/retry/decisions, pagination/search, private methods, same chat/persistence and delayed group/account switch PASS. Exact contacts restore and after-contacts verification PASS; after-contact-controls captured resume13. Evidence GROUP-LIFECYCLE-001-block12-controls-20260927.json. | 2026-09-27 block13 CLOSED: empty HU/EN calendar notices retain blurred parent and produce no download; positive ICS download and libical import four events PASS. Desktop calendar UI NOT RUN. Blocks14–16 partial evidence retained in per-block JSON; no replay of completed subchecks. | 2026-09-27 block17 CLOSED for user-agreed HTTP Help/native anonymous MCP scope: current Codex conversation directly invoked MyScoutee topic list/read successfully. MCP connection UI create/reload/secret-hide/revoke also verified. No private OAuth or Local PASS claimed. Block18 X/Back and rapid reopen checks passed; remaining checks continue. | 2026-09-27 block18 CLOSED: physical Android native-Back defect fixed in shared overlay history owner; nested Back, X/Back, rapid reopen, busy refusal, desktop Forward/Router/reload and unchanged rating dock verified. Existing frontend-sync PASS05:46:29Z; unit specs not rerun. Evidence GROUP-LIFECYCLE-001-block18-20260927.json. Normal phone logout, owned browser/tunnel cleanup complete; ENTRY untouched. User requested STOP before19. | 2026-09-27 resumed19: actual demo selector admission, denied/unsupported GPS, isolated Zoe missing/invalid Setup cancel/retry and first profile persistence/reload partially PASS. False Location required race fixed; real stale null poll retest retained accepted point over12.4s. frontend-sync PASS15:24:34Z. One ENTRY-BLOCK19 window, Zoe snapshot retained. Block19 IN PROGRESS; counts unchanged. Evidence GROUP-LIFECYCLE-001-block19-entry-20260927.json. | 2026-09-27 18:22:19.1 HTTP complete incl invitation claim/first target profile/reload/replay and GPS-denied relogin; exact scoped cleanup. Avatar wait/error boundary and Setup disabled action verified.19.2 active:53/53 seed points accepted; Firebase config404 blocks real sign-in; pending-coordinate controls/Local remain. No count change. | User scope change2026-09-27: Firebase and actual external-client/provider-configuration checks moved to DEPLOY-EXTERNAL-CONFIG-001, DEFERRED/NOT RUN. They no longer gate Group19; continue demo pending-coordinate controls. | Block19 HTTP CLOSED in user-approved demo scope:53/53 seed points; two-account real login/profile-ext unsupported pending samples rejected with original points retained and per-account acknowledgement. Earlier failure/retry/claim/cleanup evidence retained.16/48 and16/29 closed;20 active. | 2026-09-27 block20 HTTP PASS/CLOSED: stored point with denied GPS and same-session reload; tracking OFF/save/reopen/ON; &lt;5km zero writes, &gt;=5km POST200; unsupported Paris POST403 retains accepted profile/cache/baseline/session and no popup; later eligible movement POST200. Independent Mongo point47.6747/19.0354 verified, normal logout then exact original47.5147/19.0354 restore, location snapshot removed. Evidence: GROUP-LIFECYCLE-001-block20-tracking-20260927.json. HTTP17/48 (35.42%), Lifecycle17/29 closed (1–13,17–20);21 active. Local NOT RUN; older contact/badge snapshots retained. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | 2026-09-27 block21 HTTP partial: seven audited menu surfaces, profile multiselect, pricing scope and card menus exercised; HU320/EN360/desktop1100 representative checks. Notification launcher overlap and forced-sheet desktop X repaired and replayed through existing frontend-sync. Assignment basket restaged with own Group fixture and exactly restored, no assignment/share/checkout commit. Checkout optional-item menu remains NOT RUN because selected real event/date combinations returned no available slots; suitable own checkpoint required. Do not mark full21 closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP17/48 and Lifecycle17/29 unchanged. | 2026-09-27 block21 HTTP PASS/CLOSED: final checkout optional-card control used its own versioned Group slot fixture. Native pointer selected/reverted optional item; mobile X remained reachable and closed only the sheet with parent dialogs/scroll retained; desktop title/no mobile X PASS. No checkout writes; draft discarded. Exact restore-sharing completed and original contact/badge snapshots retained. Together with the recorded seven menu surfaces, profile/price controls and HU/EN smoke,21 is closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP18/48 (37.50%), Lifecycle18/29 (1–13,17–21);22 active. Local NOT RUN. | 2026-09-27 block22 HTTP PASS/CLOSED: Design Circle UI create/edit/delete persisted Base asset ownership; Main/Design Circle/Seattle Friends inventory and immediate asset counters match, event counters remain separate. Real response-stage delayed long-poll released after deletion did not resurrect count; no page reload. Own scoped fixture public Asset booked to an inaccessible Language Lab event remains in Explore (UI + three-profile authenticated reads); own/private/non-friend controls absent, foreign Event/private Asset details withheld with empty HTTP200. Event Explore UI changes with workspace. Existing Group chat preparation and tools fixtures exactly restored; no chat share submitted. Evidence GROUP-LIFECYCLE-001-block22-tools-20260927.json. HTTP19/48 (39.58%), Lifecycle19/29 (1–13,17–22);23 active. Local NOT RUN. | 2026-09-27 block23 HTTP PASS/CLOSED: independent Group Asset checkout captured HUF3200 on Design Circle payer; Maya Base reads the same stored payment as income, Base/other Group controls excluded. Real owner acceptance and payer refund request/recipient approval reversed HUF3200 on the same payer/recipient; one capture plus normal refund audit. Initial unknown provider-card fixture caused one failed attempt; repaired via snapshot-protected real provider card registration, not a manufactured payment. Card revoked and restore-sharing exactly verified. Base/Group Profile/Affiliate/API/history and bounded Feed/Impressions/Chats/Ticket scope smoke recorded; empty ticket views supported by account-scope/converter source review, no populated-ticket visual claim or exhaustive nested-screen sweep. Shared booking-row badge overlap fixed and watcher/mobile320/360/desktop1100 verified. Evidence GROUP-LIFECYCLE-001-block23-profile-payments-20260927.json. HTTP20/48 (41.67%), Lifecycle20/29 (1–13,17–23);24 next. Local NOT RUN. | 2026-09-27 block24 HTTP checklist scope PASS/CLOSED: own contact snapshot; Group Create contact candidate account resolution repaired, eight real candidates returned. Saved contact request/reject/re-request/approve passed; one Base-account conversation, same senders and read receipts under Main/Design Circle; delayed old-account HTTP response did not replace the new account contact list. Contact snapshot restored exactly. Independent free resource fixture: account-owned Asset assigned by the participating Design Circle profile; persisted request retained that participant profile. Base/Seattle Friends subjects without target Event membership returned403. Assets remain usable from any workspace; authority comes from target Event/group membership. Both Base- and Group-held tickets visible from all three workspaces; scanner rejected forged actor bodies from Base/Seattle and accepted authenticated Design Circle despite Base body, persisted correct usedByUserId and attendance. No saved contacts meant zero Event invite candidates despite prior-met profiles. Exact restore-sharing PASS. Shared empty-state spans full grid; user-requested entire contact headline row removed without replacement, watcher/UI verified. Extra forged resource-subject probe under optional-auth dev policy is separately recorded as unproven authenticated-policy boundary, not a security PASS. Evidence GROUP-LIFECYCLE-001-block24-account-contacts-20260927.json. HTTP21/48 (43.75%), Lifecycle21/29 (1–13,17–24);25 next. Local NOT RUN. | Correction:24 closure superseded by reopened forged-resource-actor repair; user requested Java verification without E2E. | 2026-09-27 block24 authorization correction and closure: user explicitly required direct forged-actor assignment rejection, then requested Java verification and excluded E2E. Reopened premature closure; removed optional-auth/demo bypass from resource-assignment submit/manage checks, using authenticated caller and existing policies. Added demo forged-subject/no-write, anonymous and valid-admin regressions; updated obsolete anonymous dev acceptance. Existing main watcher compile/restart PASS20:33:41 local. 19 focused JUnit authorization/resource-service tests PASS (zero skips/failures), reusing existing main outputs and cached test dependencies; no second main build/Gradle/server and no post-fix browser/E2E replay. Valid accepted member/admin and parent Event/generated-group assignment remain allowed; missing membership/forged actor rejected before writes.24 now closed on prior HTTP lifecycle plus this user-approved Java-only repair verification. HTTP21/48, Lifecycle21/29;25 next.24 fixtures and temporary25 notification snapshot were exactly restored.</t>
+    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup. | 2026-09-27 block11 CLOSED: approved-only contact invitations/denials, retained overlays, recipient messages/unread reset, phone/share nesting, EN desktop/HU mobile; exact fixture restore PASS; after-contacts savepoint resume12. Evidence GROUP-LIFECYCLE-001-block11-contacts-20260927.json. | 2026-09-27 block12 CLOSED: selection limits including nested/mobile; contact consent cancellation/failure/retry/decisions, pagination/search, private methods, same chat/persistence and delayed group/account switch PASS. Exact contacts restore and after-contacts verification PASS; after-contact-controls captured resume13. Evidence GROUP-LIFECYCLE-001-block12-controls-20260927.json. | 2026-09-27 block13 CLOSED: empty HU/EN calendar notices retain blurred parent and produce no download; positive ICS download and libical import four events PASS. Desktop calendar UI NOT RUN. Blocks14–16 partial evidence retained in per-block JSON; no replay of completed subchecks. | 2026-09-27 block17 CLOSED for user-agreed HTTP Help/native anonymous MCP scope: current Codex conversation directly invoked MyScoutee topic list/read successfully. MCP connection UI create/reload/secret-hide/revoke also verified. No private OAuth or Local PASS claimed. Block18 X/Back and rapid reopen checks passed; remaining checks continue. | 2026-09-27 block18 CLOSED: physical Android native-Back defect fixed in shared overlay history owner; nested Back, X/Back, rapid reopen, busy refusal, desktop Forward/Router/reload and unchanged rating dock verified. Existing frontend-sync PASS05:46:29Z; unit specs not rerun. Evidence GROUP-LIFECYCLE-001-block18-20260927.json. Normal phone logout, owned browser/tunnel cleanup complete; ENTRY untouched. User requested STOP before19. | 2026-09-27 resumed19: actual demo selector admission, denied/unsupported GPS, isolated Zoe missing/invalid Setup cancel/retry and first profile persistence/reload partially PASS. False Location required race fixed; real stale null poll retest retained accepted point over12.4s. frontend-sync PASS15:24:34Z. One ENTRY-BLOCK19 window, Zoe snapshot retained. Block19 IN PROGRESS; counts unchanged. Evidence GROUP-LIFECYCLE-001-block19-entry-20260927.json. | 2026-09-27 18:22:19.1 HTTP complete incl invitation claim/first target profile/reload/replay and GPS-denied relogin; exact scoped cleanup. Avatar wait/error boundary and Setup disabled action verified.19.2 active:53/53 seed points accepted; Firebase config404 blocks real sign-in; pending-coordinate controls/Local remain. No count change. | User scope change2026-09-27: Firebase and actual external-client/provider-configuration checks moved to DEPLOY-EXTERNAL-CONFIG-001, DEFERRED/NOT RUN. They no longer gate Group19; continue demo pending-coordinate controls. | Block19 HTTP CLOSED in user-approved demo scope:53/53 seed points; two-account real login/profile-ext unsupported pending samples rejected with original points retained and per-account acknowledgement. Earlier failure/retry/claim/cleanup evidence retained.16/48 and16/29 closed;20 active. | 2026-09-27 block20 HTTP PASS/CLOSED: stored point with denied GPS and same-session reload; tracking OFF/save/reopen/ON; &lt;5km zero writes, &gt;=5km POST200; unsupported Paris POST403 retains accepted profile/cache/baseline/session and no popup; later eligible movement POST200. Independent Mongo point47.6747/19.0354 verified, normal logout then exact original47.5147/19.0354 restore, location snapshot removed. Evidence: GROUP-LIFECYCLE-001-block20-tracking-20260927.json. HTTP17/48 (35.42%), Lifecycle17/29 closed (1–13,17–20);21 active. Local NOT RUN; older contact/badge snapshots retained. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | 2026-09-27 block21 HTTP partial: seven audited menu surfaces, profile multiselect, pricing scope and card menus exercised; HU320/EN360/desktop1100 representative checks. Notification launcher overlap and forced-sheet desktop X repaired and replayed through existing frontend-sync. Assignment basket restaged with own Group fixture and exactly restored, no assignment/share/checkout commit. Checkout optional-item menu remains NOT RUN because selected real event/date combinations returned no available slots; suitable own checkpoint required. Do not mark full21 closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP17/48 and Lifecycle17/29 unchanged. | 2026-09-27 block21 HTTP PASS/CLOSED: final checkout optional-card control used its own versioned Group slot fixture. Native pointer selected/reverted optional item; mobile X remained reachable and closed only the sheet with parent dialogs/scroll retained; desktop title/no mobile X PASS. No checkout writes; draft discarded. Exact restore-sharing completed and original contact/badge snapshots retained. Together with the recorded seven menu surfaces, profile/price controls and HU/EN smoke,21 is closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP18/48 (37.50%), Lifecycle18/29 (1–13,17–21);22 active. Local NOT RUN. | 2026-09-27 block22 HTTP PASS/CLOSED: Design Circle UI create/edit/delete persisted Base asset ownership; Main/Design Circle/Seattle Friends inventory and immediate asset counters match, event counters remain separate. Real response-stage delayed long-poll released after deletion did not resurrect count; no page reload. Own scoped fixture public Asset booked to an inaccessible Language Lab event remains in Explore (UI + three-profile authenticated reads); own/private/non-friend controls absent, foreign Event/private Asset details withheld with empty HTTP200. Event Explore UI changes with workspace. Existing Group chat preparation and tools fixtures exactly restored; no chat share submitted. Evidence GROUP-LIFECYCLE-001-block22-tools-20260927.json. HTTP19/48 (39.58%), Lifecycle19/29 (1–13,17–22);23 active. Local NOT RUN. | 2026-09-27 block23 HTTP PASS/CLOSED: independent Group Asset checkout captured HUF3200 on Design Circle payer; Maya Base reads the same stored payment as income, Base/other Group controls excluded. Real owner acceptance and payer refund request/recipient approval reversed HUF3200 on the same payer/recipient; one capture plus normal refund audit. Initial unknown provider-card fixture caused one failed attempt; repaired via snapshot-protected real provider card registration, not a manufactured payment. Card revoked and restore-sharing exactly verified. Base/Group Profile/Affiliate/API/history and bounded Feed/Impressions/Chats/Ticket scope smoke recorded; empty ticket views supported by account-scope/converter source review, no populated-ticket visual claim or exhaustive nested-screen sweep. Shared booking-row badge overlap fixed and watcher/mobile320/360/desktop1100 verified. Evidence GROUP-LIFECYCLE-001-block23-profile-payments-20260927.json. HTTP20/48 (41.67%), Lifecycle20/29 (1–13,17–23);24 next. Local NOT RUN. | 2026-09-27 block24 HTTP checklist scope PASS/CLOSED: own contact snapshot; Group Create contact candidate account resolution repaired, eight real candidates returned. Saved contact request/reject/re-request/approve passed; one Base-account conversation, same senders and read receipts under Main/Design Circle; delayed old-account HTTP response did not replace the new account contact list. Contact snapshot restored exactly. Independent free resource fixture: account-owned Asset assigned by the participating Design Circle profile; persisted request retained that participant profile. Base/Seattle Friends subjects without target Event membership returned403. Assets remain usable from any workspace; authority comes from target Event/group membership. Both Base- and Group-held tickets visible from all three workspaces; scanner rejected forged actor bodies from Base/Seattle and accepted authenticated Design Circle despite Base body, persisted correct usedByUserId and attendance. No saved contacts meant zero Event invite candidates despite prior-met profiles. Exact restore-sharing PASS. Shared empty-state spans full grid; user-requested entire contact headline row removed without replacement, watcher/UI verified. Extra forged resource-subject probe under optional-auth dev policy is separately recorded as unproven authenticated-policy boundary, not a security PASS. Evidence GROUP-LIFECYCLE-001-block24-account-contacts-20260927.json. HTTP21/48 (43.75%), Lifecycle21/29 (1–13,17–24);25 next. Local NOT RUN. | Correction:24 closure superseded by reopened forged-resource-actor repair; user requested Java verification without E2E. | 2026-09-27 block24 authorization correction and closure: user explicitly required direct forged-actor assignment rejection, then requested Java verification and excluded E2E. Reopened premature closure; removed optional-auth/demo bypass from resource-assignment submit/manage checks, using authenticated caller and existing policies. Added demo forged-subject/no-write, anonymous and valid-admin regressions; updated obsolete anonymous dev acceptance. Existing main watcher compile/restart PASS20:33:41 local. 19 focused JUnit authorization/resource-service tests PASS (zero skips/failures), reusing existing main outputs and cached test dependencies; no second main build/Gradle/server and no post-fix browser/E2E replay. Valid accepted member/admin and parent Event/generated-group assignment remain allowed; missing membership/forged actor rejected before writes.24 now closed on prior HTTP lifecycle plus this user-approved Java-only repair verification. HTTP21/48, Lifecycle21/29;25 next.24 fixtures and temporary25 notification snapshot were exactly restored. | 2026-09-27 block25 partial PASS: EN320/360/1100 and HU320 notification layout verified; remaining account notification/live-counter branch not yet executed. UI-issued Base and Photo Walks API keys used while Seattle Friends selected: Base asset and Photo Walks event created under their issuing profiles; Group JSON/multipart asset requests returned403 both from Seattle Friends and after Base selection, without created assets/external-ID mappings. Authentication filter rejects before image-controller ingestion; separate object-store inventory was not captured. Real UI Leave group caused Group key403; Base key Revoke caused401. Exact versioned restore-profile-api PASS, membership restored, generated resources/mappings/dependents and the newly created affiliate link removed; old keys retained. Shared menu checkmark moved before badges in all three list item variants; watcher PASS18:52:18.930Z and actual checked/unchecked rows share badge right edge336.125px at360px viewport. Evidence GROUP-LIFECYCLE-001-block25-notifications-api-20260927.json.25 remains IN PROGRESS for notification account scope/live counters and confirmation wording; HTTP21/48 and Lifecycle21/29 unchanged.</t>
   </si>
   <si>
     <t>180/420</t>

</xml_diff>

<commit_message>
group fix - ticket
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -3337,16 +3337,16 @@
     <t>IN PROGRESS</t>
   </si>
   <si>
-    <t>IN PROGRESS: HTTP Lifecycle21/29 closed (1–13,17–24); Group overall21/48 (43.75%).25 active: layout and API key branch PASS; notification account scope/live counters and confirmation wording remain.</t>
+    <t>IN PROGRESS: HTTP Lifecycle22/29 closed (1–13,17–25); Group overall22/48 (45.83%).26 active: Admin grants and responsibility lifecycle.</t>
   </si>
   <si>
     <t>31 focused backend moderation/chat/counter tests PASS (2026-09-25): separate scope settings, authority/foreign IDs, persisted pending count and idempotence, worker, Group support access/filter/unread. Earlier 15 filter/invitation tests PASS (2026-09-24). Frontend/backend dev watchers compiled. Full local/UI/HTTP journey NOT RUN. Profile selection correction: 21 focused Java tests PASS (2026-09-25); profile-load parameter, read-only restore, accepted-membership authority, failed-load non-commit, invite activation and removal. Added frontend HTTP parameter/retry unit cases; not executed separately from the running build watcher. | 2026-09-26: 105 focused backend tests PASS and 47 frontend tests PASS, covering explore boundaries, Base-only asset API key, contact repository account resolution and ticket account aggregation. These unit results do not close the manual local/HTTP journey. | My Tools follow-up (2026-09-26): 40 focused frontend tests PASS; 1 backend stored menu-counter test PASS. Account ownership/store/counters and stale-poll checks covered; browser journey NOT RUN. | Scope follow-up (2026-09-26): 195 backend and 32 frontend focused tests PASS. Payment payer/recipient query identity, account contacts, group event authorization and ticket scanner covered; manual local/HTTP journey NOT RUN. | Overlay navigation (2026-09-26): 27 focused frontend tests PASS; no real-device/Router/Firebase journey claimed. MCP Go race tests and image 1.3.0 initialization/discovery PASS; six generated schemas match OpenAPI. Help source parity PASS. | 2026-09-26: 13 focused frontend checks passed: popup/category/distance (5), local membership/notification lifecycle (5), workspace scopes and stale polls (3). Existing dev watchers compiled frontend/backend; added Java regression cases not run. No full-flow PASS.</t>
   </si>
   <si>
-    <t>25 notifications and scoped API keys from own baseline; fixtures restored.24 direct-actor fix passed19 Java tests; no post-fix security E2E per user.</t>
-  </si>
-  <si>
-    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup. | 2026-09-27 block11 CLOSED: approved-only contact invitations/denials, retained overlays, recipient messages/unread reset, phone/share nesting, EN desktop/HU mobile; exact fixture restore PASS; after-contacts savepoint resume12. Evidence GROUP-LIFECYCLE-001-block11-contacts-20260927.json. | 2026-09-27 block12 CLOSED: selection limits including nested/mobile; contact consent cancellation/failure/retry/decisions, pagination/search, private methods, same chat/persistence and delayed group/account switch PASS. Exact contacts restore and after-contacts verification PASS; after-contact-controls captured resume13. Evidence GROUP-LIFECYCLE-001-block12-controls-20260927.json. | 2026-09-27 block13 CLOSED: empty HU/EN calendar notices retain blurred parent and produce no download; positive ICS download and libical import four events PASS. Desktop calendar UI NOT RUN. Blocks14–16 partial evidence retained in per-block JSON; no replay of completed subchecks. | 2026-09-27 block17 CLOSED for user-agreed HTTP Help/native anonymous MCP scope: current Codex conversation directly invoked MyScoutee topic list/read successfully. MCP connection UI create/reload/secret-hide/revoke also verified. No private OAuth or Local PASS claimed. Block18 X/Back and rapid reopen checks passed; remaining checks continue. | 2026-09-27 block18 CLOSED: physical Android native-Back defect fixed in shared overlay history owner; nested Back, X/Back, rapid reopen, busy refusal, desktop Forward/Router/reload and unchanged rating dock verified. Existing frontend-sync PASS05:46:29Z; unit specs not rerun. Evidence GROUP-LIFECYCLE-001-block18-20260927.json. Normal phone logout, owned browser/tunnel cleanup complete; ENTRY untouched. User requested STOP before19. | 2026-09-27 resumed19: actual demo selector admission, denied/unsupported GPS, isolated Zoe missing/invalid Setup cancel/retry and first profile persistence/reload partially PASS. False Location required race fixed; real stale null poll retest retained accepted point over12.4s. frontend-sync PASS15:24:34Z. One ENTRY-BLOCK19 window, Zoe snapshot retained. Block19 IN PROGRESS; counts unchanged. Evidence GROUP-LIFECYCLE-001-block19-entry-20260927.json. | 2026-09-27 18:22:19.1 HTTP complete incl invitation claim/first target profile/reload/replay and GPS-denied relogin; exact scoped cleanup. Avatar wait/error boundary and Setup disabled action verified.19.2 active:53/53 seed points accepted; Firebase config404 blocks real sign-in; pending-coordinate controls/Local remain. No count change. | User scope change2026-09-27: Firebase and actual external-client/provider-configuration checks moved to DEPLOY-EXTERNAL-CONFIG-001, DEFERRED/NOT RUN. They no longer gate Group19; continue demo pending-coordinate controls. | Block19 HTTP CLOSED in user-approved demo scope:53/53 seed points; two-account real login/profile-ext unsupported pending samples rejected with original points retained and per-account acknowledgement. Earlier failure/retry/claim/cleanup evidence retained.16/48 and16/29 closed;20 active. | 2026-09-27 block20 HTTP PASS/CLOSED: stored point with denied GPS and same-session reload; tracking OFF/save/reopen/ON; &lt;5km zero writes, &gt;=5km POST200; unsupported Paris POST403 retains accepted profile/cache/baseline/session and no popup; later eligible movement POST200. Independent Mongo point47.6747/19.0354 verified, normal logout then exact original47.5147/19.0354 restore, location snapshot removed. Evidence: GROUP-LIFECYCLE-001-block20-tracking-20260927.json. HTTP17/48 (35.42%), Lifecycle17/29 closed (1–13,17–20);21 active. Local NOT RUN; older contact/badge snapshots retained. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | 2026-09-27 block21 HTTP partial: seven audited menu surfaces, profile multiselect, pricing scope and card menus exercised; HU320/EN360/desktop1100 representative checks. Notification launcher overlap and forced-sheet desktop X repaired and replayed through existing frontend-sync. Assignment basket restaged with own Group fixture and exactly restored, no assignment/share/checkout commit. Checkout optional-item menu remains NOT RUN because selected real event/date combinations returned no available slots; suitable own checkpoint required. Do not mark full21 closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP17/48 and Lifecycle17/29 unchanged. | 2026-09-27 block21 HTTP PASS/CLOSED: final checkout optional-card control used its own versioned Group slot fixture. Native pointer selected/reverted optional item; mobile X remained reachable and closed only the sheet with parent dialogs/scroll retained; desktop title/no mobile X PASS. No checkout writes; draft discarded. Exact restore-sharing completed and original contact/badge snapshots retained. Together with the recorded seven menu surfaces, profile/price controls and HU/EN smoke,21 is closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP18/48 (37.50%), Lifecycle18/29 (1–13,17–21);22 active. Local NOT RUN. | 2026-09-27 block22 HTTP PASS/CLOSED: Design Circle UI create/edit/delete persisted Base asset ownership; Main/Design Circle/Seattle Friends inventory and immediate asset counters match, event counters remain separate. Real response-stage delayed long-poll released after deletion did not resurrect count; no page reload. Own scoped fixture public Asset booked to an inaccessible Language Lab event remains in Explore (UI + three-profile authenticated reads); own/private/non-friend controls absent, foreign Event/private Asset details withheld with empty HTTP200. Event Explore UI changes with workspace. Existing Group chat preparation and tools fixtures exactly restored; no chat share submitted. Evidence GROUP-LIFECYCLE-001-block22-tools-20260927.json. HTTP19/48 (39.58%), Lifecycle19/29 (1–13,17–22);23 active. Local NOT RUN. | 2026-09-27 block23 HTTP PASS/CLOSED: independent Group Asset checkout captured HUF3200 on Design Circle payer; Maya Base reads the same stored payment as income, Base/other Group controls excluded. Real owner acceptance and payer refund request/recipient approval reversed HUF3200 on the same payer/recipient; one capture plus normal refund audit. Initial unknown provider-card fixture caused one failed attempt; repaired via snapshot-protected real provider card registration, not a manufactured payment. Card revoked and restore-sharing exactly verified. Base/Group Profile/Affiliate/API/history and bounded Feed/Impressions/Chats/Ticket scope smoke recorded; empty ticket views supported by account-scope/converter source review, no populated-ticket visual claim or exhaustive nested-screen sweep. Shared booking-row badge overlap fixed and watcher/mobile320/360/desktop1100 verified. Evidence GROUP-LIFECYCLE-001-block23-profile-payments-20260927.json. HTTP20/48 (41.67%), Lifecycle20/29 (1–13,17–23);24 next. Local NOT RUN. | 2026-09-27 block24 HTTP checklist scope PASS/CLOSED: own contact snapshot; Group Create contact candidate account resolution repaired, eight real candidates returned. Saved contact request/reject/re-request/approve passed; one Base-account conversation, same senders and read receipts under Main/Design Circle; delayed old-account HTTP response did not replace the new account contact list. Contact snapshot restored exactly. Independent free resource fixture: account-owned Asset assigned by the participating Design Circle profile; persisted request retained that participant profile. Base/Seattle Friends subjects without target Event membership returned403. Assets remain usable from any workspace; authority comes from target Event/group membership. Both Base- and Group-held tickets visible from all three workspaces; scanner rejected forged actor bodies from Base/Seattle and accepted authenticated Design Circle despite Base body, persisted correct usedByUserId and attendance. No saved contacts meant zero Event invite candidates despite prior-met profiles. Exact restore-sharing PASS. Shared empty-state spans full grid; user-requested entire contact headline row removed without replacement, watcher/UI verified. Extra forged resource-subject probe under optional-auth dev policy is separately recorded as unproven authenticated-policy boundary, not a security PASS. Evidence GROUP-LIFECYCLE-001-block24-account-contacts-20260927.json. HTTP21/48 (43.75%), Lifecycle21/29 (1–13,17–24);25 next. Local NOT RUN. | Correction:24 closure superseded by reopened forged-resource-actor repair; user requested Java verification without E2E. | 2026-09-27 block24 authorization correction and closure: user explicitly required direct forged-actor assignment rejection, then requested Java verification and excluded E2E. Reopened premature closure; removed optional-auth/demo bypass from resource-assignment submit/manage checks, using authenticated caller and existing policies. Added demo forged-subject/no-write, anonymous and valid-admin regressions; updated obsolete anonymous dev acceptance. Existing main watcher compile/restart PASS20:33:41 local. 19 focused JUnit authorization/resource-service tests PASS (zero skips/failures), reusing existing main outputs and cached test dependencies; no second main build/Gradle/server and no post-fix browser/E2E replay. Valid accepted member/admin and parent Event/generated-group assignment remain allowed; missing membership/forged actor rejected before writes.24 now closed on prior HTTP lifecycle plus this user-approved Java-only repair verification. HTTP21/48, Lifecycle21/29;25 next.24 fixtures and temporary25 notification snapshot were exactly restored. | 2026-09-27 block25 partial PASS: EN320/360/1100 and HU320 notification layout verified; remaining account notification/live-counter branch not yet executed. UI-issued Base and Photo Walks API keys used while Seattle Friends selected: Base asset and Photo Walks event created under their issuing profiles; Group JSON/multipart asset requests returned403 both from Seattle Friends and after Base selection, without created assets/external-ID mappings. Authentication filter rejects before image-controller ingestion; separate object-store inventory was not captured. Real UI Leave group caused Group key403; Base key Revoke caused401. Exact versioned restore-profile-api PASS, membership restored, generated resources/mappings/dependents and the newly created affiliate link removed; old keys retained. Shared menu checkmark moved before badges in all three list item variants; watcher PASS18:52:18.930Z and actual checked/unchecked rows share badge right edge336.125px at360px viewport. Evidence GROUP-LIFECYCLE-001-block25-notifications-api-20260927.json.25 remains IN PROGRESS for notification account scope/live counters and confirmation wording; HTTP21/48 and Lifecycle21/29 unchanged.</t>
+    <t>Execute26 from independent Admin fixture; retain14–16 partial. After whole testcase, remove evidence-proven duplicates from Group Isolation and audit remaining deployment-dependent NOT RUN scope.</t>
+  </si>
+  <si>
+    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup. | 2026-09-27 block11 CLOSED: approved-only contact invitations/denials, retained overlays, recipient messages/unread reset, phone/share nesting, EN desktop/HU mobile; exact fixture restore PASS; after-contacts savepoint resume12. Evidence GROUP-LIFECYCLE-001-block11-contacts-20260927.json. | 2026-09-27 block12 CLOSED: selection limits including nested/mobile; contact consent cancellation/failure/retry/decisions, pagination/search, private methods, same chat/persistence and delayed group/account switch PASS. Exact contacts restore and after-contacts verification PASS; after-contact-controls captured resume13. Evidence GROUP-LIFECYCLE-001-block12-controls-20260927.json. | 2026-09-27 block13 CLOSED: empty HU/EN calendar notices retain blurred parent and produce no download; positive ICS download and libical import four events PASS. Desktop calendar UI NOT RUN. Blocks14–16 partial evidence retained in per-block JSON; no replay of completed subchecks. | 2026-09-27 block17 CLOSED for user-agreed HTTP Help/native anonymous MCP scope: current Codex conversation directly invoked MyScoutee topic list/read successfully. MCP connection UI create/reload/secret-hide/revoke also verified. No private OAuth or Local PASS claimed. Block18 X/Back and rapid reopen checks passed; remaining checks continue. | 2026-09-27 block18 CLOSED: physical Android native-Back defect fixed in shared overlay history owner; nested Back, X/Back, rapid reopen, busy refusal, desktop Forward/Router/reload and unchanged rating dock verified. Existing frontend-sync PASS05:46:29Z; unit specs not rerun. Evidence GROUP-LIFECYCLE-001-block18-20260927.json. Normal phone logout, owned browser/tunnel cleanup complete; ENTRY untouched. User requested STOP before19. | 2026-09-27 resumed19: actual demo selector admission, denied/unsupported GPS, isolated Zoe missing/invalid Setup cancel/retry and first profile persistence/reload partially PASS. False Location required race fixed; real stale null poll retest retained accepted point over12.4s. frontend-sync PASS15:24:34Z. One ENTRY-BLOCK19 window, Zoe snapshot retained. Block19 IN PROGRESS; counts unchanged. Evidence GROUP-LIFECYCLE-001-block19-entry-20260927.json. | 2026-09-27 18:22:19.1 HTTP complete incl invitation claim/first target profile/reload/replay and GPS-denied relogin; exact scoped cleanup. Avatar wait/error boundary and Setup disabled action verified.19.2 active:53/53 seed points accepted; Firebase config404 blocks real sign-in; pending-coordinate controls/Local remain. No count change. | User scope change2026-09-27: Firebase and actual external-client/provider-configuration checks moved to DEPLOY-EXTERNAL-CONFIG-001, DEFERRED/NOT RUN. They no longer gate Group19; continue demo pending-coordinate controls. | Block19 HTTP CLOSED in user-approved demo scope:53/53 seed points; two-account real login/profile-ext unsupported pending samples rejected with original points retained and per-account acknowledgement. Earlier failure/retry/claim/cleanup evidence retained.16/48 and16/29 closed;20 active. | 2026-09-27 block20 HTTP PASS/CLOSED: stored point with denied GPS and same-session reload; tracking OFF/save/reopen/ON; &lt;5km zero writes, &gt;=5km POST200; unsupported Paris POST403 retains accepted profile/cache/baseline/session and no popup; later eligible movement POST200. Independent Mongo point47.6747/19.0354 verified, normal logout then exact original47.5147/19.0354 restore, location snapshot removed. Evidence: GROUP-LIFECYCLE-001-block20-tracking-20260927.json. HTTP17/48 (35.42%), Lifecycle17/29 closed (1–13,17–20);21 active. Local NOT RUN; older contact/badge snapshots retained. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | 2026-09-27 block21 HTTP partial: seven audited menu surfaces, profile multiselect, pricing scope and card menus exercised; HU320/EN360/desktop1100 representative checks. Notification launcher overlap and forced-sheet desktop X repaired and replayed through existing frontend-sync. Assignment basket restaged with own Group fixture and exactly restored, no assignment/share/checkout commit. Checkout optional-item menu remains NOT RUN because selected real event/date combinations returned no available slots; suitable own checkpoint required. Do not mark full21 closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP17/48 and Lifecycle17/29 unchanged. | 2026-09-27 block21 HTTP PASS/CLOSED: final checkout optional-card control used its own versioned Group slot fixture. Native pointer selected/reverted optional item; mobile X remained reachable and closed only the sheet with parent dialogs/scroll retained; desktop title/no mobile X PASS. No checkout writes; draft discarded. Exact restore-sharing completed and original contact/badge snapshots retained. Together with the recorded seven menu surfaces, profile/price controls and HU/EN smoke,21 is closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP18/48 (37.50%), Lifecycle18/29 (1–13,17–21);22 active. Local NOT RUN. | 2026-09-27 block22 HTTP PASS/CLOSED: Design Circle UI create/edit/delete persisted Base asset ownership; Main/Design Circle/Seattle Friends inventory and immediate asset counters match, event counters remain separate. Real response-stage delayed long-poll released after deletion did not resurrect count; no page reload. Own scoped fixture public Asset booked to an inaccessible Language Lab event remains in Explore (UI + three-profile authenticated reads); own/private/non-friend controls absent, foreign Event/private Asset details withheld with empty HTTP200. Event Explore UI changes with workspace. Existing Group chat preparation and tools fixtures exactly restored; no chat share submitted. Evidence GROUP-LIFECYCLE-001-block22-tools-20260927.json. HTTP19/48 (39.58%), Lifecycle19/29 (1–13,17–22);23 active. Local NOT RUN. | 2026-09-27 block23 HTTP PASS/CLOSED: independent Group Asset checkout captured HUF3200 on Design Circle payer; Maya Base reads the same stored payment as income, Base/other Group controls excluded. Real owner acceptance and payer refund request/recipient approval reversed HUF3200 on the same payer/recipient; one capture plus normal refund audit. Initial unknown provider-card fixture caused one failed attempt; repaired via snapshot-protected real provider card registration, not a manufactured payment. Card revoked and restore-sharing exactly verified. Base/Group Profile/Affiliate/API/history and bounded Feed/Impressions/Chats/Ticket scope smoke recorded; empty ticket views supported by account-scope/converter source review, no populated-ticket visual claim or exhaustive nested-screen sweep. Shared booking-row badge overlap fixed and watcher/mobile320/360/desktop1100 verified. Evidence GROUP-LIFECYCLE-001-block23-profile-payments-20260927.json. HTTP20/48 (41.67%), Lifecycle20/29 (1–13,17–23);24 next. Local NOT RUN. | 2026-09-27 block24 HTTP checklist scope PASS/CLOSED: own contact snapshot; Group Create contact candidate account resolution repaired, eight real candidates returned. Saved contact request/reject/re-request/approve passed; one Base-account conversation, same senders and read receipts under Main/Design Circle; delayed old-account HTTP response did not replace the new account contact list. Contact snapshot restored exactly. Independent free resource fixture: account-owned Asset assigned by the participating Design Circle profile; persisted request retained that participant profile. Base/Seattle Friends subjects without target Event membership returned403. Assets remain usable from any workspace; authority comes from target Event/group membership. Both Base- and Group-held tickets visible from all three workspaces; scanner rejected forged actor bodies from Base/Seattle and accepted authenticated Design Circle despite Base body, persisted correct usedByUserId and attendance. No saved contacts meant zero Event invite candidates despite prior-met profiles. Exact restore-sharing PASS. Shared empty-state spans full grid; user-requested entire contact headline row removed without replacement, watcher/UI verified. Extra forged resource-subject probe under optional-auth dev policy is separately recorded as unproven authenticated-policy boundary, not a security PASS. Evidence GROUP-LIFECYCLE-001-block24-account-contacts-20260927.json. HTTP21/48 (43.75%), Lifecycle21/29 (1–13,17–24);25 next. Local NOT RUN. | Correction:24 closure superseded by reopened forged-resource-actor repair; user requested Java verification without E2E. | 2026-09-27 block24 authorization correction and closure: user explicitly required direct forged-actor assignment rejection, then requested Java verification and excluded E2E. Reopened premature closure; removed optional-auth/demo bypass from resource-assignment submit/manage checks, using authenticated caller and existing policies. Added demo forged-subject/no-write, anonymous and valid-admin regressions; updated obsolete anonymous dev acceptance. Existing main watcher compile/restart PASS20:33:41 local. 19 focused JUnit authorization/resource-service tests PASS (zero skips/failures), reusing existing main outputs and cached test dependencies; no second main build/Gradle/server and no post-fix browser/E2E replay. Valid accepted member/admin and parent Event/generated-group assignment remain allowed; missing membership/forged actor rejected before writes.24 now closed on prior HTTP lifecycle plus this user-approved Java-only repair verification. HTTP21/48, Lifecycle21/29;25 next.24 fixtures and temporary25 notification snapshot were exactly restored. | 2026-09-27 block25 partial PASS: EN320/360/1100 and HU320 notification layout verified; remaining account notification/live-counter branch not yet executed. UI-issued Base and Photo Walks API keys used while Seattle Friends selected: Base asset and Photo Walks event created under their issuing profiles; Group JSON/multipart asset requests returned403 both from Seattle Friends and after Base selection, without created assets/external-ID mappings. Authentication filter rejects before image-controller ingestion; separate object-store inventory was not captured. Real UI Leave group caused Group key403; Base key Revoke caused401. Exact versioned restore-profile-api PASS, membership restored, generated resources/mappings/dependents and the newly created affiliate link removed; old keys retained. Shared menu checkmark moved before badges in all three list item variants; watcher PASS18:52:18.930Z and actual checked/unchecked rows share badge right edge336.125px at360px viewport. Evidence GROUP-LIFECYCLE-001-block25-notifications-api-20260927.json.25 remains IN PROGRESS for notification account scope/live counters and confirmation wording; HTTP21/48 and Lifecycle21/29 unchanged. | 2026-09-27 block25 HTTP PASS/CLOSED: notification layout and API-key scope evidence retained; versioned group notification inputs with actual read mutations verified All/Base/group filtering and account counter23→22→21 across Design/Seattle/Base. Original fixture counter drift recorded separately; aligned prerequisite before assertions, exactly restored afterward. Missing notification group label repaired in existing source subtitle. Real contact request/cancel/approve drove pending1→0 and account approval notification visible from Seattle; own snapshot restored. Independent two-group ticket inputs returned2 in Base/A/B; real Seattle Leave event canceled then confirmed, ticketD/member suppressed and both account ticket counters1, one Design ticket in all profiles. User-requested ticket group label added to existing metadata line; watcher/mobile PASS. Confirmation source audit99 objects/82 EN-HU keys plus bounded runtime/cancellation/320px HU check recorded separately; not every dialog executed, no extra unit runner. Exact temporary fixture/dependent cleanup PASS. Evidence block25-notifications-api-20260927.json and block25-confirmation-audit-20260927.json. HTTP22/48 (45.83%), Lifecycle22/29 (1–13,17–25);26 active. Local NOT RUN.</t>
   </si>
   <si>
     <t>180/420</t>

</xml_diff>

<commit_message>
group fix - group management
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -3343,10 +3343,10 @@
     <t>31 focused backend moderation/chat/counter tests PASS (2026-09-25): separate scope settings, authority/foreign IDs, persisted pending count and idempotence, worker, Group support access/filter/unread. Earlier 15 filter/invitation tests PASS (2026-09-24). Frontend/backend dev watchers compiled. Full local/UI/HTTP journey NOT RUN. Profile selection correction: 21 focused Java tests PASS (2026-09-25); profile-load parameter, read-only restore, accepted-membership authority, failed-load non-commit, invite activation and removal. Added frontend HTTP parameter/retry unit cases; not executed separately from the running build watcher. | 2026-09-26: 105 focused backend tests PASS and 47 frontend tests PASS, covering explore boundaries, Base-only asset API key, contact repository account resolution and ticket account aggregation. These unit results do not close the manual local/HTTP journey. | My Tools follow-up (2026-09-26): 40 focused frontend tests PASS; 1 backend stored menu-counter test PASS. Account ownership/store/counters and stale-poll checks covered; browser journey NOT RUN. | Scope follow-up (2026-09-26): 195 backend and 32 frontend focused tests PASS. Payment payer/recipient query identity, account contacts, group event authorization and ticket scanner covered; manual local/HTTP journey NOT RUN. | Overlay navigation (2026-09-26): 27 focused frontend tests PASS; no real-device/Router/Firebase journey claimed. MCP Go race tests and image 1.3.0 initialization/discovery PASS; six generated schemas match OpenAPI. Help source parity PASS. | 2026-09-26: 13 focused frontend checks passed: popup/category/distance (5), local membership/notification lifecycle (5), workspace scopes and stale polls (3). Existing dev watchers compiled frontend/backend; added Java regression cases not run. No full-flow PASS.</t>
   </si>
   <si>
-    <t>Execute26 from independent Admin fixture; retain14–16 partial. After whole testcase, remove evidence-proven duplicates from Group Isolation and audit remaining deployment-dependent NOT RUN scope.</t>
-  </si>
-  <si>
-    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup. | 2026-09-27 block11 CLOSED: approved-only contact invitations/denials, retained overlays, recipient messages/unread reset, phone/share nesting, EN desktop/HU mobile; exact fixture restore PASS; after-contacts savepoint resume12. Evidence GROUP-LIFECYCLE-001-block11-contacts-20260927.json. | 2026-09-27 block12 CLOSED: selection limits including nested/mobile; contact consent cancellation/failure/retry/decisions, pagination/search, private methods, same chat/persistence and delayed group/account switch PASS. Exact contacts restore and after-contacts verification PASS; after-contact-controls captured resume13. Evidence GROUP-LIFECYCLE-001-block12-controls-20260927.json. | 2026-09-27 block13 CLOSED: empty HU/EN calendar notices retain blurred parent and produce no download; positive ICS download and libical import four events PASS. Desktop calendar UI NOT RUN. Blocks14–16 partial evidence retained in per-block JSON; no replay of completed subchecks. | 2026-09-27 block17 CLOSED for user-agreed HTTP Help/native anonymous MCP scope: current Codex conversation directly invoked MyScoutee topic list/read successfully. MCP connection UI create/reload/secret-hide/revoke also verified. No private OAuth or Local PASS claimed. Block18 X/Back and rapid reopen checks passed; remaining checks continue. | 2026-09-27 block18 CLOSED: physical Android native-Back defect fixed in shared overlay history owner; nested Back, X/Back, rapid reopen, busy refusal, desktop Forward/Router/reload and unchanged rating dock verified. Existing frontend-sync PASS05:46:29Z; unit specs not rerun. Evidence GROUP-LIFECYCLE-001-block18-20260927.json. Normal phone logout, owned browser/tunnel cleanup complete; ENTRY untouched. User requested STOP before19. | 2026-09-27 resumed19: actual demo selector admission, denied/unsupported GPS, isolated Zoe missing/invalid Setup cancel/retry and first profile persistence/reload partially PASS. False Location required race fixed; real stale null poll retest retained accepted point over12.4s. frontend-sync PASS15:24:34Z. One ENTRY-BLOCK19 window, Zoe snapshot retained. Block19 IN PROGRESS; counts unchanged. Evidence GROUP-LIFECYCLE-001-block19-entry-20260927.json. | 2026-09-27 18:22:19.1 HTTP complete incl invitation claim/first target profile/reload/replay and GPS-denied relogin; exact scoped cleanup. Avatar wait/error boundary and Setup disabled action verified.19.2 active:53/53 seed points accepted; Firebase config404 blocks real sign-in; pending-coordinate controls/Local remain. No count change. | User scope change2026-09-27: Firebase and actual external-client/provider-configuration checks moved to DEPLOY-EXTERNAL-CONFIG-001, DEFERRED/NOT RUN. They no longer gate Group19; continue demo pending-coordinate controls. | Block19 HTTP CLOSED in user-approved demo scope:53/53 seed points; two-account real login/profile-ext unsupported pending samples rejected with original points retained and per-account acknowledgement. Earlier failure/retry/claim/cleanup evidence retained.16/48 and16/29 closed;20 active. | 2026-09-27 block20 HTTP PASS/CLOSED: stored point with denied GPS and same-session reload; tracking OFF/save/reopen/ON; &lt;5km zero writes, &gt;=5km POST200; unsupported Paris POST403 retains accepted profile/cache/baseline/session and no popup; later eligible movement POST200. Independent Mongo point47.6747/19.0354 verified, normal logout then exact original47.5147/19.0354 restore, location snapshot removed. Evidence: GROUP-LIFECYCLE-001-block20-tracking-20260927.json. HTTP17/48 (35.42%), Lifecycle17/29 closed (1–13,17–20);21 active. Local NOT RUN; older contact/badge snapshots retained. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | 2026-09-27 block21 HTTP partial: seven audited menu surfaces, profile multiselect, pricing scope and card menus exercised; HU320/EN360/desktop1100 representative checks. Notification launcher overlap and forced-sheet desktop X repaired and replayed through existing frontend-sync. Assignment basket restaged with own Group fixture and exactly restored, no assignment/share/checkout commit. Checkout optional-item menu remains NOT RUN because selected real event/date combinations returned no available slots; suitable own checkpoint required. Do not mark full21 closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP17/48 and Lifecycle17/29 unchanged. | 2026-09-27 block21 HTTP PASS/CLOSED: final checkout optional-card control used its own versioned Group slot fixture. Native pointer selected/reverted optional item; mobile X remained reachable and closed only the sheet with parent dialogs/scroll retained; desktop title/no mobile X PASS. No checkout writes; draft discarded. Exact restore-sharing completed and original contact/badge snapshots retained. Together with the recorded seven menu surfaces, profile/price controls and HU/EN smoke,21 is closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP18/48 (37.50%), Lifecycle18/29 (1–13,17–21);22 active. Local NOT RUN. | 2026-09-27 block22 HTTP PASS/CLOSED: Design Circle UI create/edit/delete persisted Base asset ownership; Main/Design Circle/Seattle Friends inventory and immediate asset counters match, event counters remain separate. Real response-stage delayed long-poll released after deletion did not resurrect count; no page reload. Own scoped fixture public Asset booked to an inaccessible Language Lab event remains in Explore (UI + three-profile authenticated reads); own/private/non-friend controls absent, foreign Event/private Asset details withheld with empty HTTP200. Event Explore UI changes with workspace. Existing Group chat preparation and tools fixtures exactly restored; no chat share submitted. Evidence GROUP-LIFECYCLE-001-block22-tools-20260927.json. HTTP19/48 (39.58%), Lifecycle19/29 (1–13,17–22);23 active. Local NOT RUN. | 2026-09-27 block23 HTTP PASS/CLOSED: independent Group Asset checkout captured HUF3200 on Design Circle payer; Maya Base reads the same stored payment as income, Base/other Group controls excluded. Real owner acceptance and payer refund request/recipient approval reversed HUF3200 on the same payer/recipient; one capture plus normal refund audit. Initial unknown provider-card fixture caused one failed attempt; repaired via snapshot-protected real provider card registration, not a manufactured payment. Card revoked and restore-sharing exactly verified. Base/Group Profile/Affiliate/API/history and bounded Feed/Impressions/Chats/Ticket scope smoke recorded; empty ticket views supported by account-scope/converter source review, no populated-ticket visual claim or exhaustive nested-screen sweep. Shared booking-row badge overlap fixed and watcher/mobile320/360/desktop1100 verified. Evidence GROUP-LIFECYCLE-001-block23-profile-payments-20260927.json. HTTP20/48 (41.67%), Lifecycle20/29 (1–13,17–23);24 next. Local NOT RUN. | 2026-09-27 block24 HTTP checklist scope PASS/CLOSED: own contact snapshot; Group Create contact candidate account resolution repaired, eight real candidates returned. Saved contact request/reject/re-request/approve passed; one Base-account conversation, same senders and read receipts under Main/Design Circle; delayed old-account HTTP response did not replace the new account contact list. Contact snapshot restored exactly. Independent free resource fixture: account-owned Asset assigned by the participating Design Circle profile; persisted request retained that participant profile. Base/Seattle Friends subjects without target Event membership returned403. Assets remain usable from any workspace; authority comes from target Event/group membership. Both Base- and Group-held tickets visible from all three workspaces; scanner rejected forged actor bodies from Base/Seattle and accepted authenticated Design Circle despite Base body, persisted correct usedByUserId and attendance. No saved contacts meant zero Event invite candidates despite prior-met profiles. Exact restore-sharing PASS. Shared empty-state spans full grid; user-requested entire contact headline row removed without replacement, watcher/UI verified. Extra forged resource-subject probe under optional-auth dev policy is separately recorded as unproven authenticated-policy boundary, not a security PASS. Evidence GROUP-LIFECYCLE-001-block24-account-contacts-20260927.json. HTTP21/48 (43.75%), Lifecycle21/29 (1–13,17–24);25 next. Local NOT RUN. | Correction:24 closure superseded by reopened forged-resource-actor repair; user requested Java verification without E2E. | 2026-09-27 block24 authorization correction and closure: user explicitly required direct forged-actor assignment rejection, then requested Java verification and excluded E2E. Reopened premature closure; removed optional-auth/demo bypass from resource-assignment submit/manage checks, using authenticated caller and existing policies. Added demo forged-subject/no-write, anonymous and valid-admin regressions; updated obsolete anonymous dev acceptance. Existing main watcher compile/restart PASS20:33:41 local. 19 focused JUnit authorization/resource-service tests PASS (zero skips/failures), reusing existing main outputs and cached test dependencies; no second main build/Gradle/server and no post-fix browser/E2E replay. Valid accepted member/admin and parent Event/generated-group assignment remain allowed; missing membership/forged actor rejected before writes.24 now closed on prior HTTP lifecycle plus this user-approved Java-only repair verification. HTTP21/48, Lifecycle21/29;25 next.24 fixtures and temporary25 notification snapshot were exactly restored. | 2026-09-27 block25 partial PASS: EN320/360/1100 and HU320 notification layout verified; remaining account notification/live-counter branch not yet executed. UI-issued Base and Photo Walks API keys used while Seattle Friends selected: Base asset and Photo Walks event created under their issuing profiles; Group JSON/multipart asset requests returned403 both from Seattle Friends and after Base selection, without created assets/external-ID mappings. Authentication filter rejects before image-controller ingestion; separate object-store inventory was not captured. Real UI Leave group caused Group key403; Base key Revoke caused401. Exact versioned restore-profile-api PASS, membership restored, generated resources/mappings/dependents and the newly created affiliate link removed; old keys retained. Shared menu checkmark moved before badges in all three list item variants; watcher PASS18:52:18.930Z and actual checked/unchecked rows share badge right edge336.125px at360px viewport. Evidence GROUP-LIFECYCLE-001-block25-notifications-api-20260927.json.25 remains IN PROGRESS for notification account scope/live counters and confirmation wording; HTTP21/48 and Lifecycle21/29 unchanged. | 2026-09-27 block25 HTTP PASS/CLOSED: notification layout and API-key scope evidence retained; versioned group notification inputs with actual read mutations verified All/Base/group filtering and account counter23→22→21 across Design/Seattle/Base. Original fixture counter drift recorded separately; aligned prerequisite before assertions, exactly restored afterward. Missing notification group label repaired in existing source subtitle. Real contact request/cancel/approve drove pending1→0 and account approval notification visible from Seattle; own snapshot restored. Independent two-group ticket inputs returned2 in Base/A/B; real Seattle Leave event canceled then confirmed, ticketD/member suppressed and both account ticket counters1, one Design ticket in all profiles. User-requested ticket group label added to existing metadata line; watcher/mobile PASS. Confirmation source audit99 objects/82 EN-HU keys plus bounded runtime/cancellation/320px HU check recorded separately; not every dialog executed, no extra unit runner. Exact temporary fixture/dependent cleanup PASS. Evidence block25-notifications-api-20260927.json and block25-confirmation-audit-20260927.json. HTTP22/48 (45.83%), Lifecycle22/29 (1–13,17–25);26 active. Local NOT RUN.</t>
+    <t>Continue26.5 normal invitation return/fresh grant;26.6 final-member deletion; finish26.7–8 UI/notifications.26.1–4 verified; retain14–16 partial. Whole-case duplicate/deployment audit queued.</t>
+  </si>
+  <si>
+    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup. | 2026-09-27 block11 CLOSED: approved-only contact invitations/denials, retained overlays, recipient messages/unread reset, phone/share nesting, EN desktop/HU mobile; exact fixture restore PASS; after-contacts savepoint resume12. Evidence GROUP-LIFECYCLE-001-block11-contacts-20260927.json. | 2026-09-27 block12 CLOSED: selection limits including nested/mobile; contact consent cancellation/failure/retry/decisions, pagination/search, private methods, same chat/persistence and delayed group/account switch PASS. Exact contacts restore and after-contacts verification PASS; after-contact-controls captured resume13. Evidence GROUP-LIFECYCLE-001-block12-controls-20260927.json. | 2026-09-27 block13 CLOSED: empty HU/EN calendar notices retain blurred parent and produce no download; positive ICS download and libical import four events PASS. Desktop calendar UI NOT RUN. Blocks14–16 partial evidence retained in per-block JSON; no replay of completed subchecks. | 2026-09-27 block17 CLOSED for user-agreed HTTP Help/native anonymous MCP scope: current Codex conversation directly invoked MyScoutee topic list/read successfully. MCP connection UI create/reload/secret-hide/revoke also verified. No private OAuth or Local PASS claimed. Block18 X/Back and rapid reopen checks passed; remaining checks continue. | 2026-09-27 block18 CLOSED: physical Android native-Back defect fixed in shared overlay history owner; nested Back, X/Back, rapid reopen, busy refusal, desktop Forward/Router/reload and unchanged rating dock verified. Existing frontend-sync PASS05:46:29Z; unit specs not rerun. Evidence GROUP-LIFECYCLE-001-block18-20260927.json. Normal phone logout, owned browser/tunnel cleanup complete; ENTRY untouched. User requested STOP before19. | 2026-09-27 resumed19: actual demo selector admission, denied/unsupported GPS, isolated Zoe missing/invalid Setup cancel/retry and first profile persistence/reload partially PASS. False Location required race fixed; real stale null poll retest retained accepted point over12.4s. frontend-sync PASS15:24:34Z. One ENTRY-BLOCK19 window, Zoe snapshot retained. Block19 IN PROGRESS; counts unchanged. Evidence GROUP-LIFECYCLE-001-block19-entry-20260927.json. | 2026-09-27 18:22:19.1 HTTP complete incl invitation claim/first target profile/reload/replay and GPS-denied relogin; exact scoped cleanup. Avatar wait/error boundary and Setup disabled action verified.19.2 active:53/53 seed points accepted; Firebase config404 blocks real sign-in; pending-coordinate controls/Local remain. No count change. | User scope change2026-09-27: Firebase and actual external-client/provider-configuration checks moved to DEPLOY-EXTERNAL-CONFIG-001, DEFERRED/NOT RUN. They no longer gate Group19; continue demo pending-coordinate controls. | Block19 HTTP CLOSED in user-approved demo scope:53/53 seed points; two-account real login/profile-ext unsupported pending samples rejected with original points retained and per-account acknowledgement. Earlier failure/retry/claim/cleanup evidence retained.16/48 and16/29 closed;20 active. | 2026-09-27 block20 HTTP PASS/CLOSED: stored point with denied GPS and same-session reload; tracking OFF/save/reopen/ON; &lt;5km zero writes, &gt;=5km POST200; unsupported Paris POST403 retains accepted profile/cache/baseline/session and no popup; later eligible movement POST200. Independent Mongo point47.6747/19.0354 verified, normal logout then exact original47.5147/19.0354 restore, location snapshot removed. Evidence: GROUP-LIFECYCLE-001-block20-tracking-20260927.json. HTTP17/48 (35.42%), Lifecycle17/29 closed (1–13,17–20);21 active. Local NOT RUN; older contact/badge snapshots retained. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | 2026-09-27 block21 HTTP partial: seven audited menu surfaces, profile multiselect, pricing scope and card menus exercised; HU320/EN360/desktop1100 representative checks. Notification launcher overlap and forced-sheet desktop X repaired and replayed through existing frontend-sync. Assignment basket restaged with own Group fixture and exactly restored, no assignment/share/checkout commit. Checkout optional-item menu remains NOT RUN because selected real event/date combinations returned no available slots; suitable own checkpoint required. Do not mark full21 closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP17/48 and Lifecycle17/29 unchanged. | 2026-09-27 block21 HTTP PASS/CLOSED: final checkout optional-card control used its own versioned Group slot fixture. Native pointer selected/reverted optional item; mobile X remained reachable and closed only the sheet with parent dialogs/scroll retained; desktop title/no mobile X PASS. No checkout writes; draft discarded. Exact restore-sharing completed and original contact/badge snapshots retained. Together with the recorded seven menu surfaces, profile/price controls and HU/EN smoke,21 is closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP18/48 (37.50%), Lifecycle18/29 (1–13,17–21);22 active. Local NOT RUN. | 2026-09-27 block22 HTTP PASS/CLOSED: Design Circle UI create/edit/delete persisted Base asset ownership; Main/Design Circle/Seattle Friends inventory and immediate asset counters match, event counters remain separate. Real response-stage delayed long-poll released after deletion did not resurrect count; no page reload. Own scoped fixture public Asset booked to an inaccessible Language Lab event remains in Explore (UI + three-profile authenticated reads); own/private/non-friend controls absent, foreign Event/private Asset details withheld with empty HTTP200. Event Explore UI changes with workspace. Existing Group chat preparation and tools fixtures exactly restored; no chat share submitted. Evidence GROUP-LIFECYCLE-001-block22-tools-20260927.json. HTTP19/48 (39.58%), Lifecycle19/29 (1–13,17–22);23 active. Local NOT RUN. | 2026-09-27 block23 HTTP PASS/CLOSED: independent Group Asset checkout captured HUF3200 on Design Circle payer; Maya Base reads the same stored payment as income, Base/other Group controls excluded. Real owner acceptance and payer refund request/recipient approval reversed HUF3200 on the same payer/recipient; one capture plus normal refund audit. Initial unknown provider-card fixture caused one failed attempt; repaired via snapshot-protected real provider card registration, not a manufactured payment. Card revoked and restore-sharing exactly verified. Base/Group Profile/Affiliate/API/history and bounded Feed/Impressions/Chats/Ticket scope smoke recorded; empty ticket views supported by account-scope/converter source review, no populated-ticket visual claim or exhaustive nested-screen sweep. Shared booking-row badge overlap fixed and watcher/mobile320/360/desktop1100 verified. Evidence GROUP-LIFECYCLE-001-block23-profile-payments-20260927.json. HTTP20/48 (41.67%), Lifecycle20/29 (1–13,17–23);24 next. Local NOT RUN. | 2026-09-27 block24 HTTP checklist scope PASS/CLOSED: own contact snapshot; Group Create contact candidate account resolution repaired, eight real candidates returned. Saved contact request/reject/re-request/approve passed; one Base-account conversation, same senders and read receipts under Main/Design Circle; delayed old-account HTTP response did not replace the new account contact list. Contact snapshot restored exactly. Independent free resource fixture: account-owned Asset assigned by the participating Design Circle profile; persisted request retained that participant profile. Base/Seattle Friends subjects without target Event membership returned403. Assets remain usable from any workspace; authority comes from target Event/group membership. Both Base- and Group-held tickets visible from all three workspaces; scanner rejected forged actor bodies from Base/Seattle and accepted authenticated Design Circle despite Base body, persisted correct usedByUserId and attendance. No saved contacts meant zero Event invite candidates despite prior-met profiles. Exact restore-sharing PASS. Shared empty-state spans full grid; user-requested entire contact headline row removed without replacement, watcher/UI verified. Extra forged resource-subject probe under optional-auth dev policy is separately recorded as unproven authenticated-policy boundary, not a security PASS. Evidence GROUP-LIFECYCLE-001-block24-account-contacts-20260927.json. HTTP21/48 (43.75%), Lifecycle21/29 (1–13,17–24);25 next. Local NOT RUN. | Correction:24 closure superseded by reopened forged-resource-actor repair; user requested Java verification without E2E. | 2026-09-27 block24 authorization correction and closure: user explicitly required direct forged-actor assignment rejection, then requested Java verification and excluded E2E. Reopened premature closure; removed optional-auth/demo bypass from resource-assignment submit/manage checks, using authenticated caller and existing policies. Added demo forged-subject/no-write, anonymous and valid-admin regressions; updated obsolete anonymous dev acceptance. Existing main watcher compile/restart PASS20:33:41 local. 19 focused JUnit authorization/resource-service tests PASS (zero skips/failures), reusing existing main outputs and cached test dependencies; no second main build/Gradle/server and no post-fix browser/E2E replay. Valid accepted member/admin and parent Event/generated-group assignment remain allowed; missing membership/forged actor rejected before writes.24 now closed on prior HTTP lifecycle plus this user-approved Java-only repair verification. HTTP21/48, Lifecycle21/29;25 next.24 fixtures and temporary25 notification snapshot were exactly restored. | 2026-09-27 block25 partial PASS: EN320/360/1100 and HU320 notification layout verified; remaining account notification/live-counter branch not yet executed. UI-issued Base and Photo Walks API keys used while Seattle Friends selected: Base asset and Photo Walks event created under their issuing profiles; Group JSON/multipart asset requests returned403 both from Seattle Friends and after Base selection, without created assets/external-ID mappings. Authentication filter rejects before image-controller ingestion; separate object-store inventory was not captured. Real UI Leave group caused Group key403; Base key Revoke caused401. Exact versioned restore-profile-api PASS, membership restored, generated resources/mappings/dependents and the newly created affiliate link removed; old keys retained. Shared menu checkmark moved before badges in all three list item variants; watcher PASS18:52:18.930Z and actual checked/unchecked rows share badge right edge336.125px at360px viewport. Evidence GROUP-LIFECYCLE-001-block25-notifications-api-20260927.json.25 remains IN PROGRESS for notification account scope/live counters and confirmation wording; HTTP21/48 and Lifecycle21/29 unchanged. | 2026-09-27 block25 HTTP PASS/CLOSED: notification layout and API-key scope evidence retained; versioned group notification inputs with actual read mutations verified All/Base/group filtering and account counter23→22→21 across Design/Seattle/Base. Original fixture counter drift recorded separately; aligned prerequisite before assertions, exactly restored afterward. Missing notification group label repaired in existing source subtitle. Real contact request/cancel/approve drove pending1→0 and account approval notification visible from Seattle; own snapshot restored. Independent two-group ticket inputs returned2 in Base/A/B; real Seattle Leave event canceled then confirmed, ticketD/member suppressed and both account ticket counters1, one Design ticket in all profiles. User-requested ticket group label added to existing metadata line; watcher/mobile PASS. Confirmation source audit99 objects/82 EN-HU keys plus bounded runtime/cancellation/320px HU check recorded separately; not every dialog executed, no extra unit runner. Exact temporary fixture/dependent cleanup PASS. Evidence block25-notifications-api-20260927.json and block25-confirmation-audit-20260927.json. HTTP22/48 (45.83%), Lifecycle22/29 (1–13,17–25);26 active. Local NOT RUN. | 2026-09-27 21:37: Block26.1–4 own HTTP execution: grants and revocations preserve provenance; Admin-first owner handover, ordinary-member fallback, sole-Admin step-down verified. Trash Restore returns former creator as Member; normal invitation return, last-member deletion and remaining notification/UI checks continue. Same-actor takeover retry200 is idempotent, competing403; pending fallback403/outsider404. See block26-admin-authority-20260927.json. Block26 remains IN PROGRESS.</t>
   </si>
   <si>
     <t>180/420</t>

</xml_diff>

<commit_message>
group fix - qa
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -3337,16 +3337,16 @@
     <t>IN PROGRESS</t>
   </si>
   <si>
-    <t>IN PROGRESS: HTTP Lifecycle22/29 closed (1–13,17–25); Group overall22/48 (45.83%).26 active: Admin grants and responsibility lifecycle.</t>
+    <t>IN PROGRESS: HTTP Lifecycle23/29 closed (1–13,17–26); Group overall23/48 (47.92%).27 active: role/editor presentation.</t>
   </si>
   <si>
     <t>31 focused backend moderation/chat/counter tests PASS (2026-09-25): separate scope settings, authority/foreign IDs, persisted pending count and idempotence, worker, Group support access/filter/unread. Earlier 15 filter/invitation tests PASS (2026-09-24). Frontend/backend dev watchers compiled. Full local/UI/HTTP journey NOT RUN. Profile selection correction: 21 focused Java tests PASS (2026-09-25); profile-load parameter, read-only restore, accepted-membership authority, failed-load non-commit, invite activation and removal. Added frontend HTTP parameter/retry unit cases; not executed separately from the running build watcher. | 2026-09-26: 105 focused backend tests PASS and 47 frontend tests PASS, covering explore boundaries, Base-only asset API key, contact repository account resolution and ticket account aggregation. These unit results do not close the manual local/HTTP journey. | My Tools follow-up (2026-09-26): 40 focused frontend tests PASS; 1 backend stored menu-counter test PASS. Account ownership/store/counters and stale-poll checks covered; browser journey NOT RUN. | Scope follow-up (2026-09-26): 195 backend and 32 frontend focused tests PASS. Payment payer/recipient query identity, account contacts, group event authorization and ticket scanner covered; manual local/HTTP journey NOT RUN. | Overlay navigation (2026-09-26): 27 focused frontend tests PASS; no real-device/Router/Firebase journey claimed. MCP Go race tests and image 1.3.0 initialization/discovery PASS; six generated schemas match OpenAPI. Help source parity PASS. | 2026-09-26: 13 focused frontend checks passed: popup/category/distance (5), local membership/notification lifecycle (5), workspace scopes and stale polls (3). Existing dev watchers compiled frontend/backend; added Java regression cases not run. No full-flow PASS.</t>
   </si>
   <si>
-    <t>Continue26.5 normal invitation return/fresh grant;26.6 final-member deletion; finish26.7–8 UI/notifications.26.1–4 verified; retain14–16 partial. Whole-case duplicate/deployment audit queued.</t>
-  </si>
-  <si>
-    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup. | 2026-09-27 block11 CLOSED: approved-only contact invitations/denials, retained overlays, recipient messages/unread reset, phone/share nesting, EN desktop/HU mobile; exact fixture restore PASS; after-contacts savepoint resume12. Evidence GROUP-LIFECYCLE-001-block11-contacts-20260927.json. | 2026-09-27 block12 CLOSED: selection limits including nested/mobile; contact consent cancellation/failure/retry/decisions, pagination/search, private methods, same chat/persistence and delayed group/account switch PASS. Exact contacts restore and after-contacts verification PASS; after-contact-controls captured resume13. Evidence GROUP-LIFECYCLE-001-block12-controls-20260927.json. | 2026-09-27 block13 CLOSED: empty HU/EN calendar notices retain blurred parent and produce no download; positive ICS download and libical import four events PASS. Desktop calendar UI NOT RUN. Blocks14–16 partial evidence retained in per-block JSON; no replay of completed subchecks. | 2026-09-27 block17 CLOSED for user-agreed HTTP Help/native anonymous MCP scope: current Codex conversation directly invoked MyScoutee topic list/read successfully. MCP connection UI create/reload/secret-hide/revoke also verified. No private OAuth or Local PASS claimed. Block18 X/Back and rapid reopen checks passed; remaining checks continue. | 2026-09-27 block18 CLOSED: physical Android native-Back defect fixed in shared overlay history owner; nested Back, X/Back, rapid reopen, busy refusal, desktop Forward/Router/reload and unchanged rating dock verified. Existing frontend-sync PASS05:46:29Z; unit specs not rerun. Evidence GROUP-LIFECYCLE-001-block18-20260927.json. Normal phone logout, owned browser/tunnel cleanup complete; ENTRY untouched. User requested STOP before19. | 2026-09-27 resumed19: actual demo selector admission, denied/unsupported GPS, isolated Zoe missing/invalid Setup cancel/retry and first profile persistence/reload partially PASS. False Location required race fixed; real stale null poll retest retained accepted point over12.4s. frontend-sync PASS15:24:34Z. One ENTRY-BLOCK19 window, Zoe snapshot retained. Block19 IN PROGRESS; counts unchanged. Evidence GROUP-LIFECYCLE-001-block19-entry-20260927.json. | 2026-09-27 18:22:19.1 HTTP complete incl invitation claim/first target profile/reload/replay and GPS-denied relogin; exact scoped cleanup. Avatar wait/error boundary and Setup disabled action verified.19.2 active:53/53 seed points accepted; Firebase config404 blocks real sign-in; pending-coordinate controls/Local remain. No count change. | User scope change2026-09-27: Firebase and actual external-client/provider-configuration checks moved to DEPLOY-EXTERNAL-CONFIG-001, DEFERRED/NOT RUN. They no longer gate Group19; continue demo pending-coordinate controls. | Block19 HTTP CLOSED in user-approved demo scope:53/53 seed points; two-account real login/profile-ext unsupported pending samples rejected with original points retained and per-account acknowledgement. Earlier failure/retry/claim/cleanup evidence retained.16/48 and16/29 closed;20 active. | 2026-09-27 block20 HTTP PASS/CLOSED: stored point with denied GPS and same-session reload; tracking OFF/save/reopen/ON; &lt;5km zero writes, &gt;=5km POST200; unsupported Paris POST403 retains accepted profile/cache/baseline/session and no popup; later eligible movement POST200. Independent Mongo point47.6747/19.0354 verified, normal logout then exact original47.5147/19.0354 restore, location snapshot removed. Evidence: GROUP-LIFECYCLE-001-block20-tracking-20260927.json. HTTP17/48 (35.42%), Lifecycle17/29 closed (1–13,17–20);21 active. Local NOT RUN; older contact/badge snapshots retained. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | 2026-09-27 block21 HTTP partial: seven audited menu surfaces, profile multiselect, pricing scope and card menus exercised; HU320/EN360/desktop1100 representative checks. Notification launcher overlap and forced-sheet desktop X repaired and replayed through existing frontend-sync. Assignment basket restaged with own Group fixture and exactly restored, no assignment/share/checkout commit. Checkout optional-item menu remains NOT RUN because selected real event/date combinations returned no available slots; suitable own checkpoint required. Do not mark full21 closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP17/48 and Lifecycle17/29 unchanged. | 2026-09-27 block21 HTTP PASS/CLOSED: final checkout optional-card control used its own versioned Group slot fixture. Native pointer selected/reverted optional item; mobile X remained reachable and closed only the sheet with parent dialogs/scroll retained; desktop title/no mobile X PASS. No checkout writes; draft discarded. Exact restore-sharing completed and original contact/badge snapshots retained. Together with the recorded seven menu surfaces, profile/price controls and HU/EN smoke,21 is closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP18/48 (37.50%), Lifecycle18/29 (1–13,17–21);22 active. Local NOT RUN. | 2026-09-27 block22 HTTP PASS/CLOSED: Design Circle UI create/edit/delete persisted Base asset ownership; Main/Design Circle/Seattle Friends inventory and immediate asset counters match, event counters remain separate. Real response-stage delayed long-poll released after deletion did not resurrect count; no page reload. Own scoped fixture public Asset booked to an inaccessible Language Lab event remains in Explore (UI + three-profile authenticated reads); own/private/non-friend controls absent, foreign Event/private Asset details withheld with empty HTTP200. Event Explore UI changes with workspace. Existing Group chat preparation and tools fixtures exactly restored; no chat share submitted. Evidence GROUP-LIFECYCLE-001-block22-tools-20260927.json. HTTP19/48 (39.58%), Lifecycle19/29 (1–13,17–22);23 active. Local NOT RUN. | 2026-09-27 block23 HTTP PASS/CLOSED: independent Group Asset checkout captured HUF3200 on Design Circle payer; Maya Base reads the same stored payment as income, Base/other Group controls excluded. Real owner acceptance and payer refund request/recipient approval reversed HUF3200 on the same payer/recipient; one capture plus normal refund audit. Initial unknown provider-card fixture caused one failed attempt; repaired via snapshot-protected real provider card registration, not a manufactured payment. Card revoked and restore-sharing exactly verified. Base/Group Profile/Affiliate/API/history and bounded Feed/Impressions/Chats/Ticket scope smoke recorded; empty ticket views supported by account-scope/converter source review, no populated-ticket visual claim or exhaustive nested-screen sweep. Shared booking-row badge overlap fixed and watcher/mobile320/360/desktop1100 verified. Evidence GROUP-LIFECYCLE-001-block23-profile-payments-20260927.json. HTTP20/48 (41.67%), Lifecycle20/29 (1–13,17–23);24 next. Local NOT RUN. | 2026-09-27 block24 HTTP checklist scope PASS/CLOSED: own contact snapshot; Group Create contact candidate account resolution repaired, eight real candidates returned. Saved contact request/reject/re-request/approve passed; one Base-account conversation, same senders and read receipts under Main/Design Circle; delayed old-account HTTP response did not replace the new account contact list. Contact snapshot restored exactly. Independent free resource fixture: account-owned Asset assigned by the participating Design Circle profile; persisted request retained that participant profile. Base/Seattle Friends subjects without target Event membership returned403. Assets remain usable from any workspace; authority comes from target Event/group membership. Both Base- and Group-held tickets visible from all three workspaces; scanner rejected forged actor bodies from Base/Seattle and accepted authenticated Design Circle despite Base body, persisted correct usedByUserId and attendance. No saved contacts meant zero Event invite candidates despite prior-met profiles. Exact restore-sharing PASS. Shared empty-state spans full grid; user-requested entire contact headline row removed without replacement, watcher/UI verified. Extra forged resource-subject probe under optional-auth dev policy is separately recorded as unproven authenticated-policy boundary, not a security PASS. Evidence GROUP-LIFECYCLE-001-block24-account-contacts-20260927.json. HTTP21/48 (43.75%), Lifecycle21/29 (1–13,17–24);25 next. Local NOT RUN. | Correction:24 closure superseded by reopened forged-resource-actor repair; user requested Java verification without E2E. | 2026-09-27 block24 authorization correction and closure: user explicitly required direct forged-actor assignment rejection, then requested Java verification and excluded E2E. Reopened premature closure; removed optional-auth/demo bypass from resource-assignment submit/manage checks, using authenticated caller and existing policies. Added demo forged-subject/no-write, anonymous and valid-admin regressions; updated obsolete anonymous dev acceptance. Existing main watcher compile/restart PASS20:33:41 local. 19 focused JUnit authorization/resource-service tests PASS (zero skips/failures), reusing existing main outputs and cached test dependencies; no second main build/Gradle/server and no post-fix browser/E2E replay. Valid accepted member/admin and parent Event/generated-group assignment remain allowed; missing membership/forged actor rejected before writes.24 now closed on prior HTTP lifecycle plus this user-approved Java-only repair verification. HTTP21/48, Lifecycle21/29;25 next.24 fixtures and temporary25 notification snapshot were exactly restored. | 2026-09-27 block25 partial PASS: EN320/360/1100 and HU320 notification layout verified; remaining account notification/live-counter branch not yet executed. UI-issued Base and Photo Walks API keys used while Seattle Friends selected: Base asset and Photo Walks event created under their issuing profiles; Group JSON/multipart asset requests returned403 both from Seattle Friends and after Base selection, without created assets/external-ID mappings. Authentication filter rejects before image-controller ingestion; separate object-store inventory was not captured. Real UI Leave group caused Group key403; Base key Revoke caused401. Exact versioned restore-profile-api PASS, membership restored, generated resources/mappings/dependents and the newly created affiliate link removed; old keys retained. Shared menu checkmark moved before badges in all three list item variants; watcher PASS18:52:18.930Z and actual checked/unchecked rows share badge right edge336.125px at360px viewport. Evidence GROUP-LIFECYCLE-001-block25-notifications-api-20260927.json.25 remains IN PROGRESS for notification account scope/live counters and confirmation wording; HTTP21/48 and Lifecycle21/29 unchanged. | 2026-09-27 block25 HTTP PASS/CLOSED: notification layout and API-key scope evidence retained; versioned group notification inputs with actual read mutations verified All/Base/group filtering and account counter23→22→21 across Design/Seattle/Base. Original fixture counter drift recorded separately; aligned prerequisite before assertions, exactly restored afterward. Missing notification group label repaired in existing source subtitle. Real contact request/cancel/approve drove pending1→0 and account approval notification visible from Seattle; own snapshot restored. Independent two-group ticket inputs returned2 in Base/A/B; real Seattle Leave event canceled then confirmed, ticketD/member suppressed and both account ticket counters1, one Design ticket in all profiles. User-requested ticket group label added to existing metadata line; watcher/mobile PASS. Confirmation source audit99 objects/82 EN-HU keys plus bounded runtime/cancellation/320px HU check recorded separately; not every dialog executed, no extra unit runner. Exact temporary fixture/dependent cleanup PASS. Evidence block25-notifications-api-20260927.json and block25-confirmation-audit-20260927.json. HTTP22/48 (45.83%), Lifecycle22/29 (1–13,17–25);26 active. Local NOT RUN. | 2026-09-27 21:37: Block26.1–4 own HTTP execution: grants and revocations preserve provenance; Admin-first owner handover, ordinary-member fallback, sole-Admin step-down verified. Trash Restore returns former creator as Member; normal invitation return, last-member deletion and remaining notification/UI checks continue. Same-actor takeover retry200 is idempotent, competing403; pending fallback403/outsider404. See block26-admin-authority-20260927.json. Block26 remains IN PROGRESS.</t>
+    <t>Execute27 role/roster/editor layout, then28 request boundaries and29 ordering. Retain14–16 partial; whole-case duplicate/deployment audit queued.</t>
+  </si>
+  <si>
+    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup. | 2026-09-27 block11 CLOSED: approved-only contact invitations/denials, retained overlays, recipient messages/unread reset, phone/share nesting, EN desktop/HU mobile; exact fixture restore PASS; after-contacts savepoint resume12. Evidence GROUP-LIFECYCLE-001-block11-contacts-20260927.json. | 2026-09-27 block12 CLOSED: selection limits including nested/mobile; contact consent cancellation/failure/retry/decisions, pagination/search, private methods, same chat/persistence and delayed group/account switch PASS. Exact contacts restore and after-contacts verification PASS; after-contact-controls captured resume13. Evidence GROUP-LIFECYCLE-001-block12-controls-20260927.json. | 2026-09-27 block13 CLOSED: empty HU/EN calendar notices retain blurred parent and produce no download; positive ICS download and libical import four events PASS. Desktop calendar UI NOT RUN. Blocks14–16 partial evidence retained in per-block JSON; no replay of completed subchecks. | 2026-09-27 block17 CLOSED for user-agreed HTTP Help/native anonymous MCP scope: current Codex conversation directly invoked MyScoutee topic list/read successfully. MCP connection UI create/reload/secret-hide/revoke also verified. No private OAuth or Local PASS claimed. Block18 X/Back and rapid reopen checks passed; remaining checks continue. | 2026-09-27 block18 CLOSED: physical Android native-Back defect fixed in shared overlay history owner; nested Back, X/Back, rapid reopen, busy refusal, desktop Forward/Router/reload and unchanged rating dock verified. Existing frontend-sync PASS05:46:29Z; unit specs not rerun. Evidence GROUP-LIFECYCLE-001-block18-20260927.json. Normal phone logout, owned browser/tunnel cleanup complete; ENTRY untouched. User requested STOP before19. | 2026-09-27 resumed19: actual demo selector admission, denied/unsupported GPS, isolated Zoe missing/invalid Setup cancel/retry and first profile persistence/reload partially PASS. False Location required race fixed; real stale null poll retest retained accepted point over12.4s. frontend-sync PASS15:24:34Z. One ENTRY-BLOCK19 window, Zoe snapshot retained. Block19 IN PROGRESS; counts unchanged. Evidence GROUP-LIFECYCLE-001-block19-entry-20260927.json. | 2026-09-27 18:22:19.1 HTTP complete incl invitation claim/first target profile/reload/replay and GPS-denied relogin; exact scoped cleanup. Avatar wait/error boundary and Setup disabled action verified.19.2 active:53/53 seed points accepted; Firebase config404 blocks real sign-in; pending-coordinate controls/Local remain. No count change. | User scope change2026-09-27: Firebase and actual external-client/provider-configuration checks moved to DEPLOY-EXTERNAL-CONFIG-001, DEFERRED/NOT RUN. They no longer gate Group19; continue demo pending-coordinate controls. | Block19 HTTP CLOSED in user-approved demo scope:53/53 seed points; two-account real login/profile-ext unsupported pending samples rejected with original points retained and per-account acknowledgement. Earlier failure/retry/claim/cleanup evidence retained.16/48 and16/29 closed;20 active. | 2026-09-27 block20 HTTP PASS/CLOSED: stored point with denied GPS and same-session reload; tracking OFF/save/reopen/ON; &lt;5km zero writes, &gt;=5km POST200; unsupported Paris POST403 retains accepted profile/cache/baseline/session and no popup; later eligible movement POST200. Independent Mongo point47.6747/19.0354 verified, normal logout then exact original47.5147/19.0354 restore, location snapshot removed. Evidence: GROUP-LIFECYCLE-001-block20-tracking-20260927.json. HTTP17/48 (35.42%), Lifecycle17/29 closed (1–13,17–20);21 active. Local NOT RUN; older contact/badge snapshots retained. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | 2026-09-27 block21 HTTP partial: seven audited menu surfaces, profile multiselect, pricing scope and card menus exercised; HU320/EN360/desktop1100 representative checks. Notification launcher overlap and forced-sheet desktop X repaired and replayed through existing frontend-sync. Assignment basket restaged with own Group fixture and exactly restored, no assignment/share/checkout commit. Checkout optional-item menu remains NOT RUN because selected real event/date combinations returned no available slots; suitable own checkpoint required. Do not mark full21 closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP17/48 and Lifecycle17/29 unchanged. | 2026-09-27 block21 HTTP PASS/CLOSED: final checkout optional-card control used its own versioned Group slot fixture. Native pointer selected/reverted optional item; mobile X remained reachable and closed only the sheet with parent dialogs/scroll retained; desktop title/no mobile X PASS. No checkout writes; draft discarded. Exact restore-sharing completed and original contact/badge snapshots retained. Together with the recorded seven menu surfaces, profile/price controls and HU/EN smoke,21 is closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP18/48 (37.50%), Lifecycle18/29 (1–13,17–21);22 active. Local NOT RUN. | 2026-09-27 block22 HTTP PASS/CLOSED: Design Circle UI create/edit/delete persisted Base asset ownership; Main/Design Circle/Seattle Friends inventory and immediate asset counters match, event counters remain separate. Real response-stage delayed long-poll released after deletion did not resurrect count; no page reload. Own scoped fixture public Asset booked to an inaccessible Language Lab event remains in Explore (UI + three-profile authenticated reads); own/private/non-friend controls absent, foreign Event/private Asset details withheld with empty HTTP200. Event Explore UI changes with workspace. Existing Group chat preparation and tools fixtures exactly restored; no chat share submitted. Evidence GROUP-LIFECYCLE-001-block22-tools-20260927.json. HTTP19/48 (39.58%), Lifecycle19/29 (1–13,17–22);23 active. Local NOT RUN. | 2026-09-27 block23 HTTP PASS/CLOSED: independent Group Asset checkout captured HUF3200 on Design Circle payer; Maya Base reads the same stored payment as income, Base/other Group controls excluded. Real owner acceptance and payer refund request/recipient approval reversed HUF3200 on the same payer/recipient; one capture plus normal refund audit. Initial unknown provider-card fixture caused one failed attempt; repaired via snapshot-protected real provider card registration, not a manufactured payment. Card revoked and restore-sharing exactly verified. Base/Group Profile/Affiliate/API/history and bounded Feed/Impressions/Chats/Ticket scope smoke recorded; empty ticket views supported by account-scope/converter source review, no populated-ticket visual claim or exhaustive nested-screen sweep. Shared booking-row badge overlap fixed and watcher/mobile320/360/desktop1100 verified. Evidence GROUP-LIFECYCLE-001-block23-profile-payments-20260927.json. HTTP20/48 (41.67%), Lifecycle20/29 (1–13,17–23);24 next. Local NOT RUN. | 2026-09-27 block24 HTTP checklist scope PASS/CLOSED: own contact snapshot; Group Create contact candidate account resolution repaired, eight real candidates returned. Saved contact request/reject/re-request/approve passed; one Base-account conversation, same senders and read receipts under Main/Design Circle; delayed old-account HTTP response did not replace the new account contact list. Contact snapshot restored exactly. Independent free resource fixture: account-owned Asset assigned by the participating Design Circle profile; persisted request retained that participant profile. Base/Seattle Friends subjects without target Event membership returned403. Assets remain usable from any workspace; authority comes from target Event/group membership. Both Base- and Group-held tickets visible from all three workspaces; scanner rejected forged actor bodies from Base/Seattle and accepted authenticated Design Circle despite Base body, persisted correct usedByUserId and attendance. No saved contacts meant zero Event invite candidates despite prior-met profiles. Exact restore-sharing PASS. Shared empty-state spans full grid; user-requested entire contact headline row removed without replacement, watcher/UI verified. Extra forged resource-subject probe under optional-auth dev policy is separately recorded as unproven authenticated-policy boundary, not a security PASS. Evidence GROUP-LIFECYCLE-001-block24-account-contacts-20260927.json. HTTP21/48 (43.75%), Lifecycle21/29 (1–13,17–24);25 next. Local NOT RUN. | Correction:24 closure superseded by reopened forged-resource-actor repair; user requested Java verification without E2E. | 2026-09-27 block24 authorization correction and closure: user explicitly required direct forged-actor assignment rejection, then requested Java verification and excluded E2E. Reopened premature closure; removed optional-auth/demo bypass from resource-assignment submit/manage checks, using authenticated caller and existing policies. Added demo forged-subject/no-write, anonymous and valid-admin regressions; updated obsolete anonymous dev acceptance. Existing main watcher compile/restart PASS20:33:41 local. 19 focused JUnit authorization/resource-service tests PASS (zero skips/failures), reusing existing main outputs and cached test dependencies; no second main build/Gradle/server and no post-fix browser/E2E replay. Valid accepted member/admin and parent Event/generated-group assignment remain allowed; missing membership/forged actor rejected before writes.24 now closed on prior HTTP lifecycle plus this user-approved Java-only repair verification. HTTP21/48, Lifecycle21/29;25 next.24 fixtures and temporary25 notification snapshot were exactly restored. | 2026-09-27 block25 partial PASS: EN320/360/1100 and HU320 notification layout verified; remaining account notification/live-counter branch not yet executed. UI-issued Base and Photo Walks API keys used while Seattle Friends selected: Base asset and Photo Walks event created under their issuing profiles; Group JSON/multipart asset requests returned403 both from Seattle Friends and after Base selection, without created assets/external-ID mappings. Authentication filter rejects before image-controller ingestion; separate object-store inventory was not captured. Real UI Leave group caused Group key403; Base key Revoke caused401. Exact versioned restore-profile-api PASS, membership restored, generated resources/mappings/dependents and the newly created affiliate link removed; old keys retained. Shared menu checkmark moved before badges in all three list item variants; watcher PASS18:52:18.930Z and actual checked/unchecked rows share badge right edge336.125px at360px viewport. Evidence GROUP-LIFECYCLE-001-block25-notifications-api-20260927.json.25 remains IN PROGRESS for notification account scope/live counters and confirmation wording; HTTP21/48 and Lifecycle21/29 unchanged. | 2026-09-27 block25 HTTP PASS/CLOSED: notification layout and API-key scope evidence retained; versioned group notification inputs with actual read mutations verified All/Base/group filtering and account counter23→22→21 across Design/Seattle/Base. Original fixture counter drift recorded separately; aligned prerequisite before assertions, exactly restored afterward. Missing notification group label repaired in existing source subtitle. Real contact request/cancel/approve drove pending1→0 and account approval notification visible from Seattle; own snapshot restored. Independent two-group ticket inputs returned2 in Base/A/B; real Seattle Leave event canceled then confirmed, ticketD/member suppressed and both account ticket counters1, one Design ticket in all profiles. User-requested ticket group label added to existing metadata line; watcher/mobile PASS. Confirmation source audit99 objects/82 EN-HU keys plus bounded runtime/cancellation/320px HU check recorded separately; not every dialog executed, no extra unit runner. Exact temporary fixture/dependent cleanup PASS. Evidence block25-notifications-api-20260927.json and block25-confirmation-audit-20260927.json. HTTP22/48 (45.83%), Lifecycle22/29 (1–13,17–25);26 active. Local NOT RUN. | 2026-09-27 21:37: Block26.1–4 own HTTP execution: grants and revocations preserve provenance; Admin-first owner handover, ordinary-member fallback, sole-Admin step-down verified. Trash Restore returns former creator as Member; normal invitation return, last-member deletion and remaining notification/UI checks continue. Same-actor takeover retry200 is idempotent, competing403; pending fallback403/outsider404. See block26-admin-authority-20260927.json. Block26 remains IN PROGRESS. | 2026-09-27 22:00: Block26 HTTP PASS/CLOSED. Own grants/revocations, Admin-first and ordinary-member fallback, sole-admin step-down, normal invite and Trash return, final-member deletion and user-corrected recovery verified. Corrected rule: Deleted card remains in Trash; any voluntarily departed Admin can restore group/responsibility, ordinary member has no Restore and direct restore/join404 until admin recovery; then Member Restore succeeds. Earlier departed Admin cancel/confirm and idempotent retry proven. Exact notification read/avatar173→172/group2→1 survives reload. Shared Deleted badge bottom-right and common X16px centered. Local25+store2+popup6+converter12 focused tests PASS (45 distinct), full Local browser NOT RUN; Java mapper spec added/not run separately. Existing dev watchers compiled, exact fixture cleanup PASS. HTTP23/48 (47.92%), Lifecycle23/29 (1–13,17–26);27 next. See block26-admin-authority-20260927.json.</t>
   </si>
   <si>
     <t>180/420</t>

</xml_diff>

<commit_message>
group fix - arrow
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -3343,10 +3343,10 @@
     <t>31 focused backend moderation/chat/counter tests PASS (2026-09-25): separate scope settings, authority/foreign IDs, persisted pending count and idempotence, worker, Group support access/filter/unread. Earlier 15 filter/invitation tests PASS (2026-09-24). Frontend/backend dev watchers compiled. Full local/UI/HTTP journey NOT RUN. Profile selection correction: 21 focused Java tests PASS (2026-09-25); profile-load parameter, read-only restore, accepted-membership authority, failed-load non-commit, invite activation and removal. Added frontend HTTP parameter/retry unit cases; not executed separately from the running build watcher. | 2026-09-26: 105 focused backend tests PASS and 47 frontend tests PASS, covering explore boundaries, Base-only asset API key, contact repository account resolution and ticket account aggregation. These unit results do not close the manual local/HTTP journey. | My Tools follow-up (2026-09-26): 40 focused frontend tests PASS; 1 backend stored menu-counter test PASS. Account ownership/store/counters and stale-poll checks covered; browser journey NOT RUN. | Scope follow-up (2026-09-26): 195 backend and 32 frontend focused tests PASS. Payment payer/recipient query identity, account contacts, group event authorization and ticket scanner covered; manual local/HTTP journey NOT RUN. | Overlay navigation (2026-09-26): 27 focused frontend tests PASS; no real-device/Router/Firebase journey claimed. MCP Go race tests and image 1.3.0 initialization/discovery PASS; six generated schemas match OpenAPI. Help source parity PASS. | 2026-09-26: 13 focused frontend checks passed: popup/category/distance (5), local membership/notification lifecycle (5), workspace scopes and stale polls (3). Existing dev watchers compiled frontend/backend; added Java regression cases not run. No full-flow PASS.</t>
   </si>
   <si>
-    <t>Execute27 role/roster/editor layout, then28 request boundaries and29 ordering. Retain14–16 partial; whole-case duplicate/deployment audit queued.</t>
-  </si>
-  <si>
-    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup. | 2026-09-27 block11 CLOSED: approved-only contact invitations/denials, retained overlays, recipient messages/unread reset, phone/share nesting, EN desktop/HU mobile; exact fixture restore PASS; after-contacts savepoint resume12. Evidence GROUP-LIFECYCLE-001-block11-contacts-20260927.json. | 2026-09-27 block12 CLOSED: selection limits including nested/mobile; contact consent cancellation/failure/retry/decisions, pagination/search, private methods, same chat/persistence and delayed group/account switch PASS. Exact contacts restore and after-contacts verification PASS; after-contact-controls captured resume13. Evidence GROUP-LIFECYCLE-001-block12-controls-20260927.json. | 2026-09-27 block13 CLOSED: empty HU/EN calendar notices retain blurred parent and produce no download; positive ICS download and libical import four events PASS. Desktop calendar UI NOT RUN. Blocks14–16 partial evidence retained in per-block JSON; no replay of completed subchecks. | 2026-09-27 block17 CLOSED for user-agreed HTTP Help/native anonymous MCP scope: current Codex conversation directly invoked MyScoutee topic list/read successfully. MCP connection UI create/reload/secret-hide/revoke also verified. No private OAuth or Local PASS claimed. Block18 X/Back and rapid reopen checks passed; remaining checks continue. | 2026-09-27 block18 CLOSED: physical Android native-Back defect fixed in shared overlay history owner; nested Back, X/Back, rapid reopen, busy refusal, desktop Forward/Router/reload and unchanged rating dock verified. Existing frontend-sync PASS05:46:29Z; unit specs not rerun. Evidence GROUP-LIFECYCLE-001-block18-20260927.json. Normal phone logout, owned browser/tunnel cleanup complete; ENTRY untouched. User requested STOP before19. | 2026-09-27 resumed19: actual demo selector admission, denied/unsupported GPS, isolated Zoe missing/invalid Setup cancel/retry and first profile persistence/reload partially PASS. False Location required race fixed; real stale null poll retest retained accepted point over12.4s. frontend-sync PASS15:24:34Z. One ENTRY-BLOCK19 window, Zoe snapshot retained. Block19 IN PROGRESS; counts unchanged. Evidence GROUP-LIFECYCLE-001-block19-entry-20260927.json. | 2026-09-27 18:22:19.1 HTTP complete incl invitation claim/first target profile/reload/replay and GPS-denied relogin; exact scoped cleanup. Avatar wait/error boundary and Setup disabled action verified.19.2 active:53/53 seed points accepted; Firebase config404 blocks real sign-in; pending-coordinate controls/Local remain. No count change. | User scope change2026-09-27: Firebase and actual external-client/provider-configuration checks moved to DEPLOY-EXTERNAL-CONFIG-001, DEFERRED/NOT RUN. They no longer gate Group19; continue demo pending-coordinate controls. | Block19 HTTP CLOSED in user-approved demo scope:53/53 seed points; two-account real login/profile-ext unsupported pending samples rejected with original points retained and per-account acknowledgement. Earlier failure/retry/claim/cleanup evidence retained.16/48 and16/29 closed;20 active. | 2026-09-27 block20 HTTP PASS/CLOSED: stored point with denied GPS and same-session reload; tracking OFF/save/reopen/ON; &lt;5km zero writes, &gt;=5km POST200; unsupported Paris POST403 retains accepted profile/cache/baseline/session and no popup; later eligible movement POST200. Independent Mongo point47.6747/19.0354 verified, normal logout then exact original47.5147/19.0354 restore, location snapshot removed. Evidence: GROUP-LIFECYCLE-001-block20-tracking-20260927.json. HTTP17/48 (35.42%), Lifecycle17/29 closed (1–13,17–20);21 active. Local NOT RUN; older contact/badge snapshots retained. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | 2026-09-27 block21 HTTP partial: seven audited menu surfaces, profile multiselect, pricing scope and card menus exercised; HU320/EN360/desktop1100 representative checks. Notification launcher overlap and forced-sheet desktop X repaired and replayed through existing frontend-sync. Assignment basket restaged with own Group fixture and exactly restored, no assignment/share/checkout commit. Checkout optional-item menu remains NOT RUN because selected real event/date combinations returned no available slots; suitable own checkpoint required. Do not mark full21 closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP17/48 and Lifecycle17/29 unchanged. | 2026-09-27 block21 HTTP PASS/CLOSED: final checkout optional-card control used its own versioned Group slot fixture. Native pointer selected/reverted optional item; mobile X remained reachable and closed only the sheet with parent dialogs/scroll retained; desktop title/no mobile X PASS. No checkout writes; draft discarded. Exact restore-sharing completed and original contact/badge snapshots retained. Together with the recorded seven menu surfaces, profile/price controls and HU/EN smoke,21 is closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP18/48 (37.50%), Lifecycle18/29 (1–13,17–21);22 active. Local NOT RUN. | 2026-09-27 block22 HTTP PASS/CLOSED: Design Circle UI create/edit/delete persisted Base asset ownership; Main/Design Circle/Seattle Friends inventory and immediate asset counters match, event counters remain separate. Real response-stage delayed long-poll released after deletion did not resurrect count; no page reload. Own scoped fixture public Asset booked to an inaccessible Language Lab event remains in Explore (UI + three-profile authenticated reads); own/private/non-friend controls absent, foreign Event/private Asset details withheld with empty HTTP200. Event Explore UI changes with workspace. Existing Group chat preparation and tools fixtures exactly restored; no chat share submitted. Evidence GROUP-LIFECYCLE-001-block22-tools-20260927.json. HTTP19/48 (39.58%), Lifecycle19/29 (1–13,17–22);23 active. Local NOT RUN. | 2026-09-27 block23 HTTP PASS/CLOSED: independent Group Asset checkout captured HUF3200 on Design Circle payer; Maya Base reads the same stored payment as income, Base/other Group controls excluded. Real owner acceptance and payer refund request/recipient approval reversed HUF3200 on the same payer/recipient; one capture plus normal refund audit. Initial unknown provider-card fixture caused one failed attempt; repaired via snapshot-protected real provider card registration, not a manufactured payment. Card revoked and restore-sharing exactly verified. Base/Group Profile/Affiliate/API/history and bounded Feed/Impressions/Chats/Ticket scope smoke recorded; empty ticket views supported by account-scope/converter source review, no populated-ticket visual claim or exhaustive nested-screen sweep. Shared booking-row badge overlap fixed and watcher/mobile320/360/desktop1100 verified. Evidence GROUP-LIFECYCLE-001-block23-profile-payments-20260927.json. HTTP20/48 (41.67%), Lifecycle20/29 (1–13,17–23);24 next. Local NOT RUN. | 2026-09-27 block24 HTTP checklist scope PASS/CLOSED: own contact snapshot; Group Create contact candidate account resolution repaired, eight real candidates returned. Saved contact request/reject/re-request/approve passed; one Base-account conversation, same senders and read receipts under Main/Design Circle; delayed old-account HTTP response did not replace the new account contact list. Contact snapshot restored exactly. Independent free resource fixture: account-owned Asset assigned by the participating Design Circle profile; persisted request retained that participant profile. Base/Seattle Friends subjects without target Event membership returned403. Assets remain usable from any workspace; authority comes from target Event/group membership. Both Base- and Group-held tickets visible from all three workspaces; scanner rejected forged actor bodies from Base/Seattle and accepted authenticated Design Circle despite Base body, persisted correct usedByUserId and attendance. No saved contacts meant zero Event invite candidates despite prior-met profiles. Exact restore-sharing PASS. Shared empty-state spans full grid; user-requested entire contact headline row removed without replacement, watcher/UI verified. Extra forged resource-subject probe under optional-auth dev policy is separately recorded as unproven authenticated-policy boundary, not a security PASS. Evidence GROUP-LIFECYCLE-001-block24-account-contacts-20260927.json. HTTP21/48 (43.75%), Lifecycle21/29 (1–13,17–24);25 next. Local NOT RUN. | Correction:24 closure superseded by reopened forged-resource-actor repair; user requested Java verification without E2E. | 2026-09-27 block24 authorization correction and closure: user explicitly required direct forged-actor assignment rejection, then requested Java verification and excluded E2E. Reopened premature closure; removed optional-auth/demo bypass from resource-assignment submit/manage checks, using authenticated caller and existing policies. Added demo forged-subject/no-write, anonymous and valid-admin regressions; updated obsolete anonymous dev acceptance. Existing main watcher compile/restart PASS20:33:41 local. 19 focused JUnit authorization/resource-service tests PASS (zero skips/failures), reusing existing main outputs and cached test dependencies; no second main build/Gradle/server and no post-fix browser/E2E replay. Valid accepted member/admin and parent Event/generated-group assignment remain allowed; missing membership/forged actor rejected before writes.24 now closed on prior HTTP lifecycle plus this user-approved Java-only repair verification. HTTP21/48, Lifecycle21/29;25 next.24 fixtures and temporary25 notification snapshot were exactly restored. | 2026-09-27 block25 partial PASS: EN320/360/1100 and HU320 notification layout verified; remaining account notification/live-counter branch not yet executed. UI-issued Base and Photo Walks API keys used while Seattle Friends selected: Base asset and Photo Walks event created under their issuing profiles; Group JSON/multipart asset requests returned403 both from Seattle Friends and after Base selection, without created assets/external-ID mappings. Authentication filter rejects before image-controller ingestion; separate object-store inventory was not captured. Real UI Leave group caused Group key403; Base key Revoke caused401. Exact versioned restore-profile-api PASS, membership restored, generated resources/mappings/dependents and the newly created affiliate link removed; old keys retained. Shared menu checkmark moved before badges in all three list item variants; watcher PASS18:52:18.930Z and actual checked/unchecked rows share badge right edge336.125px at360px viewport. Evidence GROUP-LIFECYCLE-001-block25-notifications-api-20260927.json.25 remains IN PROGRESS for notification account scope/live counters and confirmation wording; HTTP21/48 and Lifecycle21/29 unchanged. | 2026-09-27 block25 HTTP PASS/CLOSED: notification layout and API-key scope evidence retained; versioned group notification inputs with actual read mutations verified All/Base/group filtering and account counter23→22→21 across Design/Seattle/Base. Original fixture counter drift recorded separately; aligned prerequisite before assertions, exactly restored afterward. Missing notification group label repaired in existing source subtitle. Real contact request/cancel/approve drove pending1→0 and account approval notification visible from Seattle; own snapshot restored. Independent two-group ticket inputs returned2 in Base/A/B; real Seattle Leave event canceled then confirmed, ticketD/member suppressed and both account ticket counters1, one Design ticket in all profiles. User-requested ticket group label added to existing metadata line; watcher/mobile PASS. Confirmation source audit99 objects/82 EN-HU keys plus bounded runtime/cancellation/320px HU check recorded separately; not every dialog executed, no extra unit runner. Exact temporary fixture/dependent cleanup PASS. Evidence block25-notifications-api-20260927.json and block25-confirmation-audit-20260927.json. HTTP22/48 (45.83%), Lifecycle22/29 (1–13,17–25);26 active. Local NOT RUN. | 2026-09-27 21:37: Block26.1–4 own HTTP execution: grants and revocations preserve provenance; Admin-first owner handover, ordinary-member fallback, sole-Admin step-down verified. Trash Restore returns former creator as Member; normal invitation return, last-member deletion and remaining notification/UI checks continue. Same-actor takeover retry200 is idempotent, competing403; pending fallback403/outsider404. See block26-admin-authority-20260927.json. Block26 remains IN PROGRESS. | 2026-09-27 22:00: Block26 HTTP PASS/CLOSED. Own grants/revocations, Admin-first and ordinary-member fallback, sole-admin step-down, normal invite and Trash return, final-member deletion and user-corrected recovery verified. Corrected rule: Deleted card remains in Trash; any voluntarily departed Admin can restore group/responsibility, ordinary member has no Restore and direct restore/join404 until admin recovery; then Member Restore succeeds. Earlier departed Admin cancel/confirm and idempotent retry proven. Exact notification read/avatar173→172/group2→1 survives reload. Shared Deleted badge bottom-right and common X16px centered. Local25+store2+popup6+converter12 focused tests PASS (45 distinct), full Local browser NOT RUN; Java mapper spec added/not run separately. Existing dev watchers compiled, exact fixture cleanup PASS. HTTP23/48 (47.92%), Lifecycle23/29 (1–13,17–26);27 next. See block26-admin-authority-20260927.json.</t>
+    <t>HTTP26/48 (54.17%); Lifecycle26/29 (1–13,17–29);14–16 partial retained. Next InfoCard clickable-badge chevron, then remaining Group scope. Local full browser NOT RUN.</t>
+  </si>
+  <si>
+    <t>guides/qa/checklists/group/GROUP-LIFECYCLE-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=4/4/4/3/3; effort actions/extra actors/oracles/boundaries/restore/external=40/2/4/3/2/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed. | Shared UI micros appended to existing GROUP-LIFECYCLE-001 checklist; no execution or new PASS claimed. UI_NOTES_2026_09_25.md separates completed code from pending implementation. | 2026-09-26 resume: retained 10-group/27-membership baseline verified for read-only block 1/25. No manual PASS; mutation blocks not staged. guides/qa/evidence/GROUP-LIFECYCLE-001-20260926.md | NOT RUN block 19.1: complete real demo-selector entry, consent, admission before session, saved/rejected location, cancel/retry, first avatar load, reload/logout/login. No injected-session proof. | Source audit: community membership notification hook absent; Members action missing pending badge fixed and observed red in managed UI. Shared menu single-digit circle 20x20px; card numeric alignment checked after watcher deploy. Full counter/notification lifecycle is not fixed or verified. Overall remains NOT RUN. Full conversation coverage inventory in the dated execution log. | Superseding 2026-09-26 correction: member write counters, notification hooks and live store reconciliation implemented; complete lifecycle remains NOT RUN. Correct selector 2 / Groups 3 scope preserved. Retained badge-writes-ready and join snapshots exist; no product membership writes executed. Earlier absent-hook/not-staged descriptions are historical. See dated evidence follow-up and checklist 6.1.5–8. | Group/member attention writes now apply transition deltas like Activity Event, rather than recounting child collections. Versioned block-1 baseline verified without data writes; ordered browser restart in progress. | 2026-09-26 automated delegated browser continuation: creation and required/textual policy draft/save/read-only; hidden roster badge and private-roster invitation cancel/accept/reload; compact image; contextual menu/member counters. Nine focused frontend checks PASS. See GROUP-LIFECYCLE-001-members-media-policy-20260926.json. No full-case PASS. | 2026-09-26: separate checklist block 26 added for group Admin grant/revoke provenance, creator departure, Admin-first/member-fallback takeover, last-member deletion, Asset Manager icon/palette/confirmation parity and notification recipients/retry/scoped badges. Block 26 local and dev HTTP NOT RUN; closed PASS rows unchanged. | 2026-09-26 22:14: block 26 partially exercised in HTTP (grant provenance/403/revoke, ordinary-member leave, creator departure, Admin-first/member-fallback takeover, last-member deletion and Main fallback); 52 focused frontend tests PASS. Notification routing and duplicate release notification repaired/retested. Isolated admin fixture restored. Block 5 timeout/disabled selector/rollback/new-choice/late-response/reload proved; versioned after-workspace-selection checkpoint captured and verified. See dated evidence; no whole-case PASS. 2026-09-26: sequential closure map audited; earlier 2–4 evidence retained. Deferred role/layout and request/live-order checks mapped to 27–29. Current isolated moderation branch retained, support header defect open; see dated evidence.; 2026-09-26 23:17 retained checkpoint: shared read-only multi-image moderation editor and metadata verified in Group scope; 15/15 gallery tests. Group button overlap and empty read-only policy section repaired, editor/admin layout checked. App-admin companion and actor windows retained; Maya Base Feed draft NOT published. Evidence GROUP-LIFECYCLE-001-block6-resume-20260926.json. No block-6 PASS. 2026-09-27 resumed: Base Feed multi-image readonly admin PASS; app-disabled creation accepted, enabled creation under-review; full Group/nested policy readonly verified. See block6-continued evidence. Group support scope/read/reply/retry and HU verified. Late moderation response resurrected row: fixed and real delayed-response on-the-fly replay PASS; counters preserved. 2026-09-27 01:08: HTTP block 6 PASS; confirmation waits for save/failure retains state, notification delta adapters repaired and browser read/retry PASS, concurrent member/read PASS, Main realtime aggregate PASS, Event/Asset readonly previews PASS, member labels fit360px. 17 moderation/dialog +2 adapter tests PASS. Exact after-moderation-checks savepoint verified; resume7. Local NOT RUN. 2026-09-27 01:30: HTTP block7 PASS: voluntary leave→Trash→accepted Restore; admin remove→blocked→pending Restore→admin approval. Failure/delay/retry/direct403 bypass checks and live retained UI verified;41 focused frontend tests PASS. Exact after-membership-trash boundary saved for8; Local browser NOT RUN. | 2026-09-27 02:55: Block8 Group/Main Event/group-owned Event admission and replay checked; HU desktop/mobile Group/Event/Affiliate Copy PASS. Removed Group member cannot bypass blocked/pending restoration with Event link. Fresh visitor location fixture corrected by explicit request. Exact cleanup pending; no block8 closure. See GROUP-LIFECYCLE-001-block8-progress-20260927.json. | Valid Maya replay: external group Event accepted, identical replay, blocked/pending restore cannot bypass Group approval, Admin approval restores Event access; UI writes only and independent Mongo reads. See GROUP-LIFECYCLE-001-block8-maya-20260927.json. No block8 closure. Main Event Maya UI Accept updated retained card1/10→2/10; duplicate link preserved exact normalized state, base/group Event memberships and prior referrer. Registration-first source route checked; fresh-account browser PASS not claimed. Native-browser registration replay: guides/qa/evidence/GROUP-LIFECYCLE-001-block8-registration-20260927.json. New Group/Event users persist real browser coordinates through UI; accepted memberships/replay PASS. Setup Update remains open; explicit Close resumes login for existing missing-location user. Watcher build PASS; new units/live Firebase NOT RUN. Block8 CLOSED: versioned restore-sharing scope verification PASS, independent reserved resources/fresh profiles zero, exact after-membership-trash savepoint verification PASS. Evidence: GROUP-LIFECYCLE-001-block8-cleanup-20260927.json. No replay of closed1–7. | Block9 in progress: Event/Asset two-message and mixed delta UI+Mongo PASS; intentional share-token network failure after asset deletions retained picker, Retry sent only outstanding two additions (49 messages). Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. No block9 closure. | Block9 CLOSED 2026-09-27: complete chat sharing basket/delta/retry/paging/context/mobile HTTP chain, logout history race fixed and replayed. 13-scope exact cleanup, chat original41/zero paging, immutable after-chat-sharing captured resume10. Evidence GROUP-LIFECYCLE-001-block9-chat-sharing-20260927.json. Added overlay specs NOT RUN; owning watcher builds PASS. | 2026-09-27 block10 active: manual cash create/retry, Deleted state, red busy confirmation and refund request/approval replay; evidence GROUP-LIFECYCLE-001-block10-cash-20260927.json. 9/48 closed unchanged; checkout/affiliate controls pending. Cash refund live replay PASS; lost DELETE response/retry retains Deleted with one reversal. Short-window poll fix replay PASS. Checkout/negative controls remain; block10 IN PROGRESS. | Block10 latest: corrected referral prerequisite via exact versioned restore, valid cash exclusion/card EUR10 contribution+refund PASS. All eight recipient/payer denials plus unrelated deletion404 PASS with unchanged totals. Canonical header summary centralized in existing signal store; watcher03:17Z and both actor browser reads PASS. Points9/11 complete; point10 solely awaits cash-checkout accounting semantics. See block10-cash JSON pointStatus; no full block PASS. | Block10 CLOSED: final Cash-only booking accepted/no affiliate contribution; manual cash receipt separately proves history/totals/refund. Prior additional-booking-receipt expectation withdrawn as QA interpretation error; no semantics change. Barion/3DS-off restored. Exact cash restore and after-chat-sharing verification PASS; after-cash-history captured03:24:57Z resume11. Evidence block10-cash JSON finalCashBooking/cleanup. | 2026-09-27 block11 CLOSED: approved-only contact invitations/denials, retained overlays, recipient messages/unread reset, phone/share nesting, EN desktop/HU mobile; exact fixture restore PASS; after-contacts savepoint resume12. Evidence GROUP-LIFECYCLE-001-block11-contacts-20260927.json. | 2026-09-27 block12 CLOSED: selection limits including nested/mobile; contact consent cancellation/failure/retry/decisions, pagination/search, private methods, same chat/persistence and delayed group/account switch PASS. Exact contacts restore and after-contacts verification PASS; after-contact-controls captured resume13. Evidence GROUP-LIFECYCLE-001-block12-controls-20260927.json. | 2026-09-27 block13 CLOSED: empty HU/EN calendar notices retain blurred parent and produce no download; positive ICS download and libical import four events PASS. Desktop calendar UI NOT RUN. Blocks14–16 partial evidence retained in per-block JSON; no replay of completed subchecks. | 2026-09-27 block17 CLOSED for user-agreed HTTP Help/native anonymous MCP scope: current Codex conversation directly invoked MyScoutee topic list/read successfully. MCP connection UI create/reload/secret-hide/revoke also verified. No private OAuth or Local PASS claimed. Block18 X/Back and rapid reopen checks passed; remaining checks continue. | 2026-09-27 block18 CLOSED: physical Android native-Back defect fixed in shared overlay history owner; nested Back, X/Back, rapid reopen, busy refusal, desktop Forward/Router/reload and unchanged rating dock verified. Existing frontend-sync PASS05:46:29Z; unit specs not rerun. Evidence GROUP-LIFECYCLE-001-block18-20260927.json. Normal phone logout, owned browser/tunnel cleanup complete; ENTRY untouched. User requested STOP before19. | 2026-09-27 resumed19: actual demo selector admission, denied/unsupported GPS, isolated Zoe missing/invalid Setup cancel/retry and first profile persistence/reload partially PASS. False Location required race fixed; real stale null poll retest retained accepted point over12.4s. frontend-sync PASS15:24:34Z. One ENTRY-BLOCK19 window, Zoe snapshot retained. Block19 IN PROGRESS; counts unchanged. Evidence GROUP-LIFECYCLE-001-block19-entry-20260927.json. | 2026-09-27 18:22:19.1 HTTP complete incl invitation claim/first target profile/reload/replay and GPS-denied relogin; exact scoped cleanup. Avatar wait/error boundary and Setup disabled action verified.19.2 active:53/53 seed points accepted; Firebase config404 blocks real sign-in; pending-coordinate controls/Local remain. No count change. | User scope change2026-09-27: Firebase and actual external-client/provider-configuration checks moved to DEPLOY-EXTERNAL-CONFIG-001, DEFERRED/NOT RUN. They no longer gate Group19; continue demo pending-coordinate controls. | Block19 HTTP CLOSED in user-approved demo scope:53/53 seed points; two-account real login/profile-ext unsupported pending samples rejected with original points retained and per-account acknowledgement. Earlier failure/retry/claim/cleanup evidence retained.16/48 and16/29 closed;20 active. | 2026-09-27 block20 HTTP PASS/CLOSED: stored point with denied GPS and same-session reload; tracking OFF/save/reopen/ON; &lt;5km zero writes, &gt;=5km POST200; unsupported Paris POST403 retains accepted profile/cache/baseline/session and no popup; later eligible movement POST200. Independent Mongo point47.6747/19.0354 verified, normal logout then exact original47.5147/19.0354 restore, location snapshot removed. Evidence: GROUP-LIFECYCLE-001-block20-tracking-20260927.json. HTTP17/48 (35.42%), Lifecycle17/29 closed (1–13,17–20);21 active. Local NOT RUN; older contact/badge snapshots retained. | User clarification 2026-09-27: testcases are independent closed execution units. Transferred checks are CLOSED BY SCOPE TRANSFER in the source, not pending dependencies. DEPLOY-EXTERNAL-CONFIG-001 requires its own fixture, restaging, entry checkpoints, execution and cleanup; prior/cross-case evidence cannot substitute. Transfer provenance stays in the ledger, not executable cross-case references. Audit the remaining NOT RUN cases only at the current testcase boundary, before advancing to another testcase. | 2026-09-27 block21 HTTP partial: seven audited menu surfaces, profile multiselect, pricing scope and card menus exercised; HU320/EN360/desktop1100 representative checks. Notification launcher overlap and forced-sheet desktop X repaired and replayed through existing frontend-sync. Assignment basket restaged with own Group fixture and exactly restored, no assignment/share/checkout commit. Checkout optional-item menu remains NOT RUN because selected real event/date combinations returned no available slots; suitable own checkpoint required. Do not mark full21 closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP17/48 and Lifecycle17/29 unchanged. | 2026-09-27 block21 HTTP PASS/CLOSED: final checkout optional-card control used its own versioned Group slot fixture. Native pointer selected/reverted optional item; mobile X remained reachable and closed only the sheet with parent dialogs/scroll retained; desktop title/no mobile X PASS. No checkout writes; draft discarded. Exact restore-sharing completed and original contact/badge snapshots retained. Together with the recorded seven menu surfaces, profile/price controls and HU/EN smoke,21 is closed. Evidence GROUP-LIFECYCLE-001-block21-menus-20260927.json. HTTP18/48 (37.50%), Lifecycle18/29 (1–13,17–21);22 active. Local NOT RUN. | 2026-09-27 block22 HTTP PASS/CLOSED: Design Circle UI create/edit/delete persisted Base asset ownership; Main/Design Circle/Seattle Friends inventory and immediate asset counters match, event counters remain separate. Real response-stage delayed long-poll released after deletion did not resurrect count; no page reload. Own scoped fixture public Asset booked to an inaccessible Language Lab event remains in Explore (UI + three-profile authenticated reads); own/private/non-friend controls absent, foreign Event/private Asset details withheld with empty HTTP200. Event Explore UI changes with workspace. Existing Group chat preparation and tools fixtures exactly restored; no chat share submitted. Evidence GROUP-LIFECYCLE-001-block22-tools-20260927.json. HTTP19/48 (39.58%), Lifecycle19/29 (1–13,17–22);23 active. Local NOT RUN. | 2026-09-27 block23 HTTP PASS/CLOSED: independent Group Asset checkout captured HUF3200 on Design Circle payer; Maya Base reads the same stored payment as income, Base/other Group controls excluded. Real owner acceptance and payer refund request/recipient approval reversed HUF3200 on the same payer/recipient; one capture plus normal refund audit. Initial unknown provider-card fixture caused one failed attempt; repaired via snapshot-protected real provider card registration, not a manufactured payment. Card revoked and restore-sharing exactly verified. Base/Group Profile/Affiliate/API/history and bounded Feed/Impressions/Chats/Ticket scope smoke recorded; empty ticket views supported by account-scope/converter source review, no populated-ticket visual claim or exhaustive nested-screen sweep. Shared booking-row badge overlap fixed and watcher/mobile320/360/desktop1100 verified. Evidence GROUP-LIFECYCLE-001-block23-profile-payments-20260927.json. HTTP20/48 (41.67%), Lifecycle20/29 (1–13,17–23);24 next. Local NOT RUN. | 2026-09-27 block24 HTTP checklist scope PASS/CLOSED: own contact snapshot; Group Create contact candidate account resolution repaired, eight real candidates returned. Saved contact request/reject/re-request/approve passed; one Base-account conversation, same senders and read receipts under Main/Design Circle; delayed old-account HTTP response did not replace the new account contact list. Contact snapshot restored exactly. Independent free resource fixture: account-owned Asset assigned by the participating Design Circle profile; persisted request retained that participant profile. Base/Seattle Friends subjects without target Event membership returned403. Assets remain usable from any workspace; authority comes from target Event/group membership. Both Base- and Group-held tickets visible from all three workspaces; scanner rejected forged actor bodies from Base/Seattle and accepted authenticated Design Circle despite Base body, persisted correct usedByUserId and attendance. No saved contacts meant zero Event invite candidates despite prior-met profiles. Exact restore-sharing PASS. Shared empty-state spans full grid; user-requested entire contact headline row removed without replacement, watcher/UI verified. Extra forged resource-subject probe under optional-auth dev policy is separately recorded as unproven authenticated-policy boundary, not a security PASS. Evidence GROUP-LIFECYCLE-001-block24-account-contacts-20260927.json. HTTP21/48 (43.75%), Lifecycle21/29 (1–13,17–24);25 next. Local NOT RUN. | Correction:24 closure superseded by reopened forged-resource-actor repair; user requested Java verification without E2E. | 2026-09-27 block24 authorization correction and closure: user explicitly required direct forged-actor assignment rejection, then requested Java verification and excluded E2E. Reopened premature closure; removed optional-auth/demo bypass from resource-assignment submit/manage checks, using authenticated caller and existing policies. Added demo forged-subject/no-write, anonymous and valid-admin regressions; updated obsolete anonymous dev acceptance. Existing main watcher compile/restart PASS20:33:41 local. 19 focused JUnit authorization/resource-service tests PASS (zero skips/failures), reusing existing main outputs and cached test dependencies; no second main build/Gradle/server and no post-fix browser/E2E replay. Valid accepted member/admin and parent Event/generated-group assignment remain allowed; missing membership/forged actor rejected before writes.24 now closed on prior HTTP lifecycle plus this user-approved Java-only repair verification. HTTP21/48, Lifecycle21/29;25 next.24 fixtures and temporary25 notification snapshot were exactly restored. | 2026-09-27 block25 partial PASS: EN320/360/1100 and HU320 notification layout verified; remaining account notification/live-counter branch not yet executed. UI-issued Base and Photo Walks API keys used while Seattle Friends selected: Base asset and Photo Walks event created under their issuing profiles; Group JSON/multipart asset requests returned403 both from Seattle Friends and after Base selection, without created assets/external-ID mappings. Authentication filter rejects before image-controller ingestion; separate object-store inventory was not captured. Real UI Leave group caused Group key403; Base key Revoke caused401. Exact versioned restore-profile-api PASS, membership restored, generated resources/mappings/dependents and the newly created affiliate link removed; old keys retained. Shared menu checkmark moved before badges in all three list item variants; watcher PASS18:52:18.930Z and actual checked/unchecked rows share badge right edge336.125px at360px viewport. Evidence GROUP-LIFECYCLE-001-block25-notifications-api-20260927.json.25 remains IN PROGRESS for notification account scope/live counters and confirmation wording; HTTP21/48 and Lifecycle21/29 unchanged. | 2026-09-27 block25 HTTP PASS/CLOSED: notification layout and API-key scope evidence retained; versioned group notification inputs with actual read mutations verified All/Base/group filtering and account counter23→22→21 across Design/Seattle/Base. Original fixture counter drift recorded separately; aligned prerequisite before assertions, exactly restored afterward. Missing notification group label repaired in existing source subtitle. Real contact request/cancel/approve drove pending1→0 and account approval notification visible from Seattle; own snapshot restored. Independent two-group ticket inputs returned2 in Base/A/B; real Seattle Leave event canceled then confirmed, ticketD/member suppressed and both account ticket counters1, one Design ticket in all profiles. User-requested ticket group label added to existing metadata line; watcher/mobile PASS. Confirmation source audit99 objects/82 EN-HU keys plus bounded runtime/cancellation/320px HU check recorded separately; not every dialog executed, no extra unit runner. Exact temporary fixture/dependent cleanup PASS. Evidence block25-notifications-api-20260927.json and block25-confirmation-audit-20260927.json. HTTP22/48 (45.83%), Lifecycle22/29 (1–13,17–25);26 active. Local NOT RUN. | 2026-09-27 21:37: Block26.1–4 own HTTP execution: grants and revocations preserve provenance; Admin-first owner handover, ordinary-member fallback, sole-Admin step-down verified. Trash Restore returns former creator as Member; normal invitation return, last-member deletion and remaining notification/UI checks continue. Same-actor takeover retry200 is idempotent, competing403; pending fallback403/outsider404. See block26-admin-authority-20260927.json. Block26 remains IN PROGRESS. | 2026-09-27 22:00: Block26 HTTP PASS/CLOSED. Own grants/revocations, Admin-first and ordinary-member fallback, sole-admin step-down, normal invite and Trash return, final-member deletion and user-corrected recovery verified. Corrected rule: Deleted card remains in Trash; any voluntarily departed Admin can restore group/responsibility, ordinary member has no Restore and direct restore/join404 until admin recovery; then Member Restore succeeds. Earlier departed Admin cancel/confirm and idempotent retry proven. Exact notification read/avatar173→172/group2→1 survives reload. Shared Deleted badge bottom-right and common X16px centered. Local25+store2+popup6+converter12 focused tests PASS (45 distinct), full Local browser NOT RUN; Java mapper spec added/not run separately. Existing dev watchers compiled, exact fixture cleanup PASS. HTTP23/48 (47.92%), Lifecycle23/29 (1–13,17–26);27 next. See block26-admin-authority-20260927.json. | 2026-09-27: Blocks27–28 HTTP PASS/CLOSED. Three-role roster, responsive editor EN/HU, requested mobile single-column fix, normal/Admin/Operator header smoke. List summary/detail/nested-rule request boundaries verified. Existing watcher build; exact temporary fixture cleanup. Evidence block27-presentation-20260927.json and block28-requests-20260927.json. HTTP25/48, Lifecycle25/29;29 next;14–16 retained partial; Local NOT RUN. | 2026-09-27: Block29 HTTP PASS/CLOSED. Live Activities/Event Explore seven exact distance boundaries; Group save third→first, duplicate409/version2, sync200, scroll51 retained. Shared SmartList sticky-date refresh fixed and own fresh restage retest passed. Existing watcher build, exact14-event/Admin fixture cleanup. HTTP26/48; Lifecycle26/29;14–16 partial retained. Evidence block29-distance-ordering-20260927.json.</t>
   </si>
   <si>
     <t>180/420</t>

</xml_diff>

<commit_message>
group fix - isolation
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -3364,25 +3364,25 @@
     <t>DELTA only the owning workspace; no cross-workspace private detail/write, relationship, card exclusion or counter leak. Group-admin moderation is scoped to its group.</t>
   </si>
   <si>
-    <t>IN PROGRESS / OWN BASELINE VERIFIED</t>
-  </si>
-  <si>
-    <t>0/9 — baseline verified; two managed actors ready</t>
+    <t>IN PROGRESS / BLOCKS 1–2 HTTP PASS</t>
+  </si>
+  <si>
+    <t>2/9 — Event lifecycle and private-request isolation PASS</t>
   </si>
   <si>
     <t>2026-09-28</t>
   </si>
   <si>
-    <t>31 focused backend moderation/chat/counter tests PASS (2026-09-25): separate scope settings, authority/foreign IDs, persisted pending count and idempotence, worker, Group support access/filter/unread. Earlier 15 filter/invitation tests PASS (2026-09-24). Frontend/backend dev watchers compiled. Full local/UI/HTTP journey NOT RUN. Profile selection correction: 21 focused Java tests PASS (2026-09-25); profile-load parameter, read-only restore, accepted-membership authority, failed-load non-commit, invite activation and removal. Added frontend HTTP parameter/retry unit cases; not executed separately from the running build watcher.</t>
-  </si>
-  <si>
-    <t>Block1: create A Event, invite/accept A peer, compare Base/B projections. Own group-isolation fixture/savepoints; block3 includes shared Social toggle before X and fixed aggregated Social-on badge in either switch position.</t>
+    <t>31 focused backend moderation/chat/counter tests PASS (2026-09-25): separate scope settings, authority/foreign IDs, persisted pending count and idempotence, worker, Group support access/filter/unread. Earlier 15 filter/invitation tests PASS (2026-09-24). Frontend/backend dev watchers compiled. Full local/UI/HTTP journey NOT RUN. Profile selection correction: 21 focused Java tests PASS (2026-09-25); profile-load parameter, read-only restore, accepted-membership authority, failed-load non-commit, invite activation and removal. Added frontend HTTP parameter/retry unit cases; not executed separately from the running build watcher. | 2026-09-28:10 targeted policy JUnit tests PASS; existing watcher-built main classes reused.</t>
+  </si>
+  <si>
+    <t>Block3: own Home ratings/filters/Feed/Following controls and shared Social toggle/count desktop/mobile.</t>
   </si>
   <si>
     <t>IN PROGRESS</t>
   </si>
   <si>
-    <t>guides/qa/checklists/group/GROUP-ISOLATION-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=5/5/4/4/5; effort actions/extra actors/oracles/boundaries/restore/external=40/2/5/5/1/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed.; 2026-09-26 NOT RUN micros: separate direct-chat request/approve/reject; recipient-only notifications; approval saves public contact; write-side pending counter vs saved-contact count; search-row icon+label menu on mobile; SmartList live remove/insert; blurred confirmation; retry, stale version and workspace isolation. See existing GROUP-ISOLATION-001 checklist. | 2026-09-27: queued next after user-requested Group Lifecycle closure. User explicitly prohibited starting now; no fixture/browser/test action performed. | 2026-09-28: explicit full-flow automation authorized. Exact duplicate assertions removed after evidence audit; 9 unique blocks remain, no inherited PASS. Own namespace baseline verified and two managed sessions launched. Execution: guides/qa/evidence/GROUP-ISOLATION-001-20260928.md.</t>
+    <t>guides/qa/checklists/group/GROUP-ISOLATION-001.md; Added 2026-09-24. No campaign fixture or browser actions executed. Priority I/L/A/N/O=5/5/4/4/5; effort actions/extra actors/oracles/boundaries/restore/external=40/2/5/5/1/0. Finalized 2026-09-25: app-admin configurable Group review; group-admin Asset/Event/Feed scope; write-side badges propagated through signal store/SmartList without reload; Group support channel and separate unread count. Profile loading owns activeWorkspaceGroupId persistence; no per-request group header. Checklist includes shared loading state, timeout retaining prior selection, same-target retry and stale responses. Manual results remain NOT RUN. | 2026-09-25: sharing batch and discovered eventless-support regression checklist expanded; execution remains NOT RUN, no manual result claimed.; 2026-09-26 NOT RUN micros: separate direct-chat request/approve/reject; recipient-only notifications; approval saves public contact; write-side pending counter vs saved-contact count; search-row icon+label menu on mobile; SmartList live remove/insert; blurred confirmation; retry, stale version and workspace isolation. See existing GROUP-ISOLATION-001 checklist. | 2026-09-27: queued next after user-requested Group Lifecycle closure. User explicitly prohibited starting now; no fixture/browser/test action performed. | 2026-09-28: explicit full-flow automation authorized. Exact duplicate assertions removed after evidence audit; 9 unique blocks remain, no inherited PASS. Own namespace baseline verified and two managed sessions launched. Execution: guides/qa/evidence/GROUP-ISOLATION-001-20260928.md. | 2026-09-28 block1 HTTP PASS: UI create/invite/publish/accept/message; A event h1790547269571, two accepted members and two chat copies. Base/B lists and domain counters empty; A reopen intact. Own after-block1 checkpoint captured. Evidence GROUP-ISOLATION-001-block1-20260928.json. | Block2 HTTP PASS after private member/demo lifecycle authority repairs.32 negative requests403/404; forged profile/group/header rejected; Event/member/chat/notification/counter oracle unchanged. A reads and Unpublish→Publish200; exact own snapshot restored. Evidence GROUP-ISOLATION-001-block2-20260928.json.</t>
   </si>
   <si>
     <t>165/395</t>

</xml_diff>

<commit_message>
Document verified 1.3.2 images and Netcup partial deployment
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -3835,10 +3835,10 @@
     <t>Managed browser UI runs; live HTTP80; compiled local bootstrap80; seed/i18n audits; existing watcher build. Focused i18n13/13 and lazy-image/SmartList pagination15/15 passed serially with watcher stopped.</t>
   </si>
   <si>
-    <t>Retained Android Rates panels accepted; proceed with authorized1.3.2 release. Existing local persistence/native-WebView and separate Past lifecycle limitations remain.</t>
-  </si>
-  <si>
-    <t>45 contexts / 963 fields. Existing recorded scope retained. Added landing: 64 steps per viewport; feedback: 39 per viewport; Rates arrow-only, shared double-panel highlights and editable badge passed at mobile/desktop. EN/HU local/demo/e2e/prod seed parity. Landing visit visibility, internal default ON/preserved OFF, fresh-browser consent and shared guide/notification clearance above rating actions/profile eyes passed mobile/desktop. Mobile-only launcher clearance; unchanged desktop positioning; pair divider hover/tap/drag and fixed photo scale at 0/50/100% passed Home/Rates browser and Android Rates over ADB. Mobile pair image fit unified to contain on Home/Activity Rates; both targeted browser checks passed, desktop preserved. Guide screenshots removed from Git. No final form submission. Full local persistence and native WebView not claimed. guides/qa/evidence/general/EXPLANATION-GUIDE-001-20260930.md Final Android Home rail stability, mobile/desktop guide card continuity and filter badge save/reload/restore passed. No screenshots committed. User-reported Android fullscreen/drag lag confirmed; targeted follow-up measurements in progress, not a performance PASS. Follow-up: one retained list row rebuilt instead of six; one DTO snapshot per card; hidden controls excluded from launcher measurement. Native menu/guide visibility and raised list badge clearance passed. Small warm RAF-proxy medians: fullscreen 293 to 254ms, list 161 to 108ms; residual latency remains open. Final user-accepted retained-panel change: one shared loaded collection; persistent list/fullscreen DOM; z-order-only presentation; inactive new-image gating; no warm card rebuilds or switch scroll shift; saved-score paging identity preserved. Warm fullscreen median207.9→127.7ms; list103→128.1ms (dev two-RAF proxy, no universal performance claim). Rates list-scroll launchers fixed: native100-frame check0/0px movement versus48/56px before. Follow-up: panel-bottom launcher anchor56px list/96px fullscreen; native scroll0/0px. Whole-card scroll preview/adaptive prefetch withdrawn. Image-only handling preserves visible photos; only offscreen/passed photos suspend, returning once from cache. Fast-scroll requests/spinners0; sampled visible-image flickers0; focused tests15/15. See phone-image-scroll.json. Mobile photo badges/eye/image indicators follow per-image suspension; individual/pair native swipe90frames each passed; user accepted.</t>
+    <t>Recorded guide scope closed;1.3.2 partial release deployed and verified. Existing local persistence/native-WebView and separate Past lifecycle limitations remain unchanged.</t>
+  </si>
+  <si>
+    <t>45 contexts / 963 fields. Existing recorded scope retained. Added landing: 64 steps per viewport; feedback: 39 per viewport; Rates arrow-only, shared double-panel highlights and editable badge passed at mobile/desktop. EN/HU local/demo/e2e/prod seed parity. Landing visit visibility, internal default ON/preserved OFF, fresh-browser consent and shared guide/notification clearance above rating actions/profile eyes passed mobile/desktop. Mobile-only launcher clearance; unchanged desktop positioning; pair divider hover/tap/drag and fixed photo scale at 0/50/100% passed Home/Rates browser and Android Rates over ADB. Mobile pair image fit unified to contain on Home/Activity Rates; both targeted browser checks passed, desktop preserved. Guide screenshots removed from Git. No final form submission. Full local persistence and native WebView not claimed. guides/qa/evidence/general/EXPLANATION-GUIDE-001-20260930.md Final Android Home rail stability, mobile/desktop guide card continuity and filter badge save/reload/restore passed. No screenshots committed. User-reported Android fullscreen/drag lag confirmed; targeted follow-up measurements in progress, not a performance PASS. Follow-up: one retained list row rebuilt instead of six; one DTO snapshot per card; hidden controls excluded from launcher measurement. Native menu/guide visibility and raised list badge clearance passed. Small warm RAF-proxy medians: fullscreen 293 to 254ms, list 161 to 108ms; residual latency remains open. Final user-accepted retained-panel change: one shared loaded collection; persistent list/fullscreen DOM; z-order-only presentation; inactive new-image gating; no warm card rebuilds or switch scroll shift; saved-score paging identity preserved. Warm fullscreen median207.9→127.7ms; list103→128.1ms (dev two-RAF proxy, no universal performance claim). Rates list-scroll launchers fixed: native100-frame check0/0px movement versus48/56px before. Follow-up: panel-bottom launcher anchor56px list/96px fullscreen; native scroll0/0px. Whole-card scroll preview/adaptive prefetch withdrawn. Image-only handling preserves visible photos; only offscreen/passed photos suspend, returning once from cache. Fast-scroll requests/spinners0; sampled visible-image flickers0; focused tests15/15. See phone-image-scroll.json. Mobile photo badges/eye/image indicators follow per-image suspension; individual/pair native swipe90frames each passed; user accepted. Release1.3.2: both guide branches consolidated/master merged; GHCR frontend/backend images; Netcup migration010 retained-data check;8 healthy containers; publicHTTP13/13 and landing guide10/10 plus private-context denial passed. See RELEASE_1.3.2_20260930.json.</t>
   </si>
   <si>
     <t>OPERATOR-CONFIGURATION-LIFECYCLE-001</t>

</xml_diff>

<commit_message>
Close accepted guide QA scope in workbook and handoff
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -3829,16 +3829,16 @@
     <t>Available target counts; popup/menu/scroll; granular editors; slider and Save; floating guide; public landing; repeated pair targets</t>
   </si>
   <si>
-    <t>PASS (recorded guide scope)</t>
+    <t>PASS / CLOSED (recorded guide scope)</t>
   </si>
   <si>
     <t>Managed browser UI runs; live HTTP80; compiled local bootstrap80; seed/i18n audits; existing watcher build. Focused i18n13/13 and lazy-image/SmartList pagination15/15 passed serially with watcher stopped.</t>
   </si>
   <si>
-    <t>Recorded guide scope closed;1.3.2 partial release deployed and verified. Existing local persistence/native-WebView and separate Past lifecycle limitations remain unchanged.</t>
-  </si>
-  <si>
-    <t>45 contexts / 963 fields. Existing recorded scope retained. Added landing: 64 steps per viewport; feedback: 39 per viewport; Rates arrow-only, shared double-panel highlights and editable badge passed at mobile/desktop. EN/HU local/demo/e2e/prod seed parity. Landing visit visibility, internal default ON/preserved OFF, fresh-browser consent and shared guide/notification clearance above rating actions/profile eyes passed mobile/desktop. Mobile-only launcher clearance; unchanged desktop positioning; pair divider hover/tap/drag and fixed photo scale at 0/50/100% passed Home/Rates browser and Android Rates over ADB. Mobile pair image fit unified to contain on Home/Activity Rates; both targeted browser checks passed, desktop preserved. Guide screenshots removed from Git. No final form submission. Full local persistence and native WebView not claimed. guides/qa/evidence/general/EXPLANATION-GUIDE-001-20260930.md Final Android Home rail stability, mobile/desktop guide card continuity and filter badge save/reload/restore passed. No screenshots committed. User-reported Android fullscreen/drag lag confirmed; targeted follow-up measurements in progress, not a performance PASS. Follow-up: one retained list row rebuilt instead of six; one DTO snapshot per card; hidden controls excluded from launcher measurement. Native menu/guide visibility and raised list badge clearance passed. Small warm RAF-proxy medians: fullscreen 293 to 254ms, list 161 to 108ms; residual latency remains open. Final user-accepted retained-panel change: one shared loaded collection; persistent list/fullscreen DOM; z-order-only presentation; inactive new-image gating; no warm card rebuilds or switch scroll shift; saved-score paging identity preserved. Warm fullscreen median207.9→127.7ms; list103→128.1ms (dev two-RAF proxy, no universal performance claim). Rates list-scroll launchers fixed: native100-frame check0/0px movement versus48/56px before. Follow-up: panel-bottom launcher anchor56px list/96px fullscreen; native scroll0/0px. Whole-card scroll preview/adaptive prefetch withdrawn. Image-only handling preserves visible photos; only offscreen/passed photos suspend, returning once from cache. Fast-scroll requests/spinners0; sampled visible-image flickers0; focused tests15/15. See phone-image-scroll.json. Mobile photo badges/eye/image indicators follow per-image suspension; individual/pair native swipe90frames each passed; user accepted. Release1.3.2: both guide branches consolidated/master merged; GHCR frontend/backend images; Netcup migration010 retained-data check;8 healthy containers; publicHTTP13/13 and landing guide10/10 plus private-context denial passed. See RELEASE_1.3.2_20260930.json. Launcher follow-up: desktop icons remain with menus; guide above shade; bell layering unchanged; mobile menus hide both icons without hiding tour;1280/390px regression passed and user accepted.; Accepted launcher follow-up republished1.3.2: nginx-only Netcup update,13/13 HTTP PASS,8 healthy containers,7 unchanged.</t>
+    <t>None in the accepted guide scope; closed 2026-09-30 after the accepted mobile and launcher follow-ups. Release 1.3.2 deployed and verified. Local persistence/native-WebView remain unproven; EVENT-PAST-BADGES-001 is a separate open case.</t>
+  </si>
+  <si>
+    <t>45 contexts / 963 fields. Existing recorded scope retained. Added landing: 64 steps per viewport; feedback: 39 per viewport; Rates arrow-only, shared double-panel highlights and editable badge passed at mobile/desktop. EN/HU local/demo/e2e/prod seed parity. Landing visit visibility, internal default ON/preserved OFF, fresh-browser consent and shared guide/notification clearance above rating actions/profile eyes passed mobile/desktop. Mobile-only launcher clearance; unchanged desktop positioning; pair divider hover/tap/drag and fixed photo scale at 0/50/100% passed Home/Rates browser and Android Rates over ADB. Mobile pair image fit unified to contain on Home/Activity Rates; both targeted browser checks passed, desktop preserved. Guide screenshots removed from Git. No final form submission. Full local persistence and native WebView not claimed. guides/qa/evidence/general/EXPLANATION-GUIDE-001-20260930.md Final Android Home rail stability, mobile/desktop guide card continuity and filter badge save/reload/restore passed. No screenshots committed. Earlier Android fullscreen/drag lag was confirmed; the subsequent retained-panel and image-scroll fixes below were accepted and close that follow-up. No universal performance PASS is claimed. Follow-up: one retained list row rebuilt instead of six; one DTO snapshot per card; hidden controls excluded from launcher measurement. Native menu/guide visibility and raised list badge clearance passed. Small warm RAF-proxy medians: fullscreen 293 to 254ms, list 161 to 108ms; these preliminary measurements are superseded by the final user-accepted retained-panel result below. Final user-accepted retained-panel change: one shared loaded collection; persistent list/fullscreen DOM; z-order-only presentation; inactive new-image gating; no warm card rebuilds or switch scroll shift; saved-score paging identity preserved. Warm fullscreen median207.9→127.7ms; list103→128.1ms (dev two-RAF proxy, no universal performance claim). Rates list-scroll launchers fixed: native100-frame check0/0px movement versus48/56px before. Follow-up: panel-bottom launcher anchor56px list/96px fullscreen; native scroll0/0px. Whole-card scroll preview/adaptive prefetch withdrawn. Image-only handling preserves visible photos; only offscreen/passed photos suspend, returning once from cache. Fast-scroll requests/spinners0; sampled visible-image flickers0; focused tests15/15. See phone-image-scroll.json. Mobile photo badges/eye/image indicators follow per-image suspension; individual/pair native swipe90frames each passed; user accepted. Release1.3.2: both guide branches consolidated/master merged; GHCR frontend/backend images; Netcup migration010 retained-data check;8 healthy containers; publicHTTP13/13 and landing guide10/10 plus private-context denial passed. See RELEASE_1.3.2_20260930.json. Launcher follow-up: desktop icons remain with menus; guide above shade; bell layering unchanged; mobile menus hide both icons without hiding tour;1280/390px regression passed and user accepted.; Accepted launcher follow-up republished1.3.2: nginx-only Netcup update,13/13 HTTP PASS,8 healthy containers,7 unchanged. Final ledger closure 2026-09-30: PASS / CLOSED for the accepted guide scope and follow-ups; no remaining guide oracle. Local PARTIAL records the untested persistence boundary, not an open guide defect.</t>
   </si>
   <si>
     <t>OPERATOR-CONFIGURATION-LIFECYCLE-001</t>

</xml_diff>

<commit_message>
docs(qa): require template regression and fix propagation for pending cases
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -466,10 +466,10 @@
     <t>See guides/plans/MULTI_GROUP_PRODUCT_DIRECTION_2026_10.md; code/build checks do not establish manual PASS.</t>
   </si>
   <si>
-    <t>Actors: Authorized Work member API/MCP identity. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
-  </si>
-  <si>
-    <t>Prepared 2026-10-05 from user requirements. No browser actions or live data mutation performed. Preserve other completed campaign checkpoints. | 2026-10-06 conversation reconciliation: MSC-115 checklist updated; full flow remains NOT RUN.</t>
+    <t>Actors: Authorized Work member API/MCP identity. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
+  </si>
+  <si>
+    <t>Prepared 2026-10-05 from user requirements. No browser actions or live data mutation performed. Preserve other completed campaign checkpoints. | 2026-10-06 conversation reconciliation: MSC-115 checklist updated; full flow remains NOT RUN. | 2026-10-11 MSC-122 follow-up REQUIRED: for each defect record template affected/unaffected with reason, source and template fix revisions, targeted template environment/result/evidence; affected propagation or verification stays open until completed. Source PASS does not imply template PASS. See guides/qa/checklists/README.md#template-regression-and-fix-propagation--msc-122. No execution status changed by this requirement.</t>
   </si>
   <si>
     <t>P1</t>
@@ -502,10 +502,10 @@
     <t>Focused regression source prepared; execution deferred by user. 2026-10-07 Help-only watcher-AOT check PASS: enabled parent/child contexts, EN/HU in Dating/Work/Community, bounded loads and cleanup; scoped/local/Mongo seed parity PASS. Permission enforcement remains untested here.</t>
   </si>
   <si>
-    <t>Run INTEGRATION-ACCESS-001 with backend/frontend/client/MCP 1.6.0: Blocked/Write/Read/Full, default blocked main MCP, unchanged generation, API/MCP per-client caps, atomic draft save, role statistics and revoked-role denial.</t>
-  </si>
-  <si>
-    <t>MSC-116. Watcher compilation and schema generation are not behavioral QA. Existing guide/API PASS does not cover this extension. | 2026-10-07: fixed missing profile.integration-access enabled-surface registration and Work/Community child guide content; existing parent shield and level/Apply/Close steps reused. guides/qa/evidence/general/EXPLANATION-GUIDE-001-20261007.md. Section 4 now names the manual Help checks. Manual status unchanged. MSC-119 extension 2026-10-07: guides/plans/MSC-119_MCP_READ_EVENTS_ROLE_GUIDANCE.md and guides/qa/evidence/general/MSC-119_GUIDE_WIRING_20261007.md. Source/build evidence only; no functional/browser/security/load PASS claimed.</t>
+    <t>Run INTEGRATION-ACCESS-001 with backend/frontend/client/MCP 1.6.0: Blocked/Write/Read/Full, default blocked main MCP, unchanged generation, API/MCP per-client caps, atomic draft save, role statistics and revoked-role denial. | MSC-122: Template: test the retained API/MCP or guide/notification counterpart using its own catalog, actors and seeds. Follow checklist template scope and defect propagation requirements.</t>
+  </si>
+  <si>
+    <t>MSC-116. Watcher compilation and schema generation are not behavioral QA. Existing guide/API PASS does not cover this extension. | 2026-10-07: fixed missing profile.integration-access enabled-surface registration and Work/Community child guide content; existing parent shield and level/Apply/Close steps reused. guides/qa/evidence/general/EXPLANATION-GUIDE-001-20261007.md. Section 4 now names the manual Help checks. Manual status unchanged. MSC-119 extension 2026-10-07: guides/plans/MSC-119_MCP_READ_EVENTS_ROLE_GUIDANCE.md and guides/qa/evidence/general/MSC-119_GUIDE_WIRING_20261007.md. Source/build evidence only; no functional/browser/security/load PASS claimed. | 2026-10-11 MSC-122 follow-up REQUIRED: for each defect record template affected/unaffected with reason, source and template fix revisions, targeted template environment/result/evidence; affected propagation or verification stays open until completed. Source PASS does not imply template PASS. See guides/qa/checklists/README.md#template-regression-and-fix-propagation--msc-122. No execution status changed by this requirement.</t>
   </si>
   <si>
     <t>90/180</t>
@@ -538,10 +538,10 @@
     <t>Java/Go regression source prepared; execution deferred by user.</t>
   </si>
   <si>
-    <t>Run MCP-EVENTS-001 with MCP 1.6.0: Full-only Events, Read downgrade, ordinary owned-resource Events, role catalogs and node filters, role/grant revocation during delivery, queue limits/retries/idempotency and multiple users.</t>
-  </si>
-  <si>
-    <t>Source/build evidence only; no live ChatGPT callback or load test yet. MSC-119 extension 2026-10-07: guides/plans/MSC-119_MCP_READ_EVENTS_ROLE_GUIDANCE.md and guides/qa/evidence/general/MSC-119_GUIDE_WIRING_20261007.md. Source/build evidence only; no functional/browser/security/load PASS claimed.</t>
+    <t>Run MCP-EVENTS-001 with MCP 1.6.0: Full-only Events, Read downgrade, ordinary owned-resource Events, role catalogs and node filters, role/grant revocation during delivery, queue limits/retries/idempotency and multiple users. | MSC-122: Template: test the retained API/MCP or guide/notification counterpart using its own catalog, actors and seeds. Follow checklist template scope and defect propagation requirements.</t>
+  </si>
+  <si>
+    <t>Source/build evidence only; no live ChatGPT callback or load test yet. MSC-119 extension 2026-10-07: guides/plans/MSC-119_MCP_READ_EVENTS_ROLE_GUIDANCE.md and guides/qa/evidence/general/MSC-119_GUIDE_WIRING_20261007.md. Source/build evidence only; no functional/browser/security/load PASS claimed. | 2026-10-11 MSC-122 follow-up REQUIRED: for each defect record template affected/unaffected with reason, source and template fix revisions, targeted template environment/result/evidence; affected propagation or verification stays open until completed. Source PASS does not imply template PASS. See guides/qa/checklists/README.md#template-regression-and-fix-propagation--msc-122. No execution status changed by this requirement.</t>
   </si>
   <si>
     <t>CLEANUP</t>
@@ -904,7 +904,7 @@
     <t>See guides/plans/MULTI_GROUP_PRODUCT_DIRECTION_2026_10.md; code/build checks do not establish manual PASS. | 2026-10-07: compiled main-group identity/global paging checks and read-only HTTP paging/sync PASS; guides/qa/evidence/work-community/MAIN-GROUPS-20261007.md.</t>
   </si>
   <si>
-    <t>Website consent once across modes/groups; eight full EN/HU articles and unique images; green/multicolor theme; social icons/retry; aligned Read more; stable login/logout route, translated labels and ring. | Main-group landing label/icon/color after login; Groups base cards once at the entire filtered list start before pagination, never repeated per mobile page; private identity and counters retained.</t>
+    <t>Website consent once across modes/groups; eight full EN/HU articles and unique images; green/multicolor theme; social icons/retry; aligned Read more; stable login/logout route, translated labels and ring. | Main-group landing label/icon/color after login; Groups base cards once at the entire filtered list start before pagination, never repeated per mobile page; private identity and counters retained. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>ROLE-GUIDES-NOTIFICATIONS-001</t>
@@ -928,10 +928,10 @@
     <t>Compiled watcher runtime PASS; Java + isolated Mongo PASS; 222 live guide GETs PASS; seed parity PASS</t>
   </si>
   <si>
-    <t>Run checklists/general/ROLE-GUIDES-NOTIFICATIONS-001.md in EN/HU desktop/mobile Local/HTTP</t>
-  </si>
-  <si>
-    <t>Development evidence: guides/qa/evidence/general/ROLE-GUIDES-NOTIFICATIONS-001-20261007.md. No browser click-through, provider push or six-hour cycle claimed. https://github.com/fssrepository/myscoutee-roadmap/issues/156</t>
+    <t>Run checklists/general/ROLE-GUIDES-NOTIFICATIONS-001.md in EN/HU desktop/mobile Local/HTTP | MSC-122: Template: test the retained API/MCP or guide/notification counterpart using its own catalog, actors and seeds. Follow checklist template scope and defect propagation requirements.</t>
+  </si>
+  <si>
+    <t>Development evidence: guides/qa/evidence/general/ROLE-GUIDES-NOTIFICATIONS-001-20261007.md. No browser click-through, provider push or six-hour cycle claimed. https://github.com/fssrepository/myscoutee-roadmap/issues/156 | 2026-10-11 MSC-122 follow-up REQUIRED: for each defect record template affected/unaffected with reason, source and template fix revisions, targeted template environment/result/evidence; affected propagation or verification stays open until completed. Source PASS does not imply template PASS. See guides/qa/checklists/README.md#template-regression-and-fix-propagation--msc-122. No execution status changed by this requirement.</t>
   </si>
   <si>
     <t>60/120</t>
@@ -2659,7 +2659,7 @@
     <t>1. Create an event and select a Campaign through the existing selector-style control. Check capacity and priority-based invitation behavior. | 2. Open Events, select a Campaign filter and verify its title/subtitle, paging and displayed events. Clear the filter to return to all events. | 3. Check the Campaign filter in event feedback. Campaign chats use their own bucket; a whole-chat-list Campaign filter is deferred. Verify event creation, invitation, acceptance/removal and feedback notifications reach other affected participants only. | 4. Check that the scheduled random event generator does not create Work rooms.</t>
   </si>
   <si>
-    <t>Actors: Work event organizer and candidates. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Work event organizer and candidates. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-PAYMENT</t>
@@ -2671,7 +2671,7 @@
     <t>1. Open Payment history. The member control and expense/income totals share the second header row. The member button shows its avatar/count when selected and ends with a chevron; no selection shows All. Select one member with +, then confirm an empty basket to return to All. Check paging and both directions. | 2. Record cash received and bank transfer received from another member with amount/currency/note. Cash/transfer menu items and selected trigger use contextual icons/colors. Check matching historical entries, contextual method badge and payer-only notification. | 3. Retry the same save; check one receipt. Delete or request/approve a permitted manual refund and verify both histories/counters. No provider gateway is invoked for manual cash/transfer. | 4. Switch profile/group and verify filter/context isolation. Global profile totals are not replaced by the selected member subtotal. Alex’s local demo cards/payments match canonical demo amounts/dates and real counterparties.</t>
   </si>
   <si>
-    <t>Actors: Two members in each of Dating, Work and Community. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Two members in each of Dating, Work and Community. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>TOURNAMENT-001</t>
@@ -3127,7 +3127,7 @@
     <t>1. Create/operate Mingle or a Tournament in a private Community workspace using the existing controls. | 2. Check participant-only random mixing without affinity weighting, retained capacity/history rules and no automatic random-room scheduler for the Community base mode. | 3. As a participating manager start/advance manually: no own-action notification. Automatic phase changes notify affected participants. Compare the unchanged priority behavior in a Dating workspace.</t>
   </si>
   <si>
-    <t>Actors: Private Community manager; participants; Dating comparison group. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Private Community manager; participants; Dating comparison group. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>CHAT-AUTH-001</t>
@@ -3316,7 +3316,7 @@
     <t>1. Before a saved positive rating, verify the Campaign question action requires rating first. Rate, then open campaign Details through the Home eye or a campaign block in the aggregated Ratings history and choose Ask the organizer. | 2. Check the independent Campaign chat bucket, correct organizer, recipient-only new-message notification and unread badge. Reopening/retrying does not duplicate the chat or message. | 3. Create the corresponding real event: its group conversation uses the existing event chat owner and is separate from the direct Campaign question.</t>
   </si>
   <si>
-    <t>Actors: Campaign organizer and positively rating participant. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Campaign organizer and positively rating participant. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-CASE-CHAT</t>
@@ -3328,10 +3328,10 @@
     <t>1. Open the case chat from each permitted actor and inspect the Case bucket. Send a message; only other current chat participants get notification/unread increments. | 2. Mark read and reopen. Existing messages and other members’ unread counts survive case membership synchronization. | 3. Decline/remove the provider and check both HTTP and an already-open websocket against current case access. No private group membership is created. | 4. Chat Tasks opens only the target board, without an underlying Cases list or its list/counter requests. | 5. Close directly to chat; normal overview-to-board navigation retains its overview. | 6. Failed/denied detail shows a closable error without opening a Cases list; permitted retry works.</t>
   </si>
   <si>
-    <t>Actors: Manager; affected resident; invited provider. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md, MSC115-CASE-CHAT steps 1-6. Trace only requests caused by the Tasks click; one target detail, no Cases list or scheduled-task counter prefetch. CHAT-CALL-001 step 34 links this existing owner.</t>
-  </si>
-  <si>
-    <t>Prepared 2026-10-05 from user requirements. No browser actions or live data mutation performed. Preserve other completed campaign checkpoints. | 2026-10-06 conversation reconciliation: MSC-115 checklist updated; full flow remains NOT RUN. | 2026-10-07 guide expansion only: Tasks-button direct-board/close/error checks added from MSC-117 regression; no new manual run.</t>
+    <t>Actors: Manager; affected resident; invited provider. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md, MSC115-CASE-CHAT steps 1-6. Trace only requests caused by the Tasks click; one target detail, no Cases list or scheduled-task counter prefetch. CHAT-CALL-001 step 34 links this existing owner. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
+  </si>
+  <si>
+    <t>Prepared 2026-10-05 from user requirements. No browser actions or live data mutation performed. Preserve other completed campaign checkpoints. | 2026-10-06 conversation reconciliation: MSC-115 checklist updated; full flow remains NOT RUN. | 2026-10-07 guide expansion only: Tasks-button direct-board/close/error checks added from MSC-117 regression; no new manual run. | 2026-10-11 MSC-122 follow-up REQUIRED: for each defect record template affected/unaffected with reason, source and template fix revisions, targeted template environment/result/evidence; affected propagation or verification stays open until completed. Source PASS does not imply template PASS. See guides/qa/checklists/README.md#template-regression-and-fix-propagation--msc-122. No execution status changed by this requirement.</t>
   </si>
   <si>
     <t>CHAT-CALL-001</t>
@@ -3361,10 +3361,10 @@
     <t>PASS: 3 real WASM MLS, 2 PCM/FFT, 2 authenticated WebSocket tests; encrypted video control replay PASS; 4 watcher-AOT runtime checks for viewport/sender/SmartList/layout-reactivity PASS; existing watchers compile; all 50 call keys per language match live API</t>
   </si>
   <si>
-    <t>Follow guides/qa/checklists/general/CHAT-CALL-001.md steps 1-34. Revalidate the three-actor baseline after dev/demo reset; prepare at least seven distinct participants for full desktop pages. Record per-peer audio/video RTP deltas; use the linked MSC115-CASE-CHAT steps 4-6 for direct Tasks navigation and request counts.</t>
-  </si>
-  <si>
-    <t>MSC-117 https://github.com/fssrepository/myscoutee-roadmap/issues/155; guides/qa/evidence/CHAT-CALL-001-2026-10-06.json; isolated Alice admin/Bob/Carol fixture ready; browser checklist not executed by Codex | 2026-10-07 guide expansion only: 34 numbered steps; obsolete visible verification-code assertions removed; physical echo isolation and linked Tasks regression added. Earlier fixture-ready evidence is historical; revalidate after dev/demo reset. No new manual run.</t>
+    <t>Follow guides/qa/checklists/general/CHAT-CALL-001.md steps 1-34. Revalidate the three-actor baseline after dev/demo reset; prepare at least seven distinct participants for full desktop pages. Record per-peer audio/video RTP deltas; use the linked MSC115-CASE-CHAT steps 4-6 for direct Tasks navigation and request counts. | MSC-122: Template: assess/test retained chat/signaling/backend paths; minimal chat call UI is absent, so call-window steps are N/A. Follow checklist template scope and defect propagation requirements.</t>
+  </si>
+  <si>
+    <t>MSC-117 https://github.com/fssrepository/myscoutee-roadmap/issues/155; guides/qa/evidence/CHAT-CALL-001-2026-10-06.json; isolated Alice admin/Bob/Carol fixture ready; browser checklist not executed by Codex | 2026-10-07 guide expansion only: 34 numbered steps; obsolete visible verification-code assertions removed; physical echo isolation and linked Tasks regression added. Earlier fixture-ready evidence is historical; revalidate after dev/demo reset. No new manual run. | 2026-10-11 MSC-122 follow-up REQUIRED: for each defect record template affected/unaffected with reason, source and template fix revisions, targeted template environment/result/evidence; affected propagation or verification stays open until completed. Source PASS does not imply template PASS. See guides/qa/checklists/README.md#template-regression-and-fix-propagation--msc-122. No execution status changed by this requirement.</t>
   </si>
   <si>
     <t>30/60</t>
@@ -3670,7 +3670,7 @@
     <t>1. Create a Work private-group invite and a Community private-group invite using the existing invite action. Open each link in a clean prepared session. | 2. Check the relevant landing mode, then register/claim. Verify membership in the invited workspace and its base group, with the correct active profile. | 3. Switch to a Dating group from a Community account: its Dating behavior remains independent. Check joining an available base group is explicit and does not require approval. Promotional cards remain a later refinement.</t>
   </si>
   <si>
-    <t>Actors: Group manager; signed-out invitee. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Group manager; signed-out invitee. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-WORK-CAMPAIGN</t>
@@ -3682,7 +3682,7 @@
     <t>1. Open Campaigns next to Groups; create a draft through + with opportunity type, category, capacity, location, relevant filters and optional image. | 2. Save, reopen, publish, edit, unpublish, trash and restore using existing FormFlow/SmartList patterns. Observe write results without a full unrelated list reload. | 3. Check Work Home InfoCard text/images and three-dot read-only Campaign/author views while the rating bar is visible. Discovery follows opportunity/category and geographic criteria; private drafts stay private. Check the shared Dating-style frame, loading, paging and full-height empty state.</t>
   </si>
   <si>
-    <t>Actors: Work member as organizer; another Work member as participant. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Work member as organizer; another Work member as participant. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-WORK-RATING</t>
@@ -3694,7 +3694,7 @@
     <t>1. Rate two campaigns of the same author. Inspect the Ratings list: it displays people, with aggregate person rating when no Campaign filter is selected. | 2. Before the time control, open the Campaign basket popup. Select one item with +, which changes to a checkmark; inspect/remove the item in the header basket and confirm with the header checkmark. Selecting another replaces the single selection; closing cancels; confirming an empty basket returns to the aggregate view. The second header line names the selected Campaign; list paging and counters use that scope. | 3. Revise one rating. Check the corresponding write and aggregate query, including the opposite participant view. An unchanged retry must not create another notification. | 4. Use an unfiltered event for aggregate sympathy selection and a Campaign-selected event for campaign-specific selection; do not create horizontal channels or fake campaign events.</t>
   </si>
   <si>
-    <t>Owned Campaign menu → Ratings; no chooser in Activities; subtitle order; 8+9=8.5 write-side AVG and scoped scores; event priorities; per-card granular snapshot; history eye and paging.</t>
+    <t>Owned Campaign menu → Ratings; no chooser in Activities; subtitle order; 8+9=8.5 write-side AVG and scoped scores; event priorities; per-card granular snapshot; history eye and paging. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-SERVICE</t>
@@ -3706,7 +3706,7 @@
     <t>1. In base Community open the service InfoCard Home. Its header has category and Ratings controls; neither Your services nor the provisional Filters/distance popup is present. Check category selection, location-based ordering, and the two three-dot actions opening the full read-only service sheet and provider profile, including while the rating bar is visible. Empty results retain the Dating-style full-height frame/message; loading and paging use the same shared SmartList behavior. | 2. Open Your services from the sidebar Community block, not Cases or Home. Create/edit/publish/draft/trash/restore a sheet; category is on its form, without a separate category selector in the owned list. Check contextual cards/menus, a single sticky date header, + on the second row below Close, and labeled desktop List/Week/Month views. Week/Month show provider appointments. Configure staff, availability and existing pricing/slot inputs. | 3. Rate the provider through a service. Multiple services from that provider use the existing person priority. Publishing a sheet alone sends no unsolicited notification. | 4. Confirm a draft, deleted/inactive provider or another person’s private image is not exposed through discovery.</t>
   </si>
   <si>
-    <t>Actors: Anna as provider; Alex as customer; another eligible staff member. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Anna as provider; Alex as customer; another eligible staff member. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-CASE</t>
@@ -3718,7 +3718,7 @@
     <t>1. Create a case from Cases +, select the private community and a case type, then All or selected affected members with the existing basket picker. | 2. Check daily descending InfoCard groups with one sticky header, type-based card/menu colors, bottom-right contextual status badge, and the black affected-count button containing the number and chevron only. Click it to open the existing read-only member popup. Inspect status/type red unread counters across all pages, the aggregate base-group Cases badge and convenient private-group entry. | 3. Open the same case as another affected member and as a manager of multiple communities. Unrelated members cannot read it. | 4. Check lifecycle-appropriate three-dot actions: Start only while open; complete/cancel while active; reopen after completion/cancellation/deletion; no duplicate delete on deleted cases. Edit/close/reopen using these supported actions. Check targeted list/counter updates and notifications to affected others; the human actor receives none.</t>
   </si>
   <si>
-    <t>Actors: Alex; Maya; external provider Anna. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Alex; Maya; external provider Anna. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-CASE-PROVIDER</t>
@@ -3730,7 +3730,7 @@
     <t>1. As a member recommend a published service/provider. In the provider picker, + toggles to a checkmark; choosing another replaces the selection. Inspect/remove through the header basket; confirm applies and closing cancels. As manager inspect the recommendation and invite the chosen provider/staff member. | 2. As provider see the shared case in aggregate Community Cases, accept/decline and submit a quotation. As manager accept/reject the quotation. | 3. Check invitation/response/offer/decision notifications and their correct case destination. Repeating a provider invitation must preserve an accepted assignment. | 4. An external provider must not gain private-group navigation or announcement access. A declined invitation retains permitted case history but removes live case-chat access.</t>
   </si>
   <si>
-    <t>Actors: Community member; manager; external provider. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Community member; manager; external provider. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-SCHEDULE</t>
@@ -3742,7 +3742,7 @@
     <t>1. From the Cases header open Scheduled tasks and create a due date with All/selected members. Check the affected count in its SingleRow. | 2. At just before due minus 45 days, the scoped job creates nothing. At the boundary it creates one shared case and reminds all affected users, including an affected task creator. | 3. Rerun the same occurrence and simulate a delivery retry through the prepared test mechanism: no second case/reminder. Recurrence advances only after enqueueing. | 4. Check month/year recurrence and short-month dates. Edit/disable the task as permitted; Asset editor has no utility scheduling fields.</t>
   </si>
   <si>
-    <t>Actors: Manager; affected residents; selected provider when applicable. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Manager; affected residents; selected provider when applicable. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-APPOINTMENT</t>
@@ -3754,7 +3754,7 @@
     <t>1. Invite and accept the case provider/service, then open the actual existing slot picker from the case. Check day/week/month availability, templates and date overrides. | 2. Book a slot. Try an overlapping slot for that worker from another case/customer: conflict is rejected. Another worker’s capacity remains independent. | 3. Cancel a future appointment and verify availability is restored; retry save/cancel without duplicate rows or notifications. | 4. Inspect the provider’s aggregate calendar, customer and case labels, pricing snapshot and case link. Changing/unpublishing a service preserves prior bookings/audit; no fake asset/event or card charge is created.</t>
   </si>
   <si>
-    <t>Actors: Accepted case provider; two customers; second staff member. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Accepted case provider; two customers; second staff member. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-VOTING</t>
@@ -3766,7 +3766,7 @@
     <t>1. Configure apartment voting rights with one accepted assigned voter and positive weight. No Asset editor change or registration block is introduced. | 2. Publish a vote and cast each authorized ballot. Verify the first-publication rights snapshot, one final ballot per unit and denial of a replacement vote. | 3. Inspect member/admin results: correct weighted totals/counts without revealing others’ individual ballots. Unassigned residents cannot cast a unit ballot. | 4. Extend the deadline to reopen the published vote while retaining prior ballots. At expiry the Community-only job closes once and notifies participants; a cast vote notifies managers except its actor.</t>
   </si>
   <si>
-    <t>Actors: Admin; two assigned voters; unassigned resident. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Admin; two assigned voters; unassigned resident. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>SERVICE-FEEDBACK-UI-001</t>
@@ -3784,10 +3784,10 @@
     <t>Focused regression source prepared; execution deferred by user.</t>
   </si>
   <si>
-    <t>Run checklists/general/SERVICE-FEEDBACK-UI-001.md with approved feedback fixture in HTTP/local modes.</t>
-  </si>
-  <si>
-    <t>MSC-116. Watcher compilation and schema generation are not behavioral QA. Existing guide/API PASS does not cover this extension.</t>
+    <t>Run checklists/general/SERVICE-FEEDBACK-UI-001.md with approved feedback fixture in HTTP/local modes. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
+  </si>
+  <si>
+    <t>MSC-116. Watcher compilation and schema generation are not behavioral QA. Existing guide/API PASS does not cover this extension. | 2026-10-11 MSC-122 follow-up REQUIRED: for each defect record template affected/unaffected with reason, source and template fix revisions, targeted template environment/result/evidence; affected propagation or verification stays open until completed. Source PASS does not imply template PASS. See guides/qa/checklists/README.md#template-regression-and-fix-propagation--msc-122. No execution status changed by this requirement.</t>
   </si>
   <si>
     <t>P1 80</t>
@@ -3874,7 +3874,7 @@
     <t>1. Open private Community Home: newest-first SingleRow announcements grouped by day replace the rating stack, with a single sticky date header. Voting replaces Ratings in the sidebar Activities block; Your services remains in the Community block. | 2. As admin create a minimal draft with text and optional PDF/text/office attachments, then publish/edit/unpublish/trash/restore through three-dot actions and buckets. | 3. Check member visibility and color/action distinction for voting vs ordinary announcements. Members cannot publish directly; Feedback opens the existing group-admin chat. | 4. Test attachment download as a current member and denied outsider/former member. Unpublished documents remain admin/owner-only; normal feedback opening sends no notification.</t>
   </si>
   <si>
-    <t>Actors: Private Community admin; accepted resident; outsider. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Private Community admin; accepted resident; outsider. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MOBILE-PUSH-LIFECYCLE-001</t>
@@ -4210,7 +4210,7 @@
     <t>1. Switch Dating → Work → Community above the avatar. The menu structure stays consistent and all opened surfaces use the selected base group. | 2. Compare the selector red count with the existing menu counters; inspect moderation, reports, feedback, chat, content/articles, parameters, stats, metrics and graph in each scope. | 3. Change a scoped content item or parameter and return to another base group: its data is unchanged. A report retains the actor/action/event and optional group context without granting private-workspace membership. | 4. Open payment test tools from each scope and inspect their existing authorization link/context. Operator remains deployment-wide.</t>
   </si>
   <si>
-    <t>Actors: Ava; a second admin profile if needed. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | Main-group landing label/icon/color after login; Groups base cards once at the entire filtered list start before pagination, never repeated per mobile page; private identity and counters retained.</t>
+    <t>Actors: Ava; a second admin profile if needed. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | Main-group landing label/icon/color after login; Groups base cards once at the entire filtered list start before pagination, never repeated per mobile page; private identity and counters retained. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-JOBS</t>
@@ -4222,7 +4222,7 @@
     <t>1. Open Jobs in every base group. Confirm independent seeded definitions, enabled state, timing and run history. | 2. Run an available scoped job and inspect only that scope’s results, progress, counters and history. Do not enable absent/inapplicable random-room jobs in Work or Community. | 3. Inspect Community scheduled-case and vote-close jobs. Confirm shared notification/exchange/processing definitions have separate group items and that an unseeded job does not execute for that group.</t>
   </si>
   <si>
-    <t>Actors: Ava. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Ava. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>EXPLANATION-GUIDE-001</t>
@@ -4243,10 +4243,10 @@
     <t>2026-10-07: EN/HU catalog/i18n and guide-field seed parity; revision/section parity for chats, event.chat, chat.call, chat.call.volume and landing.guide across Dating/Work/Community and all three Mongo seeds. Existing watcher AOT call/guide context and intro lifecycle checks PASS. Public intro HTTP EN/HU x 3 modes PASS; private call context denial 404 PASS. Browser tour NOT RUN. Follow-up: watcher AOT launcher geometry (1500 cases, 400 Rates rechecks) and versioned introduction lifecycle/text parity PASS. See guides/qa/evidence/general/EXPLANATION-GUIDE-001-20261007.md. Consent follow-up: watcher AOT directive/service/Accept target PASS; 200 target checks reuse one index scan. Live public consent HTTP EN/HU x 3 modes PASS; private-context 404 preserved. | 2026-10-07 isolated CDP regression PASS (EN desktop / 390x844 mobile): dismissed consent stays closed on group switch; correct images on first selection; Login reopens consent; one stable consent Help step with translated label; duplicate Privacy summary removed. SW 20/20 PASS; EN/HU live seed/translation parity PASS. | Mobile header follow-up: 24 isolated CDP cases PASS (EN/HU x 320/360/390/1236px x 3 groups): full label/caret, one-line Login/Belépés, no header overlap. Translation .7 live/source/seed parity PASS. | 2026-10-07 shared missing-guide feedback: watcher-AOT DOM regression PASS for persistent centered EN/HU message, cold/cached/empty cases, X/Escape/Back/launcher/shade dismissal, Next/Back/Done and 200 viewport notifications with zero rescans.</t>
   </si>
   <si>
-    <t>Run the MSC-119 section plus retained unexecuted WebRTC/introduction/consent sections: all affected Work/Community/API/MCP and shared terms guides, EN/HU desktop/mobile local/HTTP, empty/populated and read-only/edit states; header title/X alignment; parent restoration; no business writes during guide-only navigation.</t>
-  </si>
-  <si>
-    <t>45 contexts / 963 fields. Existing recorded scope retained. Added landing: 64 steps per viewport; feedback: 39 per viewport; Rates arrow-only, shared double-panel highlights and editable badge passed at mobile/desktop. EN/HU local/demo/e2e/prod seed parity. Landing visit visibility, internal default ON/preserved OFF, fresh-browser consent and shared guide/notification clearance above rating actions/profile eyes passed mobile/desktop. Mobile-only launcher clearance; unchanged desktop positioning; pair divider hover/tap/drag and fixed photo scale at 0/50/100% passed Home/Rates browser and Android Rates over ADB. Mobile pair image fit unified to contain on Home/Activity Rates; both targeted browser checks passed, desktop preserved. Guide screenshots removed from Git. No final form submission. Full local persistence and native WebView not claimed. guides/qa/evidence/general/EXPLANATION-GUIDE-001-20260930.md Final Android Home rail stability, mobile/desktop guide card continuity and filter badge save/reload/restore passed. No screenshots committed. Earlier Android fullscreen/drag lag was confirmed; the subsequent retained-panel and image-scroll fixes below were accepted and close that follow-up. No universal performance PASS is claimed. Follow-up: one retained list row rebuilt instead of six; one DTO snapshot per card; hidden controls excluded from launcher measurement. Native menu/guide visibility and raised list badge clearance passed. Small warm RAF-proxy medians: fullscreen 293 to 254ms, list 161 to 108ms; these preliminary measurements are superseded by the final user-accepted retained-panel result below. Final user-accepted retained-panel change: one shared loaded collection; persistent list/fullscreen DOM; z-order-only presentation; inactive new-image gating; no warm card rebuilds or switch scroll shift; saved-score paging identity preserved. Warm fullscreen median207.9→127.7ms; list103→128.1ms (dev two-RAF proxy, no universal performance claim). Rates list-scroll launchers fixed: native100-frame check0/0px movement versus48/56px before. Follow-up: panel-bottom launcher anchor56px list/96px fullscreen; native scroll0/0px. Whole-card scroll preview/adaptive prefetch withdrawn. Image-only handling preserves visible photos; only offscreen/passed photos suspend, returning once from cache. Fast-scroll requests/spinners0; sampled visible-image flickers0; focused tests15/15. See phone-image-scroll.json. Mobile photo badges/eye/image indicators follow per-image suspension; individual/pair native swipe90frames each passed; user accepted. Release1.3.2: both guide branches consolidated/master merged; GHCR frontend/backend images; Netcup migration010 retained-data check;8 healthy containers; publicHTTP13/13 and landing guide10/10 plus private-context denial passed. See RELEASE_1.3.2_20260930.json. Launcher follow-up: desktop icons remain with menus; guide above shade; bell layering unchanged; mobile menus hide both icons without hiding tour;1280/390px regression passed and user accepted.; Accepted launcher follow-up republished1.3.2: nginx-only Netcup update,13/13 HTTP PASS,8 healthy containers,7 unchanged. Final ledger closure 2026-09-30: PASS / CLOSED for the accepted guide scope and follow-ups; no remaining guide oracle. Local PARTIAL records the untested persistence boundary, not an open guide defect. 2026-10-01 scoped granular-rating addendum: Home/Activity list/fullscreen CDP at1280/390; no-backdrop popup, equal-width bar, mobile menu launcher hiding, integer details, profile-count-derived main step, exact6.75 save/reload and affinity precision, EN/HU guide/i18n parity. Existing PASS/CLOSED retained; see granular-rating-checks.json and rating-step-checks.json in the linked evidence. | 2026-10-06: user explicitly reopens for expanded scope. September PASS remains historical evidence, not current completion. | 2026-10-07: Added 17 call + 7 volume catalog fields, phone steps in chats/event.chat and the one-step landing.guide intro; workspace-specific EN/HU content seeded. Existing shared guide engine/launcher reused. Watcher frontend build and backend hot-deploy PASS; check-chat-call-runtime.mjs PASS including nested guide/context/language/destruction checks. Compiled Guide first-visit/dismissal/known-visitor/transition checks PASS; consent and saved guide preference unchanged. Public intro HTTP 6/6 plus private-context denial PASS. Targeted audit-seeds.py --context chats --context event.chat --context chat.call --context chat.call.volume --context landing.guide PASS; i18n audit and sync-work-seeds.js --check PASS. Full revision audit is not a PASS: pre-existing home.game rating-details and payment.history counterparty steps are absent from global HTTP revisions; left outside this change. At that earlier checkpoint, launcher component and placeCard positioning were identical to HEAD after the positioning edits were withdrawn. No browser actions, fixture staging or full guide click-through performed. September evidence remains historical; new manual status NOT RUN. | 2026-10-07 authorized follow-up: launcher-to-launcher clearance repaired using registered references; Rates stable panel anchors and Help card placement preserved. Bounded geometry/lifecycle checks PASS; single-step HU163/EN166 introduction explains drag, red-X hide and Side menu Explanations OFF/ON. QA CSV line endings normalized. Evidence: guides/qa/evidence/general/EXPLANATION-GUIDE-001-20261007.md. Manual browser status remains NOT RUN. | 2026-10-07 consent follow-up: landing.consent one-step Accept binding; canonical source and all Mongo seeds synchronized. Introduction now explicitly names the notification bell (HU156/EN155). i18n version 2026.10.07.5. Development checks PASS; browser manual NOT RUN. | Later user-authorized fresh anonymous browser evidence: guides/qa/evidence/general/EXPLANATION-GUIDE-001-20261007.md, landing follow-up. No full manual case replay, acceptance/registration or fixture reset; historical status preserved. | Article/no-guide follow-up: shared guide feedback now remains centered until dismissed instead of flashing closed. Per-surface checklist step 9 added. Focused JSDOM evidence only; manual campaign status unchanged. guides/qa/evidence/general/EXPLANATION-GUIDE-001-20261007.md. | 2026-10-07 operator/app-admin audit: GAP, no dedicated surface registrations/catalog fields/revisions; operator launcher excluded; Explanations toggle excluded for both privileged roles. Common avatar-menu guide is not role-surface coverage. See evidence/general/EXPLANATION-GUIDE-001-20261007.md#operator--app-admin-wiring-audit. | MSC-118: prior role wiring gap implemented; 37 system contexts / 136 fields, shared launchers and role notifications have dedicated ROLE-GUIDES-NOTIFICATIONS-001 checklist/evidence. Manual role QA NOT RUN. MSC-119 extension 2026-10-07: guides/plans/MSC-119_MCP_READ_EVENTS_ROLE_GUIDANCE.md and guides/qa/evidence/general/MSC-119_GUIDE_WIRING_20261007.md. Source/build evidence only; no functional/browser/security/load PASS claimed.</t>
+    <t>Run the MSC-119 section plus retained unexecuted WebRTC/introduction/consent sections: all affected Work/Community/API/MCP and shared terms guides, EN/HU desktop/mobile local/HTTP, empty/populated and read-only/edit states; header title/X alignment; parent restoration; no business writes during guide-only navigation. | MSC-122: Template: test the retained API/MCP or guide/notification counterpart using its own catalog, actors and seeds. Follow checklist template scope and defect propagation requirements.</t>
+  </si>
+  <si>
+    <t>45 contexts / 963 fields. Existing recorded scope retained. Added landing: 64 steps per viewport; feedback: 39 per viewport; Rates arrow-only, shared double-panel highlights and editable badge passed at mobile/desktop. EN/HU local/demo/e2e/prod seed parity. Landing visit visibility, internal default ON/preserved OFF, fresh-browser consent and shared guide/notification clearance above rating actions/profile eyes passed mobile/desktop. Mobile-only launcher clearance; unchanged desktop positioning; pair divider hover/tap/drag and fixed photo scale at 0/50/100% passed Home/Rates browser and Android Rates over ADB. Mobile pair image fit unified to contain on Home/Activity Rates; both targeted browser checks passed, desktop preserved. Guide screenshots removed from Git. No final form submission. Full local persistence and native WebView not claimed. guides/qa/evidence/general/EXPLANATION-GUIDE-001-20260930.md Final Android Home rail stability, mobile/desktop guide card continuity and filter badge save/reload/restore passed. No screenshots committed. Earlier Android fullscreen/drag lag was confirmed; the subsequent retained-panel and image-scroll fixes below were accepted and close that follow-up. No universal performance PASS is claimed. Follow-up: one retained list row rebuilt instead of six; one DTO snapshot per card; hidden controls excluded from launcher measurement. Native menu/guide visibility and raised list badge clearance passed. Small warm RAF-proxy medians: fullscreen 293 to 254ms, list 161 to 108ms; these preliminary measurements are superseded by the final user-accepted retained-panel result below. Final user-accepted retained-panel change: one shared loaded collection; persistent list/fullscreen DOM; z-order-only presentation; inactive new-image gating; no warm card rebuilds or switch scroll shift; saved-score paging identity preserved. Warm fullscreen median207.9→127.7ms; list103→128.1ms (dev two-RAF proxy, no universal performance claim). Rates list-scroll launchers fixed: native100-frame check0/0px movement versus48/56px before. Follow-up: panel-bottom launcher anchor56px list/96px fullscreen; native scroll0/0px. Whole-card scroll preview/adaptive prefetch withdrawn. Image-only handling preserves visible photos; only offscreen/passed photos suspend, returning once from cache. Fast-scroll requests/spinners0; sampled visible-image flickers0; focused tests15/15. See phone-image-scroll.json. Mobile photo badges/eye/image indicators follow per-image suspension; individual/pair native swipe90frames each passed; user accepted. Release1.3.2: both guide branches consolidated/master merged; GHCR frontend/backend images; Netcup migration010 retained-data check;8 healthy containers; publicHTTP13/13 and landing guide10/10 plus private-context denial passed. See RELEASE_1.3.2_20260930.json. Launcher follow-up: desktop icons remain with menus; guide above shade; bell layering unchanged; mobile menus hide both icons without hiding tour;1280/390px regression passed and user accepted.; Accepted launcher follow-up republished1.3.2: nginx-only Netcup update,13/13 HTTP PASS,8 healthy containers,7 unchanged. Final ledger closure 2026-09-30: PASS / CLOSED for the accepted guide scope and follow-ups; no remaining guide oracle. Local PARTIAL records the untested persistence boundary, not an open guide defect. 2026-10-01 scoped granular-rating addendum: Home/Activity list/fullscreen CDP at1280/390; no-backdrop popup, equal-width bar, mobile menu launcher hiding, integer details, profile-count-derived main step, exact6.75 save/reload and affinity precision, EN/HU guide/i18n parity. Existing PASS/CLOSED retained; see granular-rating-checks.json and rating-step-checks.json in the linked evidence. | 2026-10-06: user explicitly reopens for expanded scope. September PASS remains historical evidence, not current completion. | 2026-10-07: Added 17 call + 7 volume catalog fields, phone steps in chats/event.chat and the one-step landing.guide intro; workspace-specific EN/HU content seeded. Existing shared guide engine/launcher reused. Watcher frontend build and backend hot-deploy PASS; check-chat-call-runtime.mjs PASS including nested guide/context/language/destruction checks. Compiled Guide first-visit/dismissal/known-visitor/transition checks PASS; consent and saved guide preference unchanged. Public intro HTTP 6/6 plus private-context denial PASS. Targeted audit-seeds.py --context chats --context event.chat --context chat.call --context chat.call.volume --context landing.guide PASS; i18n audit and sync-work-seeds.js --check PASS. Full revision audit is not a PASS: pre-existing home.game rating-details and payment.history counterparty steps are absent from global HTTP revisions; left outside this change. At that earlier checkpoint, launcher component and placeCard positioning were identical to HEAD after the positioning edits were withdrawn. No browser actions, fixture staging or full guide click-through performed. September evidence remains historical; new manual status NOT RUN. | 2026-10-07 authorized follow-up: launcher-to-launcher clearance repaired using registered references; Rates stable panel anchors and Help card placement preserved. Bounded geometry/lifecycle checks PASS; single-step HU163/EN166 introduction explains drag, red-X hide and Side menu Explanations OFF/ON. QA CSV line endings normalized. Evidence: guides/qa/evidence/general/EXPLANATION-GUIDE-001-20261007.md. Manual browser status remains NOT RUN. | 2026-10-07 consent follow-up: landing.consent one-step Accept binding; canonical source and all Mongo seeds synchronized. Introduction now explicitly names the notification bell (HU156/EN155). i18n version 2026.10.07.5. Development checks PASS; browser manual NOT RUN. | Later user-authorized fresh anonymous browser evidence: guides/qa/evidence/general/EXPLANATION-GUIDE-001-20261007.md, landing follow-up. No full manual case replay, acceptance/registration or fixture reset; historical status preserved. | Article/no-guide follow-up: shared guide feedback now remains centered until dismissed instead of flashing closed. Per-surface checklist step 9 added. Focused JSDOM evidence only; manual campaign status unchanged. guides/qa/evidence/general/EXPLANATION-GUIDE-001-20261007.md. | 2026-10-07 operator/app-admin audit: GAP, no dedicated surface registrations/catalog fields/revisions; operator launcher excluded; Explanations toggle excluded for both privileged roles. Common avatar-menu guide is not role-surface coverage. See evidence/general/EXPLANATION-GUIDE-001-20261007.md#operator--app-admin-wiring-audit. | MSC-118: prior role wiring gap implemented; 37 system contexts / 136 fields, shared launchers and role notifications have dedicated ROLE-GUIDES-NOTIFICATIONS-001 checklist/evidence. Manual role QA NOT RUN. MSC-119 extension 2026-10-07: guides/plans/MSC-119_MCP_READ_EVENTS_ROLE_GUIDANCE.md and guides/qa/evidence/general/MSC-119_GUIDE_WIRING_20261007.md. Source/build evidence only; no functional/browser/security/load PASS claimed. | 2026-10-11 MSC-122 follow-up REQUIRED: for each defect record template affected/unaffected with reason, source and template fix revisions, targeted template environment/result/evidence; affected propagation or verification stays open until completed. Source PASS does not imply template PASS. See guides/qa/checklists/README.md#template-regression-and-fix-propagation--msc-122. No execution status changed by this requirement.</t>
   </si>
   <si>
     <t>MSC115-GUIDES</t>
@@ -4258,7 +4258,7 @@
     <t>1. Open the guide at landing/Home mode switch, Campaign list/editor, service Home/list/editor/calendar, Cases/tasks/editors/appointments, private Home/Voting/rights and payment history/receipt. | 2. Check the explanation targets the visible control and describes the current group’s behavior in English and Hungarian. Lazy-opened popups get their own registered context. | 3. Switch modes while popups/requests are active. Check stale responses and selections do not populate another profile, no duplicate HTTP clients are used and badges clear according to existing read actions.</t>
   </si>
   <si>
-    <t>Expanded EXPLANATION-GUIDE-001 shared execution; 28 revised contexts, all new controls and EN/HU, preserve historical PASS evidence.</t>
+    <t>Expanded EXPLANATION-GUIDE-001 shared execution; 28 revised contexts, all new controls and EN/HU, preserve historical PASS evidence. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>OPERATOR-CONFIGURATION-LIFECYCLE-001</t>

</xml_diff>

<commit_message>
[MSC-122] Separate reusable application foundations and qualify version 1.4.0 delivery
</commit_message>
<xml_diff>
--- a/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
+++ b/guides/qa/matrices/ADMIN_DYNAMIC_SURFACES_QA_MATRIX.xlsx
@@ -466,10 +466,10 @@
     <t>See guides/plans/MULTI_GROUP_PRODUCT_DIRECTION_2026_10.md; code/build checks do not establish manual PASS.</t>
   </si>
   <si>
-    <t>Actors: Authorized Work member API/MCP identity. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
-  </si>
-  <si>
-    <t>Prepared 2026-10-05 from user requirements. No browser actions or live data mutation performed. Preserve other completed campaign checkpoints. | 2026-10-06 conversation reconciliation: MSC-115 checklist updated; full flow remains NOT RUN.</t>
+    <t>Actors: Authorized Work member API/MCP identity. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
+  </si>
+  <si>
+    <t>Prepared 2026-10-05 from user requirements. No browser actions or live data mutation performed. Preserve other completed campaign checkpoints. | 2026-10-06 conversation reconciliation: MSC-115 checklist updated; full flow remains NOT RUN. | 2026-10-11 MSC-122 follow-up REQUIRED: for each defect record template affected/unaffected with reason, source and template fix revisions, targeted template environment/result/evidence; affected propagation or verification stays open until completed. Source PASS does not imply template PASS. See guides/qa/checklists/README.md#template-regression-and-fix-propagation--msc-122. No execution status changed by this requirement.</t>
   </si>
   <si>
     <t>P1</t>
@@ -502,10 +502,10 @@
     <t>Focused regression source prepared; execution deferred by user. 2026-10-07 Help-only watcher-AOT check PASS: enabled parent/child contexts, EN/HU in Dating/Work/Community, bounded loads and cleanup; scoped/local/Mongo seed parity PASS. Permission enforcement remains untested here.</t>
   </si>
   <si>
-    <t>Run INTEGRATION-ACCESS-001 with backend/frontend/client/MCP 1.6.0: Blocked/Write/Read/Full, default blocked main MCP, unchanged generation, API/MCP per-client caps, atomic draft save, role statistics and revoked-role denial.</t>
-  </si>
-  <si>
-    <t>MSC-116. Watcher compilation and schema generation are not behavioral QA. Existing guide/API PASS does not cover this extension. | 2026-10-07: fixed missing profile.integration-access enabled-surface registration and Work/Community child guide content; existing parent shield and level/Apply/Close steps reused. guides/qa/evidence/general/EXPLANATION-GUIDE-001-20261007.md. Section 4 now names the manual Help checks. Manual status unchanged. MSC-119 extension 2026-10-07: guides/plans/MSC-119_MCP_READ_EVENTS_ROLE_GUIDANCE.md and guides/qa/evidence/general/MSC-119_GUIDE_WIRING_20261007.md. Source/build evidence only; no functional/browser/security/load PASS claimed.</t>
+    <t>Run INTEGRATION-ACCESS-001 with backend/frontend/client/MCP 1.6.0: Blocked/Write/Read/Full, default blocked main MCP, unchanged generation, API/MCP per-client caps, atomic draft save, role statistics and revoked-role denial. | MSC-122: Template: test the retained API/MCP or guide/notification counterpart using its own catalog, actors and seeds. Follow checklist template scope and defect propagation requirements.</t>
+  </si>
+  <si>
+    <t>MSC-116. Watcher compilation and schema generation are not behavioral QA. Existing guide/API PASS does not cover this extension. | 2026-10-07: fixed missing profile.integration-access enabled-surface registration and Work/Community child guide content; existing parent shield and level/Apply/Close steps reused. guides/qa/evidence/general/EXPLANATION-GUIDE-001-20261007.md. Section 4 now names the manual Help checks. Manual status unchanged. MSC-119 extension 2026-10-07: guides/plans/MSC-119_MCP_READ_EVENTS_ROLE_GUIDANCE.md and guides/qa/evidence/general/MSC-119_GUIDE_WIRING_20261007.md. Source/build evidence only; no functional/browser/security/load PASS claimed. | 2026-10-11 MSC-122 follow-up REQUIRED: for each defect record template affected/unaffected with reason, source and template fix revisions, targeted template environment/result/evidence; affected propagation or verification stays open until completed. Source PASS does not imply template PASS. See guides/qa/checklists/README.md#template-regression-and-fix-propagation--msc-122. No execution status changed by this requirement.</t>
   </si>
   <si>
     <t>90/180</t>
@@ -538,10 +538,10 @@
     <t>Java/Go regression source prepared; execution deferred by user.</t>
   </si>
   <si>
-    <t>Run MCP-EVENTS-001 with MCP 1.6.0: Full-only Events, Read downgrade, ordinary owned-resource Events, role catalogs and node filters, role/grant revocation during delivery, queue limits/retries/idempotency and multiple users.</t>
-  </si>
-  <si>
-    <t>Source/build evidence only; no live ChatGPT callback or load test yet. MSC-119 extension 2026-10-07: guides/plans/MSC-119_MCP_READ_EVENTS_ROLE_GUIDANCE.md and guides/qa/evidence/general/MSC-119_GUIDE_WIRING_20261007.md. Source/build evidence only; no functional/browser/security/load PASS claimed.</t>
+    <t>Run MCP-EVENTS-001 with MCP 1.6.0: Full-only Events, Read downgrade, ordinary owned-resource Events, role catalogs and node filters, role/grant revocation during delivery, queue limits/retries/idempotency and multiple users. | MSC-122: Template: test the retained API/MCP or guide/notification counterpart using its own catalog, actors and seeds. Follow checklist template scope and defect propagation requirements.</t>
+  </si>
+  <si>
+    <t>Source/build evidence only; no live ChatGPT callback or load test yet. MSC-119 extension 2026-10-07: guides/plans/MSC-119_MCP_READ_EVENTS_ROLE_GUIDANCE.md and guides/qa/evidence/general/MSC-119_GUIDE_WIRING_20261007.md. Source/build evidence only; no functional/browser/security/load PASS claimed. | 2026-10-11 MSC-122 follow-up REQUIRED: for each defect record template affected/unaffected with reason, source and template fix revisions, targeted template environment/result/evidence; affected propagation or verification stays open until completed. Source PASS does not imply template PASS. See guides/qa/checklists/README.md#template-regression-and-fix-propagation--msc-122. No execution status changed by this requirement.</t>
   </si>
   <si>
     <t>CLEANUP</t>
@@ -904,7 +904,7 @@
     <t>See guides/plans/MULTI_GROUP_PRODUCT_DIRECTION_2026_10.md; code/build checks do not establish manual PASS. | 2026-10-07: compiled main-group identity/global paging checks and read-only HTTP paging/sync PASS; guides/qa/evidence/work-community/MAIN-GROUPS-20261007.md.</t>
   </si>
   <si>
-    <t>Website consent once across modes/groups; eight full EN/HU articles and unique images; green/multicolor theme; social icons/retry; aligned Read more; stable login/logout route, translated labels and ring. | Main-group landing label/icon/color after login; Groups base cards once at the entire filtered list start before pagination, never repeated per mobile page; private identity and counters retained.</t>
+    <t>Website consent once across modes/groups; eight full EN/HU articles and unique images; green/multicolor theme; social icons/retry; aligned Read more; stable login/logout route, translated labels and ring. | Main-group landing label/icon/color after login; Groups base cards once at the entire filtered list start before pagination, never repeated per mobile page; private identity and counters retained. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>ROLE-GUIDES-NOTIFICATIONS-001</t>
@@ -928,10 +928,10 @@
     <t>Compiled watcher runtime PASS; Java + isolated Mongo PASS; 222 live guide GETs PASS; seed parity PASS</t>
   </si>
   <si>
-    <t>Run checklists/general/ROLE-GUIDES-NOTIFICATIONS-001.md in EN/HU desktop/mobile Local/HTTP</t>
-  </si>
-  <si>
-    <t>Development evidence: guides/qa/evidence/general/ROLE-GUIDES-NOTIFICATIONS-001-20261007.md. No browser click-through, provider push or six-hour cycle claimed. https://github.com/fssrepository/myscoutee-roadmap/issues/156</t>
+    <t>Run checklists/general/ROLE-GUIDES-NOTIFICATIONS-001.md in EN/HU desktop/mobile Local/HTTP | MSC-122: Template: test the retained API/MCP or guide/notification counterpart using its own catalog, actors and seeds. Follow checklist template scope and defect propagation requirements.</t>
+  </si>
+  <si>
+    <t>Development evidence: guides/qa/evidence/general/ROLE-GUIDES-NOTIFICATIONS-001-20261007.md. No browser click-through, provider push or six-hour cycle claimed. https://github.com/fssrepository/myscoutee-roadmap/issues/156 | 2026-10-11 MSC-122 follow-up REQUIRED: for each defect record template affected/unaffected with reason, source and template fix revisions, targeted template environment/result/evidence; affected propagation or verification stays open until completed. Source PASS does not imply template PASS. See guides/qa/checklists/README.md#template-regression-and-fix-propagation--msc-122. No execution status changed by this requirement.</t>
   </si>
   <si>
     <t>60/120</t>
@@ -2659,7 +2659,7 @@
     <t>1. Create an event and select a Campaign through the existing selector-style control. Check capacity and priority-based invitation behavior. | 2. Open Events, select a Campaign filter and verify its title/subtitle, paging and displayed events. Clear the filter to return to all events. | 3. Check the Campaign filter in event feedback. Campaign chats use their own bucket; a whole-chat-list Campaign filter is deferred. Verify event creation, invitation, acceptance/removal and feedback notifications reach other affected participants only. | 4. Check that the scheduled random event generator does not create Work rooms.</t>
   </si>
   <si>
-    <t>Actors: Work event organizer and candidates. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Work event organizer and candidates. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-PAYMENT</t>
@@ -2671,7 +2671,7 @@
     <t>1. Open Payment history. The member control and expense/income totals share the second header row. The member button shows its avatar/count when selected and ends with a chevron; no selection shows All. Select one member with +, then confirm an empty basket to return to All. Check paging and both directions. | 2. Record cash received and bank transfer received from another member with amount/currency/note. Cash/transfer menu items and selected trigger use contextual icons/colors. Check matching historical entries, contextual method badge and payer-only notification. | 3. Retry the same save; check one receipt. Delete or request/approve a permitted manual refund and verify both histories/counters. No provider gateway is invoked for manual cash/transfer. | 4. Switch profile/group and verify filter/context isolation. Global profile totals are not replaced by the selected member subtotal. Alex’s local demo cards/payments match canonical demo amounts/dates and real counterparties.</t>
   </si>
   <si>
-    <t>Actors: Two members in each of Dating, Work and Community. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Two members in each of Dating, Work and Community. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>TOURNAMENT-001</t>
@@ -3127,7 +3127,7 @@
     <t>1. Create/operate Mingle or a Tournament in a private Community workspace using the existing controls. | 2. Check participant-only random mixing without affinity weighting, retained capacity/history rules and no automatic random-room scheduler for the Community base mode. | 3. As a participating manager start/advance manually: no own-action notification. Automatic phase changes notify affected participants. Compare the unchanged priority behavior in a Dating workspace.</t>
   </si>
   <si>
-    <t>Actors: Private Community manager; participants; Dating comparison group. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Private Community manager; participants; Dating comparison group. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>CHAT-AUTH-001</t>
@@ -3316,7 +3316,7 @@
     <t>1. Before a saved positive rating, verify the Campaign question action requires rating first. Rate, then open campaign Details through the Home eye or a campaign block in the aggregated Ratings history and choose Ask the organizer. | 2. Check the independent Campaign chat bucket, correct organizer, recipient-only new-message notification and unread badge. Reopening/retrying does not duplicate the chat or message. | 3. Create the corresponding real event: its group conversation uses the existing event chat owner and is separate from the direct Campaign question.</t>
   </si>
   <si>
-    <t>Actors: Campaign organizer and positively rating participant. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Campaign organizer and positively rating participant. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-CASE-CHAT</t>
@@ -3328,10 +3328,10 @@
     <t>1. Open the case chat from each permitted actor and inspect the Case bucket. Send a message; only other current chat participants get notification/unread increments. | 2. Mark read and reopen. Existing messages and other members’ unread counts survive case membership synchronization. | 3. Decline/remove the provider and check both HTTP and an already-open websocket against current case access. No private group membership is created. | 4. Chat Tasks opens only the target board, without an underlying Cases list or its list/counter requests. | 5. Close directly to chat; normal overview-to-board navigation retains its overview. | 6. Failed/denied detail shows a closable error without opening a Cases list; permitted retry works.</t>
   </si>
   <si>
-    <t>Actors: Manager; affected resident; invited provider. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md, MSC115-CASE-CHAT steps 1-6. Trace only requests caused by the Tasks click; one target detail, no Cases list or scheduled-task counter prefetch. CHAT-CALL-001 step 34 links this existing owner.</t>
-  </si>
-  <si>
-    <t>Prepared 2026-10-05 from user requirements. No browser actions or live data mutation performed. Preserve other completed campaign checkpoints. | 2026-10-06 conversation reconciliation: MSC-115 checklist updated; full flow remains NOT RUN. | 2026-10-07 guide expansion only: Tasks-button direct-board/close/error checks added from MSC-117 regression; no new manual run.</t>
+    <t>Actors: Manager; affected resident; invited provider. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md, MSC115-CASE-CHAT steps 1-6. Trace only requests caused by the Tasks click; one target detail, no Cases list or scheduled-task counter prefetch. CHAT-CALL-001 step 34 links this existing owner. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
+  </si>
+  <si>
+    <t>Prepared 2026-10-05 from user requirements. No browser actions or live data mutation performed. Preserve other completed campaign checkpoints. | 2026-10-06 conversation reconciliation: MSC-115 checklist updated; full flow remains NOT RUN. | 2026-10-07 guide expansion only: Tasks-button direct-board/close/error checks added from MSC-117 regression; no new manual run. | 2026-10-11 MSC-122 follow-up REQUIRED: for each defect record template affected/unaffected with reason, source and template fix revisions, targeted template environment/result/evidence; affected propagation or verification stays open until completed. Source PASS does not imply template PASS. See guides/qa/checklists/README.md#template-regression-and-fix-propagation--msc-122. No execution status changed by this requirement.</t>
   </si>
   <si>
     <t>CHAT-CALL-001</t>
@@ -3361,10 +3361,10 @@
     <t>PASS: 3 real WASM MLS, 2 PCM/FFT, 2 authenticated WebSocket tests; encrypted video control replay PASS; 4 watcher-AOT runtime checks for viewport/sender/SmartList/layout-reactivity PASS; existing watchers compile; all 50 call keys per language match live API</t>
   </si>
   <si>
-    <t>Follow guides/qa/checklists/general/CHAT-CALL-001.md steps 1-34. Revalidate the three-actor baseline after dev/demo reset; prepare at least seven distinct participants for full desktop pages. Record per-peer audio/video RTP deltas; use the linked MSC115-CASE-CHAT steps 4-6 for direct Tasks navigation and request counts.</t>
-  </si>
-  <si>
-    <t>MSC-117 https://github.com/fssrepository/myscoutee-roadmap/issues/155; guides/qa/evidence/CHAT-CALL-001-2026-10-06.json; isolated Alice admin/Bob/Carol fixture ready; browser checklist not executed by Codex | 2026-10-07 guide expansion only: 34 numbered steps; obsolete visible verification-code assertions removed; physical echo isolation and linked Tasks regression added. Earlier fixture-ready evidence is historical; revalidate after dev/demo reset. No new manual run.</t>
+    <t>Follow guides/qa/checklists/general/CHAT-CALL-001.md steps 1-34. Revalidate the three-actor baseline after dev/demo reset; prepare at least seven distinct participants for full desktop pages. Record per-peer audio/video RTP deltas; use the linked MSC115-CASE-CHAT steps 4-6 for direct Tasks navigation and request counts. | MSC-122: Template: assess/test retained chat/signaling/backend paths; minimal chat call UI is absent, so call-window steps are N/A. Follow checklist template scope and defect propagation requirements.</t>
+  </si>
+  <si>
+    <t>MSC-117 https://github.com/fssrepository/myscoutee-roadmap/issues/155; guides/qa/evidence/CHAT-CALL-001-2026-10-06.json; isolated Alice admin/Bob/Carol fixture ready; browser checklist not executed by Codex | 2026-10-07 guide expansion only: 34 numbered steps; obsolete visible verification-code assertions removed; physical echo isolation and linked Tasks regression added. Earlier fixture-ready evidence is historical; revalidate after dev/demo reset. No new manual run. | 2026-10-11 MSC-122 follow-up REQUIRED: for each defect record template affected/unaffected with reason, source and template fix revisions, targeted template environment/result/evidence; affected propagation or verification stays open until completed. Source PASS does not imply template PASS. See guides/qa/checklists/README.md#template-regression-and-fix-propagation--msc-122. No execution status changed by this requirement.</t>
   </si>
   <si>
     <t>30/60</t>
@@ -3670,7 +3670,7 @@
     <t>1. Create a Work private-group invite and a Community private-group invite using the existing invite action. Open each link in a clean prepared session. | 2. Check the relevant landing mode, then register/claim. Verify membership in the invited workspace and its base group, with the correct active profile. | 3. Switch to a Dating group from a Community account: its Dating behavior remains independent. Check joining an available base group is explicit and does not require approval. Promotional cards remain a later refinement.</t>
   </si>
   <si>
-    <t>Actors: Group manager; signed-out invitee. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Group manager; signed-out invitee. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-WORK-CAMPAIGN</t>
@@ -3682,7 +3682,7 @@
     <t>1. Open Campaigns next to Groups; create a draft through + with opportunity type, category, capacity, location, relevant filters and optional image. | 2. Save, reopen, publish, edit, unpublish, trash and restore using existing FormFlow/SmartList patterns. Observe write results without a full unrelated list reload. | 3. Check Work Home InfoCard text/images and three-dot read-only Campaign/author views while the rating bar is visible. Discovery follows opportunity/category and geographic criteria; private drafts stay private. Check the shared Dating-style frame, loading, paging and full-height empty state.</t>
   </si>
   <si>
-    <t>Actors: Work member as organizer; another Work member as participant. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Work member as organizer; another Work member as participant. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-WORK-RATING</t>
@@ -3694,7 +3694,7 @@
     <t>1. Rate two campaigns of the same author. Inspect the Ratings list: it displays people, with aggregate person rating when no Campaign filter is selected. | 2. Before the time control, open the Campaign basket popup. Select one item with +, which changes to a checkmark; inspect/remove the item in the header basket and confirm with the header checkmark. Selecting another replaces the single selection; closing cancels; confirming an empty basket returns to the aggregate view. The second header line names the selected Campaign; list paging and counters use that scope. | 3. Revise one rating. Check the corresponding write and aggregate query, including the opposite participant view. An unchanged retry must not create another notification. | 4. Use an unfiltered event for aggregate sympathy selection and a Campaign-selected event for campaign-specific selection; do not create horizontal channels or fake campaign events.</t>
   </si>
   <si>
-    <t>Owned Campaign menu → Ratings; no chooser in Activities; subtitle order; 8+9=8.5 write-side AVG and scoped scores; event priorities; per-card granular snapshot; history eye and paging.</t>
+    <t>Owned Campaign menu → Ratings; no chooser in Activities; subtitle order; 8+9=8.5 write-side AVG and scoped scores; event priorities; per-card granular snapshot; history eye and paging. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-SERVICE</t>
@@ -3706,7 +3706,7 @@
     <t>1. In base Community open the service InfoCard Home. Its header has category and Ratings controls; neither Your services nor the provisional Filters/distance popup is present. Check category selection, location-based ordering, and the two three-dot actions opening the full read-only service sheet and provider profile, including while the rating bar is visible. Empty results retain the Dating-style full-height frame/message; loading and paging use the same shared SmartList behavior. | 2. Open Your services from the sidebar Community block, not Cases or Home. Create/edit/publish/draft/trash/restore a sheet; category is on its form, without a separate category selector in the owned list. Check contextual cards/menus, a single sticky date header, + on the second row below Close, and labeled desktop List/Week/Month views. Week/Month show provider appointments. Configure staff, availability and existing pricing/slot inputs. | 3. Rate the provider through a service. Multiple services from that provider use the existing person priority. Publishing a sheet alone sends no unsolicited notification. | 4. Confirm a draft, deleted/inactive provider or another person’s private image is not exposed through discovery.</t>
   </si>
   <si>
-    <t>Actors: Anna as provider; Alex as customer; another eligible staff member. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Anna as provider; Alex as customer; another eligible staff member. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-CASE</t>
@@ -3718,7 +3718,7 @@
     <t>1. Create a case from Cases +, select the private community and a case type, then All or selected affected members with the existing basket picker. | 2. Check daily descending InfoCard groups with one sticky header, type-based card/menu colors, bottom-right contextual status badge, and the black affected-count button containing the number and chevron only. Click it to open the existing read-only member popup. Inspect status/type red unread counters across all pages, the aggregate base-group Cases badge and convenient private-group entry. | 3. Open the same case as another affected member and as a manager of multiple communities. Unrelated members cannot read it. | 4. Check lifecycle-appropriate three-dot actions: Start only while open; complete/cancel while active; reopen after completion/cancellation/deletion; no duplicate delete on deleted cases. Edit/close/reopen using these supported actions. Check targeted list/counter updates and notifications to affected others; the human actor receives none.</t>
   </si>
   <si>
-    <t>Actors: Alex; Maya; external provider Anna. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Alex; Maya; external provider Anna. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-CASE-PROVIDER</t>
@@ -3730,7 +3730,7 @@
     <t>1. As a member recommend a published service/provider. In the provider picker, + toggles to a checkmark; choosing another replaces the selection. Inspect/remove through the header basket; confirm applies and closing cancels. As manager inspect the recommendation and invite the chosen provider/staff member. | 2. As provider see the shared case in aggregate Community Cases, accept/decline and submit a quotation. As manager accept/reject the quotation. | 3. Check invitation/response/offer/decision notifications and their correct case destination. Repeating a provider invitation must preserve an accepted assignment. | 4. An external provider must not gain private-group navigation or announcement access. A declined invitation retains permitted case history but removes live case-chat access.</t>
   </si>
   <si>
-    <t>Actors: Community member; manager; external provider. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Community member; manager; external provider. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-SCHEDULE</t>
@@ -3742,7 +3742,7 @@
     <t>1. From the Cases header open Scheduled tasks and create a due date with All/selected members. Check the affected count in its SingleRow. | 2. At just before due minus 45 days, the scoped job creates nothing. At the boundary it creates one shared case and reminds all affected users, including an affected task creator. | 3. Rerun the same occurrence and simulate a delivery retry through the prepared test mechanism: no second case/reminder. Recurrence advances only after enqueueing. | 4. Check month/year recurrence and short-month dates. Edit/disable the task as permitted; Asset editor has no utility scheduling fields.</t>
   </si>
   <si>
-    <t>Actors: Manager; affected residents; selected provider when applicable. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Manager; affected residents; selected provider when applicable. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-APPOINTMENT</t>
@@ -3754,7 +3754,7 @@
     <t>1. Invite and accept the case provider/service, then open the actual existing slot picker from the case. Check day/week/month availability, templates and date overrides. | 2. Book a slot. Try an overlapping slot for that worker from another case/customer: conflict is rejected. Another worker’s capacity remains independent. | 3. Cancel a future appointment and verify availability is restored; retry save/cancel without duplicate rows or notifications. | 4. Inspect the provider’s aggregate calendar, customer and case labels, pricing snapshot and case link. Changing/unpublishing a service preserves prior bookings/audit; no fake asset/event or card charge is created.</t>
   </si>
   <si>
-    <t>Actors: Accepted case provider; two customers; second staff member. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Accepted case provider; two customers; second staff member. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-VOTING</t>
@@ -3766,7 +3766,7 @@
     <t>1. Configure apartment voting rights with one accepted assigned voter and positive weight. No Asset editor change or registration block is introduced. | 2. Publish a vote and cast each authorized ballot. Verify the first-publication rights snapshot, one final ballot per unit and denial of a replacement vote. | 3. Inspect member/admin results: correct weighted totals/counts without revealing others’ individual ballots. Unassigned residents cannot cast a unit ballot. | 4. Extend the deadline to reopen the published vote while retaining prior ballots. At expiry the Community-only job closes once and notifies participants; a cast vote notifies managers except its actor.</t>
   </si>
   <si>
-    <t>Actors: Admin; two assigned voters; unassigned resident. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Admin; two assigned voters; unassigned resident. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>SERVICE-FEEDBACK-UI-001</t>
@@ -3784,10 +3784,10 @@
     <t>Focused regression source prepared; execution deferred by user.</t>
   </si>
   <si>
-    <t>Run checklists/general/SERVICE-FEEDBACK-UI-001.md with approved feedback fixture in HTTP/local modes.</t>
-  </si>
-  <si>
-    <t>MSC-116. Watcher compilation and schema generation are not behavioral QA. Existing guide/API PASS does not cover this extension.</t>
+    <t>Run checklists/general/SERVICE-FEEDBACK-UI-001.md with approved feedback fixture in HTTP/local modes. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
+  </si>
+  <si>
+    <t>MSC-116. Watcher compilation and schema generation are not behavioral QA. Existing guide/API PASS does not cover this extension. | 2026-10-11 MSC-122 follow-up REQUIRED: for each defect record template affected/unaffected with reason, source and template fix revisions, targeted template environment/result/evidence; affected propagation or verification stays open until completed. Source PASS does not imply template PASS. See guides/qa/checklists/README.md#template-regression-and-fix-propagation--msc-122. No execution status changed by this requirement.</t>
   </si>
   <si>
     <t>P1 80</t>
@@ -3874,7 +3874,7 @@
     <t>1. Open private Community Home: newest-first SingleRow announcements grouped by day replace the rating stack, with a single sticky date header. Voting replaces Ratings in the sidebar Activities block; Your services remains in the Community block. | 2. As admin create a minimal draft with text and optional PDF/text/office attachments, then publish/edit/unpublish/trash/restore through three-dot actions and buckets. | 3. Check member visibility and color/action distinction for voting vs ordinary announcements. Members cannot publish directly; Feedback opens the existing group-admin chat. | 4. Test attachment download as a current member and denied outsider/former member. Unpublished documents remain admin/owner-only; normal feedback opening sends no notification.</t>
   </si>
   <si>
-    <t>Actors: Private Community admin; accepted resident; outsider. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Private Community admin; accepted resident; outsider. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MOBILE-PUSH-LIFECYCLE-001</t>
@@ -4210,7 +4210,7 @@
     <t>1. Switch Dating → Work → Community above the avatar. The menu structure stays consistent and all opened surfaces use the selected base group. | 2. Compare the selector red count with the existing menu counters; inspect moderation, reports, feedback, chat, content/articles, parameters, stats, metrics and graph in each scope. | 3. Change a scoped content item or parameter and return to another base group: its data is unchanged. A report retains the actor/action/event and optional group context without granting private-workspace membership. | 4. Open payment test tools from each scope and inspect their existing authorization link/context. Operator remains deployment-wide.</t>
   </si>
   <si>
-    <t>Actors: Ava; a second admin profile if needed. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | Main-group landing label/icon/color after login; Groups base cards once at the entire filtered list start before pagination, never repeated per mobile page; private identity and counters retained.</t>
+    <t>Actors: Ava; a second admin profile if needed. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | Main-group landing label/icon/color after login; Groups base cards once at the entire filtered list start before pagination, never repeated per mobile page; private identity and counters retained. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>MSC115-JOBS</t>
@@ -4222,7 +4222,7 @@
     <t>1. Open Jobs in every base group. Confirm independent seeded definitions, enabled state, timing and run history. | 2. Run an available scoped job and inspect only that scope’s results, progress, counters and history. Do not enable absent/inapplicable random-room jobs in Work or Community. | 3. Inspect Community scheduled-case and vote-close jobs. Confirm shared notification/exchange/processing definitions have separate group items and that an unseeded job does not execute for that group.</t>
   </si>
   <si>
-    <t>Actors: Ava. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario.</t>
+    <t>Actors: Ava. Follow guides/qa/checklists/MSC-115_WORK_COMMUNITY_PAIR_QA.md and the numbered scenario. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>EXPLANATION-GUIDE-001</t>
@@ -4243,10 +4243,10 @@
     <t>2026-10-07: EN/HU catalog/i18n and guide-field seed parity; revision/section parity for chats, event.chat, chat.call, chat.call.volume and landing.guide across Dating/Work/Community and all three Mongo seeds. Existing watcher AOT call/guide context and intro lifecycle checks PASS. Public intro HTTP EN/HU x 3 modes PASS; private call context denial 404 PASS. Browser tour NOT RUN. Follow-up: watcher AOT launcher geometry (1500 cases, 400 Rates rechecks) and versioned introduction lifecycle/text parity PASS. See guides/qa/evidence/general/EXPLANATION-GUIDE-001-20261007.md. Consent follow-up: watcher AOT directive/service/Accept target PASS; 200 target checks reuse one index scan. Live public consent HTTP EN/HU x 3 modes PASS; private-context 404 preserved. | 2026-10-07 isolated CDP regression PASS (EN desktop / 390x844 mobile): dismissed consent stays closed on group switch; correct images on first selection; Login reopens consent; one stable consent Help step with translated label; duplicate Privacy summary removed. SW 20/20 PASS; EN/HU live seed/translation parity PASS. | Mobile header follow-up: 24 isolated CDP cases PASS (EN/HU x 320/360/390/1236px x 3 groups): full label/caret, one-line Login/Belépés, no header overlap. Translation .7 live/source/seed parity PASS. | 2026-10-07 shared missing-guide feedback: watcher-AOT DOM regression PASS for persistent centered EN/HU message, cold/cached/empty cases, X/Escape/Back/launcher/shade dismissal, Next/Back/Done and 200 viewport notifications with zero rescans.</t>
   </si>
   <si>
-    <t>Run the MSC-119 section plus retained unexecuted WebRTC/introduction/consent sections: all affected Work/Community/API/MCP and shared terms guides, EN/HU desktop/mobile local/HTTP, empty/populated and read-only/edit states; header title/X alignment; parent restoration; no business writes during guide-only navigation.</t>
-  </si>
-  <si>
-    <t>45 contexts / 963 fields. Existing recorded scope retained. Added landing: 64 steps per viewport; feedback: 39 per viewport; Rates arrow-only, shared double-panel highlights and editable badge passed at mobile/desktop. EN/HU local/demo/e2e/prod seed parity. Landing visit visibility, internal default ON/preserved OFF, fresh-browser consent and shared guide/notification clearance above rating actions/profile eyes passed mobile/desktop. Mobile-only launcher clearance; unchanged desktop positioning; pair divider hover/tap/drag and fixed photo scale at 0/50/100% passed Home/Rates browser and Android Rates over ADB. Mobile pair image fit unified to contain on Home/Activity Rates; both targeted browser checks passed, desktop preserved. Guide screenshots removed from Git. No final form submission. Full local persistence and native WebView not claimed. guides/qa/evidence/general/EXPLANATION-GUIDE-001-20260930.md Final Android Home rail stability, mobile/desktop guide card continuity and filter badge save/reload/restore passed. No screenshots committed. Earlier Android fullscreen/drag lag was confirmed; the subsequent retained-panel and image-scroll fixes below were accepted and close that follow-up. No universal performance PASS is claimed. Follow-up: one retained list row rebuilt instead of six; one DTO snapshot per card; hidden controls excluded from launcher measurement. Native menu/guide visibility and raised list badge clearance passed. Small warm RAF-proxy medians: fullscreen 293 to 254ms, list 161 to 108ms; these preliminary measurements are superseded by the final user-accepted retained-panel result below. Final user-accepted retained-panel change: one shared loaded collection; persistent list/fullscreen DOM; z-order-only presentation; inactive new-image gating; no warm card rebuilds or switch scroll shift; saved-score paging identity preserved. Warm fullscreen median207.9→127.7ms; list103→128.1ms (dev two-RAF proxy, no universal performance claim). Rates list-scroll launchers fixed: native100-frame check0/0px movement versus48/56px before. Follow-up: panel-bottom launcher anchor56px list/96px fullscreen; native scroll0/0px. Whole-card scroll preview/adaptive prefetch withdrawn. Image-only handling preserves visible photos; only offscreen/passed photos suspend, returning once from cache. Fast-scroll requests/spinners0; sampled visible-image flickers0; focused tests15/15. See phone-image-scroll.json. Mobile photo badges/eye/image indicators follow per-image suspension; individual/pair native swipe90frames each passed; user accepted. Release1.3.2: both guide branches consolidated/master merged; GHCR frontend/backend images; Netcup migration010 retained-data check;8 healthy containers; publicHTTP13/13 and landing guide10/10 plus private-context denial passed. See RELEASE_1.3.2_20260930.json. Launcher follow-up: desktop icons remain with menus; guide above shade; bell layering unchanged; mobile menus hide both icons without hiding tour;1280/390px regression passed and user accepted.; Accepted launcher follow-up republished1.3.2: nginx-only Netcup update,13/13 HTTP PASS,8 healthy containers,7 unchanged. Final ledger closure 2026-09-30: PASS / CLOSED for the accepted guide scope and follow-ups; no remaining guide oracle. Local PARTIAL records the untested persistence boundary, not an open guide defect. 2026-10-01 scoped granular-rating addendum: Home/Activity list/fullscreen CDP at1280/390; no-backdrop popup, equal-width bar, mobile menu launcher hiding, integer details, profile-count-derived main step, exact6.75 save/reload and affinity precision, EN/HU guide/i18n parity. Existing PASS/CLOSED retained; see granular-rating-checks.json and rating-step-checks.json in the linked evidence. | 2026-10-06: user explicitly reopens for expanded scope. September PASS remains historical evidence, not current completion. | 2026-10-07: Added 17 call + 7 volume catalog fields, phone steps in chats/event.chat and the one-step landing.guide intro; workspace-specific EN/HU content seeded. Existing shared guide engine/launcher reused. Watcher frontend build and backend hot-deploy PASS; check-chat-call-runtime.mjs PASS including nested guide/context/language/destruction checks. Compiled Guide first-visit/dismissal/known-visitor/transition checks PASS; consent and saved guide preference unchanged. Public intro HTTP 6/6 plus private-context denial PASS. Targeted audit-seeds.py --context chats --context event.chat --context chat.call --context chat.call.volume --context landing.guide PASS; i18n audit and sync-work-seeds.js --check PASS. Full revision audit is not a PASS: pre-existing home.game rating-details and payment.history counterparty steps are absent from global HTTP revisions; left outside this change. At that earlier checkpoint, launcher component and placeCard positioning were identical to HEAD after the positioning edits were withdrawn. No browser actions, fixture staging or full guide click-through performed. September evidence remains historical; new manual status NOT RUN. | 2026-10-07 authorized follow-up: launcher-to-launcher clearance repaired using registered references; Rates stable panel anchors and Help card placement preserved. Bounded geometry/lifecycle checks PASS; single-step HU163/EN166 introduction explains drag, red-X hide and Side menu Explanations OFF/ON. QA CSV line endings normalized. Evidence: guides/qa/evidence/general/EXPLANATION-GUIDE-001-20261007.md. Manual browser status remains NOT RUN. | 2026-10-07 consent follow-up: landing.consent one-step Accept binding; canonical source and all Mongo seeds synchronized. Introduction now explicitly names the notification bell (HU156/EN155). i18n version 2026.10.07.5. Development checks PASS; browser manual NOT RUN. | Later user-authorized fresh anonymous browser evidence: guides/qa/evidence/general/EXPLANATION-GUIDE-001-20261007.md, landing follow-up. No full manual case replay, acceptance/registration or fixture reset; historical status preserved. | Article/no-guide follow-up: shared guide feedback now remains centered until dismissed instead of flashing closed. Per-surface checklist step 9 added. Focused JSDOM evidence only; manual campaign status unchanged. guides/qa/evidence/general/EXPLANATION-GUIDE-001-20261007.md. | 2026-10-07 operator/app-admin audit: GAP, no dedicated surface registrations/catalog fields/revisions; operator launcher excluded; Explanations toggle excluded for both privileged roles. Common avatar-menu guide is not role-surface coverage. See evidence/general/EXPLANATION-GUIDE-001-20261007.md#operator--app-admin-wiring-audit. | MSC-118: prior role wiring gap implemented; 37 system contexts / 136 fields, shared launchers and role notifications have dedicated ROLE-GUIDES-NOTIFICATIONS-001 checklist/evidence. Manual role QA NOT RUN. MSC-119 extension 2026-10-07: guides/plans/MSC-119_MCP_READ_EVENTS_ROLE_GUIDANCE.md and guides/qa/evidence/general/MSC-119_GUIDE_WIRING_20261007.md. Source/build evidence only; no functional/browser/security/load PASS claimed.</t>
+    <t>Run the MSC-119 section plus retained unexecuted WebRTC/introduction/consent sections: all affected Work/Community/API/MCP and shared terms guides, EN/HU desktop/mobile local/HTTP, empty/populated and read-only/edit states; header title/X alignment; parent restoration; no business writes during guide-only navigation. | MSC-122: Template: test the retained API/MCP or guide/notification counterpart using its own catalog, actors and seeds. Follow checklist template scope and defect propagation requirements.</t>
+  </si>
+  <si>
+    <t>45 contexts / 963 fields. Existing recorded scope retained. Added landing: 64 steps per viewport; feedback: 39 per viewport; Rates arrow-only, shared double-panel highlights and editable badge passed at mobile/desktop. EN/HU local/demo/e2e/prod seed parity. Landing visit visibility, internal default ON/preserved OFF, fresh-browser consent and shared guide/notification clearance above rating actions/profile eyes passed mobile/desktop. Mobile-only launcher clearance; unchanged desktop positioning; pair divider hover/tap/drag and fixed photo scale at 0/50/100% passed Home/Rates browser and Android Rates over ADB. Mobile pair image fit unified to contain on Home/Activity Rates; both targeted browser checks passed, desktop preserved. Guide screenshots removed from Git. No final form submission. Full local persistence and native WebView not claimed. guides/qa/evidence/general/EXPLANATION-GUIDE-001-20260930.md Final Android Home rail stability, mobile/desktop guide card continuity and filter badge save/reload/restore passed. No screenshots committed. Earlier Android fullscreen/drag lag was confirmed; the subsequent retained-panel and image-scroll fixes below were accepted and close that follow-up. No universal performance PASS is claimed. Follow-up: one retained list row rebuilt instead of six; one DTO snapshot per card; hidden controls excluded from launcher measurement. Native menu/guide visibility and raised list badge clearance passed. Small warm RAF-proxy medians: fullscreen 293 to 254ms, list 161 to 108ms; these preliminary measurements are superseded by the final user-accepted retained-panel result below. Final user-accepted retained-panel change: one shared loaded collection; persistent list/fullscreen DOM; z-order-only presentation; inactive new-image gating; no warm card rebuilds or switch scroll shift; saved-score paging identity preserved. Warm fullscreen median207.9→127.7ms; list103→128.1ms (dev two-RAF proxy, no universal performance claim). Rates list-scroll launchers fixed: native100-frame check0/0px movement versus48/56px before. Follow-up: panel-bottom launcher anchor56px list/96px fullscreen; native scroll0/0px. Whole-card scroll preview/adaptive prefetch withdrawn. Image-only handling preserves visible photos; only offscreen/passed photos suspend, returning once from cache. Fast-scroll requests/spinners0; sampled visible-image flickers0; focused tests15/15. See phone-image-scroll.json. Mobile photo badges/eye/image indicators follow per-image suspension; individual/pair native swipe90frames each passed; user accepted. Release1.3.2: both guide branches consolidated/master merged; GHCR frontend/backend images; Netcup migration010 retained-data check;8 healthy containers; publicHTTP13/13 and landing guide10/10 plus private-context denial passed. See RELEASE_1.3.2_20260930.json. Launcher follow-up: desktop icons remain with menus; guide above shade; bell layering unchanged; mobile menus hide both icons without hiding tour;1280/390px regression passed and user accepted.; Accepted launcher follow-up republished1.3.2: nginx-only Netcup update,13/13 HTTP PASS,8 healthy containers,7 unchanged. Final ledger closure 2026-09-30: PASS / CLOSED for the accepted guide scope and follow-ups; no remaining guide oracle. Local PARTIAL records the untested persistence boundary, not an open guide defect. 2026-10-01 scoped granular-rating addendum: Home/Activity list/fullscreen CDP at1280/390; no-backdrop popup, equal-width bar, mobile menu launcher hiding, integer details, profile-count-derived main step, exact6.75 save/reload and affinity precision, EN/HU guide/i18n parity. Existing PASS/CLOSED retained; see granular-rating-checks.json and rating-step-checks.json in the linked evidence. | 2026-10-06: user explicitly reopens for expanded scope. September PASS remains historical evidence, not current completion. | 2026-10-07: Added 17 call + 7 volume catalog fields, phone steps in chats/event.chat and the one-step landing.guide intro; workspace-specific EN/HU content seeded. Existing shared guide engine/launcher reused. Watcher frontend build and backend hot-deploy PASS; check-chat-call-runtime.mjs PASS including nested guide/context/language/destruction checks. Compiled Guide first-visit/dismissal/known-visitor/transition checks PASS; consent and saved guide preference unchanged. Public intro HTTP 6/6 plus private-context denial PASS. Targeted audit-seeds.py --context chats --context event.chat --context chat.call --context chat.call.volume --context landing.guide PASS; i18n audit and sync-work-seeds.js --check PASS. Full revision audit is not a PASS: pre-existing home.game rating-details and payment.history counterparty steps are absent from global HTTP revisions; left outside this change. At that earlier checkpoint, launcher component and placeCard positioning were identical to HEAD after the positioning edits were withdrawn. No browser actions, fixture staging or full guide click-through performed. September evidence remains historical; new manual status NOT RUN. | 2026-10-07 authorized follow-up: launcher-to-launcher clearance repaired using registered references; Rates stable panel anchors and Help card placement preserved. Bounded geometry/lifecycle checks PASS; single-step HU163/EN166 introduction explains drag, red-X hide and Side menu Explanations OFF/ON. QA CSV line endings normalized. Evidence: guides/qa/evidence/general/EXPLANATION-GUIDE-001-20261007.md. Manual browser status remains NOT RUN. | 2026-10-07 consent follow-up: landing.consent one-step Accept binding; canonical source and all Mongo seeds synchronized. Introduction now explicitly names the notification bell (HU156/EN155). i18n version 2026.10.07.5. Development checks PASS; browser manual NOT RUN. | Later user-authorized fresh anonymous browser evidence: guides/qa/evidence/general/EXPLANATION-GUIDE-001-20261007.md, landing follow-up. No full manual case replay, acceptance/registration or fixture reset; historical status preserved. | Article/no-guide follow-up: shared guide feedback now remains centered until dismissed instead of flashing closed. Per-surface checklist step 9 added. Focused JSDOM evidence only; manual campaign status unchanged. guides/qa/evidence/general/EXPLANATION-GUIDE-001-20261007.md. | 2026-10-07 operator/app-admin audit: GAP, no dedicated surface registrations/catalog fields/revisions; operator launcher excluded; Explanations toggle excluded for both privileged roles. Common avatar-menu guide is not role-surface coverage. See evidence/general/EXPLANATION-GUIDE-001-20261007.md#operator--app-admin-wiring-audit. | MSC-118: prior role wiring gap implemented; 37 system contexts / 136 fields, shared launchers and role notifications have dedicated ROLE-GUIDES-NOTIFICATIONS-001 checklist/evidence. Manual role QA NOT RUN. MSC-119 extension 2026-10-07: guides/plans/MSC-119_MCP_READ_EVENTS_ROLE_GUIDANCE.md and guides/qa/evidence/general/MSC-119_GUIDE_WIRING_20261007.md. Source/build evidence only; no functional/browser/security/load PASS claimed. | 2026-10-11 MSC-122 follow-up REQUIRED: for each defect record template affected/unaffected with reason, source and template fix revisions, targeted template environment/result/evidence; affected propagation or verification stays open until completed. Source PASS does not imply template PASS. See guides/qa/checklists/README.md#template-regression-and-fix-propagation--msc-122. No execution status changed by this requirement.</t>
   </si>
   <si>
     <t>MSC115-GUIDES</t>
@@ -4258,7 +4258,7 @@
     <t>1. Open the guide at landing/Home mode switch, Campaign list/editor, service Home/list/editor/calendar, Cases/tasks/editors/appointments, private Home/Voting/rights and payment history/receipt. | 2. Check the explanation targets the visible control and describes the current group’s behavior in English and Hungarian. Lazy-opened popups get their own registered context. | 3. Switch modes while popups/requests are active. Check stale responses and selections do not populate another profile, no duplicate HTTP clients are used and badges clear according to existing read actions.</t>
   </si>
   <si>
-    <t>Expanded EXPLANATION-GUIDE-001 shared execution; 28 revised contexts, all new controls and EN/HU, preserve historical PASS evidence.</t>
+    <t>Expanded EXPLANATION-GUIDE-001 shared execution; 28 revised contexts, all new controls and EN/HU, preserve historical PASS evidence. | MSC-122: Template: assess/test affected shared functionality; omitted Work/Community product workflows are N/A with a reason. Follow checklist template scope and defect propagation requirements.</t>
   </si>
   <si>
     <t>OPERATOR-CONFIGURATION-LIFECYCLE-001</t>

</xml_diff>